<commit_message>
V5 daily refresh 2026-06-18
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -548,7 +548,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Mon 15 Jun 2026</t>
+          <t>As of Thu 18 Jun 2026</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹198,898</t>
+          <t>₹200,302</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-1,102  (-0.55%)</t>
+          <t>₹+1,404  (+0.71%)</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-0.55%</t>
+          <t>+0.15%</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.55%</t>
+          <t>+0.00%</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹61,251</t>
+          <t>₹62,655</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
@@ -795,31 +795,31 @@
         <v>4230</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>1374.7</v>
+        <v>1400.4</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>4124.1</v>
+        <v>4201.200000000001</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>-105.8999999999999</v>
+        <v>-28.79999999999973</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>-0.02503546099290777</v>
+        <v>-0.006808510638297808</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>1312.63</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1312.63</v>
+        <v>1368.1</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.0451516694551538</v>
+        <v>0.02306483861753798</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>33.1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -843,31 +843,31 @@
         <v>5209.05</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>243.65</v>
+        <v>245.3</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>5116.650000000001</v>
+        <v>5151.3</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-92.40000000000012</v>
+        <v>-57.75</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.01773835920177386</v>
+        <v>-0.01108647450110865</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>230.7</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>230.7</v>
+        <v>242.8</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.05315001026061981</v>
+        <v>0.01019160211985324</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>7.74</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -891,31 +891,31 @@
         <v>5196</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1013.9</v>
+        <v>1008.5</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>5069.5</v>
+        <v>5042.5</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-126.5000000000003</v>
+        <v>-153.5000000000002</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.02434565050038498</v>
+        <v>-0.02954195535026948</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>954.83</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>954.83</v>
+        <v>970</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.05826018345004432</v>
+        <v>0.03817550818046604</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>33.76</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -939,16 +939,16 @@
         <v>4788</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>773.45</v>
+        <v>798.1</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>4640.700000000001</v>
+        <v>4788.6</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>-147.2999999999997</v>
+        <v>0.6000000000001364</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>-0.03076441102756887</v>
+        <v>0.0001253132832080485</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>746.09</v>
@@ -957,13 +957,13 @@
         <v>746.09</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.03537397375395955</v>
+        <v>0.06516727227164515</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>22.5</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -987,16 +987,16 @@
         <v>4830</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>668.9</v>
+        <v>690.3</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4682.3</v>
+        <v>4832.099999999999</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>-147.7000000000002</v>
+        <v>2.099999999999682</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-0.03057971014492757</v>
+        <v>0.0004347826086955863</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>612.1900000000001</v>
@@ -1005,13 +1005,13 @@
         <v>612.1900000000001</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.08478098370458952</v>
+        <v>0.1131537012892944</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>34.34</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -1035,31 +1035,31 @@
         <v>3678</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1804.8</v>
+        <v>1842.1</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>3609.6</v>
+        <v>3684.2</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-68.40000000000009</v>
+        <v>6.199999999999818</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.01859706362153347</v>
+        <v>0.001685698749320233</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1729.61</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1729.61</v>
+        <v>1744.3</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.04166112588652485</v>
+        <v>0.05309158026165787</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>43.14</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -1083,31 +1083,31 @@
         <v>5198.96</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>197.28</v>
+        <v>200.52</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5129.28</v>
+        <v>5213.52</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>-69.68000000000018</v>
+        <v>14.56000000000006</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>-0.01340268053610725</v>
+        <v>0.002800560112022416</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>187.26</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>187.26</v>
+        <v>193.31</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.05079075425790759</v>
+        <v>0.03595651306602837</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>5.48</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -1131,16 +1131,16 @@
         <v>4242</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1389.1</v>
+        <v>1368.8</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4167.299999999999</v>
+        <v>4106.4</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>-74.70000000000027</v>
+        <v>-135.6000000000001</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>-0.01760961810466767</v>
+        <v>-0.031966053748232</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1324.47</v>
@@ -1149,13 +1149,13 @@
         <v>1324.47</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.04652652796774882</v>
+        <v>0.03238603156049089</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>35.79</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1179,31 +1179,31 @@
         <v>5200</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1283.2</v>
+        <v>1305.6</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>5132.8</v>
+        <v>5222.4</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>-67.19999999999982</v>
+        <v>22.39999999999964</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>-0.01292307692307689</v>
+        <v>0.004307692307692238</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1159.03</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1159.03</v>
+        <v>1212</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.09676589775561102</v>
+        <v>0.07169117647058817</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>64.73</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1227,31 +1227,31 @@
         <v>5209</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>266.05</v>
+        <v>277.1</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5321</v>
+        <v>5542</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>112.0000000000005</v>
+        <v>333.0000000000007</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.02150124784027653</v>
+        <v>0.06392781723939349</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>240.49</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>240.49</v>
+        <v>252.1357142857143</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.09607216688592371</v>
+        <v>0.09009125122441616</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>8.369999999999999</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -1275,31 +1275,31 @@
         <v>5252.55</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>272.8</v>
+        <v>298.1</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>5183.2</v>
+        <v>5663.900000000001</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-69.34999999999957</v>
+        <v>411.3500000000006</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.01320311086995832</v>
+        <v>0.07831434255742462</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>259.14</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>259.14</v>
+        <v>272.8785714285714</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.05007331378299129</v>
+        <v>0.08460727464417507</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>7.11</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1323,16 +1323,16 @@
         <v>4932</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>969.85</v>
+        <v>975.1</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>4849.25</v>
+        <v>4875.5</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-82.74999999999977</v>
+        <v>-56.49999999999977</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.01677818329278179</v>
+        <v>-0.01145579886455794</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>934.1900000000001</v>
@@ -1341,13 +1341,13 @@
         <v>934.1900000000001</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.03676857245965868</v>
+        <v>0.04195467131576245</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>25.59</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1371,16 +1371,16 @@
         <v>4387.5</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1408.3</v>
+        <v>1443.7</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4224.9</v>
+        <v>4331.1</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>-162.6000000000001</v>
+        <v>-56.39999999999986</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>-0.03705982905982909</v>
+        <v>-0.01285470085470082</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1405.17</v>
@@ -1389,13 +1389,13 @@
         <v>1405.17</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.002222537811545752</v>
+        <v>0.02668837016000552</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>38.34</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1495,7 +1495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1616,6 +1616,31 @@
         <v>0</v>
       </c>
       <c r="G4" s="15" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="n">
+        <v>200301.66</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>137646.94</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>62654.72</v>
+      </c>
+      <c r="E5" s="16" t="n">
+        <v>62353.06</v>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="15" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1699,18 +1724,18 @@
     </row>
     <row r="2">
       <c r="A2" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>1408.3</v>
+        <v>1368.8</v>
       </c>
       <c r="D2" s="15" t="n">
-        <v>1331.63</v>
+        <v>1292.57</v>
       </c>
       <c r="E2" s="15" t="n">
         <v>0.0467</v>
@@ -1719,10 +1744,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="15" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="H2" s="15" t="n">
-        <v>0.8425516224188792</v>
+        <v>0.8054424778761062</v>
       </c>
       <c r="I2" s="15" t="inlineStr">
         <is>
@@ -1737,18 +1762,18 @@
     </row>
     <row r="3">
       <c r="A3" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>1374.7</v>
+        <v>798.1</v>
       </c>
       <c r="D3" s="15" t="n">
-        <v>1308.5</v>
+        <v>753.55</v>
       </c>
       <c r="E3" s="15" t="n">
         <v>0.0467</v>
@@ -1757,10 +1782,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="15" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H3" s="15" t="n">
-        <v>0.7762733529990167</v>
+        <v>0.802551622418879</v>
       </c>
       <c r="I3" s="15" t="inlineStr">
         <is>
@@ -1775,18 +1800,18 @@
     </row>
     <row r="4">
       <c r="A4" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>243.65</v>
+        <v>782.1</v>
       </c>
       <c r="D4" s="15" t="n">
-        <v>228.17</v>
+        <v>734.78</v>
       </c>
       <c r="E4" s="15" t="n">
         <v>0.0467</v>
@@ -1795,10 +1820,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="15" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H4" s="15" t="n">
-        <v>0.7580039331366765</v>
+        <v>0.8003638151425762</v>
       </c>
       <c r="I4" s="15" t="inlineStr">
         <is>
@@ -1813,7 +1838,7 @@
     </row>
     <row r="5">
       <c r="A5" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
@@ -1821,10 +1846,10 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>809.65</v>
+        <v>820.75</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>775.54</v>
+        <v>786.95</v>
       </c>
       <c r="E5" s="15" t="n">
         <v>0.0467</v>
@@ -1833,10 +1858,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="15" t="n">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>0.7647492625368731</v>
+        <v>0.7968289085545723</v>
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
@@ -1851,18 +1876,18 @@
     </row>
     <row r="6">
       <c r="A6" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>2739.3</v>
+        <v>2406</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>2604.9</v>
+        <v>2291.79</v>
       </c>
       <c r="E6" s="15" t="n">
         <v>0.0467</v>
@@ -1871,10 +1896,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="15" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>0.7248721730580139</v>
+        <v>0.7840511307767944</v>
       </c>
       <c r="I6" s="15" t="inlineStr">
         <is>
@@ -1889,18 +1914,18 @@
     </row>
     <row r="7">
       <c r="A7" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>1013.9</v>
+        <v>975.1</v>
       </c>
       <c r="D7" s="15" t="n">
-        <v>946.39</v>
+        <v>925.24</v>
       </c>
       <c r="E7" s="15" t="n">
         <v>0.0467</v>
@@ -1909,10 +1934,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="15" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>0.7321828908554572</v>
+        <v>0.7760373647984268</v>
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
@@ -1927,18 +1952,18 @@
     </row>
     <row r="8">
       <c r="A8" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>ADANIPOWER</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>9943</v>
+        <v>230.57</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>9474.43</v>
+        <v>214.59</v>
       </c>
       <c r="E8" s="15" t="n">
         <v>0.0467</v>
@@ -1947,10 +1972,10 @@
         <v>9333</v>
       </c>
       <c r="G8" s="15" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>0.7432841691248772</v>
+        <v>0.7362684365781711</v>
       </c>
       <c r="I8" s="15" t="inlineStr">
         <is>
@@ -1965,18 +1990,18 @@
     </row>
     <row r="9">
       <c r="A9" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>197.28</v>
+        <v>6767</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>186.32</v>
+        <v>6472.43</v>
       </c>
       <c r="E9" s="15" t="n">
         <v>0.0467</v>
@@ -1985,10 +2010,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="15" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>0.7184857423795478</v>
+        <v>0.7464798426745329</v>
       </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
@@ -2003,18 +2028,18 @@
     </row>
     <row r="10">
       <c r="A10" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1389.1</v>
+        <v>9952.5</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>1317.51</v>
+        <v>9524.5</v>
       </c>
       <c r="E10" s="15" t="n">
         <v>0.0467</v>
@@ -2023,10 +2048,10 @@
         <v>9333</v>
       </c>
       <c r="G10" s="15" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>0.7370648967551623</v>
+        <v>0.7505309734513274</v>
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
@@ -2041,18 +2066,18 @@
     </row>
     <row r="11">
       <c r="A11" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>748.5</v>
+        <v>6500</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>694.35</v>
+        <v>6177.36</v>
       </c>
       <c r="E11" s="15" t="n">
         <v>0.0467</v>
@@ -2064,7 +2089,7 @@
         <v>6.4</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>0.7532300884955753</v>
+        <v>0.7924680432645035</v>
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
@@ -2079,18 +2104,18 @@
     </row>
     <row r="12">
       <c r="A12" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>SOLARINDS</t>
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>6569</v>
+        <v>17764</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>6226.71</v>
+        <v>16684</v>
       </c>
       <c r="E12" s="15" t="n">
         <v>0.0467</v>
@@ -2099,10 +2124,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>0.7686135693215339</v>
+        <v>0.7455309734513275</v>
       </c>
       <c r="I12" s="15" t="inlineStr">
         <is>
@@ -2117,18 +2142,18 @@
     </row>
     <row r="13">
       <c r="A13" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>1418.6</v>
+        <v>1443.7</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>1343.7</v>
+        <v>1373.27</v>
       </c>
       <c r="E13" s="15" t="n">
         <v>0.0467</v>
@@ -2137,10 +2162,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>0.7478613569321534</v>
+        <v>0.744346116027532</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -2155,18 +2180,18 @@
     </row>
     <row r="14">
       <c r="A14" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>OBEROIRLTY</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>1669.4</v>
+        <v>1258.2</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>1575.09</v>
+        <v>1184.36</v>
       </c>
       <c r="E14" s="15" t="n">
         <v>0.0467</v>
@@ -2175,10 +2200,10 @@
         <v>9333</v>
       </c>
       <c r="G14" s="15" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>0.7118190757128809</v>
+        <v>0.7571238938053098</v>
       </c>
       <c r="I14" s="15" t="inlineStr">
         <is>
@@ -2193,18 +2218,18 @@
     </row>
     <row r="15">
       <c r="A15" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>GPIL</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>773.45</v>
+        <v>270.55</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>728.45</v>
+        <v>255.64</v>
       </c>
       <c r="E15" s="15" t="n">
         <v>0.0467</v>
@@ -2213,10 +2238,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>6.1</v>
+        <v>6.3</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>0.7307423795476892</v>
+        <v>0.7379400196656835</v>
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
@@ -2231,18 +2256,18 @@
     </row>
     <row r="16">
       <c r="A16" s="15" t="n">
-        <v>20260615</v>
+        <v>20260618</v>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>AJANTPHARM</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>3054.4</v>
+        <v>958.75</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>2825.71</v>
+        <v>907.36</v>
       </c>
       <c r="E16" s="15" t="n">
         <v>0.0467</v>
@@ -2251,10 +2276,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="15" t="n">
-        <v>6.1</v>
+        <v>6.3</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>0.7121484759095379</v>
+        <v>0.7317600786627336</v>
       </c>
       <c r="I16" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-06-19
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -548,7 +548,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Thu 18 Jun 2026</t>
+          <t>As of Fri 19 Jun 2026</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹200,302</t>
+          <t>₹200,689</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+1,404  (+0.71%)</t>
+          <t>₹+387  (+0.19%)</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+0.15%</t>
+          <t>+0.34%</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹62,655</t>
+          <t>₹63,042</t>
         </is>
       </c>
     </row>
@@ -795,16 +795,16 @@
         <v>4230</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>1400.4</v>
+        <v>1414.8</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>4201.200000000001</v>
+        <v>4244.4</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>-28.79999999999973</v>
+        <v>14.39999999999986</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>-0.006808510638297808</v>
+        <v>0.003404255319148904</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>1312.63</v>
@@ -813,13 +813,13 @@
         <v>1368.1</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.02306483861753798</v>
+        <v>0.03300819903873342</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>33.1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -843,16 +843,16 @@
         <v>5209.05</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>245.3</v>
+        <v>246.25</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>5151.3</v>
+        <v>5171.25</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-57.75</v>
+        <v>-37.80000000000024</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.01108647450110865</v>
+        <v>-0.007256601491634797</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>230.7</v>
@@ -861,13 +861,13 @@
         <v>242.8</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.01019160211985324</v>
+        <v>0.01401015228426391</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>7.74</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -891,16 +891,16 @@
         <v>5196</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1008.5</v>
+        <v>1010</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>5042.5</v>
+        <v>5050</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-153.5000000000002</v>
+        <v>-146.0000000000002</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.02954195535026948</v>
+        <v>-0.02809853733641267</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>954.83</v>
@@ -909,13 +909,13 @@
         <v>970</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.03817550818046604</v>
+        <v>0.0396039603960396</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>33.76</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -939,16 +939,16 @@
         <v>4788</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>798.1</v>
+        <v>791.05</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>4788.6</v>
+        <v>4746.299999999999</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>0.6000000000001364</v>
+        <v>-41.70000000000027</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.0001253132832080485</v>
+        <v>-0.008709273182957451</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>746.09</v>
@@ -957,13 +957,13 @@
         <v>746.09</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.06516727227164515</v>
+        <v>0.05683585108400218</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>22.5</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -987,16 +987,16 @@
         <v>4830</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>690.3</v>
+        <v>671.05</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4832.099999999999</v>
+        <v>4697.349999999999</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>2.099999999999682</v>
+        <v>-132.6500000000003</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.0004347826086955863</v>
+        <v>-0.0274637681159421</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>612.1900000000001</v>
@@ -1005,13 +1005,13 @@
         <v>612.1900000000001</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.1131537012892944</v>
+        <v>0.0877132851501377</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>34.34</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -1035,16 +1035,16 @@
         <v>3678</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1842.1</v>
+        <v>1835.3</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>3684.2</v>
+        <v>3670.6</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>6.199999999999818</v>
+        <v>-7.400000000000091</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.001685698749320233</v>
+        <v>-0.002011963023382298</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1729.61</v>
@@ -1053,13 +1053,13 @@
         <v>1744.3</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.05309158026165787</v>
+        <v>0.04958317441290253</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>43.14</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -1083,16 +1083,16 @@
         <v>5198.96</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>200.52</v>
+        <v>198.96</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5213.52</v>
+        <v>5172.96</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>14.56000000000006</v>
+        <v>-26</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.002800560112022416</v>
+        <v>-0.005001000200040008</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>187.26</v>
@@ -1101,13 +1101,13 @@
         <v>193.31</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.03595651306602837</v>
+        <v>0.02839766787293931</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>5.48</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -1131,16 +1131,16 @@
         <v>4242</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1368.8</v>
+        <v>1412.9</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4106.4</v>
+        <v>4238.700000000001</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>-135.6000000000001</v>
+        <v>-3.299999999999727</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>-0.031966053748232</v>
+        <v>-0.0007779349363507136</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1324.47</v>
@@ -1149,13 +1149,13 @@
         <v>1324.47</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.03238603156049089</v>
+        <v>0.06258758581640601</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>35.79</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -1179,16 +1179,16 @@
         <v>5200</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1305.6</v>
+        <v>1364.2</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>5222.4</v>
+        <v>5456.8</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>22.39999999999964</v>
+        <v>256.8000000000002</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.004307692307692238</v>
+        <v>0.04938461538461542</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1159.03</v>
@@ -1197,13 +1197,13 @@
         <v>1212</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.07169117647058817</v>
+        <v>0.1115672188828618</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>64.73</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1227,31 +1227,31 @@
         <v>5209</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>277.1</v>
+        <v>275.25</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5542</v>
+        <v>5505</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>333.0000000000007</v>
+        <v>296.0000000000002</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.06392781723939349</v>
+        <v>0.05682472643501636</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>240.49</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>252.1357142857143</v>
+        <v>253.5392857142858</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.09009125122441616</v>
+        <v>0.0788763461787983</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>8.369999999999999</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -1275,31 +1275,31 @@
         <v>5252.55</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>298.1</v>
+        <v>302.3</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>5663.900000000001</v>
+        <v>5743.7</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>411.3500000000006</v>
+        <v>491.1500000000004</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.07831434255742462</v>
+        <v>0.09350696328449999</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>259.14</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>272.8785714285714</v>
+        <v>277.7535714285714</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.08460727464417507</v>
+        <v>0.08119890364349512</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>7.11</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -1323,16 +1323,16 @@
         <v>4932</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>975.1</v>
+        <v>970.3</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>4875.5</v>
+        <v>4851.5</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-56.49999999999977</v>
+        <v>-80.50000000000011</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.01145579886455794</v>
+        <v>-0.01632197891321981</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>934.1900000000001</v>
@@ -1341,13 +1341,13 @@
         <v>934.1900000000001</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.04195467131576245</v>
+        <v>0.03721529423889509</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>25.59</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1371,16 +1371,16 @@
         <v>4387.5</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1443.7</v>
+        <v>1497.8</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4331.1</v>
+        <v>4493.4</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>-56.39999999999986</v>
+        <v>105.8999999999999</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>-0.01285470085470082</v>
+        <v>0.02413675213675211</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1405.17</v>
@@ -1389,13 +1389,13 @@
         <v>1405.17</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.02668837016000552</v>
+        <v>0.06184403792228594</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>38.34</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1495,7 +1495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1641,6 +1641,31 @@
         <v>0</v>
       </c>
       <c r="G5" s="15" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>200688.9</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>137646.94</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>63041.96</v>
+      </c>
+      <c r="E6" s="16" t="n">
+        <v>62353.06</v>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="15" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1724,18 +1749,18 @@
     </row>
     <row r="2">
       <c r="A2" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>1368.8</v>
+        <v>1497.8</v>
       </c>
       <c r="D2" s="15" t="n">
-        <v>1292.57</v>
+        <v>1423.01</v>
       </c>
       <c r="E2" s="15" t="n">
         <v>0.0467</v>
@@ -1744,10 +1769,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="15" t="n">
-        <v>6.8</v>
+        <v>7</v>
       </c>
       <c r="H2" s="15" t="n">
-        <v>0.8054424778761062</v>
+        <v>0.8359390363815142</v>
       </c>
       <c r="I2" s="15" t="inlineStr">
         <is>
@@ -1762,18 +1787,18 @@
     </row>
     <row r="3">
       <c r="A3" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>798.1</v>
+        <v>1835.3</v>
       </c>
       <c r="D3" s="15" t="n">
-        <v>753.55</v>
+        <v>1755.01</v>
       </c>
       <c r="E3" s="15" t="n">
         <v>0.0467</v>
@@ -1782,10 +1807,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="15" t="n">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="H3" s="15" t="n">
-        <v>0.802551622418879</v>
+        <v>0.8156833824975418</v>
       </c>
       <c r="I3" s="15" t="inlineStr">
         <is>
@@ -1800,18 +1825,18 @@
     </row>
     <row r="4">
       <c r="A4" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>SOLARINDS</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>782.1</v>
+        <v>18052</v>
       </c>
       <c r="D4" s="15" t="n">
-        <v>734.78</v>
+        <v>16921.86</v>
       </c>
       <c r="E4" s="15" t="n">
         <v>0.0467</v>
@@ -1820,10 +1845,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="15" t="n">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
       <c r="H4" s="15" t="n">
-        <v>0.8003638151425762</v>
+        <v>0.8189970501474927</v>
       </c>
       <c r="I4" s="15" t="inlineStr">
         <is>
@@ -1838,18 +1863,18 @@
     </row>
     <row r="5">
       <c r="A5" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>820.75</v>
+        <v>1412.9</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>786.95</v>
+        <v>1333.81</v>
       </c>
       <c r="E5" s="15" t="n">
         <v>0.0467</v>
@@ -1858,10 +1883,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="15" t="n">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>0.7968289085545723</v>
+        <v>0.8182743362831859</v>
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
@@ -1876,18 +1901,18 @@
     </row>
     <row r="6">
       <c r="A6" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>2406</v>
+        <v>10066</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>2291.79</v>
+        <v>9694.139999999999</v>
       </c>
       <c r="E6" s="15" t="n">
         <v>0.0467</v>
@@ -1896,10 +1921,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="15" t="n">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>0.7840511307767944</v>
+        <v>0.8103785644051131</v>
       </c>
       <c r="I6" s="15" t="inlineStr">
         <is>
@@ -1914,18 +1939,18 @@
     </row>
     <row r="7">
       <c r="A7" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>975.1</v>
+        <v>10083</v>
       </c>
       <c r="D7" s="15" t="n">
-        <v>925.24</v>
+        <v>9644.57</v>
       </c>
       <c r="E7" s="15" t="n">
         <v>0.0467</v>
@@ -1934,10 +1959,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="15" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>0.7760373647984268</v>
+        <v>0.7759537856440512</v>
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
@@ -1952,18 +1977,18 @@
     </row>
     <row r="8">
       <c r="A8" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>ADANIPOWER</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>230.57</v>
+        <v>791.05</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>214.59</v>
+        <v>745.22</v>
       </c>
       <c r="E8" s="15" t="n">
         <v>0.0467</v>
@@ -1975,7 +2000,7 @@
         <v>6.6</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>0.7362684365781711</v>
+        <v>0.7894641101278269</v>
       </c>
       <c r="I8" s="15" t="inlineStr">
         <is>
@@ -1990,18 +2015,18 @@
     </row>
     <row r="9">
       <c r="A9" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>6767</v>
+        <v>786.9</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>6472.43</v>
+        <v>739.3099999999999</v>
       </c>
       <c r="E9" s="15" t="n">
         <v>0.0467</v>
@@ -2010,10 +2035,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="15" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>0.7464798426745329</v>
+        <v>0.7837512291052113</v>
       </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
@@ -2028,18 +2053,18 @@
     </row>
     <row r="10">
       <c r="A10" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>9952.5</v>
+        <v>1414.8</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>9524.5</v>
+        <v>1350.6</v>
       </c>
       <c r="E10" s="15" t="n">
         <v>0.0467</v>
@@ -2048,10 +2073,10 @@
         <v>9333</v>
       </c>
       <c r="G10" s="15" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>0.7505309734513274</v>
+        <v>0.7366420845624385</v>
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
@@ -2066,18 +2091,18 @@
     </row>
     <row r="11">
       <c r="A11" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>6500</v>
+        <v>3769.2</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>6177.36</v>
+        <v>3604.1</v>
       </c>
       <c r="E11" s="15" t="n">
         <v>0.0467</v>
@@ -2089,7 +2114,7 @@
         <v>6.4</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>0.7924680432645035</v>
+        <v>0.7299655850540807</v>
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
@@ -2104,18 +2129,18 @@
     </row>
     <row r="12">
       <c r="A12" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>17764</v>
+        <v>6482</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>16684</v>
+        <v>6181.43</v>
       </c>
       <c r="E12" s="15" t="n">
         <v>0.0467</v>
@@ -2124,10 +2149,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>0.7455309734513275</v>
+        <v>0.771676499508358</v>
       </c>
       <c r="I12" s="15" t="inlineStr">
         <is>
@@ -2142,18 +2167,18 @@
     </row>
     <row r="13">
       <c r="A13" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>1443.7</v>
+        <v>817.05</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>1373.27</v>
+        <v>783.09</v>
       </c>
       <c r="E13" s="15" t="n">
         <v>0.0467</v>
@@ -2162,10 +2187,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>0.744346116027532</v>
+        <v>0.7224926253687315</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -2180,18 +2205,18 @@
     </row>
     <row r="14">
       <c r="A14" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>1258.2</v>
+        <v>2414.2</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>1184.36</v>
+        <v>2309.03</v>
       </c>
       <c r="E14" s="15" t="n">
         <v>0.0467</v>
@@ -2203,7 +2228,7 @@
         <v>6.3</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>0.7571238938053098</v>
+        <v>0.7364405113077679</v>
       </c>
       <c r="I14" s="15" t="inlineStr">
         <is>
@@ -2218,18 +2243,18 @@
     </row>
     <row r="15">
       <c r="A15" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>GPIL</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>270.55</v>
+        <v>1470.8</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>255.64</v>
+        <v>1394.19</v>
       </c>
       <c r="E15" s="15" t="n">
         <v>0.0467</v>
@@ -2238,10 +2263,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>0.7379400196656835</v>
+        <v>0.7489429695181908</v>
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
@@ -2256,18 +2281,18 @@
     </row>
     <row r="16">
       <c r="A16" s="15" t="n">
-        <v>20260618</v>
+        <v>20260619</v>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>958.75</v>
+        <v>1364.2</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>907.36</v>
+        <v>1236.5</v>
       </c>
       <c r="E16" s="15" t="n">
         <v>0.0467</v>
@@ -2276,10 +2301,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="15" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>0.7317600786627336</v>
+        <v>0.7264110127826942</v>
       </c>
       <c r="I16" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-06-22
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -548,7 +548,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Fri 19 Jun 2026</t>
+          <t>As of Mon 22 Jun 2026</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹200,689</t>
+          <t>₹200,293</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+387  (+0.19%)</t>
+          <t>₹-396  (-0.20%)</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+0.34%</t>
+          <t>+0.15%</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>+0.00%</t>
+          <t>-0.20%</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹137,647</t>
+          <t>₹89,757</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹62,353</t>
+          <t>₹110,243</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹63,042</t>
+          <t>₹110,536</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>19</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -795,31 +795,31 @@
         <v>4230</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>1414.8</v>
+        <v>1401.9</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>4244.4</v>
+        <v>4205.700000000001</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>14.39999999999986</v>
+        <v>-24.29999999999973</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.003404255319148904</v>
+        <v>-0.005744680851063765</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>1312.63</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1368.1</v>
+        <v>1370.6</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.03300819903873342</v>
+        <v>0.02232684214280632</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>33.1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -843,16 +843,16 @@
         <v>5209.05</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>246.25</v>
+        <v>245.45</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>5171.25</v>
+        <v>5154.45</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-37.80000000000024</v>
+        <v>-54.60000000000048</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.007256601491634797</v>
+        <v>-0.01048175771013918</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>230.7</v>
@@ -861,13 +861,13 @@
         <v>242.8</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.01401015228426391</v>
+        <v>0.0107964962314116</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>7.74</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -891,16 +891,16 @@
         <v>5196</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1010</v>
+        <v>1014.2</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>5050</v>
+        <v>5071</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-146.0000000000002</v>
+        <v>-125</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.02809853733641267</v>
+        <v>-0.02405696689761355</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>954.83</v>
@@ -909,13 +909,13 @@
         <v>970</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.0396039603960396</v>
+        <v>0.0435811477026228</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>33.76</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -939,16 +939,16 @@
         <v>4788</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>791.05</v>
+        <v>766.15</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>4746.299999999999</v>
+        <v>4596.9</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>-41.70000000000027</v>
+        <v>-191.1000000000001</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>-0.008709273182957451</v>
+        <v>-0.03991228070175441</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>746.09</v>
@@ -957,13 +957,13 @@
         <v>746.09</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.05683585108400218</v>
+        <v>0.02618286236376682</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>22.5</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -987,16 +987,16 @@
         <v>4830</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>671.05</v>
+        <v>655.05</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4697.349999999999</v>
+        <v>4585.349999999999</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>-132.6500000000003</v>
+        <v>-244.6500000000003</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-0.0274637681159421</v>
+        <v>-0.05065217391304355</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>612.1900000000001</v>
@@ -1005,13 +1005,13 @@
         <v>612.1900000000001</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.0877132851501377</v>
+        <v>0.06543011983818015</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>34.34</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -1035,16 +1035,16 @@
         <v>3678</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1835.3</v>
+        <v>1827.2</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>3670.6</v>
+        <v>3654.4</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-7.400000000000091</v>
+        <v>-23.59999999999991</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.002011963023382298</v>
+        <v>-0.006416530723219116</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1729.61</v>
@@ -1053,13 +1053,13 @@
         <v>1744.3</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.04958317441290253</v>
+        <v>0.04536996497373035</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>43.14</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -1083,16 +1083,16 @@
         <v>5198.96</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>198.96</v>
+        <v>198.97</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5172.96</v>
+        <v>5173.22</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>-26</v>
+        <v>-25.74000000000024</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>-0.005001000200040008</v>
+        <v>-0.004950990198039653</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>187.26</v>
@@ -1101,13 +1101,13 @@
         <v>193.31</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.02839766787293931</v>
+        <v>0.02844649947228224</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>5.48</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -1131,16 +1131,16 @@
         <v>4242</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1412.9</v>
+        <v>1435.9</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4238.700000000001</v>
+        <v>4307.700000000001</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>-3.299999999999727</v>
+        <v>65.70000000000027</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>-0.0007779349363507136</v>
+        <v>0.01548797736916555</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1324.47</v>
@@ -1149,13 +1149,13 @@
         <v>1324.47</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.06258758581640601</v>
+        <v>0.07760289713768372</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>35.79</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -1179,16 +1179,16 @@
         <v>5200</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1364.2</v>
+        <v>1325.3</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>5456.8</v>
+        <v>5301.2</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>256.8000000000002</v>
+        <v>101.1999999999998</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.04938461538461542</v>
+        <v>0.01946153846153843</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1159.03</v>
@@ -1197,13 +1197,13 @@
         <v>1212</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.1115672188828618</v>
+        <v>0.08549007771825244</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>64.73</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -1227,16 +1227,16 @@
         <v>5209</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>275.25</v>
+        <v>276.25</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5505</v>
+        <v>5525</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>296.0000000000002</v>
+        <v>316.0000000000002</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.05682472643501636</v>
+        <v>0.06066423497792287</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>240.49</v>
@@ -1245,13 +1245,13 @@
         <v>253.5392857142858</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.0788763461787983</v>
+        <v>0.08221073044602437</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>8.369999999999999</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -1275,31 +1275,31 @@
         <v>5252.55</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>302.3</v>
+        <v>304.35</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>5743.7</v>
+        <v>5782.650000000001</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>491.1500000000004</v>
+        <v>530.1000000000006</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.09350696328449999</v>
+        <v>0.1009224091155726</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>259.14</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>277.7535714285714</v>
+        <v>279.75</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.08119890364349512</v>
+        <v>0.0808279940857566</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>7.11</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -1323,16 +1323,16 @@
         <v>4932</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>970.3</v>
+        <v>960.8</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>4851.5</v>
+        <v>4804</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-80.50000000000011</v>
+        <v>-128.0000000000001</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.01632197891321981</v>
+        <v>-0.02595296025952963</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>934.1900000000001</v>
@@ -1341,13 +1341,13 @@
         <v>934.1900000000001</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.03721529423889509</v>
+        <v>0.02769567027477092</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>25.59</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -1371,16 +1371,16 @@
         <v>4387.5</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1497.8</v>
+        <v>1491.9</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4493.4</v>
+        <v>4475.700000000001</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>105.8999999999999</v>
+        <v>88.20000000000027</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.02413675213675211</v>
+        <v>0.02010256410256417</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1405.17</v>
@@ -1389,17 +1389,305 @@
         <v>1405.17</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.06184403792228594</v>
+        <v>0.05813392318520009</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>38.34</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>GRANULES</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>790</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>8690</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>778.4</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>8562.4</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>-127.6000000000003</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>-0.0146835443037975</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>739.3099999999999</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>739.3099999999999</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>0.05021839671120251</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>24.04</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>RADICO</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>3770</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>7540</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>3778.6</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>7557.2</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>17.19999999999982</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>0.002281167108753292</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>3604.1</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>3604.1</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0.0461811252844969</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>81.47</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>ATUL</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>6500</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>6500</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>6546</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>6546</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="I17" s="11" t="n">
+        <v>0.007076923076923077</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>6181.43</v>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>6181.43</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>0.05569355331500148</v>
+      </c>
+      <c r="M17" s="13" t="n">
+        <v>142.71</v>
+      </c>
+      <c r="N17" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>MARICO</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>821.05</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>9031.549999999999</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>812.45</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>8936.950000000001</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>-94.599999999999</v>
+      </c>
+      <c r="I18" s="11" t="n">
+        <v>-0.01047439254612985</v>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>783.09</v>
+      </c>
+      <c r="K18" s="7" t="n">
+        <v>783.09</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>0.03613760846821344</v>
+      </c>
+      <c r="M18" s="13" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="N18" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>MANKIND</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>2426.1</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>7278.3</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>2538.3</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>7614.900000000001</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>336.6000000000008</v>
+      </c>
+      <c r="I19" s="11" t="n">
+        <v>0.04624706318783244</v>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>2309.03</v>
+      </c>
+      <c r="K19" s="7" t="n">
+        <v>2309.03</v>
+      </c>
+      <c r="L19" s="12" t="n">
+        <v>0.09032423275420556</v>
+      </c>
+      <c r="M19" s="13" t="n">
+        <v>59.36</v>
+      </c>
+      <c r="N19" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>RAINBOW</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>1475</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>8850</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>1446.8</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>8680.799999999999</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>-169.2000000000003</v>
+      </c>
+      <c r="I20" s="11" t="n">
+        <v>-0.01911864406779664</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>1394.19</v>
+      </c>
+      <c r="K20" s="7" t="n">
+        <v>1394.19</v>
+      </c>
+      <c r="L20" s="12" t="n">
+        <v>0.03636300801769415</v>
+      </c>
+      <c r="M20" s="13" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="N20" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H14">
+  <conditionalFormatting sqref="H2:H20">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1495,14 +1783,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
@@ -1667,6 +1955,31 @@
       </c>
       <c r="G6" s="15" t="n">
         <v>13</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>200292.61</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>89757.09</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>110535.52</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>110242.91</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1749,18 +2062,18 @@
     </row>
     <row r="2">
       <c r="A2" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>1497.8</v>
+        <v>10191</v>
       </c>
       <c r="D2" s="15" t="n">
-        <v>1423.01</v>
+        <v>9815</v>
       </c>
       <c r="E2" s="15" t="n">
         <v>0.0467</v>
@@ -1772,7 +2085,7 @@
         <v>7</v>
       </c>
       <c r="H2" s="15" t="n">
-        <v>0.8359390363815142</v>
+        <v>0.8203490658800394</v>
       </c>
       <c r="I2" s="15" t="inlineStr">
         <is>
@@ -1787,18 +2100,18 @@
     </row>
     <row r="3">
       <c r="A3" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>1835.3</v>
+        <v>1435.9</v>
       </c>
       <c r="D3" s="15" t="n">
-        <v>1755.01</v>
+        <v>1355.34</v>
       </c>
       <c r="E3" s="15" t="n">
         <v>0.0467</v>
@@ -1807,10 +2120,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="15" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="H3" s="15" t="n">
-        <v>0.8156833824975418</v>
+        <v>0.8156096361848575</v>
       </c>
       <c r="I3" s="15" t="inlineStr">
         <is>
@@ -1825,18 +2138,18 @@
     </row>
     <row r="4">
       <c r="A4" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>18052</v>
+        <v>1491.9</v>
       </c>
       <c r="D4" s="15" t="n">
-        <v>16921.86</v>
+        <v>1416.67</v>
       </c>
       <c r="E4" s="15" t="n">
         <v>0.0467</v>
@@ -1845,10 +2158,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="15" t="n">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="H4" s="15" t="n">
-        <v>0.8189970501474927</v>
+        <v>0.8075909537856441</v>
       </c>
       <c r="I4" s="15" t="inlineStr">
         <is>
@@ -1863,18 +2176,18 @@
     </row>
     <row r="5">
       <c r="A5" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>1412.9</v>
+        <v>2538.3</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>1333.81</v>
+        <v>2419.59</v>
       </c>
       <c r="E5" s="15" t="n">
         <v>0.0467</v>
@@ -1883,10 +2196,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="15" t="n">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>0.8182743362831859</v>
+        <v>0.8039233038348083</v>
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
@@ -1901,18 +2214,18 @@
     </row>
     <row r="6">
       <c r="A6" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>SOLARINDS</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>10066</v>
+        <v>18441</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>9694.139999999999</v>
+        <v>17315.29</v>
       </c>
       <c r="E6" s="15" t="n">
         <v>0.0467</v>
@@ -1921,10 +2234,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="15" t="n">
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>0.8103785644051131</v>
+        <v>0.7798377581120944</v>
       </c>
       <c r="I6" s="15" t="inlineStr">
         <is>
@@ -1939,18 +2252,18 @@
     </row>
     <row r="7">
       <c r="A7" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>10083</v>
+        <v>621</v>
       </c>
       <c r="D7" s="15" t="n">
-        <v>9644.57</v>
+        <v>592.4400000000001</v>
       </c>
       <c r="E7" s="15" t="n">
         <v>0.0467</v>
@@ -1959,10 +2272,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="15" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>0.7759537856440512</v>
+        <v>0.7732694198623402</v>
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
@@ -1977,18 +2290,18 @@
     </row>
     <row r="8">
       <c r="A8" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>791.05</v>
+        <v>1401.9</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>745.22</v>
+        <v>1338.11</v>
       </c>
       <c r="E8" s="15" t="n">
         <v>0.0467</v>
@@ -1997,10 +2310,10 @@
         <v>9333</v>
       </c>
       <c r="G8" s="15" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>0.7894641101278269</v>
+        <v>0.766740412979351</v>
       </c>
       <c r="I8" s="15" t="inlineStr">
         <is>
@@ -2015,18 +2328,18 @@
     </row>
     <row r="9">
       <c r="A9" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>786.9</v>
+        <v>1288.1</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>739.3099999999999</v>
+        <v>1218.93</v>
       </c>
       <c r="E9" s="15" t="n">
         <v>0.0467</v>
@@ -2035,10 +2348,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="15" t="n">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>0.7837512291052113</v>
+        <v>0.7723893805309734</v>
       </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
@@ -2053,18 +2366,18 @@
     </row>
     <row r="10">
       <c r="A10" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1414.8</v>
+        <v>812.45</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>1350.6</v>
+        <v>779.26</v>
       </c>
       <c r="E10" s="15" t="n">
         <v>0.0467</v>
@@ -2076,7 +2389,7 @@
         <v>6.4</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>0.7366420845624385</v>
+        <v>0.7512291052114061</v>
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
@@ -2091,18 +2404,18 @@
     </row>
     <row r="11">
       <c r="A11" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>3769.2</v>
+        <v>1827.2</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>3604.1</v>
+        <v>1753.19</v>
       </c>
       <c r="E11" s="15" t="n">
         <v>0.0467</v>
@@ -2114,7 +2427,7 @@
         <v>6.4</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>0.7299655850540807</v>
+        <v>0.7356243854473943</v>
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
@@ -2129,18 +2442,18 @@
     </row>
     <row r="12">
       <c r="A12" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>TIMKEN</t>
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>6482</v>
+        <v>3761</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>6181.43</v>
+        <v>3528.97</v>
       </c>
       <c r="E12" s="15" t="n">
         <v>0.0467</v>
@@ -2149,10 +2462,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>0.771676499508358</v>
+        <v>0.7422910521140609</v>
       </c>
       <c r="I12" s="15" t="inlineStr">
         <is>
@@ -2167,18 +2480,18 @@
     </row>
     <row r="13">
       <c r="A13" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>817.05</v>
+        <v>304.35</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>783.09</v>
+        <v>287.95</v>
       </c>
       <c r="E13" s="15" t="n">
         <v>0.0467</v>
@@ -2190,7 +2503,7 @@
         <v>6.3</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>0.7224926253687315</v>
+        <v>0.7164601769911505</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -2205,18 +2518,18 @@
     </row>
     <row r="14">
       <c r="A14" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>2414.2</v>
+        <v>766.15</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>2309.03</v>
+        <v>719.54</v>
       </c>
       <c r="E14" s="15" t="n">
         <v>0.0467</v>
@@ -2228,7 +2541,7 @@
         <v>6.3</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>0.7364405113077679</v>
+        <v>0.7616076696165193</v>
       </c>
       <c r="I14" s="15" t="inlineStr">
         <is>
@@ -2243,18 +2556,18 @@
     </row>
     <row r="15">
       <c r="A15" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>TRITURBINE</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>1470.8</v>
+        <v>737.3</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>1394.19</v>
+        <v>674.61</v>
       </c>
       <c r="E15" s="15" t="n">
         <v>0.0467</v>
@@ -2263,10 +2576,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>0.7489429695181908</v>
+        <v>0.713834808259587</v>
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
@@ -2281,18 +2594,18 @@
     </row>
     <row r="16">
       <c r="A16" s="15" t="n">
-        <v>20260619</v>
+        <v>20260622</v>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>1364.2</v>
+        <v>1446.8</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>1236.5</v>
+        <v>1370.6</v>
       </c>
       <c r="E16" s="15" t="n">
         <v>0.0467</v>
@@ -2304,7 +2617,7 @@
         <v>6.2</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>0.7264110127826942</v>
+        <v>0.756715830875123</v>
       </c>
       <c r="I16" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-06-27
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -20,13 +20,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="₹#,##0.00"/>
     <numFmt numFmtId="165" formatCode="₹#,##0"/>
     <numFmt numFmtId="166" formatCode="₹#,##0;[Red](₹#,##0);-"/>
     <numFmt numFmtId="167" formatCode="0.00%;[Red]-0.00%;-"/>
+    <numFmt numFmtId="168" formatCode="0.00&quot;R&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,10 +65,6 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00555555"/>
     </font>
   </fonts>
   <fills count="4">
@@ -114,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -147,8 +144,12 @@
     <xf numFmtId="2" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -548,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Mon 22 Jun 2026</t>
+          <t>As of Fri 26 Jun 2026</t>
         </is>
       </c>
     </row>
@@ -560,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹200,293</t>
+          <t>₹200,052</t>
         </is>
       </c>
     </row>
@@ -572,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-396  (-0.20%)</t>
+          <t>₹-241  (-0.12%)</t>
         </is>
       </c>
     </row>
@@ -584,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+0.15%</t>
+          <t>+0.03%</t>
         </is>
       </c>
     </row>
@@ -596,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.20%</t>
+          <t>-0.32%</t>
         </is>
       </c>
     </row>
@@ -608,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹89,757</t>
+          <t>₹109,403</t>
         </is>
       </c>
     </row>
@@ -620,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹110,243</t>
+          <t>₹89,707</t>
         </is>
       </c>
     </row>
@@ -632,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹110,536</t>
+          <t>₹90,649</t>
         </is>
       </c>
     </row>
@@ -644,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+0</t>
+          <t>₹-890</t>
         </is>
       </c>
     </row>
@@ -656,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -683,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -795,16 +796,16 @@
         <v>4230</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>1401.9</v>
+        <v>1402.6</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>4205.700000000001</v>
+        <v>4207.799999999999</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>-24.29999999999973</v>
+        <v>-22.20000000000027</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>-0.005744680851063765</v>
+        <v>-0.005248226950354674</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>1312.63</v>
@@ -813,19 +814,19 @@
         <v>1370.6</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.02232684214280632</v>
+        <v>0.02281477256523599</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>33.1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -834,46 +835,46 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>248.05</v>
+        <v>798</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>5209.05</v>
+        <v>4788</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>245.45</v>
+        <v>761.7</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>5154.45</v>
+        <v>4570.200000000001</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-54.60000000000048</v>
+        <v>-217.7999999999997</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.01048175771013918</v>
+        <v>-0.04548872180451122</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>230.7</v>
+        <v>746.09</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>242.8</v>
+        <v>750</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.0107964962314116</v>
+        <v>0.01536037810161487</v>
       </c>
       <c r="M3" s="13" t="n">
-        <v>7.74</v>
+        <v>22.5</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -882,46 +883,46 @@
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>1039.2</v>
+        <v>690</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>5196</v>
+        <v>4830</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1014.2</v>
+        <v>678.1</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>5071</v>
+        <v>4746.7</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-125</v>
+        <v>-83.29999999999984</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.02405696689761355</v>
+        <v>-0.01724637681159417</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>954.83</v>
+        <v>612.1900000000001</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>970</v>
+        <v>612.1900000000001</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.0435811477026228</v>
+        <v>0.09719805338445651</v>
       </c>
       <c r="M4" s="13" t="n">
-        <v>33.76</v>
+        <v>34.34</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -930,46 +931,46 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>798</v>
+        <v>1839</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>4788</v>
+        <v>3678</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>766.15</v>
+        <v>1796</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>4596.9</v>
+        <v>3592</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>-191.1000000000001</v>
+        <v>-86</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>-0.03991228070175441</v>
+        <v>-0.02338227297444263</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>746.09</v>
+        <v>1729.61</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>746.09</v>
+        <v>1744.3</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.02618286236376682</v>
+        <v>0.02878619153674835</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>22.5</v>
+        <v>43.14</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -978,46 +979,46 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>690</v>
+        <v>1414</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>4830</v>
+        <v>4242</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>655.05</v>
+        <v>1450</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4585.349999999999</v>
+        <v>4350</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>-244.6500000000003</v>
+        <v>108</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-0.05065217391304355</v>
+        <v>0.02545968882602546</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>612.1900000000001</v>
+        <v>1324.47</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>612.1900000000001</v>
+        <v>1331.242857142857</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.06543011983818015</v>
+        <v>0.08190147783251241</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>34.34</v>
+        <v>35.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -1026,46 +1027,46 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>1839</v>
+        <v>1300</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>3678</v>
+        <v>5200</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1827.2</v>
+        <v>1367.8</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>3654.4</v>
+        <v>5471.2</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-23.59999999999991</v>
+        <v>271.1999999999998</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.006416530723219116</v>
+        <v>0.05215384615384612</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>1729.61</v>
+        <v>1159.03</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1744.3</v>
+        <v>1214.092857142857</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.04536996497373035</v>
+        <v>0.1123754517159985</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>43.14</v>
+        <v>64.73</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -1074,46 +1075,46 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>199.96</v>
+        <v>260.45</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>5198.96</v>
+        <v>5209</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>198.97</v>
+        <v>275.3</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5173.22</v>
+        <v>5506</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>-25.74000000000024</v>
+        <v>297.0000000000005</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>-0.004950990198039653</v>
+        <v>0.05701670186216173</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>187.26</v>
+        <v>240.49</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>193.31</v>
+        <v>255.5642857142857</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.02844649947228224</v>
+        <v>0.07168802864407663</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>5.48</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -1122,46 +1123,46 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>1414</v>
+        <v>276.45</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>4242</v>
+        <v>5252.55</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1435.9</v>
+        <v>301.35</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4307.700000000001</v>
+        <v>5725.650000000001</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>65.70000000000027</v>
+        <v>473.1000000000006</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.01548797736916555</v>
+        <v>0.09007053716766154</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>1324.47</v>
+        <v>259.14</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>1324.47</v>
+        <v>279.75</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.07760289713768372</v>
+        <v>0.0716774514683923</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>35.79</v>
+        <v>7.11</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1170,238 +1171,238 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1300</v>
+        <v>1462.5</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>5200</v>
+        <v>4387.5</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1325.3</v>
+        <v>1555.2</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>5301.2</v>
+        <v>4665.6</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>101.1999999999998</v>
+        <v>278.1000000000001</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.01946153846153843</v>
+        <v>0.06338461538461541</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>1159.03</v>
+        <v>1405.17</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1212</v>
+        <v>1446.3</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.08549007771825244</v>
+        <v>0.07002314814814821</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>64.73</v>
+        <v>38.34</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>260.45</v>
+        <v>790</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>5209</v>
+        <v>8690</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>276.25</v>
+        <v>764.2</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5525</v>
+        <v>8406.200000000001</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>316.0000000000002</v>
+        <v>-283.7999999999995</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.06066423497792287</v>
+        <v>-0.03265822784810121</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>240.49</v>
+        <v>739.3099999999999</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>253.5392857142858</v>
+        <v>739.3099999999999</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.08221073044602437</v>
+        <v>0.03257000785134794</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>8.369999999999999</v>
+        <v>24.04</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>276.45</v>
+        <v>3770</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>5252.55</v>
+        <v>7540</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>304.35</v>
+        <v>3829.8</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>5782.650000000001</v>
+        <v>7659.6</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>530.1000000000006</v>
+        <v>119.6000000000004</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.1009224091155726</v>
+        <v>0.01586206896551729</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>259.14</v>
+        <v>3604.1</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>279.75</v>
+        <v>3604.1</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.0808279940857566</v>
+        <v>0.05893258133584006</v>
       </c>
       <c r="M12" s="13" t="n">
-        <v>7.11</v>
+        <v>81.47</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>986.4</v>
+        <v>6500</v>
       </c>
       <c r="D13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>6500</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>6670.5</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>6670.5</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>170.5</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0.02623076923076923</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>6181.43</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>6401.5</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>0.04032681208305224</v>
+      </c>
+      <c r="M13" s="13" t="n">
+        <v>142.71</v>
+      </c>
+      <c r="N13" s="6" t="n">
         <v>5</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>4932</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>960.8</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>4804</v>
-      </c>
-      <c r="H13" s="10" t="n">
-        <v>-128.0000000000001</v>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>-0.02595296025952963</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>934.1900000000001</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>934.1900000000001</v>
-      </c>
-      <c r="L13" s="12" t="n">
-        <v>0.02769567027477092</v>
-      </c>
-      <c r="M13" s="13" t="n">
-        <v>25.59</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>1462.5</v>
+        <v>821.05</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>4387.5</v>
+        <v>9031.549999999999</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1491.9</v>
+        <v>825.8</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4475.700000000001</v>
+        <v>9083.799999999999</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>88.20000000000027</v>
+        <v>52.25</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.02010256410256417</v>
+        <v>0.005785274952804336</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>1405.17</v>
+        <v>783.09</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>1405.17</v>
+        <v>796</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.05813392318520009</v>
+        <v>0.03608621942358919</v>
       </c>
       <c r="M14" s="13" t="n">
-        <v>38.34</v>
+        <v>16.6</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
@@ -1410,46 +1411,46 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>790</v>
+        <v>2426.1</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>8690</v>
+        <v>7278.3</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>778.4</v>
+        <v>2462.3</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>8562.4</v>
+        <v>7386.900000000001</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>-127.6000000000003</v>
+        <v>108.6000000000008</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>-0.0146835443037975</v>
+        <v>0.01492106673261625</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>739.3099999999999</v>
+        <v>2309.03</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>739.3099999999999</v>
+        <v>2309.03</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.05021839671120251</v>
+        <v>0.0622466799333956</v>
       </c>
       <c r="M15" s="13" t="n">
-        <v>24.04</v>
+        <v>59.36</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1458,236 +1459,44 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>3770</v>
+        <v>1475</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>7540</v>
+        <v>8850</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>3778.6</v>
+        <v>1434.5</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>7557.2</v>
+        <v>8607</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>17.19999999999982</v>
+        <v>-243</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.002281167108753292</v>
+        <v>-0.02745762711864407</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>3604.1</v>
+        <v>1394.19</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>3604.1</v>
+        <v>1394.19</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.0461811252844969</v>
+        <v>0.02810038340885322</v>
       </c>
       <c r="M16" s="13" t="n">
-        <v>81.47</v>
+        <v>38.1</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>ATUL</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="n">
-        <v>6500</v>
-      </c>
-      <c r="D17" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="9" t="n">
-        <v>6500</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>6546</v>
-      </c>
-      <c r="G17" s="9" t="n">
-        <v>6546</v>
-      </c>
-      <c r="H17" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="I17" s="11" t="n">
-        <v>0.007076923076923077</v>
-      </c>
-      <c r="J17" s="7" t="n">
-        <v>6181.43</v>
-      </c>
-      <c r="K17" s="7" t="n">
-        <v>6181.43</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>0.05569355331500148</v>
-      </c>
-      <c r="M17" s="13" t="n">
-        <v>142.71</v>
-      </c>
-      <c r="N17" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>MARICO</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="n">
-        <v>821.05</v>
-      </c>
-      <c r="D18" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="E18" s="9" t="n">
-        <v>9031.549999999999</v>
-      </c>
-      <c r="F18" s="7" t="n">
-        <v>812.45</v>
-      </c>
-      <c r="G18" s="9" t="n">
-        <v>8936.950000000001</v>
-      </c>
-      <c r="H18" s="10" t="n">
-        <v>-94.599999999999</v>
-      </c>
-      <c r="I18" s="11" t="n">
-        <v>-0.01047439254612985</v>
-      </c>
-      <c r="J18" s="7" t="n">
-        <v>783.09</v>
-      </c>
-      <c r="K18" s="7" t="n">
-        <v>783.09</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>0.03613760846821344</v>
-      </c>
-      <c r="M18" s="13" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="N18" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>MANKIND</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>2426.1</v>
-      </c>
-      <c r="D19" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E19" s="9" t="n">
-        <v>7278.3</v>
-      </c>
-      <c r="F19" s="7" t="n">
-        <v>2538.3</v>
-      </c>
-      <c r="G19" s="9" t="n">
-        <v>7614.900000000001</v>
-      </c>
-      <c r="H19" s="10" t="n">
-        <v>336.6000000000008</v>
-      </c>
-      <c r="I19" s="11" t="n">
-        <v>0.04624706318783244</v>
-      </c>
-      <c r="J19" s="7" t="n">
-        <v>2309.03</v>
-      </c>
-      <c r="K19" s="7" t="n">
-        <v>2309.03</v>
-      </c>
-      <c r="L19" s="12" t="n">
-        <v>0.09032423275420556</v>
-      </c>
-      <c r="M19" s="13" t="n">
-        <v>59.36</v>
-      </c>
-      <c r="N19" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>RAINBOW</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>1475</v>
-      </c>
-      <c r="D20" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="E20" s="9" t="n">
-        <v>8850</v>
-      </c>
-      <c r="F20" s="7" t="n">
-        <v>1446.8</v>
-      </c>
-      <c r="G20" s="9" t="n">
-        <v>8680.799999999999</v>
-      </c>
-      <c r="H20" s="10" t="n">
-        <v>-169.2000000000003</v>
-      </c>
-      <c r="I20" s="11" t="n">
-        <v>-0.01911864406779664</v>
-      </c>
-      <c r="J20" s="7" t="n">
-        <v>1394.19</v>
-      </c>
-      <c r="K20" s="7" t="n">
-        <v>1394.19</v>
-      </c>
-      <c r="L20" s="12" t="n">
-        <v>0.03636300801769415</v>
-      </c>
-      <c r="M20" s="13" t="n">
-        <v>38.1</v>
-      </c>
-      <c r="N20" s="6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H20">
+  <conditionalFormatting sqref="H2:H16">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1705,8 +1514,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
@@ -1768,11 +1590,184 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>No closed trades yet.</t>
-        </is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="n">
+        <v>248.05</v>
+      </c>
+      <c r="D2" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="n">
+        <v>242.8</v>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I2" s="17" t="n">
+        <v>-110.25</v>
+      </c>
+      <c r="J2" s="18" t="n">
+        <v>-0.0212</v>
+      </c>
+      <c r="K2" s="19" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="n">
+        <v>1039.2</v>
+      </c>
+      <c r="D3" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F3" s="15" t="n">
+        <v>970</v>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I3" s="17" t="n">
+        <v>-346</v>
+      </c>
+      <c r="J3" s="18" t="n">
+        <v>-0.06660000000000001</v>
+      </c>
+      <c r="K3" s="19" t="n">
+        <v>-0.82</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="n">
+        <v>199.96</v>
+      </c>
+      <c r="D4" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I4" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J4" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K4" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I5" s="17" t="n">
+        <v>-261.05</v>
+      </c>
+      <c r="J5" s="18" t="n">
+        <v>-0.0529</v>
+      </c>
+      <c r="K5" s="19" t="n">
+        <v>-1</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="I2:I5">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1783,7 +1778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1833,153 +1828,178 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="B2" s="16" t="n">
+      <c r="B2" s="20" t="n">
         <v>200000</v>
       </c>
-      <c r="C2" s="16" t="n">
+      <c r="C2" s="20" t="n">
         <v>200000</v>
       </c>
-      <c r="D2" s="16" t="n">
+      <c r="D2" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="16" t="n">
+      <c r="E2" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="16" t="n">
+      <c r="F2" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="15" t="n">
+      <c r="G2" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>2026-06-12</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n">
+      <c r="B3" s="20" t="n">
         <v>200000</v>
       </c>
-      <c r="C3" s="16" t="n">
+      <c r="C3" s="20" t="n">
         <v>200000</v>
       </c>
-      <c r="D3" s="16" t="n">
+      <c r="D3" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="E3" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="16" t="n">
+      <c r="F3" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="15" t="n">
+      <c r="G3" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="20" t="n">
         <v>198897.52</v>
       </c>
-      <c r="C4" s="16" t="n">
+      <c r="C4" s="20" t="n">
         <v>137646.94</v>
       </c>
-      <c r="D4" s="16" t="n">
+      <c r="D4" s="20" t="n">
         <v>61250.58</v>
       </c>
-      <c r="E4" s="16" t="n">
+      <c r="E4" s="20" t="n">
         <v>62353.06</v>
       </c>
-      <c r="F4" s="16" t="n">
+      <c r="F4" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="15" t="n">
+      <c r="G4" s="14" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="20" t="n">
         <v>200301.66</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="20" t="n">
         <v>137646.94</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D5" s="20" t="n">
         <v>62654.72</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="20" t="n">
         <v>62353.06</v>
       </c>
-      <c r="F5" s="16" t="n">
+      <c r="F5" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="15" t="n">
+      <c r="G5" s="14" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="20" t="n">
         <v>200688.9</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="20" t="n">
         <v>137646.94</v>
       </c>
-      <c r="D6" s="16" t="n">
+      <c r="D6" s="20" t="n">
         <v>63041.96</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="20" t="n">
         <v>62353.06</v>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="14" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="20" t="n">
         <v>200292.61</v>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="20" t="n">
         <v>89757.09</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="20" t="n">
         <v>110535.52</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="20" t="n">
         <v>110242.91</v>
       </c>
-      <c r="F7" s="16" t="n">
+      <c r="F7" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="15" t="n">
+      <c r="G7" s="14" t="n">
         <v>19</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="n">
+        <v>200052.05</v>
+      </c>
+      <c r="C8" s="20" t="n">
+        <v>109402.9</v>
+      </c>
+      <c r="D8" s="20" t="n">
+        <v>90649.14999999999</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>89706.89999999999</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <v>-890.2</v>
+      </c>
+      <c r="G8" s="14" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -2061,570 +2081,570 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="A2" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>HONASA</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="n">
+        <v>417.7</v>
+      </c>
+      <c r="D2" s="14" t="n">
+        <v>386.74</v>
+      </c>
+      <c r="E2" s="14" t="n">
+        <v>0.0467</v>
+      </c>
+      <c r="F2" s="14" t="n">
+        <v>9333</v>
+      </c>
+      <c r="G2" s="14" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="H2" s="14" t="n">
+        <v>0.8552704031465093</v>
+      </c>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>ENTER</t>
+        </is>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>RISK_NEU</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="n">
+        <v>953.2</v>
+      </c>
+      <c r="D3" s="14" t="n">
+        <v>896.01</v>
+      </c>
+      <c r="E3" s="14" t="n">
+        <v>0.0467</v>
+      </c>
+      <c r="F3" s="14" t="n">
+        <v>9333</v>
+      </c>
+      <c r="G3" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H3" s="14" t="n">
+        <v>0.8102949852507374</v>
+      </c>
+      <c r="I3" s="14" t="inlineStr">
+        <is>
+          <t>ENTER</t>
+        </is>
+      </c>
+      <c r="J3" s="14" t="inlineStr">
+        <is>
+          <t>RISK_NEU</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>OFSS</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>10974.5</v>
+      </c>
+      <c r="D4" s="14" t="n">
+        <v>10238.71</v>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>0.0467</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>9333</v>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <v>0.7795181907571289</v>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>ENTER</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>RISK_NEU</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>WELCORP</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>1455.1</v>
+      </c>
+      <c r="D5" s="14" t="n">
+        <v>1365.41</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>0.0467</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>9333</v>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>0.7973402163225172</v>
+      </c>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>ENTER</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>RISK_NEU</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>SONACOMS</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>619.25</v>
+      </c>
+      <c r="D6" s="14" t="n">
+        <v>591.46</v>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>0.0467</v>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>9333</v>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="H6" s="14" t="n">
+        <v>0.7858849557522124</v>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>ENTER</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>RISK_NEU</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>1402.6</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>1341.66</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.0467</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>9333</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>0.781086529006883</v>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>ENTER</t>
+        </is>
+      </c>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>RISK_NEU</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>9531</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>9096.139999999999</v>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>0.0467</v>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>9333</v>
+      </c>
+      <c r="G8" s="14" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>0.7733136676499508</v>
+      </c>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>ENTER</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>RISK_NEU</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>AUROPHARMA</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>1555.2</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <v>1482.6</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>0.0467</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>9333</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>0.7470403146509341</v>
+      </c>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>ENTER</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="inlineStr">
+        <is>
+          <t>RISK_NEU</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>BAJAJ-AUTO</t>
         </is>
       </c>
-      <c r="C2" s="15" t="n">
-        <v>10191</v>
-      </c>
-      <c r="D2" s="15" t="n">
-        <v>9815</v>
-      </c>
-      <c r="E2" s="15" t="n">
+      <c r="C10" s="14" t="n">
+        <v>9843</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>9444.57</v>
+      </c>
+      <c r="E10" s="14" t="n">
         <v>0.0467</v>
       </c>
-      <c r="F2" s="15" t="n">
+      <c r="F10" s="14" t="n">
         <v>9333</v>
       </c>
-      <c r="G2" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="H2" s="15" t="n">
-        <v>0.8203490658800394</v>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
+      <c r="G10" s="14" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H10" s="14" t="n">
+        <v>0.741794493608653</v>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
         <is>
           <t>ENTER</t>
         </is>
       </c>
-      <c r="J2" s="15" t="inlineStr">
+      <c r="J10" s="14" t="inlineStr">
         <is>
           <t>RISK_NEU</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B3" s="15" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
         </is>
       </c>
-      <c r="C3" s="15" t="n">
-        <v>1435.9</v>
-      </c>
-      <c r="D3" s="15" t="n">
-        <v>1355.34</v>
-      </c>
-      <c r="E3" s="15" t="n">
+      <c r="C11" s="14" t="n">
+        <v>1450</v>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>1370.83</v>
+      </c>
+      <c r="E11" s="14" t="n">
         <v>0.0467</v>
       </c>
-      <c r="F3" s="15" t="n">
+      <c r="F11" s="14" t="n">
         <v>9333</v>
       </c>
-      <c r="G3" s="15" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="H3" s="15" t="n">
-        <v>0.8156096361848575</v>
-      </c>
-      <c r="I3" s="15" t="inlineStr">
+      <c r="G11" s="14" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H11" s="14" t="n">
+        <v>0.7394788593903637</v>
+      </c>
+      <c r="I11" s="14" t="inlineStr">
         <is>
           <t>ENTER</t>
         </is>
       </c>
-      <c r="J3" s="15" t="inlineStr">
+      <c r="J11" s="14" t="inlineStr">
         <is>
           <t>RISK_NEU</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B4" s="15" t="inlineStr">
-        <is>
-          <t>AUROPHARMA</t>
-        </is>
-      </c>
-      <c r="C4" s="15" t="n">
-        <v>1491.9</v>
-      </c>
-      <c r="D4" s="15" t="n">
-        <v>1416.67</v>
-      </c>
-      <c r="E4" s="15" t="n">
+    <row r="12">
+      <c r="A12" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>SOLARINDS</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>17428</v>
+      </c>
+      <c r="D12" s="14" t="n">
+        <v>16220.29</v>
+      </c>
+      <c r="E12" s="14" t="n">
         <v>0.0467</v>
       </c>
-      <c r="F4" s="15" t="n">
+      <c r="F12" s="14" t="n">
         <v>9333</v>
       </c>
-      <c r="G4" s="15" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="H4" s="15" t="n">
-        <v>0.8075909537856441</v>
-      </c>
-      <c r="I4" s="15" t="inlineStr">
+      <c r="G12" s="14" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H12" s="14" t="n">
+        <v>0.7378023598820058</v>
+      </c>
+      <c r="I12" s="14" t="inlineStr">
         <is>
           <t>ENTER</t>
         </is>
       </c>
-      <c r="J4" s="15" t="inlineStr">
+      <c r="J12" s="14" t="inlineStr">
         <is>
           <t>RISK_NEU</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>MANKIND</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="n">
-        <v>2538.3</v>
-      </c>
-      <c r="D5" s="15" t="n">
-        <v>2419.59</v>
-      </c>
-      <c r="E5" s="15" t="n">
+    <row r="13">
+      <c r="A13" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="n">
+        <v>8592</v>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>8339.209999999999</v>
+      </c>
+      <c r="E13" s="14" t="n">
         <v>0.0467</v>
       </c>
-      <c r="F5" s="15" t="n">
+      <c r="F13" s="14" t="n">
         <v>9333</v>
       </c>
-      <c r="G5" s="15" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="H5" s="15" t="n">
-        <v>0.8039233038348083</v>
-      </c>
-      <c r="I5" s="15" t="inlineStr">
+      <c r="G13" s="14" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H13" s="14" t="n">
+        <v>0.7355555555555555</v>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
         <is>
           <t>ENTER</t>
         </is>
       </c>
-      <c r="J5" s="15" t="inlineStr">
+      <c r="J13" s="14" t="inlineStr">
         <is>
           <t>RISK_NEU</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>SOLARINDS</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="n">
-        <v>18441</v>
-      </c>
-      <c r="D6" s="15" t="n">
-        <v>17315.29</v>
-      </c>
-      <c r="E6" s="15" t="n">
+    <row r="14">
+      <c r="A14" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>942.1</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>893.91</v>
+      </c>
+      <c r="E14" s="14" t="n">
         <v>0.0467</v>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F14" s="14" t="n">
         <v>9333</v>
       </c>
-      <c r="G6" s="15" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="H6" s="15" t="n">
-        <v>0.7798377581120944</v>
-      </c>
-      <c r="I6" s="15" t="inlineStr">
+      <c r="G14" s="14" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H14" s="14" t="n">
+        <v>0.7373156342182891</v>
+      </c>
+      <c r="I14" s="14" t="inlineStr">
         <is>
           <t>ENTER</t>
         </is>
       </c>
-      <c r="J6" s="15" t="inlineStr">
+      <c r="J14" s="14" t="inlineStr">
         <is>
           <t>RISK_NEU</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B7" s="15" t="inlineStr">
-        <is>
-          <t>SONACOMS</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="n">
-        <v>621</v>
-      </c>
-      <c r="D7" s="15" t="n">
-        <v>592.4400000000001</v>
-      </c>
-      <c r="E7" s="15" t="n">
+    <row r="15">
+      <c r="A15" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>1796</v>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>1720.5</v>
+      </c>
+      <c r="E15" s="14" t="n">
         <v>0.0467</v>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="F15" s="14" t="n">
         <v>9333</v>
       </c>
-      <c r="G7" s="15" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="H7" s="15" t="n">
-        <v>0.7732694198623402</v>
-      </c>
-      <c r="I7" s="15" t="inlineStr">
+      <c r="G15" s="14" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H15" s="14" t="n">
+        <v>0.7340707964601769</v>
+      </c>
+      <c r="I15" s="14" t="inlineStr">
         <is>
           <t>ENTER</t>
         </is>
       </c>
-      <c r="J7" s="15" t="inlineStr">
+      <c r="J15" s="14" t="inlineStr">
         <is>
           <t>RISK_NEU</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>NESTLEIND</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="n">
-        <v>1401.9</v>
-      </c>
-      <c r="D8" s="15" t="n">
-        <v>1338.11</v>
-      </c>
-      <c r="E8" s="15" t="n">
+    <row r="16">
+      <c r="A16" s="14" t="n">
+        <v>20260626</v>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>VIJAYA</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>1367.8</v>
+      </c>
+      <c r="D16" s="14" t="n">
+        <v>1265.33</v>
+      </c>
+      <c r="E16" s="14" t="n">
         <v>0.0467</v>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="F16" s="14" t="n">
         <v>9333</v>
       </c>
-      <c r="G8" s="15" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="H8" s="15" t="n">
-        <v>0.766740412979351</v>
-      </c>
-      <c r="I8" s="15" t="inlineStr">
+      <c r="G16" s="14" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <v>0.7427531956735497</v>
+      </c>
+      <c r="I16" s="14" t="inlineStr">
         <is>
           <t>ENTER</t>
         </is>
       </c>
-      <c r="J8" s="15" t="inlineStr">
-        <is>
-          <t>RISK_NEU</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>MEDANTA</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="n">
-        <v>1288.1</v>
-      </c>
-      <c r="D9" s="15" t="n">
-        <v>1218.93</v>
-      </c>
-      <c r="E9" s="15" t="n">
-        <v>0.0467</v>
-      </c>
-      <c r="F9" s="15" t="n">
-        <v>9333</v>
-      </c>
-      <c r="G9" s="15" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="H9" s="15" t="n">
-        <v>0.7723893805309734</v>
-      </c>
-      <c r="I9" s="15" t="inlineStr">
-        <is>
-          <t>ENTER</t>
-        </is>
-      </c>
-      <c r="J9" s="15" t="inlineStr">
-        <is>
-          <t>RISK_NEU</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>MARICO</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="n">
-        <v>812.45</v>
-      </c>
-      <c r="D10" s="15" t="n">
-        <v>779.26</v>
-      </c>
-      <c r="E10" s="15" t="n">
-        <v>0.0467</v>
-      </c>
-      <c r="F10" s="15" t="n">
-        <v>9333</v>
-      </c>
-      <c r="G10" s="15" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="H10" s="15" t="n">
-        <v>0.7512291052114061</v>
-      </c>
-      <c r="I10" s="15" t="inlineStr">
-        <is>
-          <t>ENTER</t>
-        </is>
-      </c>
-      <c r="J10" s="15" t="inlineStr">
-        <is>
-          <t>RISK_NEU</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B11" s="15" t="inlineStr">
-        <is>
-          <t>ADANIPORTS</t>
-        </is>
-      </c>
-      <c r="C11" s="15" t="n">
-        <v>1827.2</v>
-      </c>
-      <c r="D11" s="15" t="n">
-        <v>1753.19</v>
-      </c>
-      <c r="E11" s="15" t="n">
-        <v>0.0467</v>
-      </c>
-      <c r="F11" s="15" t="n">
-        <v>9333</v>
-      </c>
-      <c r="G11" s="15" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="H11" s="15" t="n">
-        <v>0.7356243854473943</v>
-      </c>
-      <c r="I11" s="15" t="inlineStr">
-        <is>
-          <t>ENTER</t>
-        </is>
-      </c>
-      <c r="J11" s="15" t="inlineStr">
-        <is>
-          <t>RISK_NEU</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
-        <is>
-          <t>TIMKEN</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="n">
-        <v>3761</v>
-      </c>
-      <c r="D12" s="15" t="n">
-        <v>3528.97</v>
-      </c>
-      <c r="E12" s="15" t="n">
-        <v>0.0467</v>
-      </c>
-      <c r="F12" s="15" t="n">
-        <v>9333</v>
-      </c>
-      <c r="G12" s="15" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="H12" s="15" t="n">
-        <v>0.7422910521140609</v>
-      </c>
-      <c r="I12" s="15" t="inlineStr">
-        <is>
-          <t>ENTER</t>
-        </is>
-      </c>
-      <c r="J12" s="15" t="inlineStr">
-        <is>
-          <t>RISK_NEU</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B13" s="15" t="inlineStr">
-        <is>
-          <t>NYKAA</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="n">
-        <v>304.35</v>
-      </c>
-      <c r="D13" s="15" t="n">
-        <v>287.95</v>
-      </c>
-      <c r="E13" s="15" t="n">
-        <v>0.0467</v>
-      </c>
-      <c r="F13" s="15" t="n">
-        <v>9333</v>
-      </c>
-      <c r="G13" s="15" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="H13" s="15" t="n">
-        <v>0.7164601769911505</v>
-      </c>
-      <c r="I13" s="15" t="inlineStr">
-        <is>
-          <t>ENTER</t>
-        </is>
-      </c>
-      <c r="J13" s="15" t="inlineStr">
-        <is>
-          <t>RISK_NEU</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>ANTHEM</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="n">
-        <v>766.15</v>
-      </c>
-      <c r="D14" s="15" t="n">
-        <v>719.54</v>
-      </c>
-      <c r="E14" s="15" t="n">
-        <v>0.0467</v>
-      </c>
-      <c r="F14" s="15" t="n">
-        <v>9333</v>
-      </c>
-      <c r="G14" s="15" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="H14" s="15" t="n">
-        <v>0.7616076696165193</v>
-      </c>
-      <c r="I14" s="15" t="inlineStr">
-        <is>
-          <t>ENTER</t>
-        </is>
-      </c>
-      <c r="J14" s="15" t="inlineStr">
-        <is>
-          <t>RISK_NEU</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B15" s="15" t="inlineStr">
-        <is>
-          <t>TRITURBINE</t>
-        </is>
-      </c>
-      <c r="C15" s="15" t="n">
-        <v>737.3</v>
-      </c>
-      <c r="D15" s="15" t="n">
-        <v>674.61</v>
-      </c>
-      <c r="E15" s="15" t="n">
-        <v>0.0467</v>
-      </c>
-      <c r="F15" s="15" t="n">
-        <v>9333</v>
-      </c>
-      <c r="G15" s="15" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="H15" s="15" t="n">
-        <v>0.713834808259587</v>
-      </c>
-      <c r="I15" s="15" t="inlineStr">
-        <is>
-          <t>ENTER</t>
-        </is>
-      </c>
-      <c r="J15" s="15" t="inlineStr">
-        <is>
-          <t>RISK_NEU</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="n">
-        <v>20260622</v>
-      </c>
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>RAINBOW</t>
-        </is>
-      </c>
-      <c r="C16" s="15" t="n">
-        <v>1446.8</v>
-      </c>
-      <c r="D16" s="15" t="n">
-        <v>1370.6</v>
-      </c>
-      <c r="E16" s="15" t="n">
-        <v>0.0467</v>
-      </c>
-      <c r="F16" s="15" t="n">
-        <v>9333</v>
-      </c>
-      <c r="G16" s="15" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="H16" s="15" t="n">
-        <v>0.756715830875123</v>
-      </c>
-      <c r="I16" s="15" t="inlineStr">
-        <is>
-          <t>ENTER</t>
-        </is>
-      </c>
-      <c r="J16" s="15" t="inlineStr">
+      <c r="J16" s="14" t="inlineStr">
         <is>
           <t>RISK_NEU</t>
         </is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-06-29
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Fri 26 Jun 2026</t>
+          <t>As of Mon 29 Jun 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹200,052</t>
+          <t>₹201,159</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-241  (-0.12%)</t>
+          <t>₹+1,107  (+0.55%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+0.03%</t>
+          <t>+0.58%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.32%</t>
+          <t>+0.00%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹109,403</t>
+          <t>₹64,533</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹89,707</t>
+          <t>₹134,092</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹90,649</t>
+          <t>₹136,626</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹-890</t>
+          <t>₹-1,375</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -796,16 +796,16 @@
         <v>4230</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>1402.6</v>
+        <v>1387.3</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>4207.799999999999</v>
+        <v>4161.9</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>-22.20000000000027</v>
+        <v>-68.10000000000014</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>-0.005248226950354674</v>
+        <v>-0.01609929078014188</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>1312.63</v>
@@ -814,13 +814,13 @@
         <v>1370.6</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.02281477256523599</v>
+        <v>0.01203777121026458</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>33.1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>4788</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>761.7</v>
+        <v>775</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>4570.200000000001</v>
+        <v>4650</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-217.7999999999997</v>
+        <v>-138</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.04548872180451122</v>
+        <v>-0.02882205513784461</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>746.09</v>
@@ -862,13 +862,13 @@
         <v>750</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.01536037810161487</v>
+        <v>0.03225806451612903</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>22.5</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>4830</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>678.1</v>
+        <v>675.5</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>4746.7</v>
+        <v>4728.5</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-83.29999999999984</v>
+        <v>-101.5</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.01724637681159417</v>
+        <v>-0.02101449275362319</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>612.1900000000001</v>
@@ -910,13 +910,13 @@
         <v>612.1900000000001</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.09719805338445651</v>
+        <v>0.09372316802368608</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>34.34</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>3678</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1796</v>
+        <v>1776.1</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>3592</v>
+        <v>3552.2</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>-86</v>
+        <v>-125.8000000000002</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>-0.02338227297444263</v>
+        <v>-0.03420337139749869</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1729.61</v>
@@ -958,13 +958,13 @@
         <v>1744.3</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.02878619153674835</v>
+        <v>0.01790439727492819</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>43.14</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>4242</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1450</v>
+        <v>1500.3</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4350</v>
+        <v>4500.9</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>108</v>
+        <v>258.8999999999999</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.02545968882602546</v>
+        <v>0.061032531824611</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1324.47</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1331.242857142857</v>
+        <v>1372.757142857143</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.08190147783251241</v>
+        <v>0.08501156911474853</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>35.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>5200</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1367.8</v>
+        <v>1311.3</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>5471.2</v>
+        <v>5245.2</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>271.1999999999998</v>
+        <v>45.19999999999982</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.05215384615384612</v>
+        <v>0.008692307692307657</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1159.03</v>
@@ -1054,13 +1054,13 @@
         <v>1214.092857142857</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.1123754517159985</v>
+        <v>0.07413036136440387</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>64.73</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>5209</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>275.3</v>
+        <v>273.5</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5506</v>
+        <v>5470</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>297.0000000000005</v>
+        <v>261.0000000000002</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.05701670186216173</v>
+        <v>0.05010558648492997</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>240.49</v>
@@ -1102,13 +1102,13 @@
         <v>255.5642857142857</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.07168802864407663</v>
+        <v>0.06557848002089328</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>8.369999999999999</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>5252.55</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>301.35</v>
+        <v>302.05</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5725.650000000001</v>
+        <v>5738.95</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>473.1000000000006</v>
+        <v>486.4000000000004</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.09007053716766154</v>
+        <v>0.09260264062217408</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>259.14</v>
@@ -1150,13 +1150,13 @@
         <v>279.75</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.0716774514683923</v>
+        <v>0.07382883628538325</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>7.11</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>4387.5</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1555.2</v>
+        <v>1547.5</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4665.6</v>
+        <v>4642.5</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>278.1000000000001</v>
+        <v>255</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.06338461538461541</v>
+        <v>0.05811965811965812</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1405.17</v>
@@ -1198,13 +1198,13 @@
         <v>1446.3</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.07002314814814821</v>
+        <v>0.06539579967689825</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>38.34</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>8690</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>764.2</v>
+        <v>794.8</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8406.200000000001</v>
+        <v>8742.799999999999</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-283.7999999999995</v>
+        <v>52.7999999999995</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>-0.03265822784810121</v>
+        <v>0.00607594936708855</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>739.3099999999999</v>
@@ -1246,13 +1246,13 @@
         <v>739.3099999999999</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.03257000785134794</v>
+        <v>0.06981630598892805</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>24.04</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -1276,31 +1276,31 @@
         <v>7540</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>3829.8</v>
+        <v>3876.9</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>7659.6</v>
+        <v>7753.8</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>119.6000000000004</v>
+        <v>213.8000000000002</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.01586206896551729</v>
+        <v>0.02835543766578252</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>3604.1</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>3604.1</v>
+        <v>3621.964285714286</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.05893258133584006</v>
+        <v>0.0657576193055571</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>81.47</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>6500</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>6670.5</v>
+        <v>6608.5</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>6670.5</v>
+        <v>6608.5</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>170.5</v>
+        <v>108.5</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.02623076923076923</v>
+        <v>0.01669230769230769</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>6181.43</v>
@@ -1342,13 +1342,13 @@
         <v>6401.5</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.04032681208305224</v>
+        <v>0.03132329575546645</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>142.71</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>9031.549999999999</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>825.8</v>
+        <v>839.95</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>9083.799999999999</v>
+        <v>9239.450000000001</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>52.25</v>
+        <v>207.900000000001</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.005785274952804336</v>
+        <v>0.02301930454905315</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>783.09</v>
@@ -1390,13 +1390,13 @@
         <v>796</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.03608621942358919</v>
+        <v>0.05232454312756717</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>16.6</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>7278.3</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>2462.3</v>
+        <v>2486</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>7386.900000000001</v>
+        <v>7458</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>108.6000000000008</v>
+        <v>179.7000000000003</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.01492106673261625</v>
+        <v>0.02468983141667701</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>2309.03</v>
@@ -1438,65 +1438,305 @@
         <v>2309.03</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.0622466799333956</v>
+        <v>0.0711866452131938</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>59.36</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>1475</v>
+        <v>420.3</v>
       </c>
       <c r="D16" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>9246.6</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>446.45</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>9821.9</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>575.2999999999995</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>0.06221746371639299</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>386.74</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>386.74</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0.1337439802889461</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>16.71</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>952.1</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>8568.9</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>963.8</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>8674.199999999999</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>105.2999999999994</v>
+      </c>
+      <c r="I17" s="11" t="n">
+        <v>0.01228862514441753</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>896.01</v>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>896.01</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>0.07033616932973642</v>
+      </c>
+      <c r="M17" s="13" t="n">
+        <v>28.08</v>
+      </c>
+      <c r="N17" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>WELCORP</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>1465</v>
+      </c>
+      <c r="D18" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="E16" s="9" t="n">
-        <v>8850</v>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>1434.5</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>8607</v>
-      </c>
-      <c r="H16" s="10" t="n">
-        <v>-243</v>
-      </c>
-      <c r="I16" s="11" t="n">
-        <v>-0.02745762711864407</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>1394.19</v>
-      </c>
-      <c r="K16" s="7" t="n">
-        <v>1394.19</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>0.02810038340885322</v>
-      </c>
-      <c r="M16" s="13" t="n">
-        <v>38.1</v>
-      </c>
-      <c r="N16" s="6" t="n">
-        <v>5</v>
+      <c r="E18" s="9" t="n">
+        <v>8790</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>1510.8</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>9064.799999999999</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>274.7999999999997</v>
+      </c>
+      <c r="I18" s="11" t="n">
+        <v>0.03126279863481225</v>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>1365.41</v>
+      </c>
+      <c r="K18" s="7" t="n">
+        <v>1365.41</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>0.09623378342599939</v>
+      </c>
+      <c r="M18" s="13" t="n">
+        <v>45.25</v>
+      </c>
+      <c r="N18" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>SONACOMS</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>619.25</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>9288.75</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>620.75</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>9311.25</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="I19" s="11" t="n">
+        <v>0.002422285022204279</v>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>591.46</v>
+      </c>
+      <c r="K19" s="7" t="n">
+        <v>591.46</v>
+      </c>
+      <c r="L19" s="12" t="n">
+        <v>0.04718485702778891</v>
+      </c>
+      <c r="M19" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="N19" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>8700</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>8700</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>8655</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>8655</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>-45</v>
+      </c>
+      <c r="I20" s="11" t="n">
+        <v>-0.005172413793103448</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>8339.209999999999</v>
+      </c>
+      <c r="K20" s="7" t="n">
+        <v>8339.209999999999</v>
+      </c>
+      <c r="L20" s="12" t="n">
+        <v>0.03648642403235134</v>
+      </c>
+      <c r="M20" s="13" t="n">
+        <v>123.68</v>
+      </c>
+      <c r="N20" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>960.1</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>8640.9</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>956.25</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>8606.25</v>
+      </c>
+      <c r="H21" s="10" t="n">
+        <v>-34.6500000000002</v>
+      </c>
+      <c r="I21" s="11" t="n">
+        <v>-0.004009998958441853</v>
+      </c>
+      <c r="J21" s="7" t="n">
+        <v>893.91</v>
+      </c>
+      <c r="K21" s="7" t="n">
+        <v>893.91</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>0.06519215686274513</v>
+      </c>
+      <c r="M21" s="13" t="n">
+        <v>24.91</v>
+      </c>
+      <c r="N21" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H16">
+  <conditionalFormatting sqref="H2:H21">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1514,7 +1754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1590,27 +1830,27 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>248.05</v>
+        <v>1475</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>242.8</v>
+        <v>1394.19</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -1618,22 +1858,22 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-110.25</v>
+        <v>-484.86</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0548</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-0.3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -1642,10 +1882,10 @@
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>1039.2</v>
+        <v>248.05</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
@@ -1653,7 +1893,7 @@
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>970</v>
+        <v>242.8</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -1664,19 +1904,19 @@
         <v>11</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-346</v>
+        <v>-110.25</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -1685,10 +1925,10 @@
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>199.96</v>
+        <v>1039.2</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
@@ -1696,7 +1936,7 @@
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>193.31</v>
+        <v>970</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1707,19 +1947,19 @@
         <v>11</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-172.9</v>
+        <v>-346</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.06660000000000001</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -1728,10 +1968,10 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>986.4</v>
+        <v>199.96</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
@@ -1739,7 +1979,7 @@
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>193.31</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1750,17 +1990,60 @@
         <v>11</v>
       </c>
       <c r="I5" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J5" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K5" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I6" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J5" s="18" t="n">
+      <c r="J6" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K5" s="19" t="n">
+      <c r="K6" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I5">
+  <conditionalFormatting sqref="I2:I6">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1778,7 +2061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2000,6 +2283,31 @@
       </c>
       <c r="G8" s="14" t="n">
         <v>15</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="n">
+        <v>201158.99</v>
+      </c>
+      <c r="C9" s="20" t="n">
+        <v>64532.89</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <v>136626.1</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>134092.05</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>-1375.06</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -2082,30 +2390,30 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>417.7</v>
+        <v>1500.3</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>386.74</v>
+        <v>1415.27</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7.1</v>
+        <v>6.5</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8552704031465093</v>
+        <v>0.8571681415929203</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -2114,36 +2422,36 @@
       </c>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>SOLARINDS</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>953.2</v>
+        <v>17798</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>896.01</v>
+        <v>16539.57</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>7</v>
+        <v>6.2</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8102949852507374</v>
+        <v>0.8211848574237954</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -2152,36 +2460,36 @@
       </c>
       <c r="J3" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>OFSS</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>10974.5</v>
+        <v>9779</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>10238.71</v>
+        <v>9304.57</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.8</v>
+        <v>6.2</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7795181907571289</v>
+        <v>0.8009488692232055</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -2190,36 +2498,36 @@
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1455.1</v>
+        <v>956.25</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1365.41</v>
+        <v>906.42</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.7</v>
+        <v>6.2</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7973402163225172</v>
+        <v>0.7972763028515242</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -2228,36 +2536,36 @@
       </c>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>619.25</v>
+        <v>794.8</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>591.46</v>
+        <v>742.49</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.7</v>
+        <v>6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7858849557522124</v>
+        <v>0.8102704031465093</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -2266,13 +2574,13 @@
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
@@ -2280,22 +2588,22 @@
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1402.6</v>
+        <v>1387.3</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1341.66</v>
+        <v>1321.89</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.7</v>
+        <v>6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.781086529006883</v>
+        <v>0.7926106194690266</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -2304,36 +2612,36 @@
       </c>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>9531</v>
+        <v>446.45</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>9096.139999999999</v>
+        <v>413.02</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.7</v>
+        <v>6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7733136676499508</v>
+        <v>0.7875860373647984</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -2342,36 +2650,36 @@
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1555.2</v>
+        <v>839.95</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1482.6</v>
+        <v>805.14</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7470403146509341</v>
+        <v>0.7788593903638151</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -2380,36 +2688,36 @@
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>ADANIPOWER</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>9843</v>
+        <v>227.05</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>9444.57</v>
+        <v>214.06</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.741794493608653</v>
+        <v>0.7594936086529007</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -2418,36 +2726,36 @@
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1450</v>
+        <v>2170.9</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1370.83</v>
+        <v>2045.97</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7394788593903637</v>
+        <v>0.7589823008849558</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -2456,36 +2764,36 @@
       </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>17428</v>
+        <v>1510.8</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>16220.29</v>
+        <v>1420.3</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.4</v>
+        <v>5.9</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7378023598820058</v>
+        <v>0.7765339233038349</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -2494,36 +2802,36 @@
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>8592</v>
+        <v>5541.5</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>8339.209999999999</v>
+        <v>5245.64</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.4</v>
+        <v>5.9</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7355555555555555</v>
+        <v>0.7547492625368731</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -2532,36 +2840,36 @@
       </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>942.1</v>
+        <v>1547.5</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>893.91</v>
+        <v>1472.59</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.4</v>
+        <v>5.9</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7373156342182891</v>
+        <v>0.7647738446411013</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -2570,36 +2878,36 @@
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1796</v>
+        <v>963.8</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1720.5</v>
+        <v>907.64</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.4</v>
+        <v>5.9</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7340707964601769</v>
+        <v>0.75055063913471</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -2608,36 +2916,36 @@
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260626</v>
+        <v>20260629</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1367.8</v>
+        <v>2303.2</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1265.33</v>
+        <v>2201.26</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.3</v>
+        <v>5.8</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7427531956735497</v>
+        <v>0.7632792527040315</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>
@@ -2646,7 +2954,7 @@
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V5 daily refresh 2026-06-30
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Mon 29 Jun 2026</t>
+          <t>As of Tue 30 Jun 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹201,159</t>
+          <t>₹202,277</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+1,107  (+0.55%)</t>
+          <t>₹+1,118  (+0.56%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+0.58%</t>
+          <t>+1.14%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹64,533</t>
+          <t>₹73,072</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹134,092</t>
+          <t>₹125,523</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹136,626</t>
+          <t>₹129,205</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹-1,375</t>
+          <t>₹-1,405</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -796,16 +796,16 @@
         <v>4230</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>1387.3</v>
+        <v>1405.2</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>4161.9</v>
+        <v>4215.6</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>-68.10000000000014</v>
+        <v>-14.39999999999986</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>-0.01609929078014188</v>
+        <v>-0.003404255319148904</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>1312.63</v>
@@ -814,13 +814,13 @@
         <v>1370.6</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.01203777121026458</v>
+        <v>0.02462282949046409</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>33.1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>4788</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>775</v>
+        <v>770.55</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>4650</v>
+        <v>4623.299999999999</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-138</v>
+        <v>-164.7000000000003</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.02882205513784461</v>
+        <v>-0.03439849624060156</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>746.09</v>
@@ -862,13 +862,13 @@
         <v>750</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.03225806451612903</v>
+        <v>0.0266692622153007</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>22.5</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>4830</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>675.5</v>
+        <v>679.2</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>4728.5</v>
+        <v>4754.400000000001</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-101.5</v>
+        <v>-75.59999999999968</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.02101449275362319</v>
+        <v>-0.01565217391304341</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>612.1900000000001</v>
@@ -910,13 +910,13 @@
         <v>612.1900000000001</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.09372316802368608</v>
+        <v>0.09866018845700822</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>34.34</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>3678</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1776.1</v>
+        <v>1810.2</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>3552.2</v>
+        <v>3620.4</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>-125.8000000000002</v>
+        <v>-57.59999999999991</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>-0.03420337139749869</v>
+        <v>-0.01566068515497551</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1729.61</v>
@@ -958,13 +958,13 @@
         <v>1744.3</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.01790439727492819</v>
+        <v>0.03640481714727659</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>43.14</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>4242</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1500.3</v>
+        <v>1517.4</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4500.9</v>
+        <v>4552.200000000001</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>258.8999999999999</v>
+        <v>310.2000000000003</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.061032531824611</v>
+        <v>0.07312588401697319</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1324.47</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1372.757142857143</v>
+        <v>1391.807142857143</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.08501156911474853</v>
+        <v>0.08276845732361747</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>35.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -1036,31 +1036,31 @@
         <v>5200</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1311.3</v>
+        <v>1352.6</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>5245.2</v>
+        <v>5410.4</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>45.19999999999982</v>
+        <v>210.3999999999996</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.008692307692307657</v>
+        <v>0.04046153846153839</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1159.03</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1214.092857142857</v>
+        <v>1221.4</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.07413036136440387</v>
+        <v>0.09699837350288321</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>64.73</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -1084,31 +1084,31 @@
         <v>5209</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>273.5</v>
+        <v>274.75</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5470</v>
+        <v>5495</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>261.0000000000002</v>
+        <v>286.0000000000002</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.05010558648492997</v>
+        <v>0.05490497216356311</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>240.49</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>255.5642857142857</v>
+        <v>255.6500000000001</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.06557848002089328</v>
+        <v>0.06951774340309338</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>8.369999999999999</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -1132,31 +1132,31 @@
         <v>5252.55</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>302.05</v>
+        <v>310.85</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5738.95</v>
+        <v>5906.150000000001</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>486.4000000000004</v>
+        <v>653.6000000000006</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.09260264062217408</v>
+        <v>0.1244347983360464</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>259.14</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>279.75</v>
+        <v>284.4928571428572</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.07382883628538325</v>
+        <v>0.08479055125347541</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>7.11</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>4387.5</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1547.5</v>
+        <v>1578.7</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4642.5</v>
+        <v>4736.1</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>255</v>
+        <v>348.6000000000001</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.05811965811965812</v>
+        <v>0.07945299145299148</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1405.17</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1446.3</v>
+        <v>1464.164285714286</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.06539579967689825</v>
+        <v>0.0725506519830965</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>38.34</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>8690</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>794.8</v>
+        <v>813.25</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8742.799999999999</v>
+        <v>8945.75</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>52.7999999999995</v>
+        <v>255.75</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.00607594936708855</v>
+        <v>0.02943037974683544</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>739.3099999999999</v>
@@ -1246,13 +1246,13 @@
         <v>739.3099999999999</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.06981630598892805</v>
+        <v>0.09091915155241323</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>24.04</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -1276,31 +1276,31 @@
         <v>7540</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>3876.9</v>
+        <v>3945.5</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>7753.8</v>
+        <v>7891</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>213.8000000000002</v>
+        <v>351</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.02835543766578252</v>
+        <v>0.04655172413793104</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>3604.1</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>3621.964285714286</v>
+        <v>3674.064285714286</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.0657576193055571</v>
+        <v>0.06879627785723338</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>81.47</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>6500</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>6608.5</v>
+        <v>6464.5</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>6608.5</v>
+        <v>6464.5</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>108.5</v>
+        <v>-35.5</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.01669230769230769</v>
+        <v>-0.005461538461538461</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>6181.43</v>
@@ -1342,13 +1342,13 @@
         <v>6401.5</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.03132329575546645</v>
+        <v>0.009745533297238766</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>142.71</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>9031.549999999999</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>839.95</v>
+        <v>836.25</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>9239.450000000001</v>
+        <v>9198.75</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>207.900000000001</v>
+        <v>167.2000000000005</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.02301930454905315</v>
+        <v>0.01851287984897393</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>783.09</v>
@@ -1390,13 +1390,13 @@
         <v>796</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.05232454312756717</v>
+        <v>0.04813153961136024</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>16.6</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -1420,31 +1420,31 @@
         <v>7278.3</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>2486</v>
+        <v>2545.6</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>7458</v>
+        <v>7636.799999999999</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>179.7000000000003</v>
+        <v>358.5</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.02468983141667701</v>
+        <v>0.04925600758418862</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>2309.03</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>2309.03</v>
+        <v>2340.228571428572</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.0711866452131938</v>
+        <v>0.0806770225374875</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>59.36</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
@@ -1468,37 +1468,37 @@
         <v>9246.6</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>446.45</v>
+        <v>457.9</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>9821.9</v>
+        <v>10073.8</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>575.2999999999995</v>
+        <v>827.1999999999992</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.06221746371639299</v>
+        <v>0.08945990958838916</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>386.74</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>386.74</v>
+        <v>405.1107142857143</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.1337439802889461</v>
+        <v>0.1152856206907309</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -1507,46 +1507,46 @@
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>952.1</v>
+        <v>1465</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>8568.9</v>
+        <v>8790</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>963.8</v>
+        <v>1521.9</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>8674.199999999999</v>
+        <v>9131.400000000001</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>105.2999999999994</v>
+        <v>341.4000000000005</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>0.01228862514441753</v>
+        <v>0.03883959044368607</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>896.01</v>
+        <v>1365.41</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>896.01</v>
+        <v>1397.635714285714</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>0.07033616932973642</v>
+        <v>0.08165075610374251</v>
       </c>
       <c r="M17" s="13" t="n">
-        <v>28.08</v>
+        <v>45.25</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1555,46 +1555,46 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>1465</v>
+        <v>619.25</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>8790</v>
+        <v>9288.75</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>1510.8</v>
+        <v>619.9</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>9064.799999999999</v>
+        <v>9298.5</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>274.7999999999997</v>
+        <v>9.749999999999659</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>0.03126279863481225</v>
+        <v>0.001049656842955151</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>1365.41</v>
+        <v>591.46</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>1365.41</v>
+        <v>591.46</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>0.09623378342599939</v>
+        <v>0.04587836747862549</v>
       </c>
       <c r="M18" s="13" t="n">
-        <v>45.25</v>
+        <v>14</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -1603,46 +1603,46 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>619.25</v>
+        <v>8700</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>9288.75</v>
+        <v>8700</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>620.75</v>
+        <v>8682</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>9311.25</v>
+        <v>8682</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>22.5</v>
+        <v>-18</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>0.002422285022204279</v>
+        <v>-0.002068965517241379</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>591.46</v>
+        <v>8339.209999999999</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>591.46</v>
+        <v>8339.209999999999</v>
       </c>
       <c r="L19" s="12" t="n">
-        <v>0.04718485702778891</v>
+        <v>0.03948283805574762</v>
       </c>
       <c r="M19" s="13" t="n">
-        <v>14</v>
+        <v>123.68</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -1651,92 +1651,44 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>8700</v>
+        <v>960.1</v>
       </c>
       <c r="D20" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>8640.9</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>952.15</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>8569.35</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>-71.55000000000041</v>
+      </c>
+      <c r="I20" s="11" t="n">
+        <v>-0.008280387459639669</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>893.91</v>
+      </c>
+      <c r="K20" s="7" t="n">
+        <v>893.91</v>
+      </c>
+      <c r="L20" s="12" t="n">
+        <v>0.06116683295699208</v>
+      </c>
+      <c r="M20" s="13" t="n">
+        <v>24.91</v>
+      </c>
+      <c r="N20" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E20" s="9" t="n">
-        <v>8700</v>
-      </c>
-      <c r="F20" s="7" t="n">
-        <v>8655</v>
-      </c>
-      <c r="G20" s="9" t="n">
-        <v>8655</v>
-      </c>
-      <c r="H20" s="10" t="n">
-        <v>-45</v>
-      </c>
-      <c r="I20" s="11" t="n">
-        <v>-0.005172413793103448</v>
-      </c>
-      <c r="J20" s="7" t="n">
-        <v>8339.209999999999</v>
-      </c>
-      <c r="K20" s="7" t="n">
-        <v>8339.209999999999</v>
-      </c>
-      <c r="L20" s="12" t="n">
-        <v>0.03648642403235134</v>
-      </c>
-      <c r="M20" s="13" t="n">
-        <v>123.68</v>
-      </c>
-      <c r="N20" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>CGPOWER</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>960.1</v>
-      </c>
-      <c r="D21" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="E21" s="9" t="n">
-        <v>8640.9</v>
-      </c>
-      <c r="F21" s="7" t="n">
-        <v>956.25</v>
-      </c>
-      <c r="G21" s="9" t="n">
-        <v>8606.25</v>
-      </c>
-      <c r="H21" s="10" t="n">
-        <v>-34.6500000000002</v>
-      </c>
-      <c r="I21" s="11" t="n">
-        <v>-0.004009998958441853</v>
-      </c>
-      <c r="J21" s="7" t="n">
-        <v>893.91</v>
-      </c>
-      <c r="K21" s="7" t="n">
-        <v>893.91</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>0.06519215686274513</v>
-      </c>
-      <c r="M21" s="13" t="n">
-        <v>24.91</v>
-      </c>
-      <c r="N21" s="6" t="n">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H21">
+  <conditionalFormatting sqref="H2:H20">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1754,7 +1706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1830,27 +1782,27 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>1475</v>
+        <v>952.1</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>1394.19</v>
+        <v>948.8</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -1858,42 +1810,42 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-484.86</v>
+        <v>-29.7</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0035</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-1</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>248.05</v>
+        <v>1475</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>242.8</v>
+        <v>1394.19</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -1901,22 +1853,22 @@
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-110.25</v>
+        <v>-484.86</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0548</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-0.3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -1925,10 +1877,10 @@
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>1039.2</v>
+        <v>248.05</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
@@ -1936,7 +1888,7 @@
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>970</v>
+        <v>242.8</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1947,19 +1899,19 @@
         <v>11</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-346</v>
+        <v>-110.25</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -1968,10 +1920,10 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>199.96</v>
+        <v>1039.2</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
@@ -1979,7 +1931,7 @@
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>193.31</v>
+        <v>970</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1990,19 +1942,19 @@
         <v>11</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-172.9</v>
+        <v>-346</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.06660000000000001</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -2011,10 +1963,10 @@
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>986.4</v>
+        <v>199.96</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -2022,7 +1974,7 @@
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>193.31</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -2033,17 +1985,60 @@
         <v>11</v>
       </c>
       <c r="I6" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J6" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K6" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I7" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="J7" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K6" s="19" t="n">
+      <c r="K7" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I6">
+  <conditionalFormatting sqref="I2:I7">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2061,7 +2056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2308,6 +2303,31 @@
       </c>
       <c r="G9" s="14" t="n">
         <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="n">
+        <v>202277.49</v>
+      </c>
+      <c r="C10" s="20" t="n">
+        <v>73072.09</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <v>129205.4</v>
+      </c>
+      <c r="E10" s="20" t="n">
+        <v>125523.15</v>
+      </c>
+      <c r="F10" s="20" t="n">
+        <v>-1404.76</v>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -2390,18 +2410,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>SOLARINDS</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1500.3</v>
+        <v>18696</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1415.27</v>
+        <v>17409.29</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -2410,10 +2430,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8571681415929203</v>
+        <v>0.8318141592920354</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -2428,18 +2448,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>17798</v>
+        <v>1517.4</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>16539.57</v>
+        <v>1433.67</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -2451,7 +2471,7 @@
         <v>6.2</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8211848574237954</v>
+        <v>0.8186922320550639</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -2466,18 +2486,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>9779</v>
+        <v>1405.2</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>9304.57</v>
+        <v>1341.39</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -2486,10 +2506,10 @@
         <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8009488692232055</v>
+        <v>0.8060963618485742</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -2504,18 +2524,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>956.25</v>
+        <v>956.6</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>906.42</v>
+        <v>903.97</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -2524,10 +2544,10 @@
         <v>5333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.2</v>
+        <v>6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7972763028515242</v>
+        <v>0.7755752212389381</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -2542,7 +2562,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
@@ -2550,10 +2570,10 @@
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>794.8</v>
+        <v>813.25</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>742.49</v>
+        <v>760.24</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -2562,10 +2582,10 @@
         <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8102704031465093</v>
+        <v>0.8011799410029499</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -2580,18 +2600,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1387.3</v>
+        <v>1578.7</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1321.89</v>
+        <v>1502.34</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -2600,10 +2620,10 @@
         <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7926106194690266</v>
+        <v>0.7767699115044249</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -2618,18 +2638,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>446.45</v>
+        <v>5081.4</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>413.02</v>
+        <v>4761.2</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -2638,10 +2658,10 @@
         <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7875860373647984</v>
+        <v>0.7860275319567355</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -2656,18 +2676,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>839.95</v>
+        <v>457.9</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>805.14</v>
+        <v>422.71</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -2676,10 +2696,10 @@
         <v>5333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7788593903638151</v>
+        <v>0.7678810226155359</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -2694,18 +2714,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>ADANIPOWER</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>227.05</v>
+        <v>836.25</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>214.06</v>
+        <v>802.99</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -2714,10 +2734,10 @@
         <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7594936086529007</v>
+        <v>0.7629301868239922</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -2732,18 +2752,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>2170.9</v>
+        <v>9961</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>2045.97</v>
+        <v>9457.290000000001</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -2752,10 +2772,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7589823008849558</v>
+        <v>0.7527138643067848</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -2770,18 +2790,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1510.8</v>
+        <v>2295.9</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1420.3</v>
+        <v>2196.27</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -2790,10 +2810,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7765339233038349</v>
+        <v>0.7637315634218289</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -2808,18 +2828,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>5541.5</v>
+        <v>1352.6</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>5245.64</v>
+        <v>1233.99</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -2828,10 +2848,10 @@
         <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7547492625368731</v>
+        <v>0.7458357915437561</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -2846,18 +2866,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1547.5</v>
+        <v>1810.2</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1472.59</v>
+        <v>1735.64</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -2866,10 +2886,10 @@
         <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7647738446411013</v>
+        <v>0.7433824975417895</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -2884,18 +2904,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>GLAND</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>963.8</v>
+        <v>2495</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>907.64</v>
+        <v>2319.49</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -2904,10 +2924,10 @@
         <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.75055063913471</v>
+        <v>0.7357866273352999</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -2922,18 +2942,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260629</v>
+        <v>20260630</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>2303.2</v>
+        <v>3945.5</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>2201.26</v>
+        <v>3764.54</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -2942,10 +2962,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7632792527040315</v>
+        <v>0.7350245821042281</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-01
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Tue 30 Jun 2026</t>
+          <t>As of Wed 01 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹202,277</t>
+          <t>₹202,128</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+1,118  (+0.56%)</t>
+          <t>₹-149  (-0.07%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.14%</t>
+          <t>+1.06%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>+0.00%</t>
+          <t>-0.07%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹129,205</t>
+          <t>₹129,056</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
@@ -796,16 +796,16 @@
         <v>4230</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>1405.2</v>
+        <v>1453.8</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>4215.6</v>
+        <v>4361.4</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>-14.39999999999986</v>
+        <v>131.3999999999999</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>-0.003404255319148904</v>
+        <v>0.03106382978723401</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>1312.63</v>
@@ -814,13 +814,13 @@
         <v>1370.6</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.02462282949046409</v>
+        <v>0.05722933003164125</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>33.1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>4788</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>770.55</v>
+        <v>763.1</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>4623.299999999999</v>
+        <v>4578.6</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-164.7000000000003</v>
+        <v>-209.3999999999999</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.03439849624060156</v>
+        <v>-0.04373433583959897</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>746.09</v>
@@ -862,13 +862,13 @@
         <v>750</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.0266692622153007</v>
+        <v>0.0171668195518281</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>22.5</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>4830</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>679.2</v>
+        <v>645.55</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>4754.400000000001</v>
+        <v>4518.849999999999</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-75.59999999999968</v>
+        <v>-311.1500000000003</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.01565217391304341</v>
+        <v>-0.06442028985507253</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>612.1900000000001</v>
@@ -910,13 +910,13 @@
         <v>612.1900000000001</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.09866018845700822</v>
+        <v>0.05167686468902471</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>34.34</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>3678</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1810.2</v>
+        <v>1848.2</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>3620.4</v>
+        <v>3696.4</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>-57.59999999999991</v>
+        <v>18.40000000000009</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>-0.01566068515497551</v>
+        <v>0.005002718868950541</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1729.61</v>
@@ -958,13 +958,13 @@
         <v>1744.3</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.03640481714727659</v>
+        <v>0.05621685964722437</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>43.14</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>4242</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1517.4</v>
+        <v>1493.3</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4552.200000000001</v>
+        <v>4479.9</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>310.2000000000003</v>
+        <v>237.8999999999999</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.07312588401697319</v>
+        <v>0.05608203677510605</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1324.47</v>
@@ -1006,13 +1006,13 @@
         <v>1391.807142857143</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.08276845732361747</v>
+        <v>0.06796548392342933</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>35.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -1036,31 +1036,31 @@
         <v>5200</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1352.6</v>
+        <v>1369.9</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>5410.4</v>
+        <v>5479.6</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>210.3999999999996</v>
+        <v>279.6000000000004</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.04046153846153839</v>
+        <v>0.05376923076923084</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1159.03</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1221.4</v>
+        <v>1252</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.09699837350288321</v>
+        <v>0.08606467625374122</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>64.73</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>5209</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>274.75</v>
+        <v>269.45</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5495</v>
+        <v>5389</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>286.0000000000002</v>
+        <v>180</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.05490497216356311</v>
+        <v>0.03455557688615857</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>240.49</v>
@@ -1102,13 +1102,13 @@
         <v>255.6500000000001</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.06951774340309338</v>
+        <v>0.05121543885693041</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>8.369999999999999</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>5252.55</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>310.85</v>
+        <v>308.65</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5906.150000000001</v>
+        <v>5864.349999999999</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>653.6000000000006</v>
+        <v>611.7999999999997</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.1244347983360464</v>
+        <v>0.1164767589075782</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>259.14</v>
@@ -1150,13 +1150,13 @@
         <v>284.4928571428572</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.08479055125347541</v>
+        <v>0.07826710791233692</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>7.11</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>4387.5</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1578.7</v>
+        <v>1552.6</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4736.1</v>
+        <v>4657.799999999999</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>348.6000000000001</v>
+        <v>270.2999999999997</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.07945299145299148</v>
+        <v>0.06160683760683754</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1405.17</v>
@@ -1198,13 +1198,13 @@
         <v>1464.164285714286</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.0725506519830965</v>
+        <v>0.05695975414512065</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>38.34</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>8690</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>813.25</v>
+        <v>811.4</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8945.75</v>
+        <v>8925.4</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>255.75</v>
+        <v>235.3999999999997</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.02943037974683544</v>
+        <v>0.02708860759493668</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>739.3099999999999</v>
@@ -1246,13 +1246,13 @@
         <v>739.3099999999999</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.09091915155241323</v>
+        <v>0.08884643825486817</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>24.04</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -1276,31 +1276,31 @@
         <v>7540</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>3945.5</v>
+        <v>3952.6</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>7891</v>
+        <v>7905.2</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>351</v>
+        <v>365.1999999999998</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.04655172413793104</v>
+        <v>0.04843501326259945</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>3604.1</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>3674.064285714286</v>
+        <v>3676.3</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.06879627785723338</v>
+        <v>0.06990335475383286</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>81.47</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>6500</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>6464.5</v>
+        <v>6541</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>6464.5</v>
+        <v>6541</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-35.5</v>
+        <v>41</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.005461538461538461</v>
+        <v>0.006307692307692308</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>6181.43</v>
@@ -1342,13 +1342,13 @@
         <v>6401.5</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.009745533297238766</v>
+        <v>0.02132701421800948</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>142.71</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
@@ -1372,31 +1372,31 @@
         <v>9031.549999999999</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>836.25</v>
+        <v>851</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>9198.75</v>
+        <v>9361</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>167.2000000000005</v>
+        <v>329.4500000000005</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.01851287984897393</v>
+        <v>0.03647768101820845</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>783.09</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>796</v>
+        <v>800.5892857142858</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.04813153961136024</v>
+        <v>0.05923703206311894</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>16.6</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>7278.3</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>2545.6</v>
+        <v>2490.3</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>7636.799999999999</v>
+        <v>7470.900000000001</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>358.5</v>
+        <v>192.6000000000008</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.04925600758418862</v>
+        <v>0.02646222332138011</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>2309.03</v>
@@ -1438,13 +1438,13 @@
         <v>2340.228571428572</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.0806770225374875</v>
+        <v>0.06026238949983053</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>59.36</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
@@ -1468,31 +1468,31 @@
         <v>9246.6</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>457.9</v>
+        <v>466.5</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>10073.8</v>
+        <v>10263</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>827.1999999999992</v>
+        <v>1016.4</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.08945990958838916</v>
+        <v>0.1099214846538187</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>386.74</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>405.1107142857143</v>
+        <v>415.4357142857143</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.1152856206907309</v>
+        <v>0.1094625631603123</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -1516,16 +1516,16 @@
         <v>8790</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>1521.9</v>
+        <v>1477.6</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>9131.400000000001</v>
+        <v>8865.599999999999</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>341.4000000000005</v>
+        <v>75.59999999999945</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>0.03883959044368607</v>
+        <v>0.008600682593856592</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>1365.41</v>
@@ -1534,13 +1534,13 @@
         <v>1397.635714285714</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>0.08165075610374251</v>
+        <v>0.05411768118183917</v>
       </c>
       <c r="M17" s="13" t="n">
         <v>45.25</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -1564,16 +1564,16 @@
         <v>9288.75</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>619.9</v>
+        <v>619.4</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>9298.5</v>
+        <v>9291</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>9.749999999999659</v>
+        <v>2.249999999999659</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>0.001049656842955151</v>
+        <v>0.0002422285022203912</v>
       </c>
       <c r="J18" s="7" t="n">
         <v>591.46</v>
@@ -1582,13 +1582,13 @@
         <v>591.46</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>0.04587836747862549</v>
+        <v>0.04510816919599603</v>
       </c>
       <c r="M18" s="13" t="n">
         <v>14</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -1612,16 +1612,16 @@
         <v>8700</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>8682</v>
+        <v>8618.5</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>8682</v>
+        <v>8618.5</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>-18</v>
+        <v>-81.5</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>-0.002068965517241379</v>
+        <v>-0.009367816091954024</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>8339.209999999999</v>
@@ -1630,13 +1630,13 @@
         <v>8339.209999999999</v>
       </c>
       <c r="L19" s="12" t="n">
-        <v>0.03948283805574762</v>
+        <v>0.03240587109125728</v>
       </c>
       <c r="M19" s="13" t="n">
         <v>123.68</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -1660,31 +1660,31 @@
         <v>8640.9</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>952.15</v>
+        <v>976.5</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>8569.35</v>
+        <v>8788.5</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>-71.55000000000041</v>
+        <v>147.5999999999998</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>-0.008280387459639669</v>
+        <v>0.01708155400479114</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>893.91</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>893.91</v>
+        <v>902.6785714285714</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>0.06116683295699208</v>
+        <v>0.07559798112793503</v>
       </c>
       <c r="M20" s="13" t="n">
         <v>24.91</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2056,7 +2056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2327,6 +2327,31 @@
         <v>-1404.76</v>
       </c>
       <c r="G10" s="14" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="n">
+        <v>202128.09</v>
+      </c>
+      <c r="C11" s="20" t="n">
+        <v>73072.09</v>
+      </c>
+      <c r="D11" s="20" t="n">
+        <v>129056</v>
+      </c>
+      <c r="E11" s="20" t="n">
+        <v>125523.15</v>
+      </c>
+      <c r="F11" s="20" t="n">
+        <v>-1404.76</v>
+      </c>
+      <c r="G11" s="14" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2410,30 +2435,30 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>18696</v>
+        <v>1848.2</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>17409.29</v>
+        <v>1769.07</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.3</v>
+        <v>7.1</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8318141592920354</v>
+        <v>0.8376401179941003</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -2442,36 +2467,36 @@
       </c>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1517.4</v>
+        <v>1453.8</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1433.67</v>
+        <v>1385.76</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.2</v>
+        <v>6.8</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8186922320550639</v>
+        <v>0.7947984267453294</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -2480,36 +2505,36 @@
       </c>
       <c r="J3" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>ADANIPOWER</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1405.2</v>
+        <v>226.86</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1341.39</v>
+        <v>214.1</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.1</v>
+        <v>6.8</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8060963618485742</v>
+        <v>0.7809537856440512</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -2518,36 +2543,36 @@
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>SOLARINDS</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>956.6</v>
+        <v>18610</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>903.97</v>
+        <v>17390</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6</v>
+        <v>6.6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7755752212389381</v>
+        <v>0.7751819075712881</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -2556,36 +2581,36 @@
       </c>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>813.25</v>
+        <v>1493.3</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>760.24</v>
+        <v>1407.01</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>5.9</v>
+        <v>6.6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8011799410029499</v>
+        <v>0.7629203539823008</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -2594,36 +2619,36 @@
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1578.7</v>
+        <v>811.4</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1502.34</v>
+        <v>759.4400000000001</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.9</v>
+        <v>6.5</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7767699115044249</v>
+        <v>0.7706588003933137</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -2632,36 +2657,36 @@
       </c>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>5081.4</v>
+        <v>976.5</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>4761.2</v>
+        <v>927.29</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7860275319567355</v>
+        <v>0.748166175024582</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -2670,36 +2695,36 @@
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>457.9</v>
+        <v>9713.5</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>422.71</v>
+        <v>9190.360000000001</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7678810226155359</v>
+        <v>0.7434070796460177</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -2708,36 +2733,36 @@
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>836.25</v>
+        <v>1477.6</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>802.99</v>
+        <v>1388.64</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.8</v>
+        <v>6.4</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7629301868239922</v>
+        <v>0.7486676499508358</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -2746,36 +2771,36 @@
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>9961</v>
+        <v>939.7</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>9457.290000000001</v>
+        <v>886.1799999999999</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.8</v>
+        <v>6.4</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7527138643067848</v>
+        <v>0.7304375614552605</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -2784,36 +2809,36 @@
       </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>OFSS</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>2295.9</v>
+        <v>10863</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>2196.27</v>
+        <v>10135.79</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.7</v>
+        <v>6.4</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7637315634218289</v>
+        <v>0.7224827925270403</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -2822,36 +2847,36 @@
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>TATATECH</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1352.6</v>
+        <v>670.2</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1233.99</v>
+        <v>624.83</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7458357915437561</v>
+        <v>0.7116371681415929</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -2860,36 +2885,36 @@
       </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1810.2</v>
+        <v>4996</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1735.64</v>
+        <v>4656.97</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7433824975417895</v>
+        <v>0.7218534906588004</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -2898,36 +2923,36 @@
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>GLAND</t>
+          <t>NMDC</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>2495</v>
+        <v>84.3</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>2319.49</v>
+        <v>80.09</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7357866273352999</v>
+        <v>0.7074877089478859</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -2936,36 +2961,36 @@
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260630</v>
+        <v>20260701</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>3945.5</v>
+        <v>605.85</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>3764.54</v>
+        <v>570.6799999999999</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.7</v>
+        <v>6.1</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7350245821042281</v>
+        <v>0.7277335299901672</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>
@@ -2974,7 +2999,7 @@
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-02
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Wed 01 Jul 2026</t>
+          <t>As of Thu 02 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹202,128</t>
+          <t>₹203,718</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-149  (-0.07%)</t>
+          <t>₹+1,589  (+0.79%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.06%</t>
+          <t>+1.86%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.07%</t>
+          <t>+0.00%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹129,056</t>
+          <t>₹130,645</t>
         </is>
       </c>
     </row>
@@ -796,16 +796,16 @@
         <v>4230</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>1453.8</v>
+        <v>1446.2</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>4361.4</v>
+        <v>4338.6</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>131.3999999999999</v>
+        <v>108.6000000000001</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.03106382978723401</v>
+        <v>0.02567375886524826</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>1312.63</v>
@@ -814,13 +814,13 @@
         <v>1370.6</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.05722933003164125</v>
+        <v>0.05227492739593426</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>33.1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>4788</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>763.1</v>
+        <v>772.35</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>4578.6</v>
+        <v>4634.1</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-209.3999999999999</v>
+        <v>-153.8999999999999</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.04373433583959897</v>
+        <v>-0.03214285714285711</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>746.09</v>
@@ -862,13 +862,13 @@
         <v>750</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.0171668195518281</v>
+        <v>0.02893765779763064</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>22.5</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>4830</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>645.55</v>
+        <v>662.65</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>4518.849999999999</v>
+        <v>4638.55</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-311.1500000000003</v>
+        <v>-191.4500000000002</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.06442028985507253</v>
+        <v>-0.03963768115942033</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>612.1900000000001</v>
@@ -910,13 +910,13 @@
         <v>612.1900000000001</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.05167686468902471</v>
+        <v>0.0761487964989058</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>34.34</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>3678</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1848.2</v>
+        <v>1883.2</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>3696.4</v>
+        <v>3766.4</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>18.40000000000009</v>
+        <v>88.40000000000009</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.005002718868950541</v>
+        <v>0.02403480152256664</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1729.61</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1744.3</v>
+        <v>1763.992857142857</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.05621685964722437</v>
+        <v>0.0633003095035805</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>43.14</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>4242</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1493.3</v>
+        <v>1528</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4479.9</v>
+        <v>4584</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>237.8999999999999</v>
+        <v>342</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.05608203677510605</v>
+        <v>0.08062234794908062</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1324.47</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1391.807142857143</v>
+        <v>1394.757142857143</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.06796548392342933</v>
+        <v>0.08720082273747203</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>35.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>5200</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1369.9</v>
+        <v>1397.8</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>5479.6</v>
+        <v>5591.2</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>279.6000000000004</v>
+        <v>391.1999999999998</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.05376923076923084</v>
+        <v>0.0752307692307692</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1159.03</v>
@@ -1054,13 +1054,13 @@
         <v>1252</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.08606467625374122</v>
+        <v>0.1043067677779367</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>64.73</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>5209</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>269.45</v>
+        <v>274.15</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5389</v>
+        <v>5483</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>180</v>
+        <v>273.9999999999998</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.03455557688615857</v>
+        <v>0.05260126703781912</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>240.49</v>
@@ -1102,13 +1102,13 @@
         <v>255.6500000000001</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.05121543885693041</v>
+        <v>0.06748130585445883</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>8.369999999999999</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -1132,31 +1132,31 @@
         <v>5252.55</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>308.65</v>
+        <v>314</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5864.349999999999</v>
+        <v>5966</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>611.7999999999997</v>
+        <v>713.4500000000003</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.1164767589075782</v>
+        <v>0.1358292638813529</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>259.14</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>284.4928571428572</v>
+        <v>289.2285714285714</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.07826710791233692</v>
+        <v>0.07888989990900828</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>7.11</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>4387.5</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1552.6</v>
+        <v>1561</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4657.799999999999</v>
+        <v>4683</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>270.2999999999997</v>
+        <v>295.5</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.06160683760683754</v>
+        <v>0.06735042735042734</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1405.17</v>
@@ -1198,13 +1198,13 @@
         <v>1464.164285714286</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.05695975414512065</v>
+        <v>0.06203441017662678</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>38.34</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11">
@@ -1228,31 +1228,31 @@
         <v>8690</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>811.4</v>
+        <v>825.7</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8925.4</v>
+        <v>9082.700000000001</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>235.3999999999997</v>
+        <v>392.7000000000005</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.02708860759493668</v>
+        <v>0.04518987341772158</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>739.3099999999999</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>739.3099999999999</v>
+        <v>745.9107142857143</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.08884643825486817</v>
+        <v>0.09663229467637847</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>24.04</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -1276,31 +1276,31 @@
         <v>7540</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>3952.6</v>
+        <v>3972.4</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>7905.2</v>
+        <v>7944.8</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>365.1999999999998</v>
+        <v>404.8000000000002</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.04843501326259945</v>
+        <v>0.05368700265251992</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>3604.1</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>3676.3</v>
+        <v>3700.921428571429</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.06990335475383286</v>
+        <v>0.06834119711725185</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>81.47</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>6500</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>6541</v>
+        <v>6469.5</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>6541</v>
+        <v>6469.5</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>41</v>
+        <v>-30.5</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.006307692307692308</v>
+        <v>-0.004692307692307693</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>6181.43</v>
@@ -1342,13 +1342,13 @@
         <v>6401.5</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.02132701421800948</v>
+        <v>0.01051085864440838</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>142.71</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -1372,31 +1372,31 @@
         <v>9031.549999999999</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>9361</v>
+        <v>9416</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>329.4500000000005</v>
+        <v>384.4500000000005</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.03647768101820845</v>
+        <v>0.04256744412642354</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>783.09</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>800.5892857142858</v>
+        <v>805.2571428571429</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.05923703206311894</v>
+        <v>0.05927903871829104</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>16.6</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>7278.3</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>2490.3</v>
+        <v>2486.9</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>7470.900000000001</v>
+        <v>7460.700000000001</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>192.6000000000008</v>
+        <v>182.4000000000005</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.02646222332138011</v>
+        <v>0.02506079716417303</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>2309.03</v>
@@ -1438,13 +1438,13 @@
         <v>2340.228571428572</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.06026238949983053</v>
+        <v>0.05897761412659451</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>59.36</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
@@ -1468,31 +1468,31 @@
         <v>9246.6</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>466.5</v>
+        <v>469.5</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>10263</v>
+        <v>10329</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>1016.4</v>
+        <v>1082.4</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.1099214846538187</v>
+        <v>0.1170592433975731</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>386.74</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>415.4357142857143</v>
+        <v>419.8285714285714</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.1094625631603123</v>
+        <v>0.1057964399817435</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -1516,16 +1516,16 @@
         <v>8790</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>1477.6</v>
+        <v>1498.8</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>8865.599999999999</v>
+        <v>8992.799999999999</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>75.59999999999945</v>
+        <v>202.7999999999997</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>0.008600682593856592</v>
+        <v>0.02307167235494877</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>1365.41</v>
@@ -1534,13 +1534,13 @@
         <v>1397.635714285714</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>0.05411768118183917</v>
+        <v>0.06749685462655831</v>
       </c>
       <c r="M17" s="13" t="n">
         <v>45.25</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -1564,31 +1564,31 @@
         <v>9288.75</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>619.4</v>
+        <v>662.3</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>9291</v>
+        <v>9934.5</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>2.249999999999659</v>
+        <v>645.7499999999993</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>0.0002422285022203912</v>
+        <v>0.06951958013726274</v>
       </c>
       <c r="J18" s="7" t="n">
         <v>591.46</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>591.46</v>
+        <v>611.3321428571427</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>0.04510816919599603</v>
+        <v>0.07695584650891933</v>
       </c>
       <c r="M18" s="13" t="n">
         <v>14</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -1612,16 +1612,16 @@
         <v>8700</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>8618.5</v>
+        <v>8696</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>8618.5</v>
+        <v>8696</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>-81.5</v>
+        <v>-4</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>-0.009367816091954024</v>
+        <v>-0.0004597701149425287</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>8339.209999999999</v>
@@ -1630,13 +1630,13 @@
         <v>8339.209999999999</v>
       </c>
       <c r="L19" s="12" t="n">
-        <v>0.03240587109125728</v>
+        <v>0.04102920883164683</v>
       </c>
       <c r="M19" s="13" t="n">
         <v>123.68</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -1660,16 +1660,16 @@
         <v>8640.9</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>976.5</v>
+        <v>959.4</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>8788.5</v>
+        <v>8634.6</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>147.5999999999998</v>
+        <v>-6.300000000000409</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>0.01708155400479114</v>
+        <v>-0.0007290907197167435</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>893.91</v>
@@ -1678,13 +1678,13 @@
         <v>902.6785714285714</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>0.07559798112793503</v>
+        <v>0.05912177253640664</v>
       </c>
       <c r="M20" s="13" t="n">
         <v>24.91</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -2056,7 +2056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2352,6 +2352,31 @@
         <v>-1404.76</v>
       </c>
       <c r="G11" s="14" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="n">
+        <v>203717.54</v>
+      </c>
+      <c r="C12" s="20" t="n">
+        <v>73072.09</v>
+      </c>
+      <c r="D12" s="20" t="n">
+        <v>130645.45</v>
+      </c>
+      <c r="E12" s="20" t="n">
+        <v>125523.15</v>
+      </c>
+      <c r="F12" s="20" t="n">
+        <v>-1404.76</v>
+      </c>
+      <c r="G12" s="14" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2435,18 +2460,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1848.2</v>
+        <v>1528</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1769.07</v>
+        <v>1439.17</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -2455,10 +2480,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8376401179941003</v>
+        <v>0.8016420845624386</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -2473,18 +2498,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1453.8</v>
+        <v>959.4</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1385.76</v>
+        <v>909.11</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -2496,7 +2521,7 @@
         <v>6.8</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.7947984267453294</v>
+        <v>0.7959537856440511</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -2511,18 +2536,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>ADANIPOWER</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>226.86</v>
+        <v>1883.2</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>214.1</v>
+        <v>1803.73</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -2534,7 +2559,7 @@
         <v>6.8</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7809537856440512</v>
+        <v>0.7942625368731564</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -2549,18 +2574,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>18610</v>
+        <v>825.7</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>17390</v>
+        <v>772.51</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -2569,10 +2594,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7751819075712881</v>
+        <v>0.8127138643067846</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -2587,18 +2612,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1493.3</v>
+        <v>662.3</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1407.01</v>
+        <v>628.3200000000001</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -2607,10 +2632,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7629203539823008</v>
+        <v>0.7684267453294003</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -2625,18 +2650,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>BSE</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>811.4</v>
+        <v>3834.7</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>759.4400000000001</v>
+        <v>3603.03</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -2648,7 +2673,7 @@
         <v>6.5</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7706588003933137</v>
+        <v>0.7209783677482793</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -2663,18 +2688,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>976.5</v>
+        <v>772.35</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>927.29</v>
+        <v>727.95</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -2683,10 +2708,10 @@
         <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.748166175024582</v>
+        <v>0.7537069813176007</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -2701,7 +2726,7 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
@@ -2709,10 +2734,10 @@
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>9713.5</v>
+        <v>9635</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>9190.360000000001</v>
+        <v>9114.709999999999</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -2721,10 +2746,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7434070796460177</v>
+        <v>0.7266273352999016</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -2739,18 +2764,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1477.6</v>
+        <v>9857</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1388.64</v>
+        <v>9438.860000000001</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -2762,7 +2787,7 @@
         <v>6.4</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7486676499508358</v>
+        <v>0.7348672566371681</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -2777,18 +2802,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>OFSS</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>939.7</v>
+        <v>10986</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>886.1799999999999</v>
+        <v>10226</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -2800,7 +2825,7 @@
         <v>6.4</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7304375614552605</v>
+        <v>0.7348328416912489</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -2815,18 +2840,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>OFSS</t>
+          <t>SOLARINDS</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>10863</v>
+        <v>18659</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>10135.79</v>
+        <v>17449</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -2835,10 +2860,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7224827925270403</v>
+        <v>0.7311504424778761</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -2853,18 +2878,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>TATATECH</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>670.2</v>
+        <v>1446.2</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>624.83</v>
+        <v>1384.8</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -2873,10 +2898,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7116371681415929</v>
+        <v>0.7208800393313668</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -2891,18 +2916,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>4996</v>
+        <v>962.35</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>4656.97</v>
+        <v>914.71</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -2911,10 +2936,10 @@
         <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7218534906588004</v>
+        <v>0.7453638151425762</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -2929,18 +2954,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>NMDC</t>
+          <t>THERMAX</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>84.3</v>
+        <v>4917</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>80.09</v>
+        <v>4522.46</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -2949,10 +2974,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7074877089478859</v>
+        <v>0.72055063913471</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -2967,7 +2992,7 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260701</v>
+        <v>20260702</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
@@ -2975,10 +3000,10 @@
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>605.85</v>
+        <v>594</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>570.6799999999999</v>
+        <v>558.33</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -2987,10 +3012,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7277335299901672</v>
+        <v>0.749228121927237</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-03
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Thu 02 Jul 2026</t>
+          <t>As of Fri 03 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹203,718</t>
+          <t>₹202,887</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+1,589  (+0.79%)</t>
+          <t>₹-831  (-0.41%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.86%</t>
+          <t>+1.44%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>+0.00%</t>
+          <t>-0.41%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹73,072</t>
+          <t>₹81,196</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹125,523</t>
+          <t>₹116,882</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹130,645</t>
+          <t>₹121,691</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹-1,405</t>
+          <t>₹-1,922</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -796,31 +796,31 @@
         <v>4230</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>1446.2</v>
+        <v>1459.8</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>4338.6</v>
+        <v>4379.4</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>108.6000000000001</v>
+        <v>149.3999999999999</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.02567375886524826</v>
+        <v>0.03531914893617018</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>1312.63</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1370.6</v>
+        <v>1371.878571428571</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.05227492739593426</v>
+        <v>0.06022840702248841</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>33.1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>4788</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>772.35</v>
+        <v>770.9</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>4634.1</v>
+        <v>4625.4</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-153.8999999999999</v>
+        <v>-162.6000000000001</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.03214285714285711</v>
+        <v>-0.03395989974937346</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>746.09</v>
@@ -862,13 +862,13 @@
         <v>750</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.02893765779763064</v>
+        <v>0.02711116876378256</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>22.5</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>4830</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>662.65</v>
+        <v>680.65</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>4638.55</v>
+        <v>4764.55</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-191.4500000000002</v>
+        <v>-65.45000000000016</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.03963768115942033</v>
+        <v>-0.01355072463768119</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>612.1900000000001</v>
@@ -910,13 +910,13 @@
         <v>612.1900000000001</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.0761487964989058</v>
+        <v>0.1005803276280025</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>34.34</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>3678</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1883.2</v>
+        <v>1874.2</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>3766.4</v>
+        <v>3748.4</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>88.40000000000009</v>
+        <v>70.40000000000009</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.02403480152256664</v>
+        <v>0.01914083741163678</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1729.61</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1763.992857142857</v>
+        <v>1767.271428571428</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.0633003095035805</v>
+        <v>0.05705291400521372</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>43.14</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>4242</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1528</v>
+        <v>1542.3</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4584</v>
+        <v>4626.9</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>342</v>
+        <v>384.8999999999999</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.08062234794908062</v>
+        <v>0.09073550212164071</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1324.47</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1394.757142857143</v>
+        <v>1409.035714285714</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.08720082273747203</v>
+        <v>0.08640620223969768</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>35.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>5200</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1397.8</v>
+        <v>1365.2</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>5591.2</v>
+        <v>5460.8</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>391.1999999999998</v>
+        <v>260.8000000000002</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.0752307692307692</v>
+        <v>0.05015384615384619</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1159.03</v>
@@ -1054,13 +1054,13 @@
         <v>1252</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.1043067677779367</v>
+        <v>0.08291825373571642</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>64.73</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8">
@@ -1084,31 +1084,31 @@
         <v>5209</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>274.15</v>
+        <v>270.8</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5483</v>
+        <v>5416</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>273.9999999999998</v>
+        <v>207.0000000000005</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.05260126703781912</v>
+        <v>0.03973891341908244</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>240.49</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>255.6500000000001</v>
+        <v>256.2178571428572</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.06748130585445883</v>
+        <v>0.05384838573538699</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>8.369999999999999</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>5252.55</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>314</v>
+        <v>310.3</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5966</v>
+        <v>5895.7</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>713.4500000000003</v>
+        <v>643.1500000000004</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.1358292638813529</v>
+        <v>0.1224452884789294</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>259.14</v>
@@ -1150,13 +1150,13 @@
         <v>289.2285714285714</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.07888989990900828</v>
+        <v>0.06790663413286693</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>7.11</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>4387.5</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1561</v>
+        <v>1620.5</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4683</v>
+        <v>4861.5</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>295.5</v>
+        <v>474</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.06735042735042734</v>
+        <v>0.108034188034188</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1405.17</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1464.164285714286</v>
+        <v>1502.471428571428</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.06203441017662678</v>
+        <v>0.07283466302287671</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>38.34</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11">
@@ -1228,31 +1228,31 @@
         <v>8690</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>825.7</v>
+        <v>833.8</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>9082.700000000001</v>
+        <v>9171.799999999999</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>392.7000000000005</v>
+        <v>481.7999999999995</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.04518987341772158</v>
+        <v>0.05544303797468349</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>739.3099999999999</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>745.9107142857143</v>
+        <v>757.8357142857143</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.09663229467637847</v>
+        <v>0.09110612342802311</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>24.04</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>7540</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>3972.4</v>
+        <v>3892.3</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>7944.8</v>
+        <v>7784.6</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>404.8000000000002</v>
+        <v>244.6000000000004</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.05368700265251992</v>
+        <v>0.03244031830238732</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>3604.1</v>
@@ -1294,13 +1294,13 @@
         <v>3700.921428571429</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.06834119711725185</v>
+        <v>0.04916850485023543</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>81.47</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>6500</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>6469.5</v>
+        <v>6556.5</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>6469.5</v>
+        <v>6556.5</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-30.5</v>
+        <v>56.5</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.004692307692307693</v>
+        <v>0.008692307692307692</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>6181.43</v>
@@ -1342,13 +1342,13 @@
         <v>6401.5</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.01051085864440838</v>
+        <v>0.02364066193853428</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>142.71</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>9031.549999999999</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>856</v>
+        <v>838.55</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>9416</v>
+        <v>9224.049999999999</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>384.4500000000005</v>
+        <v>192.5</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.04256744412642354</v>
+        <v>0.02131417087875282</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>783.09</v>
@@ -1390,13 +1390,13 @@
         <v>805.2571428571429</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.05927903871829104</v>
+        <v>0.03970288848948433</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>16.6</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>7278.3</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>2486.9</v>
+        <v>2528.6</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>7460.700000000001</v>
+        <v>7585.799999999999</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>182.4000000000005</v>
+        <v>307.5</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.02506079716417303</v>
+        <v>0.04224887679815342</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>2309.03</v>
@@ -1438,13 +1438,13 @@
         <v>2340.228571428572</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.05897761412659451</v>
+        <v>0.07449633337476379</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>59.36</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16">
@@ -1468,31 +1468,31 @@
         <v>9246.6</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>469.5</v>
+        <v>461.75</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>10329</v>
+        <v>10158.5</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>1082.4</v>
+        <v>911.8999999999997</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.1170592433975731</v>
+        <v>0.09862003330954078</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>386.74</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>419.8285714285714</v>
+        <v>420.1285714285714</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.1057964399817435</v>
+        <v>0.09013844844922279</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
@@ -1516,16 +1516,16 @@
         <v>8790</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>1498.8</v>
+        <v>1439.3</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>8992.799999999999</v>
+        <v>8635.799999999999</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>202.7999999999997</v>
+        <v>-154.2000000000003</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>0.02307167235494877</v>
+        <v>-0.01754266211604099</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>1365.41</v>
@@ -1534,13 +1534,13 @@
         <v>1397.635714285714</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>0.06749685462655831</v>
+        <v>0.02894760349773195</v>
       </c>
       <c r="M17" s="13" t="n">
         <v>45.25</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
@@ -1564,31 +1564,31 @@
         <v>9288.75</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>662.3</v>
+        <v>660.1</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>9934.5</v>
+        <v>9901.5</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>645.7499999999993</v>
+        <v>612.7500000000003</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>0.06951958013726274</v>
+        <v>0.06596689543802992</v>
       </c>
       <c r="J18" s="7" t="n">
         <v>591.46</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>611.3321428571427</v>
+        <v>611.342857142857</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>0.07695584650891933</v>
+        <v>0.07386326747029689</v>
       </c>
       <c r="M18" s="13" t="n">
         <v>14</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
@@ -1612,83 +1612,35 @@
         <v>8700</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>8696</v>
+        <v>8893.5</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>8696</v>
+        <v>8893.5</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>-4</v>
+        <v>193.5</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>-0.0004597701149425287</v>
+        <v>0.02224137931034483</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>8339.209999999999</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>8339.209999999999</v>
+        <v>8503.071428571429</v>
       </c>
       <c r="L19" s="12" t="n">
-        <v>0.04102920883164683</v>
+        <v>0.04390044093198073</v>
       </c>
       <c r="M19" s="13" t="n">
         <v>123.68</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>CGPOWER</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>960.1</v>
-      </c>
-      <c r="D20" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="E20" s="9" t="n">
-        <v>8640.9</v>
-      </c>
-      <c r="F20" s="7" t="n">
-        <v>959.4</v>
-      </c>
-      <c r="G20" s="9" t="n">
-        <v>8634.6</v>
-      </c>
-      <c r="H20" s="10" t="n">
-        <v>-6.300000000000409</v>
-      </c>
-      <c r="I20" s="11" t="n">
-        <v>-0.0007290907197167435</v>
-      </c>
-      <c r="J20" s="7" t="n">
-        <v>893.91</v>
-      </c>
-      <c r="K20" s="7" t="n">
-        <v>902.6785714285714</v>
-      </c>
-      <c r="L20" s="12" t="n">
-        <v>0.05912177253640664</v>
-      </c>
-      <c r="M20" s="13" t="n">
-        <v>24.91</v>
-      </c>
-      <c r="N20" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H20">
+  <conditionalFormatting sqref="H2:H19">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1706,7 +1658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1782,7 +1734,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -1791,18 +1743,18 @@
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>952.1</v>
+        <v>960.1</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>948.8</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -1810,42 +1762,42 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-29.7</v>
+        <v>-516.79</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.0598</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>1475</v>
+        <v>952.1</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>1394.19</v>
+        <v>948.8</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -1853,42 +1805,42 @@
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-484.86</v>
+        <v>-29.7</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0035</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-1</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>248.05</v>
+        <v>1475</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>242.8</v>
+        <v>1394.19</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1896,22 +1848,22 @@
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-110.25</v>
+        <v>-484.86</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0548</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-0.3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -1920,10 +1872,10 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>1039.2</v>
+        <v>248.05</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
@@ -1931,7 +1883,7 @@
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>970</v>
+        <v>242.8</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1942,19 +1894,19 @@
         <v>11</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-346</v>
+        <v>-110.25</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -1963,10 +1915,10 @@
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>199.96</v>
+        <v>1039.2</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -1974,7 +1926,7 @@
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>193.31</v>
+        <v>970</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -1985,19 +1937,19 @@
         <v>11</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>-172.9</v>
+        <v>-346</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.06660000000000001</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -2006,10 +1958,10 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>986.4</v>
+        <v>199.96</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
@@ -2017,7 +1969,7 @@
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>193.31</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -2028,17 +1980,60 @@
         <v>11</v>
       </c>
       <c r="I7" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J7" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K7" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I8" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J7" s="18" t="n">
+      <c r="J8" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K7" s="19" t="n">
+      <c r="K8" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I7">
+  <conditionalFormatting sqref="I2:I8">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2056,7 +2051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2378,6 +2373,31 @@
       </c>
       <c r="G12" s="14" t="n">
         <v>19</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="n">
+        <v>202886.9</v>
+      </c>
+      <c r="C13" s="20" t="n">
+        <v>81196.2</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <v>121690.7</v>
+      </c>
+      <c r="E13" s="20" t="n">
+        <v>116882.25</v>
+      </c>
+      <c r="F13" s="20" t="n">
+        <v>-1921.55</v>
+      </c>
+      <c r="G13" s="14" t="n">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -2460,7 +2480,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -2468,10 +2488,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1528</v>
+        <v>1542.3</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1439.17</v>
+        <v>1453.46</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -2480,10 +2500,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.8</v>
+        <v>7</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8016420845624386</v>
+        <v>0.8264454277286135</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -2498,7 +2518,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
@@ -2506,10 +2526,10 @@
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>959.4</v>
+        <v>892.55</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>909.11</v>
+        <v>836</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -2518,10 +2538,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.8</v>
+        <v>7</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.7959537856440511</v>
+        <v>0.7961799410029499</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -2536,18 +2556,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1883.2</v>
+        <v>833.8</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1803.73</v>
+        <v>783.16</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -2556,10 +2576,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7942625368731564</v>
+        <v>0.8129301868239921</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -2574,18 +2594,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>825.7</v>
+        <v>1439.3</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>772.51</v>
+        <v>1342.31</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -2594,10 +2614,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8127138643067846</v>
+        <v>0.7727728613569321</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -2612,18 +2632,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>662.3</v>
+        <v>8893.5</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>628.3200000000001</v>
+        <v>8633.209999999999</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -2632,10 +2652,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7684267453294003</v>
+        <v>0.7722959685349067</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -2650,18 +2670,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>BSE</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>3834.7</v>
+        <v>1620.5</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>3603.03</v>
+        <v>1541.81</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -2670,10 +2690,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7209783677482793</v>
+        <v>0.7688200589970501</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -2688,18 +2708,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>772.35</v>
+        <v>838.55</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>727.95</v>
+        <v>802.13</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -2708,10 +2728,10 @@
         <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7537069813176007</v>
+        <v>0.7575663716814159</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -2726,18 +2746,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>9635</v>
+        <v>5478</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>9114.709999999999</v>
+        <v>5171.64</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -2746,10 +2766,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7266273352999016</v>
+        <v>0.7476745329400196</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -2764,18 +2784,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>9857</v>
+        <v>7552.5</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>9438.860000000001</v>
+        <v>7128.14</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -2784,10 +2804,10 @@
         <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7348672566371681</v>
+        <v>0.7650491642084563</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -2802,18 +2822,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>OFSS</t>
+          <t>SOLARINDS</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>10986</v>
+        <v>18514</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>10226</v>
+        <v>17279.57</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -2825,7 +2845,7 @@
         <v>6.4</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7348328416912489</v>
+        <v>0.7397738446411013</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -2840,18 +2860,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>18659</v>
+        <v>1778.9</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>17449</v>
+        <v>1680.3</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -2860,10 +2880,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7311504424778761</v>
+        <v>0.753874139626352</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -2878,18 +2898,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1446.2</v>
+        <v>1874.2</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1384.8</v>
+        <v>1796.91</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -2898,10 +2918,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7208800393313668</v>
+        <v>0.7318879056047197</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -2916,18 +2936,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>962.35</v>
+        <v>1459.8</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>914.71</v>
+        <v>1401.19</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -2936,10 +2956,10 @@
         <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7453638151425762</v>
+        <v>0.7400737463126844</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -2954,18 +2974,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>THERMAX</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>4917</v>
+        <v>578.55</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>4522.46</v>
+        <v>541.78</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -2977,7 +2997,7 @@
         <v>6.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.72055063913471</v>
+        <v>0.7740363815142576</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -2992,18 +3012,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260702</v>
+        <v>20260703</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>594</v>
+        <v>955.1</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>558.33</v>
+        <v>908.65</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -3012,10 +3032,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.749228121927237</v>
+        <v>0.7628564405113076</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-06
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Fri 03 Jul 2026</t>
+          <t>As of Mon 06 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹202,887</t>
+          <t>₹205,022</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-831  (-0.41%)</t>
+          <t>₹+2,135  (+1.05%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.44%</t>
+          <t>+2.51%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.41%</t>
+          <t>+0.00%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹81,196</t>
+          <t>₹32,316</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹116,882</t>
+          <t>₹165,762</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹121,691</t>
+          <t>₹172,706</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>24</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -796,31 +796,31 @@
         <v>4230</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>1459.8</v>
+        <v>1473.7</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>4379.4</v>
+        <v>4421.1</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>149.3999999999999</v>
+        <v>191.1000000000001</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.03531914893617018</v>
+        <v>0.04517730496453904</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>1312.63</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1371.878571428571</v>
+        <v>1386.914285714286</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.06022840702248841</v>
+        <v>0.05888967516164378</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>33.1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>4788</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>770.9</v>
+        <v>774.05</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>4625.4</v>
+        <v>4644.299999999999</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-162.6000000000001</v>
+        <v>-143.7000000000003</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.03395989974937346</v>
+        <v>-0.03001253132832086</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>746.09</v>
@@ -862,13 +862,13 @@
         <v>750</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.02711116876378256</v>
+        <v>0.03107034429300427</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>22.5</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>4830</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>680.65</v>
+        <v>684.15</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>4764.55</v>
+        <v>4789.05</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-65.45000000000016</v>
+        <v>-40.95000000000016</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.01355072463768119</v>
+        <v>-0.008478260869565251</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>612.1900000000001</v>
@@ -910,13 +910,13 @@
         <v>612.1900000000001</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.1005803276280025</v>
+        <v>0.1051816122195424</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>34.34</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>3678</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1874.2</v>
+        <v>1864.4</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>3748.4</v>
+        <v>3728.8</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>70.40000000000009</v>
+        <v>50.80000000000018</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.01914083741163678</v>
+        <v>0.0138118542686243</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1729.61</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1767.271428571428</v>
+        <v>1768.707142857143</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.05705291400521372</v>
+        <v>0.05132635547246154</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>43.14</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>4242</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1542.3</v>
+        <v>1529.2</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4626.9</v>
+        <v>4587.6</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>384.8999999999999</v>
+        <v>345.6000000000001</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.09073550212164071</v>
+        <v>0.08147100424328151</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1324.47</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1409.035714285714</v>
+        <v>1414.35</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.08640620223969768</v>
+        <v>0.07510462987182849</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>35.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>5200</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1365.2</v>
+        <v>1347.4</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>5460.8</v>
+        <v>5389.6</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>260.8000000000002</v>
+        <v>189.6000000000004</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.05015384615384619</v>
+        <v>0.03646153846153853</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1159.03</v>
@@ -1054,13 +1054,13 @@
         <v>1252</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.08291825373571642</v>
+        <v>0.07080302805403005</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>64.73</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -1084,31 +1084,31 @@
         <v>5209</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>270.8</v>
+        <v>272.3</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5416</v>
+        <v>5446</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>207.0000000000005</v>
+        <v>237.0000000000005</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.03973891341908244</v>
+        <v>0.04549817623344221</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>240.49</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>256.2178571428572</v>
+        <v>256.7214285714286</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.05384838573538699</v>
+        <v>0.05721105923089027</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>8.369999999999999</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>5252.55</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>310.3</v>
+        <v>313.5</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5895.7</v>
+        <v>5956.5</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>643.1500000000004</v>
+        <v>703.9500000000003</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.1224452884789294</v>
+        <v>0.1340206185567011</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>259.14</v>
@@ -1150,13 +1150,13 @@
         <v>289.2285714285714</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.06790663413286693</v>
+        <v>0.07742082478924593</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>7.11</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>4387.5</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1620.5</v>
+        <v>1594.6</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4861.5</v>
+        <v>4783.799999999999</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>474</v>
+        <v>396.2999999999997</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.108034188034188</v>
+        <v>0.09032478632478626</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1405.17</v>
@@ -1198,13 +1198,13 @@
         <v>1502.471428571428</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.07283466302287671</v>
+        <v>0.05777534894554848</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>38.34</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11">
@@ -1228,31 +1228,31 @@
         <v>8690</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>833.8</v>
+        <v>854.2</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>9171.799999999999</v>
+        <v>9396.200000000001</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>481.7999999999995</v>
+        <v>706.2000000000005</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.05544303797468349</v>
+        <v>0.08126582278481019</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>739.3099999999999</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>757.8357142857143</v>
+        <v>774.0785714285714</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.09110612342802311</v>
+        <v>0.09379703649195577</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>24.04</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
@@ -1276,31 +1276,31 @@
         <v>7540</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>3892.3</v>
+        <v>4106.7</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>7784.6</v>
+        <v>8213.4</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>244.6000000000004</v>
+        <v>673.3999999999996</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.03244031830238732</v>
+        <v>0.08931034482758615</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>3604.1</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>3700.921428571429</v>
+        <v>3795.664285714286</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.04916850485023543</v>
+        <v>0.07573860137962701</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>81.47</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>6500</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>6556.5</v>
+        <v>6460</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>6556.5</v>
+        <v>6460</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>56.5</v>
+        <v>-40</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.008692307692307692</v>
+        <v>-0.006153846153846154</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>6181.43</v>
@@ -1342,13 +1342,13 @@
         <v>6401.5</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.02364066193853428</v>
+        <v>0.009055727554179566</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>142.71</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>9031.549999999999</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>838.55</v>
+        <v>838.1</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>9224.049999999999</v>
+        <v>9219.1</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>192.5</v>
+        <v>187.5500000000008</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.02131417087875282</v>
+        <v>0.02076609219901354</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>783.09</v>
@@ -1390,13 +1390,13 @@
         <v>805.2571428571429</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.03970288848948433</v>
+        <v>0.0391872773450151</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>16.6</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>7278.3</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>2528.6</v>
+        <v>2541.5</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>7585.799999999999</v>
+        <v>7624.5</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>307.5</v>
+        <v>346.2000000000003</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.04224887679815342</v>
+        <v>0.04756605251226251</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>2309.03</v>
@@ -1438,13 +1438,13 @@
         <v>2340.228571428572</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.07449633337476379</v>
+        <v>0.07919395182822263</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>59.36</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>9246.6</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>461.75</v>
+        <v>468.9</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>10158.5</v>
+        <v>10315.8</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>911.8999999999997</v>
+        <v>1069.199999999999</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.09862003330954078</v>
+        <v>0.1156316916488222</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>386.74</v>
@@ -1486,13 +1486,13 @@
         <v>420.1285714285714</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.09013844844922279</v>
+        <v>0.1040124303080158</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
@@ -1516,16 +1516,16 @@
         <v>8790</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>1439.3</v>
+        <v>1543.6</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>8635.799999999999</v>
+        <v>9261.599999999999</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>-154.2000000000003</v>
+        <v>471.5999999999995</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>-0.01754266211604099</v>
+        <v>0.05365187713310574</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>1365.41</v>
@@ -1534,13 +1534,13 @@
         <v>1397.635714285714</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>0.02894760349773195</v>
+        <v>0.09456095213415752</v>
       </c>
       <c r="M17" s="13" t="n">
         <v>45.25</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
@@ -1564,31 +1564,31 @@
         <v>9288.75</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>660.1</v>
+        <v>667.5</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>9901.5</v>
+        <v>10012.5</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>612.7500000000003</v>
+        <v>723.75</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>0.06596689543802992</v>
+        <v>0.07791683488090433</v>
       </c>
       <c r="J18" s="7" t="n">
         <v>591.46</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>611.342857142857</v>
+        <v>617.5178571428571</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>0.07386326747029689</v>
+        <v>0.07487961476725527</v>
       </c>
       <c r="M18" s="13" t="n">
         <v>14</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
@@ -1612,35 +1612,323 @@
         <v>8700</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>8893.5</v>
+        <v>8888.5</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>8893.5</v>
+        <v>8888.5</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>193.5</v>
+        <v>188.5</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>0.02224137931034483</v>
+        <v>0.02166666666666667</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>8339.209999999999</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>8503.071428571429</v>
+        <v>8510.25</v>
       </c>
       <c r="L19" s="12" t="n">
-        <v>0.04390044093198073</v>
+        <v>0.04255498678067166</v>
       </c>
       <c r="M19" s="13" t="n">
         <v>123.68</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>900</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>925.05</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>9250.5</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>250.4999999999995</v>
+      </c>
+      <c r="I20" s="11" t="n">
+        <v>0.02783333333333328</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>836</v>
+      </c>
+      <c r="K20" s="7" t="n">
+        <v>836</v>
+      </c>
+      <c r="L20" s="12" t="n">
+        <v>0.09626506675314843</v>
+      </c>
+      <c r="M20" s="13" t="n">
+        <v>29.64</v>
+      </c>
+      <c r="N20" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>5479</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>5479</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>5578.5</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>5578.5</v>
+      </c>
+      <c r="H21" s="10" t="n">
+        <v>99.5</v>
+      </c>
+      <c r="I21" s="11" t="n">
+        <v>0.01816024822047819</v>
+      </c>
+      <c r="J21" s="7" t="n">
+        <v>5171.64</v>
+      </c>
+      <c r="K21" s="7" t="n">
+        <v>5171.64</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>0.07293358429685394</v>
+      </c>
+      <c r="M21" s="13" t="n">
+        <v>153.54</v>
+      </c>
+      <c r="N21" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>NAVINFLUOR</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>7579.5</v>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>7579.5</v>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>7729</v>
+      </c>
+      <c r="G22" s="9" t="n">
+        <v>7729</v>
+      </c>
+      <c r="H22" s="10" t="n">
+        <v>149.5</v>
+      </c>
+      <c r="I22" s="11" t="n">
+        <v>0.01972425621742859</v>
+      </c>
+      <c r="J22" s="7" t="n">
+        <v>7128.14</v>
+      </c>
+      <c r="K22" s="7" t="n">
+        <v>7128.14</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>0.07774097554664247</v>
+      </c>
+      <c r="M22" s="13" t="n">
+        <v>209.96</v>
+      </c>
+      <c r="N22" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>IPCALAB</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>1798.5</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>8992.5</v>
+      </c>
+      <c r="F23" s="7" t="n">
+        <v>1782.4</v>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>8912</v>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>-80.49999999999955</v>
+      </c>
+      <c r="I23" s="11" t="n">
+        <v>-0.008951904364748351</v>
+      </c>
+      <c r="J23" s="7" t="n">
+        <v>1680.3</v>
+      </c>
+      <c r="K23" s="7" t="n">
+        <v>1680.3</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>0.05728231597845609</v>
+      </c>
+      <c r="M23" s="13" t="n">
+        <v>50.24</v>
+      </c>
+      <c r="N23" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>ELGIEQUIP</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>571.5</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>9144</v>
+      </c>
+      <c r="F24" s="7" t="n">
+        <v>591.95</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>9471.200000000001</v>
+      </c>
+      <c r="H24" s="10" t="n">
+        <v>327.2000000000007</v>
+      </c>
+      <c r="I24" s="11" t="n">
+        <v>0.03578302712160988</v>
+      </c>
+      <c r="J24" s="7" t="n">
+        <v>541.78</v>
+      </c>
+      <c r="K24" s="7" t="n">
+        <v>541.78</v>
+      </c>
+      <c r="L24" s="12" t="n">
+        <v>0.08475377988005756</v>
+      </c>
+      <c r="M24" s="13" t="n">
+        <v>18.67</v>
+      </c>
+      <c r="N24" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>965</v>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>8685</v>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>958.5</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>8626.5</v>
+      </c>
+      <c r="H25" s="10" t="n">
+        <v>-58.5</v>
+      </c>
+      <c r="I25" s="11" t="n">
+        <v>-0.006735751295336788</v>
+      </c>
+      <c r="J25" s="7" t="n">
+        <v>908.65</v>
+      </c>
+      <c r="K25" s="7" t="n">
+        <v>908.65</v>
+      </c>
+      <c r="L25" s="12" t="n">
+        <v>0.05200834637454358</v>
+      </c>
+      <c r="M25" s="13" t="n">
+        <v>23.48</v>
+      </c>
+      <c r="N25" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H19">
+  <conditionalFormatting sqref="H2:H25">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2051,7 +2339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2398,6 +2686,31 @@
       </c>
       <c r="G13" s="14" t="n">
         <v>18</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="n">
+        <v>205022.25</v>
+      </c>
+      <c r="C14" s="20" t="n">
+        <v>32316.2</v>
+      </c>
+      <c r="D14" s="20" t="n">
+        <v>172706.05</v>
+      </c>
+      <c r="E14" s="20" t="n">
+        <v>165762.25</v>
+      </c>
+      <c r="F14" s="20" t="n">
+        <v>-1921.55</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -2480,18 +2793,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1542.3</v>
+        <v>854.2</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1453.46</v>
+        <v>800.79</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -2500,10 +2813,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8264454277286135</v>
+        <v>0.8175138132607304</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -2518,18 +2831,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>ADANIPOWER</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>892.55</v>
+        <v>219.85</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>836</v>
+        <v>207.35</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -2538,10 +2851,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.7961799410029499</v>
+        <v>0.7845731902626522</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -2556,18 +2869,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>833.8</v>
+        <v>1543.6</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>783.16</v>
+        <v>1431.87</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -2576,10 +2889,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8129301868239921</v>
+        <v>0.7852578475336323</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -2594,18 +2907,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1439.3</v>
+        <v>1529.2</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1342.31</v>
+        <v>1443.9</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -2614,10 +2927,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7727728613569321</v>
+        <v>0.7829256085842409</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -2632,18 +2945,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>8893.5</v>
+        <v>925.05</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>8633.209999999999</v>
+        <v>865.78</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -2652,10 +2965,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7722959685349067</v>
+        <v>0.7747217328635491</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -2670,18 +2983,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1620.5</v>
+        <v>1782.4</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1541.81</v>
+        <v>1681.91</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -2693,7 +3006,7 @@
         <v>6.6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7688200589970501</v>
+        <v>0.7937029548366432</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -2708,18 +3021,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>838.55</v>
+        <v>958.5</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>802.13</v>
+        <v>911.55</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -2731,7 +3044,7 @@
         <v>6.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7575663716814159</v>
+        <v>0.8071358504163997</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -2746,18 +3059,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>BSE</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>5478</v>
+        <v>3802.7</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>5171.64</v>
+        <v>3575.97</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -2766,10 +3079,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7476745329400196</v>
+        <v>0.729642456758488</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -2784,18 +3097,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>7552.5</v>
+        <v>6857.5</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>7128.14</v>
+        <v>6612.07</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -2807,7 +3120,7 @@
         <v>6.5</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7650491642084563</v>
+        <v>0.7557795483664317</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -2822,18 +3135,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>18514</v>
+        <v>1022.9</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>17279.57</v>
+        <v>965.67</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -2842,10 +3155,10 @@
         <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7397738446411013</v>
+        <v>0.769477698590647</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -2860,18 +3173,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>SOLARINDS</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1778.9</v>
+        <v>18539</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1680.3</v>
+        <v>17317.29</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -2883,7 +3196,7 @@
         <v>6.4</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.753874139626352</v>
+        <v>0.7512992472773863</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -2898,18 +3211,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1874.2</v>
+        <v>8888.5</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1796.91</v>
+        <v>8633</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -2921,7 +3234,7 @@
         <v>6.4</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7318879056047197</v>
+        <v>0.7390304692504805</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -2936,18 +3249,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1459.8</v>
+        <v>980.05</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1401.19</v>
+        <v>936.51</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -2959,7 +3272,7 @@
         <v>6.4</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7400737463126844</v>
+        <v>0.7424767777065984</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -2974,7 +3287,7 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
@@ -2982,10 +3295,10 @@
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>578.55</v>
+        <v>591.95</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>541.78</v>
+        <v>554.61</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -2997,7 +3310,7 @@
         <v>6.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7740363815142576</v>
+        <v>0.7750730701473414</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3012,18 +3325,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260703</v>
+        <v>20260706</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>955.1</v>
+        <v>2390</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>908.65</v>
+        <v>2297.11</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -3032,10 +3345,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7628564405113076</v>
+        <v>0.7366051409352979</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-07
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Mon 06 Jul 2026</t>
+          <t>As of Tue 07 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹205,022</t>
+          <t>₹203,935</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+2,135  (+1.05%)</t>
+          <t>₹-1,088  (-0.53%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.51%</t>
+          <t>+1.97%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>+0.00%</t>
+          <t>-0.53%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹32,316</t>
+          <t>₹37,740</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹165,762</t>
+          <t>₹160,283</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹172,706</t>
+          <t>₹166,195</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹-1,922</t>
+          <t>₹-1,977</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -796,31 +796,31 @@
         <v>4230</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>1473.7</v>
+        <v>1471.8</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>4421.1</v>
+        <v>4415.4</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>191.1000000000001</v>
+        <v>185.3999999999999</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.04517730496453904</v>
+        <v>0.04382978723404252</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>1312.63</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1386.914285714286</v>
+        <v>1388.671428571429</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.05888967516164378</v>
+        <v>0.05648088831945331</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>33.1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>4788</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>774.05</v>
+        <v>766.65</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>4644.299999999999</v>
+        <v>4599.9</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-143.7000000000003</v>
+        <v>-188.1000000000001</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.03001253132832086</v>
+        <v>-0.03928571428571431</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>746.09</v>
@@ -862,13 +862,13 @@
         <v>750</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.03107034429300427</v>
+        <v>0.02171786343181371</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>22.5</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -892,31 +892,31 @@
         <v>4830</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>684.15</v>
+        <v>643.55</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>4789.05</v>
+        <v>4504.849999999999</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-40.95000000000016</v>
+        <v>-325.1500000000003</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.008478260869565251</v>
+        <v>-0.06731884057971022</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>612.1900000000001</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>612.1900000000001</v>
+        <v>630.05</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.1051816122195424</v>
+        <v>0.02097739103410769</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>34.34</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>3678</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1864.4</v>
+        <v>1833.9</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>3728.8</v>
+        <v>3667.8</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>50.80000000000018</v>
+        <v>-10.19999999999982</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.0138118542686243</v>
+        <v>-0.002773246329526867</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1729.61</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1768.707142857143</v>
+        <v>1770.5</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.05132635547246154</v>
+        <v>0.03457113255902726</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>43.14</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>4242</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1529.2</v>
+        <v>1477.4</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4587.6</v>
+        <v>4432.200000000001</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>345.6000000000001</v>
+        <v>190.2000000000003</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.08147100424328151</v>
+        <v>0.0448373408769449</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1324.47</v>
@@ -1006,13 +1006,13 @@
         <v>1414.35</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.07510462987182849</v>
+        <v>0.04267632327061065</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>35.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>5200</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1347.4</v>
+        <v>1339.4</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>5389.6</v>
+        <v>5357.6</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>189.6000000000004</v>
+        <v>157.6000000000004</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.03646153846153853</v>
+        <v>0.03030769230769238</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1159.03</v>
@@ -1054,13 +1054,13 @@
         <v>1252</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.07080302805403005</v>
+        <v>0.06525309840226974</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>64.73</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
@@ -1084,31 +1084,31 @@
         <v>5209</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>272.3</v>
+        <v>268.5</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5446</v>
+        <v>5370</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>237.0000000000005</v>
+        <v>161.0000000000002</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.04549817623344221</v>
+        <v>0.03090804377039743</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>240.49</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>256.7214285714286</v>
+        <v>257.8464285714286</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.05721105923089027</v>
+        <v>0.03967810587922313</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>8.369999999999999</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>5252.55</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>313.5</v>
+        <v>315.2</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5956.5</v>
+        <v>5988.8</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>703.9500000000003</v>
+        <v>736.25</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.1340206185567011</v>
+        <v>0.1401700126605173</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>259.14</v>
@@ -1150,13 +1150,13 @@
         <v>289.2285714285714</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.07742082478924593</v>
+        <v>0.08239666424945619</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>7.11</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>4387.5</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1594.6</v>
+        <v>1583.1</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4783.799999999999</v>
+        <v>4749.299999999999</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>396.2999999999997</v>
+        <v>361.7999999999997</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.09032478632478626</v>
+        <v>0.08246153846153841</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1405.17</v>
@@ -1198,13 +1198,13 @@
         <v>1502.471428571428</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.05777534894554848</v>
+        <v>0.05093081386429892</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>38.34</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11">
@@ -1228,31 +1228,31 @@
         <v>8690</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>854.2</v>
+        <v>863.55</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>9396.200000000001</v>
+        <v>9499.049999999999</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>706.2000000000005</v>
+        <v>809.0499999999995</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.08126582278481019</v>
+        <v>0.09310126582278476</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>739.3099999999999</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>774.0785714285714</v>
+        <v>781.7249999999999</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.09379703649195577</v>
+        <v>0.09475421226333165</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>24.04</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>7540</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>4106.7</v>
+        <v>4098.6</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>8213.4</v>
+        <v>8197.200000000001</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>673.3999999999996</v>
+        <v>657.2000000000007</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.08931034482758615</v>
+        <v>0.08716180371352794</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>3604.1</v>
@@ -1294,13 +1294,13 @@
         <v>3795.664285714286</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.07573860137962701</v>
+        <v>0.07391199782504142</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>81.47</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>6500</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>6460</v>
+        <v>6432.5</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>6460</v>
+        <v>6432.5</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-40</v>
+        <v>-67.5</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.006153846153846154</v>
+        <v>-0.01038461538461538</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>6181.43</v>
@@ -1342,13 +1342,13 @@
         <v>6401.5</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.009055727554179566</v>
+        <v>0.004819277108433735</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>142.71</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>9031.549999999999</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>838.1</v>
+        <v>847.65</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>9219.1</v>
+        <v>9324.15</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>187.5500000000008</v>
+        <v>292.6000000000003</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.02076609219901354</v>
+        <v>0.03239753973570431</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>783.09</v>
@@ -1390,13 +1390,13 @@
         <v>805.2571428571429</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.0391872773450151</v>
+        <v>0.05001221865493672</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>16.6</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>7278.3</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>2541.5</v>
+        <v>2527.4</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>7624.5</v>
+        <v>7582.200000000001</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>346.2000000000003</v>
+        <v>303.9000000000005</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.04756605251226251</v>
+        <v>0.04175425580149218</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>2309.03</v>
@@ -1438,13 +1438,13 @@
         <v>2340.228571428572</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.07919395182822263</v>
+        <v>0.07405690771996039</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>59.36</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>9246.6</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>468.9</v>
+        <v>464.85</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>10315.8</v>
+        <v>10226.7</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>1069.199999999999</v>
+        <v>980.1000000000003</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.1156316916488222</v>
+        <v>0.1059957173447538</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>386.74</v>
@@ -1486,13 +1486,13 @@
         <v>420.1285714285714</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.1040124303080158</v>
+        <v>0.09620614944913121</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
@@ -1516,16 +1516,16 @@
         <v>8790</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>1543.6</v>
+        <v>1541</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>9261.599999999999</v>
+        <v>9246</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>471.5999999999995</v>
+        <v>456</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>0.05365187713310574</v>
+        <v>0.05187713310580205</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>1365.41</v>
@@ -1534,13 +1534,13 @@
         <v>1397.635714285714</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>0.09456095213415752</v>
+        <v>0.09303328080096408</v>
       </c>
       <c r="M17" s="13" t="n">
         <v>45.25</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18">
@@ -1564,31 +1564,31 @@
         <v>9288.75</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>667.5</v>
+        <v>671.2</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>10012.5</v>
+        <v>10068</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>723.75</v>
+        <v>779.2500000000007</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>0.07791683488090433</v>
+        <v>0.08389180460234162</v>
       </c>
       <c r="J18" s="7" t="n">
         <v>591.46</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>617.5178571428571</v>
+        <v>621.0571428571428</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>0.07487961476725527</v>
+        <v>0.07470628298995415</v>
       </c>
       <c r="M18" s="13" t="n">
         <v>14</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
@@ -1612,16 +1612,16 @@
         <v>8700</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>8888.5</v>
+        <v>8837</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>8888.5</v>
+        <v>8837</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>188.5</v>
+        <v>137</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>0.02166666666666667</v>
+        <v>0.01574712643678161</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>8339.209999999999</v>
@@ -1630,13 +1630,13 @@
         <v>8510.25</v>
       </c>
       <c r="L19" s="12" t="n">
-        <v>0.04255498678067166</v>
+        <v>0.03697521783410659</v>
       </c>
       <c r="M19" s="13" t="n">
         <v>123.68</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20">
@@ -1660,37 +1660,37 @@
         <v>9000</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>925.05</v>
+        <v>910.5</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>9250.5</v>
+        <v>9105</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>250.4999999999995</v>
+        <v>105</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>0.02783333333333328</v>
+        <v>0.01166666666666667</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>836</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>836</v>
+        <v>887.1</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>0.09626506675314843</v>
+        <v>0.02570016474464577</v>
       </c>
       <c r="M20" s="13" t="n">
         <v>29.64</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
@@ -1699,46 +1699,46 @@
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>5479</v>
+        <v>7579.5</v>
       </c>
       <c r="D21" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>5479</v>
+        <v>7579.5</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>5578.5</v>
+        <v>7547</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>5578.5</v>
+        <v>7547</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>99.5</v>
+        <v>-32.5</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>0.01816024822047819</v>
+        <v>-0.004287881786397519</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>5171.64</v>
+        <v>7128.14</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>5171.64</v>
+        <v>7128.14</v>
       </c>
       <c r="L21" s="12" t="n">
-        <v>0.07293358429685394</v>
+        <v>0.05550019875447193</v>
       </c>
       <c r="M21" s="13" t="n">
-        <v>153.54</v>
+        <v>209.96</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1747,46 +1747,46 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>7579.5</v>
+        <v>1798.5</v>
       </c>
       <c r="D22" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>8992.5</v>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>1793.1</v>
+      </c>
+      <c r="G22" s="9" t="n">
+        <v>8965.5</v>
+      </c>
+      <c r="H22" s="10" t="n">
+        <v>-27.00000000000045</v>
+      </c>
+      <c r="I22" s="11" t="n">
+        <v>-0.003002502085070943</v>
+      </c>
+      <c r="J22" s="7" t="n">
+        <v>1680.3</v>
+      </c>
+      <c r="K22" s="7" t="n">
+        <v>1680.3</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>0.06290781328425629</v>
+      </c>
+      <c r="M22" s="13" t="n">
+        <v>50.24</v>
+      </c>
+      <c r="N22" s="6" t="n">
         <v>1</v>
-      </c>
-      <c r="E22" s="9" t="n">
-        <v>7579.5</v>
-      </c>
-      <c r="F22" s="7" t="n">
-        <v>7729</v>
-      </c>
-      <c r="G22" s="9" t="n">
-        <v>7729</v>
-      </c>
-      <c r="H22" s="10" t="n">
-        <v>149.5</v>
-      </c>
-      <c r="I22" s="11" t="n">
-        <v>0.01972425621742859</v>
-      </c>
-      <c r="J22" s="7" t="n">
-        <v>7128.14</v>
-      </c>
-      <c r="K22" s="7" t="n">
-        <v>7128.14</v>
-      </c>
-      <c r="L22" s="12" t="n">
-        <v>0.07774097554664247</v>
-      </c>
-      <c r="M22" s="13" t="n">
-        <v>209.96</v>
-      </c>
-      <c r="N22" s="6" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
@@ -1795,46 +1795,46 @@
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>1798.5</v>
+        <v>571.5</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>8992.5</v>
+        <v>9144</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>1782.4</v>
+        <v>589</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>8912</v>
+        <v>9424</v>
       </c>
       <c r="H23" s="10" t="n">
-        <v>-80.49999999999955</v>
+        <v>280</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>-0.008951904364748351</v>
+        <v>0.03062117235345582</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>1680.3</v>
+        <v>541.78</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>1680.3</v>
+        <v>571.1</v>
       </c>
       <c r="L23" s="12" t="n">
-        <v>0.05728231597845609</v>
+        <v>0.03039049235993205</v>
       </c>
       <c r="M23" s="13" t="n">
-        <v>50.24</v>
+        <v>18.67</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1843,92 +1843,44 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>571.5</v>
+        <v>965</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>9144</v>
+        <v>8685</v>
       </c>
       <c r="F24" s="7" t="n">
-        <v>591.95</v>
+        <v>961.6</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>9471.200000000001</v>
+        <v>8654.4</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>327.2000000000007</v>
+        <v>-30.5999999999998</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>0.03578302712160988</v>
+        <v>-0.003523316062176142</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>541.78</v>
+        <v>908.65</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>541.78</v>
+        <v>933</v>
       </c>
       <c r="L24" s="12" t="n">
-        <v>0.08475377988005756</v>
+        <v>0.02974209650582365</v>
       </c>
       <c r="M24" s="13" t="n">
-        <v>18.67</v>
+        <v>23.48</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>SHYAMMETL</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="n">
-        <v>965</v>
-      </c>
-      <c r="D25" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="E25" s="9" t="n">
-        <v>8685</v>
-      </c>
-      <c r="F25" s="7" t="n">
-        <v>958.5</v>
-      </c>
-      <c r="G25" s="9" t="n">
-        <v>8626.5</v>
-      </c>
-      <c r="H25" s="10" t="n">
-        <v>-58.5</v>
-      </c>
-      <c r="I25" s="11" t="n">
-        <v>-0.006735751295336788</v>
-      </c>
-      <c r="J25" s="7" t="n">
-        <v>908.65</v>
-      </c>
-      <c r="K25" s="7" t="n">
-        <v>908.65</v>
-      </c>
-      <c r="L25" s="12" t="n">
-        <v>0.05200834637454358</v>
-      </c>
-      <c r="M25" s="13" t="n">
-        <v>23.48</v>
-      </c>
-      <c r="N25" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H25">
+  <conditionalFormatting sqref="H2:H24">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1946,10 +1898,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -2022,27 +1974,27 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>960.1</v>
+        <v>5479</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>5424</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -2050,22 +2002,22 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-516.79</v>
+        <v>-55</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.01</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -2074,18 +2026,18 @@
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>952.1</v>
+        <v>960.1</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>948.8</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -2093,42 +2045,42 @@
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-29.7</v>
+        <v>-516.79</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.0598</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>1475</v>
+        <v>952.1</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>1394.19</v>
+        <v>948.8</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -2136,42 +2088,42 @@
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-484.86</v>
+        <v>-29.7</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0035</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-1</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>248.05</v>
+        <v>1475</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>242.8</v>
+        <v>1394.19</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -2179,22 +2131,22 @@
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-110.25</v>
+        <v>-484.86</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0548</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-0.3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -2203,10 +2155,10 @@
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>1039.2</v>
+        <v>248.05</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -2214,7 +2166,7 @@
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>970</v>
+        <v>242.8</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -2225,19 +2177,19 @@
         <v>11</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>-346</v>
+        <v>-110.25</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -2246,10 +2198,10 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>199.96</v>
+        <v>1039.2</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
@@ -2257,7 +2209,7 @@
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>193.31</v>
+        <v>970</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -2268,19 +2220,19 @@
         <v>11</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>-172.9</v>
+        <v>-346</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.06660000000000001</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -2289,10 +2241,10 @@
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>986.4</v>
+        <v>199.96</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
@@ -2300,7 +2252,7 @@
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>193.31</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -2311,17 +2263,60 @@
         <v>11</v>
       </c>
       <c r="I8" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J8" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K8" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I9" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J8" s="18" t="n">
+      <c r="J9" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K8" s="19" t="n">
+      <c r="K9" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I8">
+  <conditionalFormatting sqref="I2:I9">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2339,7 +2334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2711,6 +2706,31 @@
       </c>
       <c r="G14" s="14" t="n">
         <v>24</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="n">
+        <v>203934.75</v>
+      </c>
+      <c r="C15" s="20" t="n">
+        <v>37740.2</v>
+      </c>
+      <c r="D15" s="20" t="n">
+        <v>166194.55</v>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>160283.25</v>
+      </c>
+      <c r="F15" s="20" t="n">
+        <v>-1976.55</v>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -2793,18 +2813,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>854.2</v>
+        <v>2422</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>800.79</v>
+        <v>2327.06</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -2813,10 +2833,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8175138132607304</v>
+        <v>0.8359455076873799</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -2831,18 +2851,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>ADANIPOWER</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>219.85</v>
+        <v>863.55</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>207.35</v>
+        <v>809</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -2851,10 +2871,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.7845731902626522</v>
+        <v>0.8253263132607304</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -2869,18 +2889,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>SOLARINDS</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1543.6</v>
+        <v>18268</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1431.87</v>
+        <v>17022.71</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -2892,7 +2912,7 @@
         <v>6.8</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7852578475336323</v>
+        <v>0.8012942424727738</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -2907,18 +2927,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>BSE</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1529.2</v>
+        <v>3683.4</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1443.9</v>
+        <v>3466.51</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -2927,10 +2947,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7829256085842409</v>
+        <v>0.7593399663677131</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -2945,18 +2965,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>925.05</v>
+        <v>1024.5</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>865.78</v>
+        <v>966.11</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -2968,7 +2988,7 @@
         <v>6.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7747217328635491</v>
+        <v>0.7954306133888533</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -2983,18 +3003,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1782.4</v>
+        <v>1477.4</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1681.91</v>
+        <v>1387.47</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -3003,10 +3023,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7937029548366432</v>
+        <v>0.7799987988468929</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3021,18 +3041,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>958.5</v>
+        <v>971.9</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>911.55</v>
+        <v>928.62</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -3044,7 +3064,7 @@
         <v>6.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.8071358504163997</v>
+        <v>0.7767036354900705</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3059,18 +3079,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>BSE</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>3802.7</v>
+        <v>1471.8</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>3575.97</v>
+        <v>1415.11</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -3082,7 +3102,7 @@
         <v>6.6</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.729642456758488</v>
+        <v>0.7726357303010891</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3097,18 +3117,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>6857.5</v>
+        <v>643.55</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>6612.07</v>
+        <v>580.4299999999999</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -3117,10 +3137,10 @@
         <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7557795483664317</v>
+        <v>0.731179932735426</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3135,18 +3155,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1022.9</v>
+        <v>1833.9</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>965.67</v>
+        <v>1753.99</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -3158,7 +3178,7 @@
         <v>6.5</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.769477698590647</v>
+        <v>0.7545073270339526</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3173,18 +3193,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>18539</v>
+        <v>6771.5</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>17317.29</v>
+        <v>6513.71</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -3193,10 +3213,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7512992472773863</v>
+        <v>0.7593459721332478</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3211,18 +3231,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ADANIPOWER</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>8888.5</v>
+        <v>218.07</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>8633</v>
+        <v>205.2</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -3231,10 +3251,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7390304692504805</v>
+        <v>0.7347964045483664</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3249,18 +3269,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>980.05</v>
+        <v>961.6</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>936.51</v>
+        <v>913.5599999999999</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -3272,7 +3292,7 @@
         <v>6.4</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7424767777065984</v>
+        <v>0.7611036595131326</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3287,18 +3307,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>591.95</v>
+        <v>8837</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>554.61</v>
+        <v>8573</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -3307,10 +3327,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7750730701473414</v>
+        <v>0.7468679932735427</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3325,18 +3345,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260706</v>
+        <v>20260707</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>2390</v>
+        <v>766.65</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>2297.11</v>
+        <v>724.61</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -3345,10 +3365,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7366051409352979</v>
+        <v>0.7611487027546444</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-08
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Tue 07 Jul 2026</t>
+          <t>As of Wed 08 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹203,935</t>
+          <t>₹201,907</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-1,088  (-0.53%)</t>
+          <t>₹-2,028  (-0.99%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.97%</t>
+          <t>+0.95%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.53%</t>
+          <t>-1.52%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹37,740</t>
+          <t>₹71,333</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹160,283</t>
+          <t>₹125,957</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹166,195</t>
+          <t>₹130,573</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹-1,977</t>
+          <t>₹-2,710</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -796,16 +796,16 @@
         <v>4230</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>1471.8</v>
+        <v>1450.5</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>4415.4</v>
+        <v>4351.5</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>185.3999999999999</v>
+        <v>121.5</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.04382978723404252</v>
+        <v>0.02872340425531915</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>1312.63</v>
@@ -814,19 +814,19 @@
         <v>1388.671428571429</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.05648088831945331</v>
+        <v>0.04262569557295513</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>33.1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -835,46 +835,46 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>798</v>
+        <v>690</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>4788</v>
+        <v>4830</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>766.65</v>
+        <v>640.85</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>4599.9</v>
+        <v>4485.95</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-188.1000000000001</v>
+        <v>-344.0499999999998</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.03928571428571431</v>
+        <v>-0.07123188405797098</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>746.09</v>
+        <v>612.1900000000001</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>750</v>
+        <v>630.05</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.02171786343181371</v>
+        <v>0.01685261761722722</v>
       </c>
       <c r="M3" s="13" t="n">
-        <v>22.5</v>
+        <v>34.34</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -883,46 +883,46 @@
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>690</v>
+        <v>1839</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>4830</v>
+        <v>3678</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>643.55</v>
+        <v>1791.7</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>4504.849999999999</v>
+        <v>3583.4</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-325.1500000000003</v>
+        <v>-94.59999999999991</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.06731884057971022</v>
+        <v>-0.02572050027188687</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>612.1900000000001</v>
+        <v>1729.61</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>630.05</v>
+        <v>1770.5</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.02097739103410769</v>
+        <v>0.01183233800301392</v>
       </c>
       <c r="M4" s="13" t="n">
-        <v>34.34</v>
+        <v>43.14</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -931,46 +931,46 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>1839</v>
+        <v>1414</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>3678</v>
+        <v>4242</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1833.9</v>
+        <v>1469.2</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>3667.8</v>
+        <v>4407.6</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>-10.19999999999982</v>
+        <v>165.6000000000001</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>-0.002773246329526867</v>
+        <v>0.03903818953323907</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>1729.61</v>
+        <v>1324.47</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1770.5</v>
+        <v>1414.35</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.03457113255902726</v>
+        <v>0.03733324258099655</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>43.14</v>
+        <v>35.79</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -979,46 +979,46 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>1414</v>
+        <v>1300</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>4242</v>
+        <v>5200</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1477.4</v>
+        <v>1326</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4432.200000000001</v>
+        <v>5304</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>190.2000000000003</v>
+        <v>104</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.0448373408769449</v>
+        <v>0.02</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>1324.47</v>
+        <v>1159.03</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1414.35</v>
+        <v>1252</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.04267632327061065</v>
+        <v>0.05580693815987934</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>35.79</v>
+        <v>64.73</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -1027,46 +1027,46 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>1300</v>
+        <v>276.45</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>5200</v>
+        <v>5252.55</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1339.4</v>
+        <v>317.95</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>5357.6</v>
+        <v>6041.05</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>157.6000000000004</v>
+        <v>788.5</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.03030769230769238</v>
+        <v>0.1501175619461024</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>1159.03</v>
+        <v>259.14</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1252</v>
+        <v>293.9928571428571</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.06525309840226974</v>
+        <v>0.07534877451531014</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>64.73</v>
+        <v>7.11</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -1075,142 +1075,142 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>260.45</v>
+        <v>1462.5</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>5209</v>
+        <v>4387.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>268.5</v>
+        <v>1557.4</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5370</v>
+        <v>4672.200000000001</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>161.0000000000002</v>
+        <v>284.7000000000003</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.03090804377039743</v>
+        <v>0.06488888888888895</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>240.49</v>
+        <v>1405.17</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>257.8464285714286</v>
+        <v>1502.471428571428</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.03967810587922313</v>
+        <v>0.0352694050523769</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>8.369999999999999</v>
+        <v>38.34</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>276.45</v>
+        <v>790</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>5252.55</v>
+        <v>8690</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>315.2</v>
+        <v>859.55</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5988.8</v>
+        <v>9455.049999999999</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>736.25</v>
+        <v>765.0499999999995</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.1401700126605173</v>
+        <v>0.08803797468354424</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>259.14</v>
+        <v>739.3099999999999</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>289.2285714285714</v>
+        <v>786.6535714285715</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.08239666424945619</v>
+        <v>0.0848076651403973</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>7.11</v>
+        <v>24.04</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1462.5</v>
+        <v>3770</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>4387.5</v>
+        <v>7540</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1583.1</v>
+        <v>4077.6</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4749.299999999999</v>
+        <v>8155.2</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>361.7999999999997</v>
+        <v>615.1999999999998</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.08246153846153841</v>
+        <v>0.0815915119363395</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>1405.17</v>
+        <v>3604.1</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1502.471428571428</v>
+        <v>3808.65</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.05093081386429892</v>
+        <v>0.06595791642142432</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>38.34</v>
+        <v>81.47</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -1219,46 +1219,46 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>790</v>
+        <v>821.05</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>11</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>8690</v>
+        <v>9031.549999999999</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>863.55</v>
+        <v>840.1</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>9499.049999999999</v>
+        <v>9241.1</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>809.0499999999995</v>
+        <v>209.5500000000008</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.09310126582278476</v>
+        <v>0.02320199744229958</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>739.3099999999999</v>
+        <v>783.09</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>781.7249999999999</v>
+        <v>805.2571428571429</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.09475421226333165</v>
+        <v>0.0414746543778802</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>24.04</v>
+        <v>16.6</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1267,190 +1267,190 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>3770</v>
+        <v>2426.1</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>7540</v>
+        <v>7278.3</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>4098.6</v>
+        <v>2491.2</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>8197.200000000001</v>
+        <v>7473.599999999999</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>657.2000000000007</v>
+        <v>195.2999999999997</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.08716180371352794</v>
+        <v>0.02683318906887594</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>3604.1</v>
+        <v>2309.03</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>3795.664285714286</v>
+        <v>2340.7</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.07391199782504142</v>
+        <v>0.06041265253693</v>
       </c>
       <c r="M12" s="13" t="n">
-        <v>81.47</v>
+        <v>59.36</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>6500</v>
+        <v>420.3</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>6500</v>
+        <v>9246.6</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>6432.5</v>
+        <v>467.6</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>6432.5</v>
+        <v>10287.2</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-67.5</v>
+        <v>1040.6</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.01038461538461538</v>
+        <v>0.112538662859862</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>6181.43</v>
+        <v>386.74</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>6401.5</v>
+        <v>420.1285714285714</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.004819277108433735</v>
+        <v>0.1015214469021143</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>142.71</v>
+        <v>16.71</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>821.05</v>
+        <v>1465</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>9031.549999999999</v>
+        <v>8790</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>847.65</v>
+        <v>1529.2</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>9324.15</v>
+        <v>9175.200000000001</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>292.6000000000003</v>
+        <v>385.2000000000003</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.03239753973570431</v>
+        <v>0.04382252559726966</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>783.09</v>
+        <v>1365.41</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>805.2571428571429</v>
+        <v>1397.635714285714</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.05001221865493672</v>
+        <v>0.08603471469676019</v>
       </c>
       <c r="M14" s="13" t="n">
-        <v>16.6</v>
+        <v>45.25</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>2426.1</v>
+        <v>619.25</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>7278.3</v>
+        <v>9288.75</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>2527.4</v>
+        <v>662.05</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>7582.200000000001</v>
+        <v>9930.75</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>303.9000000000005</v>
+        <v>641.9999999999993</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.04175425580149218</v>
+        <v>0.06911586596689537</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>2309.03</v>
+        <v>591.46</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>2340.228571428572</v>
+        <v>621.0571428571428</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.07405690771996039</v>
+        <v>0.06191806833752305</v>
       </c>
       <c r="M15" s="13" t="n">
-        <v>59.36</v>
+        <v>14</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1459,428 +1459,188 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>420.3</v>
+        <v>8700</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>9246.6</v>
+        <v>8700</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>464.85</v>
+        <v>8753.5</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>10226.7</v>
+        <v>8753.5</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>980.1000000000003</v>
+        <v>53.5</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.1059957173447538</v>
+        <v>0.006149425287356322</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>386.74</v>
+        <v>8339.209999999999</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>420.1285714285714</v>
+        <v>8510.25</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.09620614944913121</v>
+        <v>0.02778888444622151</v>
       </c>
       <c r="M16" s="13" t="n">
-        <v>16.71</v>
+        <v>123.68</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>1465</v>
+        <v>900</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>8790</v>
+        <v>9000</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>1541</v>
+        <v>908.1</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>9246</v>
+        <v>9081</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>456</v>
+        <v>81.00000000000023</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>0.05187713310580205</v>
+        <v>0.009000000000000025</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>1365.41</v>
+        <v>836</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>1397.635714285714</v>
+        <v>887.1</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>0.09303328080096408</v>
+        <v>0.02312520647505781</v>
       </c>
       <c r="M17" s="13" t="n">
-        <v>45.25</v>
+        <v>29.64</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>619.25</v>
+        <v>7579.5</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>9288.75</v>
+        <v>7579.5</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>671.2</v>
+        <v>7363</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>10068</v>
+        <v>7363</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>779.2500000000007</v>
+        <v>-216.5</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>0.08389180460234162</v>
+        <v>-0.02856388943861732</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>591.46</v>
+        <v>7128.14</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>621.0571428571428</v>
+        <v>7128.14</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>0.07470628298995415</v>
+        <v>0.03189732446013849</v>
       </c>
       <c r="M18" s="13" t="n">
-        <v>14</v>
+        <v>209.96</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>8700</v>
+        <v>1798.5</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>8700</v>
+        <v>8992.5</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>8837</v>
+        <v>1762.4</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>8837</v>
+        <v>8812</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>137</v>
+        <v>-180.4999999999995</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>0.01574712643678161</v>
+        <v>-0.02007228245760351</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>8339.209999999999</v>
+        <v>1680.3</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>8510.25</v>
+        <v>1680.3</v>
       </c>
       <c r="L19" s="12" t="n">
-        <v>0.03697521783410659</v>
+        <v>0.04658420335905591</v>
       </c>
       <c r="M19" s="13" t="n">
-        <v>123.68</v>
+        <v>50.24</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>CGPOWER</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>900</v>
-      </c>
-      <c r="D20" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="E20" s="9" t="n">
-        <v>9000</v>
-      </c>
-      <c r="F20" s="7" t="n">
-        <v>910.5</v>
-      </c>
-      <c r="G20" s="9" t="n">
-        <v>9105</v>
-      </c>
-      <c r="H20" s="10" t="n">
-        <v>105</v>
-      </c>
-      <c r="I20" s="11" t="n">
-        <v>0.01166666666666667</v>
-      </c>
-      <c r="J20" s="7" t="n">
-        <v>836</v>
-      </c>
-      <c r="K20" s="7" t="n">
-        <v>887.1</v>
-      </c>
-      <c r="L20" s="12" t="n">
-        <v>0.02570016474464577</v>
-      </c>
-      <c r="M20" s="13" t="n">
-        <v>29.64</v>
-      </c>
-      <c r="N20" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>NAVINFLUOR</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>7579.5</v>
-      </c>
-      <c r="D21" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="9" t="n">
-        <v>7579.5</v>
-      </c>
-      <c r="F21" s="7" t="n">
-        <v>7547</v>
-      </c>
-      <c r="G21" s="9" t="n">
-        <v>7547</v>
-      </c>
-      <c r="H21" s="10" t="n">
-        <v>-32.5</v>
-      </c>
-      <c r="I21" s="11" t="n">
-        <v>-0.004287881786397519</v>
-      </c>
-      <c r="J21" s="7" t="n">
-        <v>7128.14</v>
-      </c>
-      <c r="K21" s="7" t="n">
-        <v>7128.14</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>0.05550019875447193</v>
-      </c>
-      <c r="M21" s="13" t="n">
-        <v>209.96</v>
-      </c>
-      <c r="N21" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>IPCALAB</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="n">
-        <v>1798.5</v>
-      </c>
-      <c r="D22" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="E22" s="9" t="n">
-        <v>8992.5</v>
-      </c>
-      <c r="F22" s="7" t="n">
-        <v>1793.1</v>
-      </c>
-      <c r="G22" s="9" t="n">
-        <v>8965.5</v>
-      </c>
-      <c r="H22" s="10" t="n">
-        <v>-27.00000000000045</v>
-      </c>
-      <c r="I22" s="11" t="n">
-        <v>-0.003002502085070943</v>
-      </c>
-      <c r="J22" s="7" t="n">
-        <v>1680.3</v>
-      </c>
-      <c r="K22" s="7" t="n">
-        <v>1680.3</v>
-      </c>
-      <c r="L22" s="12" t="n">
-        <v>0.06290781328425629</v>
-      </c>
-      <c r="M22" s="13" t="n">
-        <v>50.24</v>
-      </c>
-      <c r="N22" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>ELGIEQUIP</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="n">
-        <v>571.5</v>
-      </c>
-      <c r="D23" s="8" t="n">
-        <v>16</v>
-      </c>
-      <c r="E23" s="9" t="n">
-        <v>9144</v>
-      </c>
-      <c r="F23" s="7" t="n">
-        <v>589</v>
-      </c>
-      <c r="G23" s="9" t="n">
-        <v>9424</v>
-      </c>
-      <c r="H23" s="10" t="n">
-        <v>280</v>
-      </c>
-      <c r="I23" s="11" t="n">
-        <v>0.03062117235345582</v>
-      </c>
-      <c r="J23" s="7" t="n">
-        <v>541.78</v>
-      </c>
-      <c r="K23" s="7" t="n">
-        <v>571.1</v>
-      </c>
-      <c r="L23" s="12" t="n">
-        <v>0.03039049235993205</v>
-      </c>
-      <c r="M23" s="13" t="n">
-        <v>18.67</v>
-      </c>
-      <c r="N23" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>SHYAMMETL</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="n">
-        <v>965</v>
-      </c>
-      <c r="D24" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="E24" s="9" t="n">
-        <v>8685</v>
-      </c>
-      <c r="F24" s="7" t="n">
-        <v>961.6</v>
-      </c>
-      <c r="G24" s="9" t="n">
-        <v>8654.4</v>
-      </c>
-      <c r="H24" s="10" t="n">
-        <v>-30.5999999999998</v>
-      </c>
-      <c r="I24" s="11" t="n">
-        <v>-0.003523316062176142</v>
-      </c>
-      <c r="J24" s="7" t="n">
-        <v>908.65</v>
-      </c>
-      <c r="K24" s="7" t="n">
-        <v>933</v>
-      </c>
-      <c r="L24" s="12" t="n">
-        <v>0.02974209650582365</v>
-      </c>
-      <c r="M24" s="13" t="n">
-        <v>23.48</v>
-      </c>
-      <c r="N24" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H24">
+  <conditionalFormatting sqref="H2:H19">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1898,7 +1658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1974,27 +1734,27 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>5479</v>
+        <v>798</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>5424</v>
+        <v>750</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -2002,42 +1762,42 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-55</v>
+        <v>-288</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0602</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-0.18</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>960.1</v>
+        <v>260.45</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>257.85</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -2045,42 +1805,42 @@
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-516.79</v>
+        <v>-52.07</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.01</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>952.1</v>
+        <v>6500</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>948.8</v>
+        <v>6401.5</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -2088,42 +1848,42 @@
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-29.7</v>
+        <v>-98.5</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.0152</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>1475</v>
+        <v>571.5</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>1394.19</v>
+        <v>571.1</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -2131,42 +1891,42 @@
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-484.86</v>
+        <v>-6.4</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0007</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-1</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>248.05</v>
+        <v>965</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>242.8</v>
+        <v>933</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -2174,42 +1934,42 @@
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>-110.25</v>
+        <v>-288</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0332</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>-0.3</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>1039.2</v>
+        <v>5479</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>970</v>
+        <v>5424</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -2217,42 +1977,42 @@
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>-346</v>
+        <v>-55</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.01</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>199.96</v>
+        <v>960.1</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>193.31</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -2260,63 +2020,278 @@
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>-172.9</v>
+        <v>-516.79</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.0598</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>952.1</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="n">
+        <v>948.8</v>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="17" t="n">
+        <v>-29.7</v>
+      </c>
+      <c r="J9" s="18" t="n">
+        <v>-0.0035</v>
+      </c>
+      <c r="K9" s="19" t="n">
+        <v>-0.06</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>RAINBOW</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>1475</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>1394.19</v>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="I10" s="17" t="n">
+        <v>-484.86</v>
+      </c>
+      <c r="J10" s="18" t="n">
+        <v>-0.0548</v>
+      </c>
+      <c r="K10" s="19" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>248.05</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="n">
+        <v>242.8</v>
+      </c>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H11" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I11" s="17" t="n">
+        <v>-110.25</v>
+      </c>
+      <c r="J11" s="18" t="n">
+        <v>-0.0212</v>
+      </c>
+      <c r="K11" s="19" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>1039.2</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="n">
+        <v>970</v>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I12" s="17" t="n">
+        <v>-346</v>
+      </c>
+      <c r="J12" s="18" t="n">
+        <v>-0.06660000000000001</v>
+      </c>
+      <c r="K12" s="19" t="n">
+        <v>-0.82</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>199.96</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H13" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I13" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J13" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K13" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
           <t>SHYAMMETL</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C14" s="15" t="n">
         <v>986.4</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D14" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F14" s="15" t="n">
         <v>934.1900000000001</v>
       </c>
-      <c r="G9" s="14" t="inlineStr">
+      <c r="G14" s="14" t="inlineStr">
         <is>
           <t>STOP_LOSS</t>
         </is>
       </c>
-      <c r="H9" s="14" t="n">
+      <c r="H14" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="I9" s="17" t="n">
+      <c r="I14" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J9" s="18" t="n">
+      <c r="J14" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K9" s="19" t="n">
+      <c r="K14" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I9">
+  <conditionalFormatting sqref="I2:I14">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2334,7 +2309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2731,6 +2706,31 @@
       </c>
       <c r="G15" s="14" t="n">
         <v>23</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="n">
+        <v>201906.53</v>
+      </c>
+      <c r="C16" s="20" t="n">
+        <v>71333.23</v>
+      </c>
+      <c r="D16" s="20" t="n">
+        <v>130573.3</v>
+      </c>
+      <c r="E16" s="20" t="n">
+        <v>125957.25</v>
+      </c>
+      <c r="F16" s="20" t="n">
+        <v>-2709.52</v>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -2813,7 +2813,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -2821,22 +2821,22 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>2422</v>
+        <v>2435.8</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>2327.06</v>
+        <v>2337.94</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.9</v>
+        <v>6.4</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8359455076873799</v>
+        <v>0.8688361006746658</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -2845,36 +2845,36 @@
       </c>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>863.55</v>
+        <v>8753.5</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>809</v>
+        <v>8473.709999999999</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.9</v>
+        <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8253263132607304</v>
+        <v>0.8145659112026825</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -2883,36 +2883,36 @@
       </c>
       <c r="J3" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>18268</v>
+        <v>943.75</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>17022.71</v>
+        <v>897.61</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.8</v>
+        <v>6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8012942424727738</v>
+        <v>0.803014786086535</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -2921,36 +2921,36 @@
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>BSE</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>3683.4</v>
+        <v>1043.9</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>3466.51</v>
+        <v>981.51</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.8</v>
+        <v>6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7593399663677131</v>
+        <v>0.8007807134488749</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -2959,36 +2959,36 @@
       </c>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1024.5</v>
+        <v>748.45</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>966.11</v>
+        <v>707.9</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.7</v>
+        <v>5.9</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7954306133888533</v>
+        <v>0.8087565143618956</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -2997,36 +2997,36 @@
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1477.4</v>
+        <v>859.55</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1387.47</v>
+        <v>808.29</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.7</v>
+        <v>5.9</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7799987988468929</v>
+        <v>0.7955429644891528</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3035,36 +3035,36 @@
       </c>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>971.9</v>
+        <v>1450.5</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>928.62</v>
+        <v>1391.17</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.6</v>
+        <v>5.9</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7767036354900705</v>
+        <v>0.7830444794570355</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3073,36 +3073,36 @@
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1471.8</v>
+        <v>6755</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1415.11</v>
+        <v>6493.5</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.6</v>
+        <v>5.9</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7726357303010891</v>
+        <v>0.7825405001413971</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3111,36 +3111,36 @@
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>643.55</v>
+        <v>928.35</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>580.4299999999999</v>
+        <v>879.21</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.6</v>
+        <v>5.8</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.731179932735426</v>
+        <v>0.7840170888377167</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3149,36 +3149,36 @@
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1833.9</v>
+        <v>1529.2</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1753.99</v>
+        <v>1415.6</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.5</v>
+        <v>5.7</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7545073270339526</v>
+        <v>0.7461782410212904</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3187,36 +3187,36 @@
       </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>6771.5</v>
+        <v>1469.2</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>6513.71</v>
+        <v>1376.47</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.5</v>
+        <v>5.7</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7593459721332478</v>
+        <v>0.7366602028037005</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3225,36 +3225,36 @@
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>ADANIPOWER</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>218.07</v>
+        <v>2665.9</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>205.2</v>
+        <v>2561.37</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.5</v>
+        <v>5.7</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7347964045483664</v>
+        <v>0.7321748878923767</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3263,36 +3263,36 @@
       </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>961.6</v>
+        <v>840.1</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>913.5599999999999</v>
+        <v>805.58</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.4</v>
+        <v>5.6</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7611036595131326</v>
+        <v>0.7403981335595684</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3301,36 +3301,36 @@
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>8837</v>
+        <v>662.05</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>8573</v>
+        <v>626.41</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.4</v>
+        <v>5.6</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7468679932735427</v>
+        <v>0.7366349533389892</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3339,36 +3339,36 @@
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260707</v>
+        <v>20260708</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>766.65</v>
+        <v>4667</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>724.61</v>
+        <v>4308.83</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.3</v>
+        <v>5.5</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7611487027546444</v>
+        <v>0.7420534884660446</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-09
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Wed 08 Jul 2026</t>
+          <t>As of Thu 09 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹201,907</t>
+          <t>₹204,306</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-2,028  (-0.99%)</t>
+          <t>₹+2,400  (+1.19%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+0.95%</t>
+          <t>+2.15%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.52%</t>
+          <t>-0.35%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹130,573</t>
+          <t>₹132,973</t>
         </is>
       </c>
     </row>
@@ -796,16 +796,16 @@
         <v>4230</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>1450.5</v>
+        <v>1463.2</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>4351.5</v>
+        <v>4389.6</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>121.5</v>
+        <v>159.6000000000001</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.02872340425531915</v>
+        <v>0.03773049645390074</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>1312.63</v>
@@ -814,13 +814,13 @@
         <v>1388.671428571429</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.04262569557295513</v>
+        <v>0.05093532765758028</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>33.1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>4830</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>640.85</v>
+        <v>650.05</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>4485.95</v>
+        <v>4550.349999999999</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-344.0499999999998</v>
+        <v>-279.6500000000003</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.07123188405797098</v>
+        <v>-0.05789855072463775</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>612.1900000000001</v>
@@ -862,13 +862,13 @@
         <v>630.05</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.01685261761722722</v>
+        <v>0.03076686408737789</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>34.34</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>3678</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1791.7</v>
+        <v>1800.1</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>3583.4</v>
+        <v>3600.2</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-94.59999999999991</v>
+        <v>-77.80000000000018</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.02572050027188687</v>
+        <v>-0.02115280043501908</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1729.61</v>
@@ -910,13 +910,13 @@
         <v>1770.5</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.01183233800301392</v>
+        <v>0.01644353091494912</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>43.14</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>4242</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1469.2</v>
+        <v>1507.4</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>4407.6</v>
+        <v>4522.200000000001</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>165.6000000000001</v>
+        <v>280.2000000000003</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.03903818953323907</v>
+        <v>0.06605374823196612</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1324.47</v>
@@ -958,13 +958,13 @@
         <v>1414.35</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.03733324258099655</v>
+        <v>0.06172880456415031</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>35.79</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>5200</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1326</v>
+        <v>1377.8</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>5304</v>
+        <v>5511.2</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>104</v>
+        <v>311.1999999999998</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.02</v>
+        <v>0.05984615384615381</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1159.03</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1252</v>
+        <v>1261.4</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.05580693815987934</v>
+        <v>0.08448250834663948</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>64.73</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
@@ -1036,31 +1036,31 @@
         <v>5252.55</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>317.95</v>
+        <v>324.05</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>6041.05</v>
+        <v>6156.95</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>788.5</v>
+        <v>904.4000000000004</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.1501175619461024</v>
+        <v>0.1721830349068549</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>259.14</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>293.9928571428571</v>
+        <v>299.5892857142857</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.07534877451531014</v>
+        <v>0.07548438292150683</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>7.11</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>4387.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1557.4</v>
+        <v>1587.4</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>4672.200000000001</v>
+        <v>4762.200000000001</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>284.7000000000003</v>
+        <v>374.7000000000003</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.06488888888888895</v>
+        <v>0.08540170940170946</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1405.17</v>
@@ -1102,13 +1102,13 @@
         <v>1502.471428571428</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.0352694050523769</v>
+        <v>0.05350168289566069</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>38.34</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -1132,31 +1132,31 @@
         <v>8690</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>859.55</v>
+        <v>882.05</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>9455.049999999999</v>
+        <v>9702.549999999999</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>765.0499999999995</v>
+        <v>1012.549999999999</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.08803797468354424</v>
+        <v>0.1165189873417721</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>739.3099999999999</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>786.6535714285715</v>
+        <v>801.8</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.0848076651403973</v>
+        <v>0.0909812368913327</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>24.04</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>7540</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4077.6</v>
+        <v>4089</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>8155.2</v>
+        <v>8178</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>615.1999999999998</v>
+        <v>638</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.0815915119363395</v>
+        <v>0.08461538461538462</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>3604.1</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>3808.65</v>
+        <v>3813.921428571429</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.06595791642142432</v>
+        <v>0.06727282255528765</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>81.47</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11">
@@ -1228,31 +1228,31 @@
         <v>9031.549999999999</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>840.1</v>
+        <v>860.05</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>9241.1</v>
+        <v>9460.549999999999</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>209.5500000000008</v>
+        <v>429</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.02320199744229958</v>
+        <v>0.04750015224407771</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>783.09</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>805.2571428571429</v>
+        <v>807.8071428571428</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.0414746543778802</v>
+        <v>0.06074397667909672</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>16.6</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>7278.3</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>2491.2</v>
+        <v>2532</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>7473.599999999999</v>
+        <v>7596</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>195.2999999999997</v>
+        <v>317.7000000000003</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.02683318906887594</v>
+        <v>0.04365030295536049</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>2309.03</v>
@@ -1294,13 +1294,13 @@
         <v>2340.7</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.06041265253693</v>
+        <v>0.07555292259083736</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>59.36</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>9246.6</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>467.6</v>
+        <v>471.6</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>10287.2</v>
+        <v>10375.2</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>1040.6</v>
+        <v>1128.6</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.112538662859862</v>
+        <v>0.1220556745182013</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>386.74</v>
@@ -1342,13 +1342,13 @@
         <v>420.1285714285714</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.1015214469021143</v>
+        <v>0.1091421301344967</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -1372,31 +1372,31 @@
         <v>8790</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1529.2</v>
+        <v>1601.9</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>9175.200000000001</v>
+        <v>9611.400000000001</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>385.2000000000003</v>
+        <v>821.4000000000005</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.04382252559726966</v>
+        <v>0.09344709897610928</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1365.41</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>1397.635714285714</v>
+        <v>1421.75</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.08603471469676019</v>
+        <v>0.1124602035083339</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>45.25</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>9288.75</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>662.05</v>
+        <v>670.75</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>9930.75</v>
+        <v>10061.25</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>641.9999999999993</v>
+        <v>772.5</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.06911586596689537</v>
+        <v>0.08316511909568026</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>591.46</v>
@@ -1438,13 +1438,13 @@
         <v>621.0571428571428</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.06191806833752305</v>
+        <v>0.07408551195357015</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>14</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>8700</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>8753.5</v>
+        <v>8845.5</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>8753.5</v>
+        <v>8845.5</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>53.5</v>
+        <v>145.5</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.006149425287356322</v>
+        <v>0.01672413793103448</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>8339.209999999999</v>
@@ -1486,13 +1486,13 @@
         <v>8510.25</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.02778888444622151</v>
+        <v>0.03790062743768018</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>123.68</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
@@ -1516,16 +1516,16 @@
         <v>9000</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>908.1</v>
+        <v>910.9</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>9081</v>
+        <v>9109</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>81.00000000000023</v>
+        <v>108.9999999999998</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>0.009000000000000025</v>
+        <v>0.01211111111111109</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>836</v>
@@ -1534,13 +1534,13 @@
         <v>887.1</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>0.02312520647505781</v>
+        <v>0.02612800526951362</v>
       </c>
       <c r="M17" s="13" t="n">
         <v>29.64</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -1564,16 +1564,16 @@
         <v>7579.5</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>7363</v>
+        <v>7689</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>7363</v>
+        <v>7689</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>-216.5</v>
+        <v>109.5</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>-0.02856388943861732</v>
+        <v>0.01444686324955472</v>
       </c>
       <c r="J18" s="7" t="n">
         <v>7128.14</v>
@@ -1582,13 +1582,13 @@
         <v>7128.14</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>0.03189732446013849</v>
+        <v>0.07294316556119126</v>
       </c>
       <c r="M18" s="13" t="n">
         <v>209.96</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -1612,16 +1612,16 @@
         <v>8992.5</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>1762.4</v>
+        <v>1770.4</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>8812</v>
+        <v>8852</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>-180.4999999999995</v>
+        <v>-140.4999999999995</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>-0.02007228245760351</v>
+        <v>-0.01562413122046145</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>1680.3</v>
@@ -1630,13 +1630,13 @@
         <v>1680.3</v>
       </c>
       <c r="L19" s="12" t="n">
-        <v>0.04658420335905591</v>
+        <v>0.05089245368278363</v>
       </c>
       <c r="M19" s="13" t="n">
         <v>50.24</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -2309,7 +2309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2730,6 +2730,31 @@
         <v>-2709.52</v>
       </c>
       <c r="G16" s="14" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="n">
+        <v>204306.38</v>
+      </c>
+      <c r="C17" s="20" t="n">
+        <v>71333.23</v>
+      </c>
+      <c r="D17" s="20" t="n">
+        <v>132973.15</v>
+      </c>
+      <c r="E17" s="20" t="n">
+        <v>125957.25</v>
+      </c>
+      <c r="F17" s="20" t="n">
+        <v>-2709.52</v>
+      </c>
+      <c r="G17" s="14" t="n">
         <v>18</v>
       </c>
     </row>
@@ -2813,18 +2838,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>2435.8</v>
+        <v>8845.5</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>2337.94</v>
+        <v>8559.139999999999</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -2833,10 +2858,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8688361006746658</v>
+        <v>0.8715317335272492</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -2851,18 +2876,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SOLARINDS</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>8753.5</v>
+        <v>17380</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>8473.709999999999</v>
+        <v>16069.71</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -2874,7 +2899,7 @@
         <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8145659112026825</v>
+        <v>0.8091423261826849</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -2889,18 +2914,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>943.75</v>
+        <v>882.05</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>897.61</v>
+        <v>828.55</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -2912,7 +2937,7 @@
         <v>6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.803014786086535</v>
+        <v>0.8182392033288894</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -2927,7 +2952,7 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
@@ -2935,10 +2960,10 @@
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1043.9</v>
+        <v>1089.2</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>981.51</v>
+        <v>1024.8</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -2950,7 +2975,7 @@
         <v>6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8007807134488749</v>
+        <v>0.80683957500101</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -2965,18 +2990,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>748.45</v>
+        <v>951.45</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>707.9</v>
+        <v>904.41</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -2985,10 +3010,10 @@
         <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8087565143618956</v>
+        <v>0.801893709853351</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -3003,18 +3028,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>859.55</v>
+        <v>1507.4</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>808.29</v>
+        <v>1414.13</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -3023,10 +3048,10 @@
         <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7955429644891528</v>
+        <v>0.7924847493233143</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3041,7 +3066,7 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
@@ -3049,10 +3074,10 @@
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1450.5</v>
+        <v>1463.2</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1391.17</v>
+        <v>1403.23</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -3064,7 +3089,7 @@
         <v>5.9</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7830444794570355</v>
+        <v>0.7929806488102452</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3079,18 +3104,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>6755</v>
+        <v>860.05</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>6493.5</v>
+        <v>825.22</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -3102,7 +3127,7 @@
         <v>5.9</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7825405001413971</v>
+        <v>0.7915848584010019</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3117,18 +3142,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>928.35</v>
+        <v>6813</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>879.21</v>
+        <v>6533.5</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -3137,10 +3162,10 @@
         <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7840170888377167</v>
+        <v>0.7829737809558437</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3155,18 +3180,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1529.2</v>
+        <v>9074</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1415.6</v>
+        <v>8560.43</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -3175,10 +3200,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7461782410212904</v>
+        <v>0.7720155132711186</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3193,18 +3218,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1469.2</v>
+        <v>1601.9</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1376.47</v>
+        <v>1481.8</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -3213,10 +3238,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7366602028037005</v>
+        <v>0.7699400072718459</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3231,18 +3256,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>2665.9</v>
+        <v>1938.7</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>2561.37</v>
+        <v>1870</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -3251,10 +3276,10 @@
         <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7321748878923767</v>
+        <v>0.7540449642467579</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3269,18 +3294,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>840.1</v>
+        <v>2444.5</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>805.58</v>
+        <v>2345.24</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -3289,10 +3314,10 @@
         <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7403981335595684</v>
+        <v>0.7827374459661456</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3307,18 +3332,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>662.05</v>
+        <v>1481.5</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>626.41</v>
+        <v>1402.26</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -3330,7 +3355,7 @@
         <v>5.6</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7366349533389892</v>
+        <v>0.761648083060639</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3345,18 +3370,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260708</v>
+        <v>20260709</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>4667</v>
+        <v>7689</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>4308.83</v>
+        <v>7212.57</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -3365,10 +3390,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7420534884660446</v>
+        <v>0.753375348442613</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-10
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Thu 09 Jul 2026</t>
+          <t>As of Fri 10 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹204,306</t>
+          <t>₹204,751</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+2,400  (+1.19%)</t>
+          <t>₹+445  (+0.22%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.15%</t>
+          <t>+2.38%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.35%</t>
+          <t>-0.13%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹71,333</t>
+          <t>₹105,114</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹125,957</t>
+          <t>₹94,137</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹132,973</t>
+          <t>₹99,637</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹-2,710</t>
+          <t>₹-749</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -697,7 +697,7 @@
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
@@ -778,869 +778,533 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C2" s="7" t="n">
-        <v>1410</v>
+        <v>790</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E2" s="9" t="n">
-        <v>4230</v>
+        <v>8690</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>1463.2</v>
+        <v>889.85</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>4389.6</v>
+        <v>9788.35</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>159.6000000000001</v>
+        <v>1098.35</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.03773049645390074</v>
+        <v>0.1263924050632912</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>1312.63</v>
+        <v>739.3099999999999</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1388.671428571429</v>
+        <v>809.3107142857143</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.05093532765758028</v>
+        <v>0.09050883375207699</v>
       </c>
       <c r="M2" s="13" t="n">
-        <v>33.1</v>
+        <v>24.04</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>690</v>
+        <v>3770</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>4830</v>
+        <v>7540</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>650.05</v>
+        <v>4073.7</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>4550.349999999999</v>
+        <v>8147.4</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-279.6500000000003</v>
+        <v>607.3999999999996</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.05789855072463775</v>
+        <v>0.08055702917771879</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>612.1900000000001</v>
+        <v>3604.1</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>630.05</v>
+        <v>3813.921428571429</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.03076686408737789</v>
+        <v>0.0637696863854901</v>
       </c>
       <c r="M3" s="13" t="n">
-        <v>34.34</v>
+        <v>81.47</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>1839</v>
+        <v>821.05</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>3678</v>
+        <v>9031.549999999999</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1800.1</v>
+        <v>852.5</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>3600.2</v>
+        <v>9377.5</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-77.80000000000018</v>
+        <v>345.9500000000005</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.02115280043501908</v>
+        <v>0.03830460995067297</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>1729.61</v>
+        <v>783.09</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1770.5</v>
+        <v>807.8071428571428</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.01644353091494912</v>
+        <v>0.05242563887725182</v>
       </c>
       <c r="M4" s="13" t="n">
-        <v>43.14</v>
+        <v>16.6</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>1414</v>
+        <v>2426.1</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>4242</v>
+        <v>7278.3</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1507.4</v>
+        <v>2525.1</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>4522.200000000001</v>
+        <v>7575.299999999999</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>280.2000000000003</v>
+        <v>297</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.06605374823196612</v>
+        <v>0.04080623222455793</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>1324.47</v>
+        <v>2309.03</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1414.35</v>
+        <v>2340.7</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.06172880456415031</v>
+        <v>0.07302681081937352</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>35.79</v>
+        <v>59.36</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>1300</v>
+        <v>420.3</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>5200</v>
+        <v>9246.6</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1377.8</v>
+        <v>472.1</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>5511.2</v>
+        <v>10386.2</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>311.1999999999998</v>
+        <v>1139.6</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.05984615384615381</v>
+        <v>0.1232453009754937</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>1159.03</v>
+        <v>386.74</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1261.4</v>
+        <v>420.4464285714286</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.08448250834663948</v>
+        <v>0.1094123521045783</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>64.73</v>
+        <v>16.71</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>276.45</v>
+        <v>1465</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>5252.55</v>
+        <v>8790</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>324.05</v>
+        <v>1612.6</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>6156.95</v>
+        <v>9675.599999999999</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>904.4000000000004</v>
+        <v>885.5999999999995</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.1721830349068549</v>
+        <v>0.1007508532423208</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>259.14</v>
+        <v>1365.41</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>299.5892857142857</v>
+        <v>1432.192857142857</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.07548438292150683</v>
+        <v>0.1118734607820556</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>7.11</v>
+        <v>45.25</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>1462.5</v>
+        <v>619.25</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>4387.5</v>
+        <v>9288.75</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1587.4</v>
+        <v>668.55</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>4762.200000000001</v>
+        <v>10028.25</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>374.7000000000003</v>
+        <v>739.4999999999993</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.08540170940170946</v>
+        <v>0.07961243439644725</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>1405.17</v>
+        <v>591.46</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>1502.471428571428</v>
+        <v>621.0571428571428</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.05350168289566069</v>
+        <v>0.07103860166458326</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>38.34</v>
+        <v>14</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>790</v>
+        <v>8700</v>
       </c>
       <c r="D9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>8700</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>8841</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>8841</v>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>141</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>0.01620689655172414</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>8339.209999999999</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>8510.25</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>0.03741092636579572</v>
+      </c>
+      <c r="M9" s="13" t="n">
+        <v>123.68</v>
+      </c>
+      <c r="N9" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="E9" s="9" t="n">
-        <v>8690</v>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>882.05</v>
-      </c>
-      <c r="G9" s="9" t="n">
-        <v>9702.549999999999</v>
-      </c>
-      <c r="H9" s="10" t="n">
-        <v>1012.549999999999</v>
-      </c>
-      <c r="I9" s="11" t="n">
-        <v>0.1165189873417721</v>
-      </c>
-      <c r="J9" s="7" t="n">
-        <v>739.3099999999999</v>
-      </c>
-      <c r="K9" s="7" t="n">
-        <v>801.8</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>0.0909812368913327</v>
-      </c>
-      <c r="M9" s="13" t="n">
-        <v>24.04</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>3770</v>
+        <v>900</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>7540</v>
+        <v>9000</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4089</v>
+        <v>916.6</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>8178</v>
+        <v>9166</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>638</v>
+        <v>166.0000000000002</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.08461538461538462</v>
+        <v>0.01844444444444447</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>3604.1</v>
+        <v>836</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>3813.921428571429</v>
+        <v>887.1</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.06727282255528765</v>
+        <v>0.03218415884791621</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>81.47</v>
+        <v>29.64</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>821.05</v>
+        <v>7579.5</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>9031.549999999999</v>
+        <v>7579.5</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>860.05</v>
+        <v>7712</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>9460.549999999999</v>
+        <v>7712</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>429</v>
+        <v>132.5</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.04750015224407771</v>
+        <v>0.0174813642060822</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>783.09</v>
+        <v>7128.14</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>807.8071428571428</v>
+        <v>7128.14</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.06074397667909672</v>
+        <v>0.07570798755186718</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>16.6</v>
+        <v>209.96</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>2426.1</v>
+        <v>1798.5</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>7278.3</v>
+        <v>8992.5</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>2532</v>
+        <v>1787.9</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>7596</v>
+        <v>8939.5</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>317.7000000000003</v>
+        <v>-52.99999999999955</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.04365030295536049</v>
+        <v>-0.005893800389213183</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>2309.03</v>
+        <v>1680.3</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>2340.7</v>
+        <v>1680.3</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.07555292259083736</v>
+        <v>0.06018233681973272</v>
       </c>
       <c r="M12" s="13" t="n">
-        <v>59.36</v>
+        <v>50.24</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>HONASA</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>420.3</v>
-      </c>
-      <c r="D13" s="8" t="n">
-        <v>22</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>9246.6</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>471.6</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>10375.2</v>
-      </c>
-      <c r="H13" s="10" t="n">
-        <v>1128.6</v>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>0.1220556745182013</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>386.74</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>420.1285714285714</v>
-      </c>
-      <c r="L13" s="12" t="n">
-        <v>0.1091421301344967</v>
-      </c>
-      <c r="M13" s="13" t="n">
-        <v>16.71</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>WELCORP</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>1465</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="E14" s="9" t="n">
-        <v>8790</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>1601.9</v>
-      </c>
-      <c r="G14" s="9" t="n">
-        <v>9611.400000000001</v>
-      </c>
-      <c r="H14" s="10" t="n">
-        <v>821.4000000000005</v>
-      </c>
-      <c r="I14" s="11" t="n">
-        <v>0.09344709897610928</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>1365.41</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>1421.75</v>
-      </c>
-      <c r="L14" s="12" t="n">
-        <v>0.1124602035083339</v>
-      </c>
-      <c r="M14" s="13" t="n">
-        <v>45.25</v>
-      </c>
-      <c r="N14" s="6" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>SONACOMS</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>619.25</v>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="E15" s="9" t="n">
-        <v>9288.75</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>670.75</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>10061.25</v>
-      </c>
-      <c r="H15" s="10" t="n">
-        <v>772.5</v>
-      </c>
-      <c r="I15" s="11" t="n">
-        <v>0.08316511909568026</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>591.46</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>621.0571428571428</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>0.07408551195357015</v>
-      </c>
-      <c r="M15" s="13" t="n">
-        <v>14</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>APOLLOHOSP</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>8700</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <v>8700</v>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>8845.5</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>8845.5</v>
-      </c>
-      <c r="H16" s="10" t="n">
-        <v>145.5</v>
-      </c>
-      <c r="I16" s="11" t="n">
-        <v>0.01672413793103448</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>8339.209999999999</v>
-      </c>
-      <c r="K16" s="7" t="n">
-        <v>8510.25</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>0.03790062743768018</v>
-      </c>
-      <c r="M16" s="13" t="n">
-        <v>123.68</v>
-      </c>
-      <c r="N16" s="6" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>CGPOWER</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="n">
-        <v>900</v>
-      </c>
-      <c r="D17" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="E17" s="9" t="n">
-        <v>9000</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>910.9</v>
-      </c>
-      <c r="G17" s="9" t="n">
-        <v>9109</v>
-      </c>
-      <c r="H17" s="10" t="n">
-        <v>108.9999999999998</v>
-      </c>
-      <c r="I17" s="11" t="n">
-        <v>0.01211111111111109</v>
-      </c>
-      <c r="J17" s="7" t="n">
-        <v>836</v>
-      </c>
-      <c r="K17" s="7" t="n">
-        <v>887.1</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>0.02612800526951362</v>
-      </c>
-      <c r="M17" s="13" t="n">
-        <v>29.64</v>
-      </c>
-      <c r="N17" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>NAVINFLUOR</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="n">
-        <v>7579.5</v>
-      </c>
-      <c r="D18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="9" t="n">
-        <v>7579.5</v>
-      </c>
-      <c r="F18" s="7" t="n">
-        <v>7689</v>
-      </c>
-      <c r="G18" s="9" t="n">
-        <v>7689</v>
-      </c>
-      <c r="H18" s="10" t="n">
-        <v>109.5</v>
-      </c>
-      <c r="I18" s="11" t="n">
-        <v>0.01444686324955472</v>
-      </c>
-      <c r="J18" s="7" t="n">
-        <v>7128.14</v>
-      </c>
-      <c r="K18" s="7" t="n">
-        <v>7128.14</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>0.07294316556119126</v>
-      </c>
-      <c r="M18" s="13" t="n">
-        <v>209.96</v>
-      </c>
-      <c r="N18" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>IPCALAB</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>1798.5</v>
-      </c>
-      <c r="D19" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="E19" s="9" t="n">
-        <v>8992.5</v>
-      </c>
-      <c r="F19" s="7" t="n">
-        <v>1770.4</v>
-      </c>
-      <c r="G19" s="9" t="n">
-        <v>8852</v>
-      </c>
-      <c r="H19" s="10" t="n">
-        <v>-140.4999999999995</v>
-      </c>
-      <c r="I19" s="11" t="n">
-        <v>-0.01562413122046145</v>
-      </c>
-      <c r="J19" s="7" t="n">
-        <v>1680.3</v>
-      </c>
-      <c r="K19" s="7" t="n">
-        <v>1680.3</v>
-      </c>
-      <c r="L19" s="12" t="n">
-        <v>0.05089245368278363</v>
-      </c>
-      <c r="M19" s="13" t="n">
-        <v>50.24</v>
-      </c>
-      <c r="N19" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H19">
+  <conditionalFormatting sqref="H2:H12">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1658,7 +1322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1734,7 +1398,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -1743,41 +1407,41 @@
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>798</v>
+        <v>1410</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>750</v>
+        <v>1455.2</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-288</v>
+        <v>135.6</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.0321</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-0.92</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -1786,276 +1450,276 @@
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>260.45</v>
+        <v>690</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>257.85</v>
+        <v>660.45</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-52.07</v>
+        <v>-206.85</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0428</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-0.13</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>6500</v>
+        <v>1839</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>6401.5</v>
+        <v>1828.1</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-98.5</v>
+        <v>-21.8</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.0059</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>571.5</v>
+        <v>1414</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>571.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-6.4</v>
+        <v>371.4</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.0007</v>
+        <v>0.0876</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-0.01</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>965</v>
+        <v>1300</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>933</v>
+        <v>1389.1</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>-288</v>
+        <v>356.4</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>-0.0332</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>-0.57</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>5479</v>
+        <v>276.45</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>5424</v>
+        <v>330.1</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>-55</v>
+        <v>1019.35</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>-0.01</v>
+        <v>0.1941</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>-0.18</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>960.1</v>
+        <v>1462.5</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>1564.7</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>-516.79</v>
+        <v>306.6</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>-0.0598</v>
+        <v>0.0699</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>-0.87</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>952.1</v>
+        <v>798</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>948.8</v>
+        <v>750</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
@@ -2063,42 +1727,42 @@
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>-29.7</v>
+        <v>-288</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.0602</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1475</v>
+        <v>260.45</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>1394.19</v>
+        <v>257.85</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
@@ -2106,42 +1770,42 @@
         </is>
       </c>
       <c r="H10" s="14" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>-484.86</v>
+        <v>-52.07</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.01</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>-1</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>248.05</v>
+        <v>6500</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>242.8</v>
+        <v>6401.5</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
@@ -2149,42 +1813,42 @@
         </is>
       </c>
       <c r="H11" s="14" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>-110.25</v>
+        <v>-98.5</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0152</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>-0.3</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>1039.2</v>
+        <v>571.5</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>970</v>
+        <v>571.1</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -2192,42 +1856,42 @@
         </is>
       </c>
       <c r="H12" s="14" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>-346</v>
+        <v>-6.4</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0007</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>199.96</v>
+        <v>965</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>193.31</v>
+        <v>933</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
@@ -2235,63 +1899,364 @@
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>-172.9</v>
+        <v>-288</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.0332</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>5479</v>
+      </c>
+      <c r="D14" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="n">
+        <v>5424</v>
+      </c>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="17" t="n">
+        <v>-55</v>
+      </c>
+      <c r="J14" s="18" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="K14" s="19" t="n">
+        <v>-0.18</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>960.1</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="n">
+        <v>902.6799999999999</v>
+      </c>
+      <c r="G15" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I15" s="17" t="n">
+        <v>-516.79</v>
+      </c>
+      <c r="J15" s="18" t="n">
+        <v>-0.0598</v>
+      </c>
+      <c r="K15" s="19" t="n">
+        <v>-0.87</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>952.1</v>
+      </c>
+      <c r="D16" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>948.8</v>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H16" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="17" t="n">
+        <v>-29.7</v>
+      </c>
+      <c r="J16" s="18" t="n">
+        <v>-0.0035</v>
+      </c>
+      <c r="K16" s="19" t="n">
+        <v>-0.06</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>RAINBOW</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="n">
+        <v>1475</v>
+      </c>
+      <c r="D17" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="n">
+        <v>1394.19</v>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="I17" s="17" t="n">
+        <v>-484.86</v>
+      </c>
+      <c r="J17" s="18" t="n">
+        <v>-0.0548</v>
+      </c>
+      <c r="K17" s="19" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="n">
+        <v>248.05</v>
+      </c>
+      <c r="D18" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F18" s="15" t="n">
+        <v>242.8</v>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I18" s="17" t="n">
+        <v>-110.25</v>
+      </c>
+      <c r="J18" s="18" t="n">
+        <v>-0.0212</v>
+      </c>
+      <c r="K18" s="19" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="n">
+        <v>1039.2</v>
+      </c>
+      <c r="D19" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="n">
+        <v>970</v>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I19" s="17" t="n">
+        <v>-346</v>
+      </c>
+      <c r="J19" s="18" t="n">
+        <v>-0.06660000000000001</v>
+      </c>
+      <c r="K19" s="19" t="n">
+        <v>-0.82</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="n">
+        <v>199.96</v>
+      </c>
+      <c r="D20" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I20" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J20" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K20" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
           <t>SHYAMMETL</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C21" s="15" t="n">
         <v>986.4</v>
       </c>
-      <c r="D14" s="16" t="n">
+      <c r="D21" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="F14" s="15" t="n">
+      <c r="F21" s="15" t="n">
         <v>934.1900000000001</v>
       </c>
-      <c r="G14" s="14" t="inlineStr">
+      <c r="G21" s="14" t="inlineStr">
         <is>
           <t>STOP_LOSS</t>
         </is>
       </c>
-      <c r="H14" s="14" t="n">
+      <c r="H21" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="I14" s="17" t="n">
+      <c r="I21" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J14" s="18" t="n">
+      <c r="J21" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K14" s="19" t="n">
+      <c r="K21" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I14">
+  <conditionalFormatting sqref="I2:I21">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2309,7 +2274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2756,6 +2721,31 @@
       </c>
       <c r="G17" s="14" t="n">
         <v>18</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="n">
+        <v>204751.08</v>
+      </c>
+      <c r="C18" s="20" t="n">
+        <v>105113.98</v>
+      </c>
+      <c r="D18" s="20" t="n">
+        <v>99637.10000000001</v>
+      </c>
+      <c r="E18" s="20" t="n">
+        <v>94137.2</v>
+      </c>
+      <c r="F18" s="20" t="n">
+        <v>-748.8200000000001</v>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -2838,30 +2828,30 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>8845.5</v>
+        <v>2435.5</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8559.139999999999</v>
+        <v>2335.46</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8715317335272492</v>
+        <v>0.863963963963964</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -2870,36 +2860,36 @@
       </c>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>17380</v>
+        <v>1117.2</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>16069.71</v>
+        <v>1050.57</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.1</v>
+        <v>6.9</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8091423261826849</v>
+        <v>0.8223407263766008</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -2908,36 +2898,36 @@
       </c>
       <c r="J3" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>882.05</v>
+        <v>8841</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>828.55</v>
+        <v>8553.290000000001</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6</v>
+        <v>6.9</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8182392033288894</v>
+        <v>0.821985213913465</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -2946,36 +2936,36 @@
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1089.2</v>
+        <v>889.85</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1024.8</v>
+        <v>836.16</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6</v>
+        <v>6.8</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.80683957500101</v>
+        <v>0.8252201753322829</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -2984,36 +2974,36 @@
       </c>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>951.45</v>
+        <v>1265</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>904.41</v>
+        <v>1182.49</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6</v>
+        <v>6.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.801893709853351</v>
+        <v>0.8061265301175615</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -3022,36 +3012,36 @@
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1507.4</v>
+        <v>2525.1</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1414.13</v>
+        <v>2384.96</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6</v>
+        <v>6.7</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7924847493233143</v>
+        <v>0.7980921504464106</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3060,36 +3050,36 @@
       </c>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1463.2</v>
+        <v>968</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1403.23</v>
+        <v>920.8099999999999</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.9</v>
+        <v>6.7</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7929806488102452</v>
+        <v>0.792481719387549</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3098,36 +3088,36 @@
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>860.05</v>
+        <v>1455.2</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>825.22</v>
+        <v>1396.59</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.9</v>
+        <v>6.6</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7915848584010019</v>
+        <v>0.7830747788146892</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3136,36 +3126,36 @@
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>6813</v>
+        <v>1537.8</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>6533.5</v>
+        <v>1442.61</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.9</v>
+        <v>6.6</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7829737809558437</v>
+        <v>0.7731971882196097</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3174,36 +3164,36 @@
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>SOLARINDS</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>9074</v>
+        <v>18236</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>8560.43</v>
+        <v>16870.14</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.9</v>
+        <v>6.6</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7720155132711186</v>
+        <v>0.7649466731305297</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3212,36 +3202,36 @@
       </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1601.9</v>
+        <v>1564.7</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1481.8</v>
+        <v>1479.99</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.9</v>
+        <v>6.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7699400072718459</v>
+        <v>0.7551993697733609</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3250,36 +3240,36 @@
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1938.7</v>
+        <v>9210.5</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1870</v>
+        <v>8693.5</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.9</v>
+        <v>6.5</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7540449642467579</v>
+        <v>0.7459964448753686</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3288,36 +3278,36 @@
       </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>2444.5</v>
+        <v>1612.6</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>2345.24</v>
+        <v>1492.33</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.7</v>
+        <v>6.4</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7827374459661456</v>
+        <v>0.7421373166888863</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3326,36 +3316,36 @@
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1481.5</v>
+        <v>576.35</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1402.26</v>
+        <v>535.64</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.6</v>
+        <v>6.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.761648083060639</v>
+        <v>0.7722801276612936</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3364,36 +3354,36 @@
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260709</v>
+        <v>20260710</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>CAPLIPOINT</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>7689</v>
+        <v>2583.6</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>7212.57</v>
+        <v>2377.59</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0467</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>5333</v>
+        <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.6</v>
+        <v>6.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.753375348442613</v>
+        <v>0.7458530279158082</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>
@@ -3402,7 +3392,7 @@
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-12
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -820,7 +820,7 @@
         <v>24.04</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
@@ -868,7 +868,7 @@
         <v>81.47</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -916,7 +916,7 @@
         <v>16.6</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -964,7 +964,7 @@
         <v>59.36</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -1012,7 +1012,7 @@
         <v>16.71</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -1060,7 +1060,7 @@
         <v>45.25</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
@@ -1108,7 +1108,7 @@
         <v>14</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
@@ -1156,7 +1156,7 @@
         <v>123.68</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10">
@@ -1204,7 +1204,7 @@
         <v>29.64</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -1252,7 +1252,7 @@
         <v>209.96</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -1300,7 +1300,7 @@
         <v>50.24</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2851,7 +2851,7 @@
         <v>7</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.863963963963964</v>
+        <v>0.8645719891095451</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -2889,7 +2889,7 @@
         <v>6.9</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8223407263766008</v>
+        <v>0.8231342088404869</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -2927,7 +2927,7 @@
         <v>6.9</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.821985213913465</v>
+        <v>0.8227808696348494</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -2965,7 +2965,7 @@
         <v>6.8</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8252201753322829</v>
+        <v>0.8260009609224855</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -3003,7 +3003,7 @@
         <v>6.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8061265301175615</v>
+        <v>0.8069927130044843</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -3041,7 +3041,7 @@
         <v>6.7</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7980921504464106</v>
+        <v>0.7989950352338244</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3079,7 +3079,7 @@
         <v>6.7</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.792481719387549</v>
+        <v>0.7934096732863549</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3114,10 +3114,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7830747788146892</v>
+        <v>0.7840446828955797</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3155,7 +3155,7 @@
         <v>6.6</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7731971882196097</v>
+        <v>0.7742102418321589</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3193,7 +3193,7 @@
         <v>6.6</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7649466731305297</v>
+        <v>0.7646570707879565</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3231,7 +3231,7 @@
         <v>6.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7551993697733609</v>
+        <v>0.7562930413196669</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3269,7 +3269,7 @@
         <v>6.5</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7459964448753686</v>
+        <v>0.7471312459961563</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3307,7 +3307,7 @@
         <v>6.4</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7421373166888863</v>
+        <v>0.7419492713004484</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3345,7 +3345,7 @@
         <v>6.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7722801276612936</v>
+        <v>0.7732973654708519</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3383,7 +3383,7 @@
         <v>6.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7458530279158082</v>
+        <v>0.7469881085842408</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-13
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Fri 10 Jul 2026</t>
+          <t>As of Mon 13 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹204,751</t>
+          <t>₹204,806</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+445  (+0.22%)</t>
+          <t>₹+55  (+0.03%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.38%</t>
+          <t>+2.40%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.13%</t>
+          <t>-0.11%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹105,114</t>
+          <t>₹71,410</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹94,137</t>
+          <t>₹127,842</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹99,637</t>
+          <t>₹133,397</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -697,7 +697,7 @@
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
@@ -796,31 +796,31 @@
         <v>8690</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>889.85</v>
+        <v>897.65</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>9788.35</v>
+        <v>9874.15</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>1098.35</v>
+        <v>1184.15</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.1263924050632912</v>
+        <v>0.1362658227848101</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>739.3099999999999</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>809.3107142857143</v>
+        <v>817.7428571428571</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.09050883375207699</v>
+        <v>0.08901815056775229</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>24.04</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>7540</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>4073.7</v>
+        <v>4045.4</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8147.4</v>
+        <v>8090.8</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>607.3999999999996</v>
+        <v>550.8000000000002</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.08055702917771879</v>
+        <v>0.07305039787798411</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>3604.1</v>
@@ -862,13 +862,13 @@
         <v>3813.921428571429</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.0637696863854901</v>
+        <v>0.0572201936591119</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>81.47</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -892,31 +892,31 @@
         <v>9031.549999999999</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>852.5</v>
+        <v>846.75</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9377.5</v>
+        <v>9314.25</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>345.9500000000005</v>
+        <v>282.7000000000005</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.03830460995067297</v>
+        <v>0.03130138237622562</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>783.09</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>807.8071428571428</v>
+        <v>808.5785714285714</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.05242563887725182</v>
+        <v>0.04507992745370957</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>16.6</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>7278.3</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>2525.1</v>
+        <v>2507.5</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>7575.299999999999</v>
+        <v>7522.5</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>297</v>
+        <v>244.2000000000003</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.04080623222455793</v>
+        <v>0.03355179094019212</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>2309.03</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>2340.7</v>
+        <v>2348.371428571429</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.07302681081937352</v>
+        <v>0.06346104543512318</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>59.36</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>9246.6</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>472.1</v>
+        <v>472.25</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>10386.2</v>
+        <v>10389.5</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>1139.6</v>
+        <v>1142.9</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.1232453009754937</v>
+        <v>0.1236021889126814</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>386.74</v>
@@ -1006,13 +1006,13 @@
         <v>420.4464285714286</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.1094123521045783</v>
+        <v>0.1096952280117975</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -1036,31 +1036,31 @@
         <v>8790</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1612.6</v>
+        <v>1619.9</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>9675.599999999999</v>
+        <v>9719.400000000001</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>885.5999999999995</v>
+        <v>929.4000000000005</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.1007508532423208</v>
+        <v>0.1057337883959045</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1365.41</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1432.192857142857</v>
+        <v>1437.992857142857</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.1118734607820556</v>
+        <v>0.112295291596483</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>45.25</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>9288.75</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>668.55</v>
+        <v>670.85</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>10028.25</v>
+        <v>10062.75</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>739.4999999999993</v>
+        <v>774.0000000000003</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.07961243439644725</v>
+        <v>0.08332660476382725</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>591.46</v>
@@ -1102,13 +1102,13 @@
         <v>621.0571428571428</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.07103860166458326</v>
+        <v>0.07422353304443199</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>14</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>8700</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>8841</v>
+        <v>8782.5</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8841</v>
+        <v>8782.5</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>141</v>
+        <v>82.5</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.01620689655172414</v>
+        <v>0.009482758620689655</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>8339.209999999999</v>
@@ -1150,13 +1150,13 @@
         <v>8510.25</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.03741092636579572</v>
+        <v>0.03099914602903501</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>123.68</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>9000</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>916.6</v>
+        <v>905.5</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9166</v>
+        <v>9055</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>166.0000000000002</v>
+        <v>55</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.01844444444444447</v>
+        <v>0.006111111111111111</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>836</v>
@@ -1198,13 +1198,13 @@
         <v>887.1</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.03218415884791621</v>
+        <v>0.02032026504693537</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>29.64</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>7579.5</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>7712</v>
+        <v>7637</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>7712</v>
+        <v>7637</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>132.5</v>
+        <v>57.5</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.0174813642060822</v>
+        <v>0.007586252391318688</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>7128.14</v>
@@ -1246,13 +1246,13 @@
         <v>7128.14</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.07570798755186718</v>
+        <v>0.06663087599842867</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>209.96</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>8992.5</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>1787.9</v>
+        <v>1823.3</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>8939.5</v>
+        <v>9116.5</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-52.99999999999955</v>
+        <v>123.9999999999998</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.005893800389213183</v>
+        <v>0.01378926883514037</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1680.3</v>
@@ -1294,17 +1294,209 @@
         <v>1680.3</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.06018233681973272</v>
+        <v>0.07842922174079965</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>50.24</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>JBCHEPHARM</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>2415.2</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>7245.6</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>2460</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>7380</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>134.4000000000005</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0.01854918847300438</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>2335.46</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>2335.46</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>0.05062601626016259</v>
+      </c>
+      <c r="M13" s="13" t="n">
+        <v>49.27</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>PREMIERENE</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>1114.9</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>8919.200000000001</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>1109.5</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>8876</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>-43.20000000000073</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>-0.004843483720513132</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>1050.57</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>1050.57</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>0.05311401532221727</v>
+      </c>
+      <c r="M14" s="13" t="n">
+        <v>32.69</v>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>SAILIFE</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>1269</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>8883</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>1272.1</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>8904.699999999999</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>21.69999999999936</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>0.002442868400315137</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>1182.49</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>1182.49</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>0.07044257526923976</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>39.97</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>FORTIS</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>961.85</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>8656.65</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>963.5</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>8671.5</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>14.8499999999998</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>0.001715444196080446</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>920.8099999999999</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>920.8099999999999</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0.04430721328489887</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>23.22</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H12">
+  <conditionalFormatting sqref="H2:H16">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2274,7 +2466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2746,6 +2938,31 @@
       </c>
       <c r="G18" s="14" t="n">
         <v>11</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n">
+        <v>204806.08</v>
+      </c>
+      <c r="C19" s="20" t="n">
+        <v>71409.53</v>
+      </c>
+      <c r="D19" s="20" t="n">
+        <v>133396.55</v>
+      </c>
+      <c r="E19" s="20" t="n">
+        <v>127841.65</v>
+      </c>
+      <c r="F19" s="20" t="n">
+        <v>-748.8200000000001</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -2828,18 +3045,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>2435.5</v>
+        <v>8782.5</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>2335.46</v>
+        <v>8485.43</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -2851,7 +3068,7 @@
         <v>7</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8645719891095451</v>
+        <v>0.8336533071748878</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -2866,18 +3083,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1117.2</v>
+        <v>2460</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1050.57</v>
+        <v>2361.46</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -2889,7 +3106,7 @@
         <v>6.9</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8231342088404869</v>
+        <v>0.8428551409352978</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -2904,18 +3121,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>8841</v>
+        <v>1029.35</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>8553.290000000001</v>
+        <v>970.3</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -2924,10 +3141,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8227808696348494</v>
+        <v>0.8033211883408071</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -2942,18 +3159,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>889.85</v>
+        <v>1272.1</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>836.16</v>
+        <v>1192.16</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -2962,10 +3179,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.8</v>
+        <v>6.6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8260009609224855</v>
+        <v>0.7913526985906471</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -2980,18 +3197,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1265</v>
+        <v>897.65</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1182.49</v>
+        <v>844.38</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -3000,10 +3217,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8069927130044843</v>
+        <v>0.7857823510570147</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -3018,18 +3235,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>2525.1</v>
+        <v>1427</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>2384.96</v>
+        <v>1366.46</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -3038,10 +3255,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7989950352338244</v>
+        <v>0.7741231582319026</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3056,18 +3273,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>968</v>
+        <v>1558.6</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>920.8099999999999</v>
+        <v>1464.94</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -3076,10 +3293,10 @@
         <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7934096732863549</v>
+        <v>0.7500630605381166</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3094,18 +3311,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>OFSS</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1455.2</v>
+        <v>11746</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1396.59</v>
+        <v>10897.07</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -3114,10 +3331,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7840446828955797</v>
+        <v>0.7312780269058297</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3132,18 +3349,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1537.8</v>
+        <v>1823.3</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1442.61</v>
+        <v>1710.01</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -3152,10 +3369,10 @@
         <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7742102418321589</v>
+        <v>0.7715146540679052</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3170,18 +3387,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>18236</v>
+        <v>9306.5</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>16870.14</v>
+        <v>8776.57</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -3190,10 +3407,10 @@
         <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7646570707879565</v>
+        <v>0.7337183696348495</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3208,18 +3425,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1564.7</v>
+        <v>1109.5</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1479.99</v>
+        <v>1044.11</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -3228,10 +3445,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7562930413196669</v>
+        <v>0.738540999359385</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3246,18 +3463,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>9210.5</v>
+        <v>1921.4</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>8693.5</v>
+        <v>1855.64</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -3266,10 +3483,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7471312459961563</v>
+        <v>0.7156159913516976</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3284,18 +3501,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1612.6</v>
+        <v>963.5</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1492.33</v>
+        <v>917.0599999999999</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -3304,10 +3521,10 @@
         <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7419492713004484</v>
+        <v>0.7145399583600256</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3322,18 +3539,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>576.35</v>
+        <v>1810.3</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>535.64</v>
+        <v>1726.07</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -3342,10 +3559,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7732973654708519</v>
+        <v>0.712533031710442</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3360,18 +3577,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260710</v>
+        <v>20260713</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>CAPLIPOINT</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>2583.6</v>
+        <v>6264</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>2377.59</v>
+        <v>5941.21</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -3380,10 +3597,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7469881085842408</v>
+        <v>0.7234835442024343</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-14
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Mon 13 Jul 2026</t>
+          <t>As of Tue 14 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹204,806</t>
+          <t>₹205,528</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+55  (+0.03%)</t>
+          <t>₹+722  (+0.35%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.40%</t>
+          <t>+2.76%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.11%</t>
+          <t>+0.00%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹133,397</t>
+          <t>₹134,118</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -796,31 +796,31 @@
         <v>8690</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>897.65</v>
+        <v>895.1</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>9874.15</v>
+        <v>9846.1</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>1184.15</v>
+        <v>1156.1</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.1362658227848101</v>
+        <v>0.1330379746835443</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>739.3099999999999</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>817.7428571428571</v>
+        <v>820.6357142857142</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.08901815056775229</v>
+        <v>0.08319102414734195</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>24.04</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>7540</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>4045.4</v>
+        <v>4051.2</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8090.8</v>
+        <v>8102.4</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>550.8000000000002</v>
+        <v>562.3999999999996</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.07305039787798411</v>
+        <v>0.07458885941644558</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>3604.1</v>
@@ -862,13 +862,13 @@
         <v>3813.921428571429</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.0572201936591119</v>
+        <v>0.05856994752877445</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>81.47</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -892,31 +892,31 @@
         <v>9031.549999999999</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>846.75</v>
+        <v>848.25</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9314.25</v>
+        <v>9330.75</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>282.7000000000005</v>
+        <v>299.2000000000005</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.03130138237622562</v>
+        <v>0.03312831130869015</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>783.09</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>808.5785714285714</v>
+        <v>810.2285714285714</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.04507992745370957</v>
+        <v>0.04482337585785865</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>16.6</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>7278.3</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>2507.5</v>
+        <v>2531.1</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>7522.5</v>
+        <v>7593.299999999999</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>244.2000000000003</v>
+        <v>315</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.03355179094019212</v>
+        <v>0.04327933720786448</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>2309.03</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>2348.371428571429</v>
+        <v>2358.721428571428</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.06346104543512318</v>
+        <v>0.06810421217200895</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>59.36</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>9246.6</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>472.25</v>
+        <v>474.4</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>10389.5</v>
+        <v>10436.8</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>1142.9</v>
+        <v>1190.199999999999</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.1236021889126814</v>
+        <v>0.1287175826790387</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>386.74</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>420.4464285714286</v>
+        <v>422.5428571428571</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.1096952280117975</v>
+        <v>0.1093110093953264</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -1036,31 +1036,31 @@
         <v>8790</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1619.9</v>
+        <v>1683.4</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>9719.400000000001</v>
+        <v>10100.4</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>929.4000000000005</v>
+        <v>1310.400000000001</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.1057337883959045</v>
+        <v>0.1490784982935154</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1365.41</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1437.992857142857</v>
+        <v>1490.692857142857</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.112295291596483</v>
+        <v>0.1144749571445543</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>45.25</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>9288.75</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>670.85</v>
+        <v>666.8</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>10062.75</v>
+        <v>10002</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>774.0000000000003</v>
+        <v>713.2499999999993</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.08332660476382725</v>
+        <v>0.07678643520387558</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>591.46</v>
@@ -1102,13 +1102,13 @@
         <v>621.0571428571428</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.07422353304443199</v>
+        <v>0.06860056560116547</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>14</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>8700</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>8782.5</v>
+        <v>8900.5</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8782.5</v>
+        <v>8900.5</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>82.5</v>
+        <v>200.5</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.009482758620689655</v>
+        <v>0.02304597701149425</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>8339.209999999999</v>
@@ -1150,13 +1150,13 @@
         <v>8510.25</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.03099914602903501</v>
+        <v>0.04384585135666536</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>123.68</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>9000</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>905.5</v>
+        <v>913.85</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9055</v>
+        <v>9138.5</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>55</v>
+        <v>138.5000000000002</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.006111111111111111</v>
+        <v>0.01538888888888891</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>836</v>
@@ -1198,13 +1198,13 @@
         <v>887.1</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.02032026504693537</v>
+        <v>0.02927176232423264</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>29.64</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -1228,31 +1228,31 @@
         <v>7579.5</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>7637</v>
+        <v>7586</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>7637</v>
+        <v>7586</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>57.5</v>
+        <v>6.5</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.007586252391318688</v>
+        <v>0.0008575763572795039</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>7128.14</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>7128.14</v>
+        <v>7164.5</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.06663087599842867</v>
+        <v>0.05556287898760875</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>209.96</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>8992.5</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>1823.3</v>
+        <v>1840.4</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>9116.5</v>
+        <v>9202</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>123.9999999999998</v>
+        <v>209.5000000000005</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.01378926883514037</v>
+        <v>0.0232971921045316</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1680.3</v>
@@ -1294,13 +1294,13 @@
         <v>1680.3</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.07842922174079965</v>
+        <v>0.08699195826994138</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>50.24</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -1324,31 +1324,31 @@
         <v>7245.6</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>2460</v>
+        <v>2487.6</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>7380</v>
+        <v>7462.799999999999</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>134.4000000000005</v>
+        <v>217.2000000000003</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.01854918847300438</v>
+        <v>0.02997681351440878</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>2335.46</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>2335.46</v>
+        <v>2337.814285714285</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.05062601626016259</v>
+        <v>0.06021294190614051</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>49.27</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>8919.200000000001</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1109.5</v>
+        <v>1100.9</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>8876</v>
+        <v>8807.200000000001</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>-43.20000000000073</v>
+        <v>-112</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>-0.004843483720513132</v>
+        <v>-0.01255718001614494</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1050.57</v>
@@ -1390,13 +1390,13 @@
         <v>1050.57</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.05311401532221727</v>
+        <v>0.04571714052139172</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>32.69</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>8883</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1272.1</v>
+        <v>1268.8</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>8904.699999999999</v>
+        <v>8881.6</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>21.69999999999936</v>
+        <v>-1.400000000000318</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.002442868400315137</v>
+        <v>-0.0001576044129235977</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>1182.49</v>
@@ -1438,13 +1438,13 @@
         <v>1182.49</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.07044257526923976</v>
+        <v>0.06802490542244637</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>39.97</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1468,31 +1468,31 @@
         <v>8656.65</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>963.5</v>
+        <v>969.75</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>8671.5</v>
+        <v>8727.75</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>14.8499999999998</v>
+        <v>71.0999999999998</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.001715444196080446</v>
+        <v>0.008213338878203438</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>920.8099999999999</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>920.8099999999999</v>
+        <v>935.6</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.04430721328489887</v>
+        <v>0.03521526166537765</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>23.22</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2962,6 +2962,31 @@
         <v>-748.8200000000001</v>
       </c>
       <c r="G19" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B20" s="20" t="n">
+        <v>205527.63</v>
+      </c>
+      <c r="C20" s="20" t="n">
+        <v>71409.53</v>
+      </c>
+      <c r="D20" s="20" t="n">
+        <v>134118.1</v>
+      </c>
+      <c r="E20" s="20" t="n">
+        <v>127841.65</v>
+      </c>
+      <c r="F20" s="20" t="n">
+        <v>-748.8200000000001</v>
+      </c>
+      <c r="G20" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3045,18 +3070,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>8782.5</v>
+        <v>2487.6</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8485.43</v>
+        <v>2387.74</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -3065,10 +3090,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7</v>
+        <v>7.1</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8336533071748878</v>
+        <v>0.8612496263079223</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -3083,18 +3108,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>2460</v>
+        <v>8900.5</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>2361.46</v>
+        <v>8596.860000000001</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -3103,10 +3128,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8428551409352978</v>
+        <v>0.8325430991529646</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -3121,18 +3146,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1029.35</v>
+        <v>1555.4</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>970.3</v>
+        <v>1491.86</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -3141,10 +3166,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8033211883408071</v>
+        <v>0.7929207772795218</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -3159,18 +3184,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1272.1</v>
+        <v>1683.4</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1192.16</v>
+        <v>1554.93</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -3179,10 +3204,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7913526985906471</v>
+        <v>0.7670911808669656</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -3197,18 +3222,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>897.65</v>
+        <v>7188.5</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>844.38</v>
+        <v>6877.29</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -3217,10 +3242,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7857823510570147</v>
+        <v>0.7628440458395616</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -3235,18 +3260,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>ADANIPOWER</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1427</v>
+        <v>226.17</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1366.46</v>
+        <v>213.68</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -3255,10 +3280,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7741231582319026</v>
+        <v>0.7545969108121575</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3273,18 +3298,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1558.6</v>
+        <v>1100.9</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1464.94</v>
+        <v>1036.13</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -3296,7 +3321,7 @@
         <v>6.5</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7500630605381166</v>
+        <v>0.7612137518684605</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3311,18 +3336,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>OFSS</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>11746</v>
+        <v>9532.5</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>10897.07</v>
+        <v>8992.360000000001</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -3334,7 +3359,7 @@
         <v>6.5</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7312780269058297</v>
+        <v>0.7433492775286498</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3349,18 +3374,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1823.3</v>
+        <v>1427.1</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1710.01</v>
+        <v>1364.84</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -3369,10 +3394,10 @@
         <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7715146540679052</v>
+        <v>0.7489606377678126</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3387,18 +3412,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>9306.5</v>
+        <v>1821.9</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>8776.57</v>
+        <v>1739.2</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -3407,10 +3432,10 @@
         <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7337183696348495</v>
+        <v>0.7467324364723468</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3425,18 +3450,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1109.5</v>
+        <v>1942.6</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1044.11</v>
+        <v>1873.47</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -3445,10 +3470,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.738540999359385</v>
+        <v>0.7474080717488789</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3463,18 +3488,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1921.4</v>
+        <v>1035.95</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1855.64</v>
+        <v>976.61</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -3483,10 +3508,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7156159913516976</v>
+        <v>0.7570672645739911</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3501,18 +3526,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>963.5</v>
+        <v>1484.1</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>917.0599999999999</v>
+        <v>1406.96</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -3521,10 +3546,10 @@
         <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7145399583600256</v>
+        <v>0.7788978574987544</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3539,18 +3564,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1810.3</v>
+        <v>1268.8</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1726.07</v>
+        <v>1188.27</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -3559,10 +3584,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.712533031710442</v>
+        <v>0.7521155954160439</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3577,7 +3602,7 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260713</v>
+        <v>20260714</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
@@ -3585,10 +3610,10 @@
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>6264</v>
+        <v>6072</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>5941.21</v>
+        <v>5724.71</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -3597,10 +3622,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7234835442024343</v>
+        <v>0.7390503238664673</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-15
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Tue 14 Jul 2026</t>
+          <t>As of Wed 15 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹205,528</t>
+          <t>₹205,966</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+722  (+0.35%)</t>
+          <t>₹+439  (+0.21%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.76%</t>
+          <t>+2.98%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹134,118</t>
+          <t>₹134,557</t>
         </is>
       </c>
     </row>
@@ -796,31 +796,31 @@
         <v>8690</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>895.1</v>
+        <v>898.05</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>9846.1</v>
+        <v>9878.549999999999</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>1156.1</v>
+        <v>1188.549999999999</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.1330379746835443</v>
+        <v>0.1367721518987341</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>739.3099999999999</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>820.6357142857142</v>
+        <v>823.4571428571428</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.08319102414734195</v>
+        <v>0.08306091770264146</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>24.04</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>7540</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>4051.2</v>
+        <v>4090</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8102.4</v>
+        <v>8180</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>562.3999999999996</v>
+        <v>640</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.07458885941644558</v>
+        <v>0.08488063660477453</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>3604.1</v>
@@ -862,13 +862,13 @@
         <v>3813.921428571429</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.05856994752877445</v>
+        <v>0.06750087320991961</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>81.47</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -892,31 +892,31 @@
         <v>9031.549999999999</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>848.25</v>
+        <v>844.45</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9330.75</v>
+        <v>9288.950000000001</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>299.2000000000005</v>
+        <v>257.400000000001</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.03312831130869015</v>
+        <v>0.02850009134644673</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>783.09</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>810.2285714285714</v>
+        <v>811.1071428571428</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.04482337585785865</v>
+        <v>0.03948470263823467</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>16.6</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>7278.3</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>2531.1</v>
+        <v>2543.1</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>7593.299999999999</v>
+        <v>7629.299999999999</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>315</v>
+        <v>351</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.04327933720786448</v>
+        <v>0.04822554717447756</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>2309.03</v>
@@ -958,13 +958,13 @@
         <v>2358.721428571428</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.06810421217200895</v>
+        <v>0.07250150266547593</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>59.36</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>9246.6</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>474.4</v>
+        <v>470.75</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>10436.8</v>
+        <v>10356.5</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>1190.199999999999</v>
+        <v>1109.9</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.1287175826790387</v>
+        <v>0.1200333095408042</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>386.74</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>422.5428571428571</v>
+        <v>424.3107142857143</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.1093110093953264</v>
+        <v>0.09864957135270459</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -1036,31 +1036,31 @@
         <v>8790</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1683.4</v>
+        <v>1680.1</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>10100.4</v>
+        <v>10080.6</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>1310.400000000001</v>
+        <v>1290.599999999999</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.1490784982935154</v>
+        <v>0.1468259385665528</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1365.41</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1490.692857142857</v>
+        <v>1494.785714285714</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.1144749571445543</v>
+        <v>0.1102995569991581</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>45.25</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>9288.75</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>666.8</v>
+        <v>669.2</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>10002</v>
+        <v>10038</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>713.2499999999993</v>
+        <v>749.2500000000007</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.07678643520387558</v>
+        <v>0.08066209123940257</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>591.46</v>
@@ -1102,13 +1102,13 @@
         <v>621.0571428571428</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.06860056560116547</v>
+        <v>0.07194091025531563</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>14</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>8700</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>8900.5</v>
+        <v>8934</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8900.5</v>
+        <v>8934</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>200.5</v>
+        <v>234</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.02304597701149425</v>
+        <v>0.02689655172413793</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>8339.209999999999</v>
@@ -1150,13 +1150,13 @@
         <v>8510.25</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.04384585135666536</v>
+        <v>0.04743116185359302</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>123.68</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>9000</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>913.85</v>
+        <v>929.15</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9138.5</v>
+        <v>9291.5</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>138.5000000000002</v>
+        <v>291.4999999999998</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.01538888888888891</v>
+        <v>0.03238888888888886</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>836</v>
@@ -1198,13 +1198,13 @@
         <v>887.1</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.02927176232423264</v>
+        <v>0.04525641715546463</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>29.64</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>7579.5</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>7586</v>
+        <v>7618</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>7586</v>
+        <v>7618</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>6.5</v>
+        <v>38.5</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.0008575763572795039</v>
+        <v>0.005079490731578601</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>7128.14</v>
@@ -1246,13 +1246,13 @@
         <v>7164.5</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.05556287898760875</v>
+        <v>0.0595300603833027</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>209.96</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -1276,31 +1276,31 @@
         <v>8992.5</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>1840.4</v>
+        <v>1878</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>9202</v>
+        <v>9390</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>209.5000000000005</v>
+        <v>397.5</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.0232971921045316</v>
+        <v>0.04420350291909925</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1680.3</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>1680.3</v>
+        <v>1705.135714285714</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.08699195826994138</v>
+        <v>0.09204701049748994</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>50.24</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
@@ -1324,31 +1324,31 @@
         <v>7245.6</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>2487.6</v>
+        <v>2506</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>7462.799999999999</v>
+        <v>7518</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>217.2000000000003</v>
+        <v>272.4000000000005</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.02997681351440878</v>
+        <v>0.03759523020867845</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>2335.46</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>2337.814285714285</v>
+        <v>2349.7</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.06021294190614051</v>
+        <v>0.06237031125299289</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>49.27</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>8919.200000000001</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1100.9</v>
+        <v>1090.7</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>8807.200000000001</v>
+        <v>8725.6</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>-112</v>
+        <v>-193.6000000000004</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>-0.01255718001614494</v>
+        <v>-0.0217059825993363</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1050.57</v>
@@ -1390,13 +1390,13 @@
         <v>1050.57</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.04571714052139172</v>
+        <v>0.03679288530301651</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>32.69</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>8883</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1268.8</v>
+        <v>1263.2</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>8881.6</v>
+        <v>8842.4</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>-1.400000000000318</v>
+        <v>-40.59999999999968</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>-0.0001576044129235977</v>
+        <v>-0.004570527974783258</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>1182.49</v>
@@ -1438,13 +1438,13 @@
         <v>1182.49</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.06802490542244637</v>
+        <v>0.06389328689043701</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>39.97</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>8656.65</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>969.75</v>
+        <v>976.15</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>8727.75</v>
+        <v>8785.35</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>71.0999999999998</v>
+        <v>128.6999999999996</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.008213338878203438</v>
+        <v>0.01486718303269736</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>920.8099999999999</v>
@@ -1486,13 +1486,13 @@
         <v>935.6</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.03521526166537765</v>
+        <v>0.04154074681145311</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>23.22</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2987,6 +2987,31 @@
         <v>-748.8200000000001</v>
       </c>
       <c r="G20" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="n">
+        <v>205966.28</v>
+      </c>
+      <c r="C21" s="20" t="n">
+        <v>71409.53</v>
+      </c>
+      <c r="D21" s="20" t="n">
+        <v>134556.75</v>
+      </c>
+      <c r="E21" s="20" t="n">
+        <v>127841.65</v>
+      </c>
+      <c r="F21" s="20" t="n">
+        <v>-748.8200000000001</v>
+      </c>
+      <c r="G21" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3070,18 +3095,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>2487.6</v>
+        <v>8934</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>2387.74</v>
+        <v>8637.43</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -3093,7 +3118,7 @@
         <v>7.1</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8612496263079223</v>
+        <v>0.8442527348777349</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -3108,18 +3133,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>8900.5</v>
+        <v>2506</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>8596.860000000001</v>
+        <v>2401.8</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -3131,7 +3156,7 @@
         <v>7</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8325430991529646</v>
+        <v>0.848067487129987</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -3146,7 +3171,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
@@ -3154,10 +3179,10 @@
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1555.4</v>
+        <v>1568.8</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1491.86</v>
+        <v>1505.23</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -3169,7 +3194,7 @@
         <v>6.7</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7929207772795218</v>
+        <v>0.7990548584298585</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -3184,18 +3209,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1683.4</v>
+        <v>2543.1</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1554.93</v>
+        <v>2412.1</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -3207,7 +3232,7 @@
         <v>6.7</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7670911808669656</v>
+        <v>0.7874276061776062</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -3222,18 +3247,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>7188.5</v>
+        <v>750.8</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>6877.29</v>
+        <v>719.5700000000001</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -3242,10 +3267,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7628440458395616</v>
+        <v>0.7896657818532818</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -3260,18 +3285,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>ADANIPOWER</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>226.17</v>
+        <v>7273</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>213.68</v>
+        <v>6951.93</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -3280,10 +3305,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7545969108121575</v>
+        <v>0.7622767857142856</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3298,18 +3323,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1100.9</v>
+        <v>9324.5</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1036.13</v>
+        <v>8769.57</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -3321,7 +3346,7 @@
         <v>6.5</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7612137518684605</v>
+        <v>0.7509069337194337</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3336,18 +3361,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>9532.5</v>
+        <v>1951.5</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>8992.360000000001</v>
+        <v>1883.64</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -3359,7 +3384,7 @@
         <v>6.5</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7433492775286498</v>
+        <v>0.7355312902187903</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3374,18 +3399,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1427.1</v>
+        <v>5549.5</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1364.84</v>
+        <v>5267.14</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -3397,7 +3422,7 @@
         <v>6.5</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7489606377678126</v>
+        <v>0.7498391248391248</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3412,18 +3437,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1821.9</v>
+        <v>929.15</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1739.2</v>
+        <v>872.4299999999999</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -3435,7 +3460,7 @@
         <v>6.5</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7467324364723468</v>
+        <v>0.7398648648648649</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3450,18 +3475,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1942.6</v>
+        <v>1033.75</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1873.47</v>
+        <v>973.91</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -3470,10 +3495,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7474080717488789</v>
+        <v>0.7602216055341054</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3488,18 +3513,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1035.95</v>
+        <v>1424.4</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>976.61</v>
+        <v>1362.86</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -3511,7 +3536,7 @@
         <v>6.4</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7570672645739911</v>
+        <v>0.7337636743886744</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3526,18 +3551,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1484.1</v>
+        <v>7618</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1406.96</v>
+        <v>7191.79</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -3549,7 +3574,7 @@
         <v>6.3</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7788978574987544</v>
+        <v>0.7503478925353926</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3564,18 +3589,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1268.8</v>
+        <v>4828.5</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1188.27</v>
+        <v>4507.54</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -3587,7 +3612,7 @@
         <v>6.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7521155954160439</v>
+        <v>0.7457046332046332</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3602,18 +3627,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260714</v>
+        <v>20260715</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>6072</v>
+        <v>1501.6</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>5724.71</v>
+        <v>1421.94</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -3625,7 +3650,7 @@
         <v>6.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7390503238664673</v>
+        <v>0.7544401544401544</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-16
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Wed 15 Jul 2026</t>
+          <t>As of Thu 16 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹205,966</t>
+          <t>₹206,098</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+439  (+0.21%)</t>
+          <t>₹+131  (+0.06%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.98%</t>
+          <t>+3.05%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹134,557</t>
+          <t>₹134,688</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -796,31 +796,31 @@
         <v>8690</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>898.05</v>
+        <v>903.25</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>9878.549999999999</v>
+        <v>9935.75</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>1188.549999999999</v>
+        <v>1245.75</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.1367721518987341</v>
+        <v>0.1433544303797468</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>739.3099999999999</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>823.4571428571428</v>
+        <v>830.2214285714285</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.08306091770264146</v>
+        <v>0.08085089557550121</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>24.04</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>7540</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>4090</v>
+        <v>4106</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8180</v>
+        <v>8212</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>640</v>
+        <v>672</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.08488063660477453</v>
+        <v>0.08912466843501327</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>3604.1</v>
@@ -862,13 +862,13 @@
         <v>3813.921428571429</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.06750087320991961</v>
+        <v>0.0711345765778303</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>81.47</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -892,31 +892,31 @@
         <v>9031.549999999999</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>844.45</v>
+        <v>839.35</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9288.950000000001</v>
+        <v>9232.85</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>257.400000000001</v>
+        <v>201.3000000000008</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.02850009134644673</v>
+        <v>0.02228853297606731</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>783.09</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>811.1071428571428</v>
+        <v>811.6642857142856</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.03948470263823467</v>
+        <v>0.03298470755431515</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>16.6</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>7278.3</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>2543.1</v>
+        <v>2546</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>7629.299999999999</v>
+        <v>7638</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>351</v>
+        <v>359.7000000000003</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.04822554717447756</v>
+        <v>0.04942088124974242</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>2309.03</v>
@@ -958,13 +958,13 @@
         <v>2358.721428571428</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.07250150266547593</v>
+        <v>0.07355796206935268</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>59.36</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>9246.6</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>470.75</v>
+        <v>470.1</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>10356.5</v>
+        <v>10342.2</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>1109.9</v>
+        <v>1095.6</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.1200333095408042</v>
+        <v>0.1184867951463241</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>386.74</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>424.3107142857143</v>
+        <v>425.7571428571429</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.09864957135270459</v>
+        <v>0.09432643510499288</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -1036,31 +1036,31 @@
         <v>8790</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1680.1</v>
+        <v>1684</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>10080.6</v>
+        <v>10104</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>1290.599999999999</v>
+        <v>1314</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.1468259385665528</v>
+        <v>0.1494880546075085</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1365.41</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1494.785714285714</v>
+        <v>1498.128571428571</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.1102995569991581</v>
+        <v>0.1103749575839837</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>45.25</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -1084,31 +1084,31 @@
         <v>9288.75</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>669.2</v>
+        <v>683.4</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>10038</v>
+        <v>10251</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>749.2500000000007</v>
+        <v>962.2499999999997</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.08066209123940257</v>
+        <v>0.1035930561162696</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>591.46</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>621.0571428571428</v>
+        <v>626.1964285714286</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.07194091025531563</v>
+        <v>0.08370437727329737</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>14</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>8700</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>8934</v>
+        <v>8888</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8934</v>
+        <v>8888</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>234</v>
+        <v>188</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.02689655172413793</v>
+        <v>0.02160919540229885</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>8339.209999999999</v>
@@ -1150,13 +1150,13 @@
         <v>8510.25</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.04743116185359302</v>
+        <v>0.04250112511251125</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>123.68</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>9000</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>929.15</v>
+        <v>921.95</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9291.5</v>
+        <v>9219.5</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>291.4999999999998</v>
+        <v>219.5000000000005</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.03238888888888886</v>
+        <v>0.02438888888888894</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>836</v>
@@ -1198,13 +1198,13 @@
         <v>887.1</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.04525641715546463</v>
+        <v>0.03780031455068065</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>29.64</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>7579.5</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>7618</v>
+        <v>7650</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>7618</v>
+        <v>7650</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>38.5</v>
+        <v>70.5</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.005079490731578601</v>
+        <v>0.009301405105877696</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>7128.14</v>
@@ -1246,13 +1246,13 @@
         <v>7164.5</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.0595300603833027</v>
+        <v>0.0634640522875817</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>209.96</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -1276,31 +1276,31 @@
         <v>8992.5</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>1878</v>
+        <v>1890.2</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>9390</v>
+        <v>9451</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>397.5</v>
+        <v>458.5000000000002</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.04420350291909925</v>
+        <v>0.05098693355574092</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1680.3</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>1705.135714285714</v>
+        <v>1718.814285714286</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.09204701049748994</v>
+        <v>0.09067067732817392</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>50.24</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>7245.6</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>2506</v>
+        <v>2408.9</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>7518</v>
+        <v>7226.700000000001</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>272.4000000000005</v>
+        <v>-18.89999999999918</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.03759523020867845</v>
+        <v>-0.002608479629016118</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>2335.46</v>
@@ -1342,13 +1342,13 @@
         <v>2349.7</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.06237031125299289</v>
+        <v>0.02457553240068092</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>49.27</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>8919.200000000001</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1090.7</v>
+        <v>1100.6</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>8725.6</v>
+        <v>8804.799999999999</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>-193.6000000000004</v>
+        <v>-114.4000000000015</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>-0.0217059825993363</v>
+        <v>-0.0128262624450625</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1050.57</v>
@@ -1390,13 +1390,13 @@
         <v>1050.57</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.03679288530301651</v>
+        <v>0.04545702344175902</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>32.69</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>8883</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1263.2</v>
+        <v>1294.9</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>8842.4</v>
+        <v>9064.300000000001</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>-40.59999999999968</v>
+        <v>181.3000000000006</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>-0.004570527974783258</v>
+        <v>0.02040977147360133</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>1182.49</v>
@@ -1438,13 +1438,13 @@
         <v>1182.49</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.06389328689043701</v>
+        <v>0.08680979226195079</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>39.97</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>8656.65</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>976.15</v>
+        <v>963.1</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>8785.35</v>
+        <v>8667.9</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>128.6999999999996</v>
+        <v>11.25</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.01486718303269736</v>
+        <v>0.001299578936424598</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>920.8099999999999</v>
@@ -1486,13 +1486,13 @@
         <v>935.6</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.04154074681145311</v>
+        <v>0.02855362890665559</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>23.22</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3012,6 +3012,31 @@
         <v>-748.8200000000001</v>
       </c>
       <c r="G21" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="n">
+        <v>206097.53</v>
+      </c>
+      <c r="C22" s="20" t="n">
+        <v>71409.53</v>
+      </c>
+      <c r="D22" s="20" t="n">
+        <v>134688</v>
+      </c>
+      <c r="E22" s="20" t="n">
+        <v>127841.65</v>
+      </c>
+      <c r="F22" s="20" t="n">
+        <v>-748.8200000000001</v>
+      </c>
+      <c r="G22" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3095,18 +3120,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>8934</v>
+        <v>2408.9</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8637.43</v>
+        <v>2289.39</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -3115,10 +3140,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8442527348777349</v>
+        <v>0.8516087516087516</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -3133,18 +3158,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>2506</v>
+        <v>1294.9</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>2401.8</v>
+        <v>1217.41</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -3153,10 +3178,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.848067487129987</v>
+        <v>0.8358892374517375</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -3171,18 +3196,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1568.8</v>
+        <v>1826.4</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1505.23</v>
+        <v>1746.27</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -3191,10 +3216,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7990548584298585</v>
+        <v>0.7982685810810811</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -3209,18 +3234,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>2543.1</v>
+        <v>9215</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>2412.1</v>
+        <v>8644.860000000001</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -3229,10 +3254,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7874276061776062</v>
+        <v>0.7828969594594595</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -3247,18 +3272,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>750.8</v>
+        <v>5592</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>719.5700000000001</v>
+        <v>5302.07</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -3267,10 +3292,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7896657818532818</v>
+        <v>0.7842040701415701</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -3285,18 +3310,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>7273</v>
+        <v>722.35</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>6951.93</v>
+        <v>671.14</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -3305,10 +3330,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7622767857142856</v>
+        <v>0.7557030244530244</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3323,18 +3348,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>9324.5</v>
+        <v>7316</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>8769.57</v>
+        <v>6988.57</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -3343,10 +3368,10 @@
         <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7509069337194337</v>
+        <v>0.7568593146718147</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3361,18 +3386,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1951.5</v>
+        <v>8888</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1883.64</v>
+        <v>8600.709999999999</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -3384,7 +3409,7 @@
         <v>6.5</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7355312902187903</v>
+        <v>0.7631957850707851</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3399,18 +3424,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>5549.5</v>
+        <v>7650</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>5267.14</v>
+        <v>7233</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -3422,7 +3447,7 @@
         <v>6.5</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7498391248391248</v>
+        <v>0.7804315476190476</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3437,18 +3462,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>929.15</v>
+        <v>581.6</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>872.4299999999999</v>
+        <v>543.89</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -3457,10 +3482,10 @@
         <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7398648648648649</v>
+        <v>0.7745455276705276</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3475,18 +3500,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1033.75</v>
+        <v>758.95</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>973.91</v>
+        <v>728.51</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -3498,7 +3523,7 @@
         <v>6.4</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7602216055341054</v>
+        <v>0.765558638996139</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3513,18 +3538,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1424.4</v>
+        <v>1559.6</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1362.86</v>
+        <v>1496.53</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -3533,10 +3558,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7337636743886744</v>
+        <v>0.7394465894465895</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3551,18 +3576,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>JSWDULUX</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>7618</v>
+        <v>3080.2</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>7191.79</v>
+        <v>2862.51</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -3574,7 +3599,7 @@
         <v>6.3</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7503478925353926</v>
+        <v>0.7709821428571429</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3589,18 +3614,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>4828.5</v>
+        <v>1490.8</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>4507.54</v>
+        <v>1410.91</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -3609,10 +3634,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7457046332046332</v>
+        <v>0.7629122425997426</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3627,18 +3652,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260715</v>
+        <v>20260716</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1501.6</v>
+        <v>1040.5</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1421.94</v>
+        <v>979.47</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -3650,7 +3675,7 @@
         <v>6.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7544401544401544</v>
+        <v>0.7358309202059202</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-17
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Thu 16 Jul 2026</t>
+          <t>As of Fri 17 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹206,098</t>
+          <t>₹204,735</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+131  (+0.06%)</t>
+          <t>₹-1,363  (-0.66%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+3.05%</t>
+          <t>+2.37%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>+0.00%</t>
+          <t>-0.66%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹71,410</t>
+          <t>₹106,031</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹127,842</t>
+          <t>₹95,302</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹134,688</t>
+          <t>₹98,704</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹-749</t>
+          <t>₹+1,333</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -778,725 +778,533 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C2" s="7" t="n">
-        <v>790</v>
+        <v>420.3</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E2" s="9" t="n">
-        <v>8690</v>
+        <v>9246.6</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>903.25</v>
+        <v>466.95</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>9935.75</v>
+        <v>10272.9</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>1245.75</v>
+        <v>1026.299999999999</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.1433544303797468</v>
+        <v>0.1109921484653818</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>739.3099999999999</v>
+        <v>386.74</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>830.2214285714285</v>
+        <v>430.3535714285714</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.08085089557550121</v>
+        <v>0.07837333455708018</v>
       </c>
       <c r="M2" s="13" t="n">
-        <v>24.04</v>
+        <v>16.71</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>3770</v>
+        <v>1465</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>7540</v>
+        <v>8790</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>4106</v>
+        <v>1581.5</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8212</v>
+        <v>9489</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>672</v>
+        <v>699</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.08912466843501327</v>
+        <v>0.0795221843003413</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>3604.1</v>
+        <v>1365.41</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>3813.921428571429</v>
+        <v>1498.128571428571</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.0711345765778303</v>
+        <v>0.0527166794634389</v>
       </c>
       <c r="M3" s="13" t="n">
-        <v>81.47</v>
+        <v>45.25</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>821.05</v>
+        <v>619.25</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>9031.549999999999</v>
+        <v>9288.75</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>839.35</v>
+        <v>704.85</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9232.85</v>
+        <v>10572.75</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>201.3000000000008</v>
+        <v>1284</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.02228853297606731</v>
+        <v>0.1382317319337909</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>783.09</v>
+        <v>591.46</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>811.6642857142856</v>
+        <v>646.0285714285715</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.03298470755431515</v>
+        <v>0.08345240628705193</v>
       </c>
       <c r="M4" s="13" t="n">
-        <v>16.6</v>
+        <v>14</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>2426.1</v>
+        <v>8700</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>7278.3</v>
+        <v>8700</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>2546</v>
+        <v>8826</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>7638</v>
+        <v>8826</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>359.7000000000003</v>
+        <v>126</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.04942088124974242</v>
+        <v>0.01448275862068966</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>2309.03</v>
+        <v>8339.209999999999</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>2358.721428571428</v>
+        <v>8510.25</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.07355796206935268</v>
+        <v>0.03577498300475867</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>59.36</v>
+        <v>123.68</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>420.3</v>
+        <v>900</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>9246.6</v>
+        <v>9000</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>470.1</v>
+        <v>905</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>10342.2</v>
+        <v>9050</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>1095.6</v>
+        <v>50</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.1184867951463241</v>
+        <v>0.005555555555555556</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>386.74</v>
+        <v>836</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>425.7571428571429</v>
+        <v>887.1</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.09432643510499288</v>
+        <v>0.01977900552486185</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>16.71</v>
+        <v>29.64</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>1465</v>
+        <v>7579.5</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>8790</v>
+        <v>7579.5</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1684</v>
+        <v>7579</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>10104</v>
+        <v>7579</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>1314</v>
+        <v>-0.5</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.1494880546075085</v>
+        <v>-6.596741209842338e-05</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>1365.41</v>
+        <v>7128.14</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1498.128571428571</v>
+        <v>7164.5</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.1103749575839837</v>
+        <v>0.05469059242644148</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>45.25</v>
+        <v>209.96</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>619.25</v>
+        <v>1798.5</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>9288.75</v>
+        <v>8992.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>683.4</v>
+        <v>1900.6</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>10251</v>
+        <v>9503</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>962.2499999999997</v>
+        <v>510.4999999999995</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.1035930561162696</v>
+        <v>0.05676953016402553</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>591.46</v>
+        <v>1680.3</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>626.1964285714286</v>
+        <v>1718.814285714286</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.08370437727329737</v>
+        <v>0.09564648757535212</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>14</v>
+        <v>50.24</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>8700</v>
+        <v>2415.2</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>8700</v>
+        <v>7245.6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>8888</v>
+        <v>2415.2</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8888</v>
+        <v>7245.599999999999</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>188</v>
+        <v>0</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.02160919540229885</v>
+        <v>0</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>8339.209999999999</v>
+        <v>2335.46</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>8510.25</v>
+        <v>2349.7</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.04250112511251125</v>
+        <v>0.02711990725405764</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>123.68</v>
+        <v>49.27</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>900</v>
+        <v>1114.9</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>9000</v>
+        <v>8919.200000000001</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>921.95</v>
+        <v>1086.2</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9219.5</v>
+        <v>8689.6</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>219.5000000000005</v>
+        <v>-229.6000000000004</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.02438888888888894</v>
+        <v>-0.02574221903309718</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>836</v>
+        <v>1050.57</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>887.1</v>
+        <v>1050.57</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.03780031455068065</v>
+        <v>0.03280243049162227</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>29.64</v>
+        <v>32.69</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>7579.5</v>
+        <v>1269</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>7579.5</v>
+        <v>8883</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>7650</v>
+        <v>1272</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>7650</v>
+        <v>8904</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>70.5</v>
+        <v>21</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.009301405105877696</v>
+        <v>0.002364066193853428</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>7128.14</v>
+        <v>1182.49</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>7164.5</v>
+        <v>1182.807142857143</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.0634640522875817</v>
+        <v>0.07012017070979329</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>209.96</v>
+        <v>39.97</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>1798.5</v>
+        <v>961.85</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>8992.5</v>
+        <v>8656.65</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>1890.2</v>
+        <v>952.45</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>9451</v>
+        <v>8572.050000000001</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>458.5000000000002</v>
+        <v>-84.5999999999998</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.05098693355574092</v>
+        <v>-0.009772833601912957</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>1680.3</v>
+        <v>920.8099999999999</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>1718.814285714286</v>
+        <v>935.6</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.09067067732817392</v>
+        <v>0.01769121738673948</v>
       </c>
       <c r="M12" s="13" t="n">
-        <v>50.24</v>
+        <v>23.22</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>JBCHEPHARM</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>2415.2</v>
-      </c>
-      <c r="D13" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>7245.6</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>2408.9</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>7226.700000000001</v>
-      </c>
-      <c r="H13" s="10" t="n">
-        <v>-18.89999999999918</v>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>-0.002608479629016118</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>2335.46</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>2349.7</v>
-      </c>
-      <c r="L13" s="12" t="n">
-        <v>0.02457553240068092</v>
-      </c>
-      <c r="M13" s="13" t="n">
-        <v>49.27</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>PREMIERENE</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>1114.9</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="E14" s="9" t="n">
-        <v>8919.200000000001</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>1100.6</v>
-      </c>
-      <c r="G14" s="9" t="n">
-        <v>8804.799999999999</v>
-      </c>
-      <c r="H14" s="10" t="n">
-        <v>-114.4000000000015</v>
-      </c>
-      <c r="I14" s="11" t="n">
-        <v>-0.0128262624450625</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>1050.57</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>1050.57</v>
-      </c>
-      <c r="L14" s="12" t="n">
-        <v>0.04545702344175902</v>
-      </c>
-      <c r="M14" s="13" t="n">
-        <v>32.69</v>
-      </c>
-      <c r="N14" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>SAILIFE</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>1269</v>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="E15" s="9" t="n">
-        <v>8883</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>1294.9</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>9064.300000000001</v>
-      </c>
-      <c r="H15" s="10" t="n">
-        <v>181.3000000000006</v>
-      </c>
-      <c r="I15" s="11" t="n">
-        <v>0.02040977147360133</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>1182.49</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>1182.49</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>0.08680979226195079</v>
-      </c>
-      <c r="M15" s="13" t="n">
-        <v>39.97</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>FORTIS</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>961.85</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <v>8656.65</v>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>963.1</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>8667.9</v>
-      </c>
-      <c r="H16" s="10" t="n">
-        <v>11.25</v>
-      </c>
-      <c r="I16" s="11" t="n">
-        <v>0.001299578936424598</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>920.8099999999999</v>
-      </c>
-      <c r="K16" s="7" t="n">
-        <v>935.6</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>0.02855362890665559</v>
-      </c>
-      <c r="M16" s="13" t="n">
-        <v>23.22</v>
-      </c>
-      <c r="N16" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H16">
+  <conditionalFormatting sqref="H2:H12">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1514,7 +1322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1590,27 +1398,27 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>1410</v>
+        <v>790</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>1455.2</v>
+        <v>880.8</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -1621,39 +1429,39 @@
         <v>25</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>135.6</v>
+        <v>998.8</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.1149</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>0.46</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>690</v>
+        <v>3770</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>660.45</v>
+        <v>4097.9</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -1664,39 +1472,39 @@
         <v>25</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-206.85</v>
+        <v>655.8</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-0.38</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>1839</v>
+        <v>821.05</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>1828.1</v>
+        <v>844</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1707,39 +1515,39 @@
         <v>25</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-21.8</v>
+        <v>252.45</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0059</v>
+        <v>0.028</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-0.1</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>1414</v>
+        <v>2426.1</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>3</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>1537.8</v>
+        <v>2484.2</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1750,19 +1558,19 @@
         <v>25</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>371.4</v>
+        <v>174.3</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>0.0876</v>
+        <v>0.0239</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>1.38</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -1771,10 +1579,10 @@
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>1300</v>
+        <v>1410</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -1782,7 +1590,7 @@
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>1389.1</v>
+        <v>1455.2</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -1793,19 +1601,19 @@
         <v>25</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>356.4</v>
+        <v>135.6</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>0.0321</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>0.63</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -1814,10 +1622,10 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>276.45</v>
+        <v>690</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
@@ -1825,7 +1633,7 @@
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>330.1</v>
+        <v>660.45</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -1836,19 +1644,19 @@
         <v>25</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>1019.35</v>
+        <v>-206.85</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>0.1941</v>
+        <v>-0.0428</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>3.1</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -1857,10 +1665,10 @@
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>1462.5</v>
+        <v>1839</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
@@ -1868,7 +1676,7 @@
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>1564.7</v>
+        <v>1828.1</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -1879,19 +1687,19 @@
         <v>25</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>306.6</v>
+        <v>-21.8</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>0.0699</v>
+        <v>-0.0059</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>1.78</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -1900,41 +1708,41 @@
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>798</v>
+        <v>1414</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>750</v>
+        <v>1537.8</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>-288</v>
+        <v>371.4</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.0876</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>-0.92</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -1943,139 +1751,139 @@
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>260.45</v>
+        <v>1300</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>257.85</v>
+        <v>1389.1</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H10" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>-52.07</v>
+        <v>356.4</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>-0.01</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>-0.13</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>6500</v>
+        <v>276.45</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>6401.5</v>
+        <v>330.1</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H11" s="14" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>-98.5</v>
+        <v>1019.35</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>-0.0152</v>
+        <v>0.1941</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>-0.31</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>571.5</v>
+        <v>1462.5</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>571.1</v>
+        <v>1564.7</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H12" s="14" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>-6.4</v>
+        <v>306.6</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>-0.0007</v>
+        <v>0.0699</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>-0.01</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>965</v>
+        <v>798</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
@@ -2083,7 +1891,7 @@
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>933</v>
+        <v>750</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
@@ -2091,42 +1899,42 @@
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="I13" s="17" t="n">
         <v>-288</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0602</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>5479</v>
+        <v>260.45</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>5424</v>
+        <v>257.85</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
@@ -2134,42 +1942,42 @@
         </is>
       </c>
       <c r="H14" s="14" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>-55</v>
+        <v>-52.07</v>
       </c>
       <c r="J14" s="18" t="n">
         <v>-0.01</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>-0.18</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>960.1</v>
+        <v>6500</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>6401.5</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
@@ -2177,42 +1985,42 @@
         </is>
       </c>
       <c r="H15" s="14" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>-516.79</v>
+        <v>-98.5</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.0152</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>952.1</v>
+        <v>571.5</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>948.8</v>
+        <v>571.1</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
@@ -2220,42 +2028,42 @@
         </is>
       </c>
       <c r="H16" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>-29.7</v>
+        <v>-6.4</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.0007</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>1475</v>
+        <v>965</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>1394.19</v>
+        <v>933</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -2263,42 +2071,42 @@
         </is>
       </c>
       <c r="H17" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>-484.86</v>
+        <v>-288</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0332</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>-1</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>248.05</v>
+        <v>5479</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>242.8</v>
+        <v>5424</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -2306,42 +2114,42 @@
         </is>
       </c>
       <c r="H18" s="14" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>-110.25</v>
+        <v>-55</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.01</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>-0.3</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>1039.2</v>
+        <v>960.1</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>970</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
@@ -2349,42 +2157,42 @@
         </is>
       </c>
       <c r="H19" s="14" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>-346</v>
+        <v>-516.79</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0598</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>199.96</v>
+        <v>952.1</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>193.31</v>
+        <v>948.8</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -2392,42 +2200,42 @@
         </is>
       </c>
       <c r="H20" s="14" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>-172.9</v>
+        <v>-29.7</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.0035</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>986.4</v>
+        <v>1475</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>1394.19</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -2435,20 +2243,192 @@
         </is>
       </c>
       <c r="H21" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>-261.05</v>
+        <v>-484.86</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>-0.0529</v>
+        <v>-0.0548</v>
       </c>
       <c r="K21" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="n">
+        <v>248.05</v>
+      </c>
+      <c r="D22" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="n">
+        <v>242.8</v>
+      </c>
+      <c r="G22" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H22" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I22" s="17" t="n">
+        <v>-110.25</v>
+      </c>
+      <c r="J22" s="18" t="n">
+        <v>-0.0212</v>
+      </c>
+      <c r="K22" s="19" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>1039.2</v>
+      </c>
+      <c r="D23" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F23" s="15" t="n">
+        <v>970</v>
+      </c>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H23" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I23" s="17" t="n">
+        <v>-346</v>
+      </c>
+      <c r="J23" s="18" t="n">
+        <v>-0.06660000000000001</v>
+      </c>
+      <c r="K23" s="19" t="n">
+        <v>-0.82</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>199.96</v>
+      </c>
+      <c r="D24" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F24" s="15" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I24" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J24" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K24" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D25" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F25" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H25" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I25" s="17" t="n">
+        <v>-261.05</v>
+      </c>
+      <c r="J25" s="18" t="n">
+        <v>-0.0529</v>
+      </c>
+      <c r="K25" s="19" t="n">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I21">
+  <conditionalFormatting sqref="I2:I25">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2466,7 +2446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3038,6 +3018,31 @@
       </c>
       <c r="G22" s="14" t="n">
         <v>15</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="n">
+        <v>204734.63</v>
+      </c>
+      <c r="C23" s="20" t="n">
+        <v>106030.73</v>
+      </c>
+      <c r="D23" s="20" t="n">
+        <v>98703.89999999999</v>
+      </c>
+      <c r="E23" s="20" t="n">
+        <v>95301.8</v>
+      </c>
+      <c r="F23" s="20" t="n">
+        <v>1332.53</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -3120,18 +3125,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>2408.9</v>
+        <v>880.8</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>2289.39</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -3140,10 +3145,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7.2</v>
+        <v>6.9</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8516087516087516</v>
+        <v>0.8443043240062497</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -3158,18 +3163,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1294.9</v>
+        <v>777</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1217.41</v>
+        <v>744.8</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -3178,10 +3183,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8358892374517375</v>
+        <v>0.8257969279467564</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -3196,18 +3201,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1826.4</v>
+        <v>8862</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1746.27</v>
+        <v>8315.07</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -3216,10 +3221,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7982685810810811</v>
+        <v>0.7796796055434938</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -3234,18 +3239,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>9215</v>
+        <v>1566.1</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>8644.860000000001</v>
+        <v>1504.37</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -3254,10 +3259,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.8</v>
+        <v>6.6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7828969594594595</v>
+        <v>0.7821287259298337</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -3272,7 +3277,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
@@ -3280,10 +3285,10 @@
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>5592</v>
+        <v>5448</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>5302.07</v>
+        <v>5157.93</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -3292,10 +3297,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7842040701415701</v>
+        <v>0.7660217519225696</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -3310,18 +3315,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>722.35</v>
+        <v>1932.6</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>671.14</v>
+        <v>1868.37</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -3330,10 +3335,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7557030244530244</v>
+        <v>0.7646297912058925</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3348,18 +3353,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>7316</v>
+        <v>2190.5</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>6988.57</v>
+        <v>2067.2</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -3371,7 +3376,7 @@
         <v>6.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7568593146718147</v>
+        <v>0.7569719781669135</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3386,18 +3391,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>8888</v>
+        <v>741.55</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>8600.709999999999</v>
+        <v>687.5700000000001</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -3406,10 +3411,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7631957850707851</v>
+        <v>0.74493537325244</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3424,18 +3429,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>7650</v>
+        <v>844</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>7233</v>
+        <v>811.3099999999999</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -3447,7 +3452,7 @@
         <v>6.5</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7804315476190476</v>
+        <v>0.7583406042651624</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3462,18 +3467,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>581.6</v>
+        <v>7247.5</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>543.89</v>
+        <v>6931.93</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -3482,10 +3487,10 @@
         <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7745455276705276</v>
+        <v>0.7459793437899478</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3500,18 +3505,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>758.95</v>
+        <v>1341.3</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>728.51</v>
+        <v>1223.64</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -3523,7 +3528,7 @@
         <v>6.4</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.765558638996139</v>
+        <v>0.7441003997321591</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3538,18 +3543,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1559.6</v>
+        <v>1086.2</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1496.53</v>
+        <v>1025.69</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -3561,7 +3566,7 @@
         <v>6.3</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7394465894465895</v>
+        <v>0.7282927175699532</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3576,18 +3581,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>JSWDULUX</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>3080.2</v>
+        <v>7579</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>2862.51</v>
+        <v>7157.86</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -3599,7 +3604,7 @@
         <v>6.3</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7709821428571429</v>
+        <v>0.750858308138709</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3614,18 +3619,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1490.8</v>
+        <v>1427.2</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1410.91</v>
+        <v>1370.09</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -3634,10 +3639,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7629122425997426</v>
+        <v>0.7250552929001887</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3652,18 +3657,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260716</v>
+        <v>20260717</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1040.5</v>
+        <v>1493.4</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>979.47</v>
+        <v>1417.66</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -3672,10 +3677,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7358309202059202</v>
+        <v>0.7486171702209686</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-20
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Fri 17 Jul 2026</t>
+          <t>As of Mon 20 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹204,735</t>
+          <t>₹205,146</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-1,363  (-0.66%)</t>
+          <t>₹+412  (+0.20%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.37%</t>
+          <t>+2.57%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.66%</t>
+          <t>-0.46%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹106,031</t>
+          <t>₹74,218</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹95,302</t>
+          <t>₹126,600</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹98,704</t>
+          <t>₹130,928</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+1,333</t>
+          <t>₹+818</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -796,31 +796,31 @@
         <v>9246.6</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>466.95</v>
+        <v>457.55</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>10272.9</v>
+        <v>10066.1</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>1026.299999999999</v>
+        <v>819.5</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.1109921484653818</v>
+        <v>0.08862717106828456</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>386.74</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>430.3535714285714</v>
+        <v>430.3857142857142</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.07837333455708018</v>
+        <v>0.05936899948483394</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8790</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1581.5</v>
+        <v>1615.8</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9489</v>
+        <v>9694.799999999999</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>699</v>
+        <v>904.7999999999997</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.0795221843003413</v>
+        <v>0.1029351535836177</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1365.41</v>
@@ -862,13 +862,13 @@
         <v>1498.128571428571</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.0527166794634389</v>
+        <v>0.07282549113221226</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>45.25</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -892,31 +892,31 @@
         <v>9288.75</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>704.85</v>
+        <v>714.55</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>10572.75</v>
+        <v>10718.25</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>1284</v>
+        <v>1429.499999999999</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.1382317319337909</v>
+        <v>0.1538958417440451</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>591.46</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>646.0285714285715</v>
+        <v>655.2785714285714</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.08345240628705193</v>
+        <v>0.08294930875576041</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>14</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>8700</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>8826</v>
+        <v>8905</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>8826</v>
+        <v>8905</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>126</v>
+        <v>205</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.01448275862068966</v>
+        <v>0.0235632183908046</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>8339.209999999999</v>
@@ -958,13 +958,13 @@
         <v>8510.25</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.03577498300475867</v>
+        <v>0.04432902863559798</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>123.68</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>9000</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>905</v>
+        <v>912.45</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9050</v>
+        <v>9124.5</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>50</v>
+        <v>124.5000000000005</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.005555555555555556</v>
+        <v>0.01383333333333338</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>836</v>
@@ -1006,13 +1006,13 @@
         <v>887.1</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.01977900552486185</v>
+        <v>0.02778234423804046</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>29.64</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -1036,31 +1036,31 @@
         <v>7579.5</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>7579</v>
+        <v>7861.5</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>7579</v>
+        <v>7861.5</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-0.5</v>
+        <v>282</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-6.596741209842338e-05</v>
+        <v>0.03720562042351078</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>7128.14</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>7164.5</v>
+        <v>7289</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.05469059242644148</v>
+        <v>0.07282325255994403</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>209.96</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>8992.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1900.6</v>
+        <v>1838.6</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>9503</v>
+        <v>9193</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>510.4999999999995</v>
+        <v>200.4999999999995</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.05676953016402553</v>
+        <v>0.02229635807617454</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1680.3</v>
@@ -1102,13 +1102,13 @@
         <v>1718.814285714286</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.09564648757535212</v>
+        <v>0.06515050271169054</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>50.24</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -1156,13 +1156,13 @@
         <v>49.27</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1171,46 +1171,46 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1114.9</v>
+        <v>1269</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>8919.200000000001</v>
+        <v>8883</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1086.2</v>
+        <v>1297</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>8689.6</v>
+        <v>9079</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>-229.6000000000004</v>
+        <v>196</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>-0.02574221903309718</v>
+        <v>0.02206461780929866</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>1050.57</v>
+        <v>1182.49</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1050.57</v>
+        <v>1185.2</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.03280243049162227</v>
+        <v>0.08619892058596758</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>32.69</v>
+        <v>39.97</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -1219,92 +1219,284 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>1269</v>
+        <v>961.85</v>
       </c>
       <c r="D11" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>8656.65</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>951.2</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>8560.800000000001</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>-95.8499999999998</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>-0.01107241253833756</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>920.8099999999999</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>935.6</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>0.0164003364171573</v>
+      </c>
+      <c r="M11" s="13" t="n">
+        <v>23.22</v>
+      </c>
+      <c r="N11" s="6" t="n">
         <v>7</v>
-      </c>
-      <c r="E11" s="9" t="n">
-        <v>8883</v>
-      </c>
-      <c r="F11" s="7" t="n">
-        <v>1272</v>
-      </c>
-      <c r="G11" s="9" t="n">
-        <v>8904</v>
-      </c>
-      <c r="H11" s="10" t="n">
-        <v>21</v>
-      </c>
-      <c r="I11" s="11" t="n">
-        <v>0.002364066193853428</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>1182.49</v>
-      </c>
-      <c r="K11" s="7" t="n">
-        <v>1182.807142857143</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>0.07012017070979329</v>
-      </c>
-      <c r="M11" s="13" t="n">
-        <v>39.97</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>961.85</v>
+        <v>880.8</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>8656.65</v>
+        <v>8808</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>952.45</v>
+        <v>876.1</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>8572.050000000001</v>
+        <v>8761</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-84.5999999999998</v>
+        <v>-46.99999999999932</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.009772833601912957</v>
+        <v>-0.005336058128973583</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>920.8099999999999</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>935.6</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.01769121738673948</v>
+        <v>0.04926378267321078</v>
       </c>
       <c r="M12" s="13" t="n">
-        <v>23.22</v>
+        <v>24.22</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>4</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>ANTHEM</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>777</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>9324</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>791.55</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>9498.599999999999</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>174.5999999999995</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0.01872586872586867</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>744.8</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>744.8</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>0.05906133535468385</v>
+      </c>
+      <c r="M13" s="13" t="n">
+        <v>17.34</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>8847</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>8847</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>8885</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>8885</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>0.004295241324742851</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>8315.07</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>8315.07</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>0.06414518851997753</v>
+      </c>
+      <c r="M14" s="13" t="n">
+        <v>254.57</v>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>1560</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>7800</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>1565.8</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>7829</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>28.99999999999977</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>0.003717948717948689</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>1504.37</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>1504.37</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>0.03923234129518461</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>30.61</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>5438</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>5438</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>5506</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>5506</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>68</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>0.01250459727841118</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>5157.93</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>5157.93</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0.06321649110061746</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>143.39</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H12">
+  <conditionalFormatting sqref="H2:H16">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1322,7 +1514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1398,50 +1590,50 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>790</v>
+        <v>1114.9</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>880.8</v>
+        <v>1050.57</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>998.8</v>
+        <v>-514.64</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0577</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -1450,10 +1642,10 @@
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>3770</v>
+        <v>790</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
@@ -1461,7 +1653,7 @@
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>4097.9</v>
+        <v>880.8</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -1472,19 +1664,19 @@
         <v>25</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>655.8</v>
+        <v>998.8</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.1149</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>1.98</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -1493,10 +1685,10 @@
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>821.05</v>
+        <v>3770</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
@@ -1504,7 +1696,7 @@
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>844</v>
+        <v>4097.9</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1515,19 +1707,19 @@
         <v>25</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>252.45</v>
+        <v>655.8</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>0.028</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>0.6</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -1536,10 +1728,10 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>2426.1</v>
+        <v>821.05</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
@@ -1547,7 +1739,7 @@
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>2484.2</v>
+        <v>844</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1558,39 +1750,39 @@
         <v>25</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>174.3</v>
+        <v>252.45</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.028</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>1410</v>
+        <v>2426.1</v>
       </c>
       <c r="D6" s="16" t="n">
         <v>3</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>1455.2</v>
+        <v>2484.2</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -1601,19 +1793,19 @@
         <v>25</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>135.6</v>
+        <v>174.3</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.0239</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>0.46</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -1622,10 +1814,10 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>690</v>
+        <v>1410</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
@@ -1633,7 +1825,7 @@
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>660.45</v>
+        <v>1455.2</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -1644,19 +1836,19 @@
         <v>25</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>-206.85</v>
+        <v>135.6</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.0321</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -1665,10 +1857,10 @@
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>1839</v>
+        <v>690</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
@@ -1676,7 +1868,7 @@
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>1828.1</v>
+        <v>660.45</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -1687,19 +1879,19 @@
         <v>25</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>-21.8</v>
+        <v>-206.85</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>-0.0059</v>
+        <v>-0.0428</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>-0.1</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -1708,10 +1900,10 @@
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>1414</v>
+        <v>1839</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
@@ -1719,7 +1911,7 @@
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>1537.8</v>
+        <v>1828.1</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
@@ -1730,19 +1922,19 @@
         <v>25</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>371.4</v>
+        <v>-21.8</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>0.0876</v>
+        <v>-0.0059</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>1.38</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -1751,10 +1943,10 @@
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1300</v>
+        <v>1414</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
@@ -1762,7 +1954,7 @@
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>1389.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
@@ -1773,19 +1965,19 @@
         <v>25</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>356.4</v>
+        <v>371.4</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>0.0876</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>0.63</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -1794,10 +1986,10 @@
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>276.45</v>
+        <v>1300</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
@@ -1805,7 +1997,7 @@
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>330.1</v>
+        <v>1389.1</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
@@ -1816,19 +2008,19 @@
         <v>25</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>1019.35</v>
+        <v>356.4</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>3.1</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -1837,10 +2029,10 @@
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>1462.5</v>
+        <v>276.45</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
@@ -1848,7 +2040,7 @@
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>1564.7</v>
+        <v>330.1</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -1859,19 +2051,19 @@
         <v>25</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>306.6</v>
+        <v>1019.35</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.1941</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>1.78</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -1880,41 +2072,41 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>798</v>
+        <v>1462.5</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>750</v>
+        <v>1564.7</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>-288</v>
+        <v>306.6</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.0699</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>-0.92</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -1923,10 +2115,10 @@
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>260.45</v>
+        <v>798</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
@@ -1934,7 +2126,7 @@
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>257.85</v>
+        <v>750</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
@@ -1945,31 +2137,31 @@
         <v>23</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>-52.07</v>
+        <v>-288</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0602</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>-0.13</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>6500</v>
+        <v>260.45</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
@@ -1977,7 +2169,7 @@
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>6401.5</v>
+        <v>257.85</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
@@ -1985,65 +2177,65 @@
         </is>
       </c>
       <c r="H15" s="14" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>-98.5</v>
+        <v>-52.07</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.01</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>571.5</v>
+        <v>6500</v>
       </c>
       <c r="D16" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>6401.5</v>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H16" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="E16" s="14" t="inlineStr">
-        <is>
-          <t>2026-07-08</t>
-        </is>
-      </c>
-      <c r="F16" s="15" t="n">
-        <v>571.1</v>
-      </c>
-      <c r="G16" s="14" t="inlineStr">
-        <is>
-          <t>STOP_LOSS</t>
-        </is>
-      </c>
-      <c r="H16" s="14" t="n">
-        <v>2</v>
-      </c>
       <c r="I16" s="17" t="n">
-        <v>-6.4</v>
+        <v>-98.5</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.0152</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -2052,10 +2244,10 @@
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>965</v>
+        <v>571.5</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
@@ -2063,7 +2255,7 @@
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>933</v>
+        <v>571.1</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -2074,19 +2266,19 @@
         <v>2</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>-288</v>
+        <v>-6.4</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0007</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -2095,18 +2287,18 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>5479</v>
+        <v>965</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>5424</v>
+        <v>933</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -2114,42 +2306,42 @@
         </is>
       </c>
       <c r="H18" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>-55</v>
+        <v>-288</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0332</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>-0.18</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>960.1</v>
+        <v>5479</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>5424</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
@@ -2157,22 +2349,22 @@
         </is>
       </c>
       <c r="H19" s="14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>-516.79</v>
+        <v>-55</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.01</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -2181,18 +2373,18 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>952.1</v>
+        <v>960.1</v>
       </c>
       <c r="D20" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>948.8</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -2200,42 +2392,42 @@
         </is>
       </c>
       <c r="H20" s="14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>-29.7</v>
+        <v>-516.79</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.0598</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>1475</v>
+        <v>952.1</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>1394.19</v>
+        <v>948.8</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -2243,42 +2435,42 @@
         </is>
       </c>
       <c r="H21" s="14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>-484.86</v>
+        <v>-29.7</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0035</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>-1</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>248.05</v>
+        <v>1475</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>242.8</v>
+        <v>1394.19</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -2286,22 +2478,22 @@
         </is>
       </c>
       <c r="H22" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>-110.25</v>
+        <v>-484.86</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0548</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>-0.3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
@@ -2310,10 +2502,10 @@
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>1039.2</v>
+        <v>248.05</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
@@ -2321,7 +2513,7 @@
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>970</v>
+        <v>242.8</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -2332,19 +2524,19 @@
         <v>11</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>-346</v>
+        <v>-110.25</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -2353,10 +2545,10 @@
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>199.96</v>
+        <v>1039.2</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
@@ -2364,7 +2556,7 @@
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>193.31</v>
+        <v>970</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -2375,19 +2567,19 @@
         <v>11</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>-172.9</v>
+        <v>-346</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.06660000000000001</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -2396,10 +2588,10 @@
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>986.4</v>
+        <v>199.96</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
@@ -2407,7 +2599,7 @@
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>193.31</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -2418,17 +2610,60 @@
         <v>11</v>
       </c>
       <c r="I25" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J25" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K25" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D26" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G26" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H26" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I26" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J25" s="18" t="n">
+      <c r="J26" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K25" s="19" t="n">
+      <c r="K26" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I25">
+  <conditionalFormatting sqref="I2:I26">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2446,7 +2681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3043,6 +3278,31 @@
       </c>
       <c r="G23" s="14" t="n">
         <v>11</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="n">
+        <v>205146.44</v>
+      </c>
+      <c r="C24" s="20" t="n">
+        <v>74218.28999999999</v>
+      </c>
+      <c r="D24" s="20" t="n">
+        <v>130928.15</v>
+      </c>
+      <c r="E24" s="20" t="n">
+        <v>126599.6</v>
+      </c>
+      <c r="F24" s="20" t="n">
+        <v>817.89</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -3125,18 +3385,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>880.8</v>
+        <v>7861.5</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>832.9400000000001</v>
+        <v>7417</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -3148,7 +3408,7 @@
         <v>6.9</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8443043240062497</v>
+        <v>0.8277640033884996</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -3163,18 +3423,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>777</v>
+        <v>1055</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>744.8</v>
+        <v>985.6900000000001</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -3183,10 +3443,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8257969279467564</v>
+        <v>0.8045941031839501</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -3201,18 +3461,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>8862</v>
+        <v>8905</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>8315.07</v>
+        <v>8606.93</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -3221,10 +3481,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7796796055434938</v>
+        <v>0.8027221636810679</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -3239,18 +3499,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>SOLARINDS</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1566.1</v>
+        <v>19028</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1504.37</v>
+        <v>17859.86</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -3259,10 +3519,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.6</v>
+        <v>6.8</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7821287259298337</v>
+        <v>0.7914636666046819</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -3277,18 +3537,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>5448</v>
+        <v>1559.6</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>5157.93</v>
+        <v>1481.97</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -3300,7 +3560,7 @@
         <v>6.6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7660217519225696</v>
+        <v>0.7839242546333601</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -3315,18 +3575,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1932.6</v>
+        <v>4132.4</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1868.37</v>
+        <v>3947.11</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -3338,7 +3598,7 @@
         <v>6.6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7646297912058925</v>
+        <v>0.7708227442715758</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3353,18 +3613,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>2190.5</v>
+        <v>769.9</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>2067.2</v>
+        <v>712.78</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -3376,7 +3636,7 @@
         <v>6.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7569719781669135</v>
+        <v>0.7314882538895432</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3391,18 +3651,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>741.55</v>
+        <v>1297</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>687.5700000000001</v>
+        <v>1222.24</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -3411,10 +3671,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.74493537325244</v>
+        <v>0.7829583255852393</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3429,18 +3689,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>844</v>
+        <v>2565.8</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>811.3099999999999</v>
+        <v>2434.01</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -3452,7 +3712,7 @@
         <v>6.5</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7583406042651624</v>
+        <v>0.7566189384078184</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3467,18 +3727,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>7247.5</v>
+        <v>1956.4</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>6931.93</v>
+        <v>1893.21</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -3490,7 +3750,7 @@
         <v>6.5</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7459793437899478</v>
+        <v>0.7480929358044588</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3505,18 +3765,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1341.3</v>
+        <v>323.5</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1223.64</v>
+        <v>307.96</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -3525,10 +3785,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7441003997321591</v>
+        <v>0.752547573296969</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3543,18 +3803,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1086.2</v>
+        <v>7318</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1025.69</v>
+        <v>6989.5</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -3563,10 +3823,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7282927175699532</v>
+        <v>0.7405029029525403</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3581,18 +3841,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>7579</v>
+        <v>1565.8</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>7157.86</v>
+        <v>1504.57</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -3604,7 +3864,7 @@
         <v>6.3</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.750858308138709</v>
+        <v>0.7382921134734189</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3619,18 +3879,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1427.2</v>
+        <v>588</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1370.09</v>
+        <v>552.46</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -3639,10 +3899,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7250552929001887</v>
+        <v>0.7631418004504225</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3657,7 +3917,7 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260717</v>
+        <v>20260720</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
@@ -3665,10 +3925,10 @@
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1493.4</v>
+        <v>1492.3</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1417.66</v>
+        <v>1417.84</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -3680,7 +3940,7 @@
         <v>6.1</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7486171702209686</v>
+        <v>0.7466238971879585</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-21
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Mon 20 Jul 2026</t>
+          <t>As of Tue 21 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹205,146</t>
+          <t>₹205,545</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+412  (+0.20%)</t>
+          <t>₹+399  (+0.19%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.57%</t>
+          <t>+2.77%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.46%</t>
+          <t>-0.27%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹130,928</t>
+          <t>₹131,327</t>
         </is>
       </c>
     </row>
@@ -796,16 +796,16 @@
         <v>9246.6</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>457.55</v>
+        <v>451.1</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>10066.1</v>
+        <v>9924.200000000001</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>819.5</v>
+        <v>677.6000000000003</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.08862717106828456</v>
+        <v>0.07328098976921249</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>386.74</v>
@@ -814,13 +814,13 @@
         <v>430.3857142857142</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.05936899948483394</v>
+        <v>0.04591949836906623</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8790</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1615.8</v>
+        <v>1628.9</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9694.799999999999</v>
+        <v>9773.400000000001</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>904.7999999999997</v>
+        <v>983.4000000000005</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.1029351535836177</v>
+        <v>0.1118771331058021</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1365.41</v>
@@ -862,13 +862,13 @@
         <v>1498.128571428571</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.07282549113221226</v>
+        <v>0.08028204835866457</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>45.25</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -892,31 +892,31 @@
         <v>9288.75</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>714.55</v>
+        <v>732.75</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>10718.25</v>
+        <v>10991.25</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>1429.499999999999</v>
+        <v>1702.5</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.1538958417440451</v>
+        <v>0.1832862333467905</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>591.46</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>655.2785714285714</v>
+        <v>671.9678571428572</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.08294930875576041</v>
+        <v>0.08295072379002777</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>14</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>8700</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>8905</v>
+        <v>8926.5</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>8905</v>
+        <v>8926.5</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>205</v>
+        <v>226.5</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.0235632183908046</v>
+        <v>0.02603448275862069</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>8339.209999999999</v>
@@ -958,13 +958,13 @@
         <v>8510.25</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.04432902863559798</v>
+        <v>0.04663081834985717</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>123.68</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>9000</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>912.45</v>
+        <v>914.85</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9124.5</v>
+        <v>9148.5</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>124.5000000000005</v>
+        <v>148.5000000000002</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.01383333333333338</v>
+        <v>0.01650000000000003</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>836</v>
@@ -1006,13 +1006,13 @@
         <v>887.1</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.02778234423804046</v>
+        <v>0.03033284144941794</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>29.64</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>7579.5</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>7861.5</v>
+        <v>7882</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>7861.5</v>
+        <v>7882</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>282</v>
+        <v>302.5</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.03720562042351078</v>
+        <v>0.03991028431954614</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>7128.14</v>
@@ -1054,13 +1054,13 @@
         <v>7289</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.07282325255994403</v>
+        <v>0.07523471200202994</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>209.96</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -1084,31 +1084,31 @@
         <v>8992.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1838.6</v>
+        <v>1799</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>9193</v>
+        <v>8995</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>200.4999999999995</v>
+        <v>2.5</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.02229635807617454</v>
+        <v>0.0002780094523213789</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1680.3</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>1718.814285714286</v>
+        <v>1722.657142857143</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.06515050271169054</v>
+        <v>0.04243627412054329</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>50.24</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -1156,7 +1156,7 @@
         <v>49.27</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>8883</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1297</v>
+        <v>1288.7</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9079</v>
+        <v>9020.9</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>196</v>
+        <v>137.9000000000003</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.02206461780929866</v>
+        <v>0.01552403467297088</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1182.49</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1185.2</v>
+        <v>1187.221428571428</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.08619892058596758</v>
+        <v>0.07874491458723655</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>39.97</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>8656.65</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>951.2</v>
+        <v>969</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8560.800000000001</v>
+        <v>8721</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-95.8499999999998</v>
+        <v>64.3499999999998</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>-0.01107241253833756</v>
+        <v>0.007433591516348679</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>920.8099999999999</v>
@@ -1246,13 +1246,13 @@
         <v>935.6</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.0164003364171573</v>
+        <v>0.03446852425180597</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>23.22</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>8808</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>876.1</v>
+        <v>875.7</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>8761</v>
+        <v>8757</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-46.99999999999932</v>
+        <v>-50.99999999999909</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.005336058128973583</v>
+        <v>-0.00579019073569472</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>832.9400000000001</v>
@@ -1294,13 +1294,13 @@
         <v>832.9400000000001</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.04926378267321078</v>
+        <v>0.04882950782231357</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>24.22</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1348,7 +1348,7 @@
         <v>17.34</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1372,31 +1372,31 @@
         <v>8847</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>8885</v>
+        <v>8903.5</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>8885</v>
+        <v>8903.5</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>38</v>
+        <v>56.5</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.004295241324742851</v>
+        <v>0.006386345653893975</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>8315.07</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>8315.07</v>
+        <v>8791</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.06414518851997753</v>
+        <v>0.01263548042904476</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>254.57</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1420,31 +1420,31 @@
         <v>7800</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1565.8</v>
+        <v>1591.3</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>7829</v>
+        <v>7956.5</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>28.99999999999977</v>
+        <v>156.4999999999998</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.003717948717948689</v>
+        <v>0.02006410256410254</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>1504.37</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>1504.37</v>
+        <v>1547.4</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.03923234129518461</v>
+        <v>0.02758750706969136</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>30.61</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1468,31 +1468,31 @@
         <v>5438</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>5506</v>
+        <v>5583</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>5506</v>
+        <v>5583</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>68</v>
+        <v>145</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.01250459727841118</v>
+        <v>0.02666421478484737</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>5157.93</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>5157.93</v>
+        <v>5381</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.06321649110061746</v>
+        <v>0.03618126455310765</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>143.39</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2681,7 +2681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3302,6 +3302,31 @@
         <v>817.89</v>
       </c>
       <c r="G24" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n">
+        <v>205545.24</v>
+      </c>
+      <c r="C25" s="20" t="n">
+        <v>74218.28999999999</v>
+      </c>
+      <c r="D25" s="20" t="n">
+        <v>131326.95</v>
+      </c>
+      <c r="E25" s="20" t="n">
+        <v>126599.6</v>
+      </c>
+      <c r="F25" s="20" t="n">
+        <v>817.89</v>
+      </c>
+      <c r="G25" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3385,18 +3410,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>7861.5</v>
+        <v>875.7</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>7417</v>
+        <v>824.74</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -3405,10 +3430,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8277640033884996</v>
+        <v>0.841421310357652</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -3423,18 +3448,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1055</v>
+        <v>7882</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>985.6900000000001</v>
+        <v>7455.14</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -3443,10 +3468,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8045941031839501</v>
+        <v>0.8105694332527531</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -3461,18 +3486,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>8905</v>
+        <v>1593.2</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>8606.93</v>
+        <v>1509.59</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -3481,10 +3506,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8027221636810679</v>
+        <v>0.7869377466476579</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -3499,18 +3524,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>19028</v>
+        <v>601</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>17859.86</v>
+        <v>564.96</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -3519,10 +3544,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.8</v>
+        <v>6.6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7914636666046819</v>
+        <v>0.8171832062645922</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -3537,18 +3562,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1559.6</v>
+        <v>1062.65</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1481.97</v>
+        <v>990.03</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -3560,7 +3585,7 @@
         <v>6.6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7839242546333601</v>
+        <v>0.7804985640199178</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -3575,18 +3600,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>4132.4</v>
+        <v>1846.5</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>3947.11</v>
+        <v>1777.26</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -3598,7 +3623,7 @@
         <v>6.6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7708227442715758</v>
+        <v>0.7782578152441167</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3613,18 +3638,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>769.9</v>
+        <v>1591.3</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>712.78</v>
+        <v>1528.33</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -3636,7 +3661,7 @@
         <v>6.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7314882538895432</v>
+        <v>0.7640633070931218</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3651,18 +3676,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1297</v>
+        <v>10403.5</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1222.24</v>
+        <v>9979.790000000001</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -3674,7 +3699,7 @@
         <v>6.5</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7829583255852393</v>
+        <v>0.7385700117771028</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3689,18 +3714,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>2565.8</v>
+        <v>1961.9</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>2434.01</v>
+        <v>1898.56</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -3712,7 +3737,7 @@
         <v>6.5</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7566189384078184</v>
+        <v>0.756176780511994</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3727,18 +3752,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1956.4</v>
+        <v>1432.5</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1893.21</v>
+        <v>1378.66</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -3747,10 +3772,10 @@
         <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7480929358044588</v>
+        <v>0.7343932725882766</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3765,18 +3790,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>323.5</v>
+        <v>8926.5</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>307.96</v>
+        <v>8637.209999999999</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -3785,10 +3810,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.752547573296969</v>
+        <v>0.7502334758982625</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3803,18 +3828,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>7318</v>
+        <v>1342.6</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>6989.5</v>
+        <v>1281.94</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -3823,10 +3848,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7405029029525403</v>
+        <v>0.770245253001095</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3841,18 +3866,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1565.8</v>
+        <v>1288.7</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1504.57</v>
+        <v>1215.51</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -3864,7 +3889,7 @@
         <v>6.3</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7382921134734189</v>
+        <v>0.7625240190913035</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3879,18 +3904,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>588</v>
+        <v>1799</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>552.46</v>
+        <v>1680.37</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -3902,7 +3927,7 @@
         <v>6.2</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7631418004504225</v>
+        <v>0.7258486745593917</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3917,7 +3942,7 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260720</v>
+        <v>20260721</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
@@ -3925,10 +3950,10 @@
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1492.3</v>
+        <v>1483.7</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1417.84</v>
+        <v>1410.33</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -3940,7 +3965,7 @@
         <v>6.1</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7466238971879585</v>
+        <v>0.7551695282960392</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-22
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Tue 21 Jul 2026</t>
+          <t>As of Wed 22 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹205,545</t>
+          <t>₹204,165</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+399  (+0.19%)</t>
+          <t>₹-1,380  (-0.67%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.77%</t>
+          <t>+2.08%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.27%</t>
+          <t>-0.94%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹74,218</t>
+          <t>₹91,485</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹126,600</t>
+          <t>₹108,468</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹131,327</t>
+          <t>₹112,680</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+818</t>
+          <t>₹-47</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>13</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -796,16 +796,16 @@
         <v>9246.6</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>451.1</v>
+        <v>456.65</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>9924.200000000001</v>
+        <v>10046.3</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>677.6000000000003</v>
+        <v>799.6999999999992</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.07328098976921249</v>
+        <v>0.08648584344515814</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>386.74</v>
@@ -814,13 +814,13 @@
         <v>430.3857142857142</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.04591949836906623</v>
+        <v>0.0575151335033083</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8790</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1628.9</v>
+        <v>1611.8</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9773.400000000001</v>
+        <v>9670.799999999999</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>983.4000000000005</v>
+        <v>880.7999999999997</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.1118771331058021</v>
+        <v>0.1002047781569966</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1365.41</v>
@@ -862,13 +862,13 @@
         <v>1498.128571428571</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.08028204835866457</v>
+        <v>0.07052452448903622</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>45.25</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -892,31 +892,31 @@
         <v>9288.75</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>732.75</v>
+        <v>726.5</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>10991.25</v>
+        <v>10897.5</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>1702.5</v>
+        <v>1608.75</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.1832862333467905</v>
+        <v>0.173193379087606</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>591.46</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>671.9678571428572</v>
+        <v>679.6178571428571</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.08295072379002777</v>
+        <v>0.06453151115917807</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>14</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>8700</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>8926.5</v>
+        <v>8938</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>8926.5</v>
+        <v>8938</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>226.5</v>
+        <v>238</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.02603448275862069</v>
+        <v>0.02735632183908046</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>8339.209999999999</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>8510.25</v>
+        <v>8516.928571428571</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.04663081834985717</v>
+        <v>0.04711025157433759</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>123.68</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>9000</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>914.85</v>
+        <v>912.85</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9148.5</v>
+        <v>9128.5</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>148.5000000000002</v>
+        <v>128.5000000000002</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.01650000000000003</v>
+        <v>0.0142777777777778</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>836</v>
@@ -1006,13 +1006,13 @@
         <v>887.1</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.03033284144941794</v>
+        <v>0.02820835843785945</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>29.64</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>7579.5</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>7882</v>
+        <v>7789</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>7882</v>
+        <v>7789</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>302.5</v>
+        <v>209.5</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.03991028431954614</v>
+        <v>0.0276403456692394</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>7128.14</v>
@@ -1054,13 +1054,13 @@
         <v>7289</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.07523471200202994</v>
+        <v>0.06419309282321223</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>209.96</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>8992.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1799</v>
+        <v>1788.5</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>8995</v>
+        <v>8942.5</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>2.5</v>
+        <v>-50</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.0002780094523213789</v>
+        <v>-0.005560189046427579</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1680.3</v>
@@ -1102,13 +1102,13 @@
         <v>1722.657142857143</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.04243627412054329</v>
+        <v>0.03681456927193592</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>50.24</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -1156,7 +1156,7 @@
         <v>49.27</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>8883</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1288.7</v>
+        <v>1250.5</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9020.9</v>
+        <v>8753.5</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>137.9000000000003</v>
+        <v>-129.5</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.01552403467297088</v>
+        <v>-0.01457840819542947</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1182.49</v>
@@ -1198,13 +1198,13 @@
         <v>1187.221428571428</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.07874491458723655</v>
+        <v>0.05060261609641879</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>39.97</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>8656.65</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>969</v>
+        <v>949.85</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8721</v>
+        <v>8548.65</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>64.3499999999998</v>
+        <v>-108</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.007433591516348679</v>
+        <v>-0.01247595778967614</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>920.8099999999999</v>
@@ -1246,19 +1246,19 @@
         <v>935.6</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.03446852425180597</v>
+        <v>0.01500236879507291</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>23.22</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1267,46 +1267,46 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>880.8</v>
+        <v>8847</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>8808</v>
+        <v>8847</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>875.7</v>
+        <v>9090.5</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>8757</v>
+        <v>9090.5</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-50.99999999999909</v>
+        <v>243.5</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.00579019073569472</v>
+        <v>0.02752345427828642</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>832.9400000000001</v>
+        <v>8315.07</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>832.9400000000001</v>
+        <v>8791</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.04882950782231357</v>
+        <v>0.03294648259171663</v>
       </c>
       <c r="M12" s="13" t="n">
-        <v>24.22</v>
+        <v>254.57</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -1315,46 +1315,46 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>777</v>
+        <v>1560</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>9324</v>
+        <v>7800</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>791.55</v>
+        <v>1608.6</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>9498.599999999999</v>
+        <v>8043</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>174.5999999999995</v>
+        <v>242.9999999999995</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.01872586872586867</v>
+        <v>0.03115384615384609</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>744.8</v>
+        <v>1504.37</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>744.8</v>
+        <v>1547.4</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.05906133535468385</v>
+        <v>0.03804550540842958</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>17.34</v>
+        <v>30.61</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1363,140 +1363,44 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>8847</v>
+        <v>5438</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>8847</v>
+        <v>5438</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>8903.5</v>
+        <v>5586</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>8903.5</v>
+        <v>5586</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>56.5</v>
+        <v>148</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.006386345653893975</v>
+        <v>0.02721588819418904</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>8315.07</v>
+        <v>5157.93</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>8791</v>
+        <v>5381</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.01263548042904476</v>
+        <v>0.03669889008234873</v>
       </c>
       <c r="M14" s="13" t="n">
-        <v>254.57</v>
+        <v>143.39</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>PIDILITIND</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>1560</v>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="E15" s="9" t="n">
-        <v>7800</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>1591.3</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>7956.5</v>
-      </c>
-      <c r="H15" s="10" t="n">
-        <v>156.4999999999998</v>
-      </c>
-      <c r="I15" s="11" t="n">
-        <v>0.02006410256410254</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>1504.37</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>1547.4</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>0.02758750706969136</v>
-      </c>
-      <c r="M15" s="13" t="n">
-        <v>30.61</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>CUMMINSIND</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>5438</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <v>5438</v>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>5583</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>5583</v>
-      </c>
-      <c r="H16" s="10" t="n">
-        <v>145</v>
-      </c>
-      <c r="I16" s="11" t="n">
-        <v>0.02666421478484737</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>5157.93</v>
-      </c>
-      <c r="K16" s="7" t="n">
-        <v>5381</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>0.03618126455310765</v>
-      </c>
-      <c r="M16" s="13" t="n">
-        <v>143.39</v>
-      </c>
-      <c r="N16" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H16">
+  <conditionalFormatting sqref="H2:H14">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1514,7 +1418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1590,27 +1494,27 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>1114.9</v>
+        <v>880.8</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>1050.57</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -1618,13 +1522,13 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-514.64</v>
+        <v>-478.6</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0577</v>
+        <v>-0.0543</v>
       </c>
       <c r="K2" s="19" t="n">
         <v>-1</v>
@@ -1633,93 +1537,93 @@
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>790</v>
+        <v>777</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>880.8</v>
+        <v>744.8</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>998.8</v>
+        <v>-386.4</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0414</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>3770</v>
+        <v>1114.9</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>4097.9</v>
+        <v>1050.57</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>655.8</v>
+        <v>-514.64</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>-0.0577</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>1.98</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -1728,7 +1632,7 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>821.05</v>
+        <v>790</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>11</v>
@@ -1739,7 +1643,7 @@
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>844</v>
+        <v>880.8</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1750,19 +1654,19 @@
         <v>25</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>252.45</v>
+        <v>998.8</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>0.028</v>
+        <v>0.1149</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>0.6</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -1771,10 +1675,10 @@
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>2426.1</v>
+        <v>3770</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -1782,7 +1686,7 @@
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>2484.2</v>
+        <v>4097.9</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -1793,39 +1697,39 @@
         <v>25</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>174.3</v>
+        <v>655.8</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>0.5</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>1410</v>
+        <v>821.05</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>1455.2</v>
+        <v>844</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -1836,39 +1740,39 @@
         <v>25</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>135.6</v>
+        <v>252.45</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.028</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>0.46</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>690</v>
+        <v>2426.1</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>660.45</v>
+        <v>2484.2</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -1879,19 +1783,19 @@
         <v>25</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>-206.85</v>
+        <v>174.3</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.0239</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -1900,10 +1804,10 @@
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>1839</v>
+        <v>1410</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
@@ -1911,7 +1815,7 @@
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>1828.1</v>
+        <v>1455.2</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
@@ -1922,19 +1826,19 @@
         <v>25</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>-21.8</v>
+        <v>135.6</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>-0.0059</v>
+        <v>0.0321</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>-0.1</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -1943,10 +1847,10 @@
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1414</v>
+        <v>690</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
@@ -1954,7 +1858,7 @@
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>1537.8</v>
+        <v>660.45</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
@@ -1965,19 +1869,19 @@
         <v>25</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>371.4</v>
+        <v>-206.85</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>0.0876</v>
+        <v>-0.0428</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>1.38</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -1986,10 +1890,10 @@
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>1300</v>
+        <v>1839</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
@@ -1997,7 +1901,7 @@
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>1389.1</v>
+        <v>1828.1</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
@@ -2008,19 +1912,19 @@
         <v>25</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>356.4</v>
+        <v>-21.8</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>-0.0059</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>0.63</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -2029,10 +1933,10 @@
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>276.45</v>
+        <v>1414</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
@@ -2040,7 +1944,7 @@
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>330.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -2051,19 +1955,19 @@
         <v>25</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>1019.35</v>
+        <v>371.4</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.0876</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>3.1</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -2072,10 +1976,10 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>1462.5</v>
+        <v>1300</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
@@ -2083,7 +1987,7 @@
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>1564.7</v>
+        <v>1389.1</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
@@ -2094,19 +1998,19 @@
         <v>25</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>306.6</v>
+        <v>356.4</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>1.78</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -2115,41 +2019,41 @@
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>798</v>
+        <v>276.45</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>750</v>
+        <v>330.1</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H14" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>-288</v>
+        <v>1019.35</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.1941</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>-0.92</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -2158,53 +2062,53 @@
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>260.45</v>
+        <v>1462.5</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>257.85</v>
+        <v>1564.7</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H15" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>-52.07</v>
+        <v>306.6</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>-0.01</v>
+        <v>0.0699</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>-0.13</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>6500</v>
+        <v>798</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
@@ -2212,7 +2116,7 @@
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>6401.5</v>
+        <v>750</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
@@ -2220,34 +2124,34 @@
         </is>
       </c>
       <c r="H16" s="14" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>-98.5</v>
+        <v>-288</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.0602</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>571.5</v>
+        <v>260.45</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
@@ -2255,7 +2159,7 @@
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>571.1</v>
+        <v>257.85</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -2263,34 +2167,34 @@
         </is>
       </c>
       <c r="H17" s="14" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>-6.4</v>
+        <v>-52.07</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.01</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>965</v>
+        <v>6500</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
@@ -2298,7 +2202,7 @@
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>933</v>
+        <v>6401.5</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -2306,22 +2210,22 @@
         </is>
       </c>
       <c r="H18" s="14" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>-288</v>
+        <v>-98.5</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0152</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -2330,18 +2234,18 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>5479</v>
+        <v>571.5</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>5424</v>
+        <v>571.1</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
@@ -2349,42 +2253,42 @@
         </is>
       </c>
       <c r="H19" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>-55</v>
+        <v>-6.4</v>
       </c>
       <c r="J19" s="18" t="n">
+        <v>-0.0007</v>
+      </c>
+      <c r="K19" s="19" t="n">
         <v>-0.01</v>
-      </c>
-      <c r="K19" s="19" t="n">
-        <v>-0.18</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>960.1</v>
+        <v>965</v>
       </c>
       <c r="D20" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>933</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -2392,42 +2296,42 @@
         </is>
       </c>
       <c r="H20" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>-516.79</v>
+        <v>-288</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.0332</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>952.1</v>
+        <v>5479</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>948.8</v>
+        <v>5424</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -2438,39 +2342,39 @@
         <v>1</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>-29.7</v>
+        <v>-55</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.01</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>1475</v>
+        <v>960.1</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>1394.19</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -2478,42 +2382,42 @@
         </is>
       </c>
       <c r="H22" s="14" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>-484.86</v>
+        <v>-516.79</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0598</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>-1</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>248.05</v>
+        <v>952.1</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>242.8</v>
+        <v>948.8</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -2521,42 +2425,42 @@
         </is>
       </c>
       <c r="H23" s="14" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>-110.25</v>
+        <v>-29.7</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0035</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>-0.3</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>1039.2</v>
+        <v>1475</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>970</v>
+        <v>1394.19</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -2564,22 +2468,22 @@
         </is>
       </c>
       <c r="H24" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>-346</v>
+        <v>-484.86</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0548</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>-0.82</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -2588,10 +2492,10 @@
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>199.96</v>
+        <v>248.05</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
@@ -2599,7 +2503,7 @@
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>193.31</v>
+        <v>242.8</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -2610,19 +2514,19 @@
         <v>11</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>-172.9</v>
+        <v>-110.25</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.0212</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
@@ -2631,7 +2535,7 @@
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>986.4</v>
+        <v>1039.2</v>
       </c>
       <c r="D26" s="16" t="n">
         <v>5</v>
@@ -2642,7 +2546,7 @@
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>970</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
@@ -2653,17 +2557,103 @@
         <v>11</v>
       </c>
       <c r="I26" s="17" t="n">
+        <v>-346</v>
+      </c>
+      <c r="J26" s="18" t="n">
+        <v>-0.06660000000000001</v>
+      </c>
+      <c r="K26" s="19" t="n">
+        <v>-0.82</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="n">
+        <v>199.96</v>
+      </c>
+      <c r="D27" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="G27" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H27" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I27" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J27" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K27" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D28" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F28" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G28" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I28" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J26" s="18" t="n">
+      <c r="J28" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K26" s="19" t="n">
+      <c r="K28" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I26">
+  <conditionalFormatting sqref="I2:I28">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2681,7 +2671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3328,6 +3318,31 @@
       </c>
       <c r="G25" s="14" t="n">
         <v>15</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="n">
+        <v>204165.14</v>
+      </c>
+      <c r="C26" s="20" t="n">
+        <v>91485.28999999999</v>
+      </c>
+      <c r="D26" s="20" t="n">
+        <v>112679.85</v>
+      </c>
+      <c r="E26" s="20" t="n">
+        <v>108467.6</v>
+      </c>
+      <c r="F26" s="20" t="n">
+        <v>-47.11</v>
+      </c>
+      <c r="G26" s="14" t="n">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -3410,30 +3425,30 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>875.7</v>
+        <v>9090.5</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>824.74</v>
+        <v>8589.5</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7</v>
+        <v>6.2</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.841421310357652</v>
+        <v>0.8206484570475396</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -3442,13 +3457,13 @@
       </c>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
@@ -3456,22 +3471,22 @@
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>7882</v>
+        <v>7789</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>7455.14</v>
+        <v>7360.57</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.7</v>
+        <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8105694332527531</v>
+        <v>0.8339720600500417</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -3480,36 +3495,36 @@
       </c>
       <c r="J3" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1593.2</v>
+        <v>1533.6</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1509.59</v>
+        <v>1450.07</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.7</v>
+        <v>6.1</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7869377466476579</v>
+        <v>0.8122685571309425</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -3518,36 +3533,36 @@
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>601</v>
+        <v>853.8</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>564.96</v>
+        <v>797.86</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8171832062645922</v>
+        <v>0.818281901584654</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -3556,36 +3571,36 @@
       </c>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1062.65</v>
+        <v>326.6</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>990.03</v>
+        <v>310.44</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7804985640199178</v>
+        <v>0.8014512093411177</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -3594,36 +3609,36 @@
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1846.5</v>
+        <v>1353.4</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1777.26</v>
+        <v>1288.41</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.6</v>
+        <v>5.9</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7782578152441167</v>
+        <v>0.8078440366972477</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3632,36 +3647,36 @@
       </c>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1591.3</v>
+        <v>1250.5</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1528.33</v>
+        <v>1175.64</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.6</v>
+        <v>5.9</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7640633070931218</v>
+        <v>0.8031588824020016</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3670,36 +3685,36 @@
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>10403.5</v>
+        <v>1943</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>9979.790000000001</v>
+        <v>1876.67</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.5</v>
+        <v>5.9</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7385700117771028</v>
+        <v>0.7778231859883237</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3708,36 +3723,36 @@
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1961.9</v>
+        <v>1608.6</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1898.56</v>
+        <v>1543.36</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.5</v>
+        <v>5.9</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.756176780511994</v>
+        <v>0.7746497080900752</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3746,36 +3761,36 @@
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1432.5</v>
+        <v>1819.4</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1378.66</v>
+        <v>1751.19</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.4</v>
+        <v>5.8</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7343932725882766</v>
+        <v>0.7544787322768974</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3784,36 +3799,36 @@
       </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>8926.5</v>
+        <v>1489.9</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>8637.209999999999</v>
+        <v>1414.13</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.4</v>
+        <v>5.6</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7502334758982625</v>
+        <v>0.7853336113427856</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3822,36 +3837,36 @@
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>CAPLIPOINT</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1342.6</v>
+        <v>2480.6</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1281.94</v>
+        <v>2283.19</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.3</v>
+        <v>5.6</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.770245253001095</v>
+        <v>0.7533236030025021</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3860,36 +3875,36 @@
       </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1288.7</v>
+        <v>1577.8</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1215.51</v>
+        <v>1498.01</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.3</v>
+        <v>5.6</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7625240190913035</v>
+        <v>0.736743119266055</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3898,36 +3913,36 @@
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1799</v>
+        <v>1415.1</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1680.37</v>
+        <v>1358.21</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.2</v>
+        <v>5.6</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7258486745593917</v>
+        <v>0.7360425354462051</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3936,36 +3951,36 @@
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260721</v>
+        <v>20260722</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1483.7</v>
+        <v>2185.5</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1410.33</v>
+        <v>2081.01</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0267</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>9333</v>
+        <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7551695282960392</v>
+        <v>0.7346267723102585</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>
@@ -3974,7 +3989,7 @@
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>RISK_NEU</t>
+          <t>RISK_OFF</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-23
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Wed 22 Jul 2026</t>
+          <t>As of Thu 23 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹204,165</t>
+          <t>₹202,796</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-1,380  (-0.67%)</t>
+          <t>₹-1,369  (-0.67%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.08%</t>
+          <t>+1.40%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.94%</t>
+          <t>-1.60%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹91,485</t>
+          <t>₹100,356</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹108,468</t>
+          <t>₹99,468</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹112,680</t>
+          <t>₹102,440</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹-47</t>
+          <t>₹-176</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -796,16 +796,16 @@
         <v>9246.6</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>456.65</v>
+        <v>445.45</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>10046.3</v>
+        <v>9799.9</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>799.6999999999992</v>
+        <v>553.2999999999995</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.08648584344515814</v>
+        <v>0.05983821080180818</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>386.74</v>
@@ -814,13 +814,13 @@
         <v>430.3857142857142</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.0575151335033083</v>
+        <v>0.03381812933951228</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>16.71</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -844,31 +844,31 @@
         <v>8790</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1611.8</v>
+        <v>1612.8</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9670.799999999999</v>
+        <v>9676.799999999999</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>880.7999999999997</v>
+        <v>886.7999999999997</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.1002047781569966</v>
+        <v>0.1008873720136518</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1365.41</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>1498.128571428571</v>
+        <v>1506.7</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.07052452448903622</v>
+        <v>0.06578621031746026</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>45.25</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9288.75</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>726.5</v>
+        <v>719.75</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>10897.5</v>
+        <v>10796.25</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>1608.75</v>
+        <v>1507.5</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.173193379087606</v>
+        <v>0.1622930964876867</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>591.46</v>
@@ -910,13 +910,13 @@
         <v>679.6178571428571</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.06453151115917807</v>
+        <v>0.05575844787376571</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>14</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
@@ -940,37 +940,37 @@
         <v>8700</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>8938</v>
+        <v>8862</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>8938</v>
+        <v>8862</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>238</v>
+        <v>162</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.02735632183908046</v>
+        <v>0.01862068965517241</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>8339.209999999999</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>8516.928571428571</v>
+        <v>8535.464285714286</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.04711025157433759</v>
+        <v>0.03684672921301216</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>123.68</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -979,46 +979,46 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>900</v>
+        <v>7579.5</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>9000</v>
+        <v>7579.5</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>912.85</v>
+        <v>7673.5</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9128.5</v>
+        <v>7673.5</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>128.5000000000002</v>
+        <v>94</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.0142777777777778</v>
+        <v>0.0124018734745036</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>836</v>
+        <v>7128.14</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>887.1</v>
+        <v>7289</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.02820835843785945</v>
+        <v>0.05010751286896462</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>29.64</v>
+        <v>209.96</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -1027,94 +1027,94 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>7579.5</v>
+        <v>1798.5</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>7579.5</v>
+        <v>8992.5</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>7789</v>
+        <v>1771.2</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>7789</v>
+        <v>8856</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>209.5</v>
+        <v>-136.4999999999998</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.0276403456692394</v>
+        <v>-0.01517931609674726</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>7128.14</v>
+        <v>1680.3</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>7289</v>
+        <v>1722.657142857143</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.06419309282321223</v>
+        <v>0.02740676216285988</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>209.96</v>
+        <v>50.24</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>1798.5</v>
+        <v>2415.2</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>8992.5</v>
+        <v>7245.6</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1788.5</v>
+        <v>2415.2</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>8942.5</v>
+        <v>7245.599999999999</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>-50</v>
+        <v>0</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>-0.005560189046427579</v>
+        <v>0</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>1680.3</v>
+        <v>2335.46</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>1722.657142857143</v>
+        <v>2349.7</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.03681456927193592</v>
+        <v>0.02711990725405764</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>50.24</v>
+        <v>49.27</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -1123,46 +1123,46 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>2415.2</v>
+        <v>1269</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>7245.6</v>
+        <v>8883</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>2415.2</v>
+        <v>1240.3</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>7245.599999999999</v>
+        <v>8682.1</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>0</v>
+        <v>-200.9000000000003</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0</v>
+        <v>-0.02261623325453116</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>2335.46</v>
+        <v>1182.49</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>2349.7</v>
+        <v>1187.221428571428</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.02711990725405764</v>
+        <v>0.04279494592322152</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>49.27</v>
+        <v>39.97</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1171,94 +1171,94 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1269</v>
+        <v>961.85</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>8883</v>
+        <v>8656.65</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1250.5</v>
+        <v>943.65</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>8753.5</v>
+        <v>8492.85</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>-129.5</v>
+        <v>-163.8000000000004</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>-0.01457840819542947</v>
+        <v>-0.0189218693143422</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>1182.49</v>
+        <v>920.8099999999999</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1187.221428571428</v>
+        <v>935.6</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.05060261609641879</v>
+        <v>0.008530705240290313</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>39.97</v>
+        <v>23.22</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>961.85</v>
+        <v>8847</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>8656.65</v>
+        <v>8847</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>949.85</v>
+        <v>8935</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8548.65</v>
+        <v>8935</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-108</v>
+        <v>88</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>-0.01247595778967614</v>
+        <v>0.009946874646772918</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>920.8099999999999</v>
+        <v>8315.07</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>935.6</v>
+        <v>8791</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.01500236879507291</v>
+        <v>0.01611639619473979</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>23.22</v>
+        <v>254.57</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1267,46 +1267,46 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>8847</v>
+        <v>1560</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>8847</v>
+        <v>7800</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>9090.5</v>
+        <v>1564.2</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>9090.5</v>
+        <v>7821</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>243.5</v>
+        <v>21.00000000000023</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.02752345427828642</v>
+        <v>0.002692307692307721</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>8315.07</v>
+        <v>1504.37</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>8791</v>
+        <v>1547.4</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.03294648259171663</v>
+        <v>0.01074031453778286</v>
       </c>
       <c r="M12" s="13" t="n">
-        <v>254.57</v>
+        <v>30.61</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -1315,92 +1315,44 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>1560</v>
+        <v>5438</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>7800</v>
+        <v>5438</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1608.6</v>
+        <v>5599</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>8043</v>
+        <v>5599</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>242.9999999999995</v>
+        <v>161</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.03115384615384609</v>
+        <v>0.02960647296800294</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>1504.37</v>
+        <v>5157.93</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>1547.4</v>
+        <v>5381</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.03804550540842958</v>
+        <v>0.03893552420075013</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>30.61</v>
+        <v>143.39</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>CUMMINSIND</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>5438</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="9" t="n">
-        <v>5438</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>5586</v>
-      </c>
-      <c r="G14" s="9" t="n">
-        <v>5586</v>
-      </c>
-      <c r="H14" s="10" t="n">
-        <v>148</v>
-      </c>
-      <c r="I14" s="11" t="n">
-        <v>0.02721588819418904</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>5157.93</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>5381</v>
-      </c>
-      <c r="L14" s="12" t="n">
-        <v>0.03669889008234873</v>
-      </c>
-      <c r="M14" s="13" t="n">
-        <v>143.39</v>
-      </c>
-      <c r="N14" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H14">
+  <conditionalFormatting sqref="H2:H13">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1418,7 +1370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1494,27 +1446,27 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>880.8</v>
+        <v>900</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>10</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>832.9400000000001</v>
+        <v>887.1</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -1522,22 +1474,22 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-478.6</v>
+        <v>-129</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0543</v>
+        <v>-0.0143</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -1546,10 +1498,10 @@
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>777</v>
+        <v>880.8</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
@@ -1557,7 +1509,7 @@
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>744.8</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -1568,10 +1520,10 @@
         <v>2</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-386.4</v>
+        <v>-478.6</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0414</v>
+        <v>-0.0543</v>
       </c>
       <c r="K3" s="19" t="n">
         <v>-1</v>
@@ -1580,27 +1532,27 @@
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>1114.9</v>
+        <v>777</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>1050.57</v>
+        <v>744.8</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1608,13 +1560,13 @@
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-514.64</v>
+        <v>-386.4</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0577</v>
+        <v>-0.0414</v>
       </c>
       <c r="K4" s="19" t="n">
         <v>-1</v>
@@ -1623,50 +1575,50 @@
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>790</v>
+        <v>1114.9</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>880.8</v>
+        <v>1050.57</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>998.8</v>
+        <v>-514.64</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0577</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -1675,10 +1627,10 @@
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>3770</v>
+        <v>790</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -1686,7 +1638,7 @@
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>4097.9</v>
+        <v>880.8</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -1697,19 +1649,19 @@
         <v>25</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>655.8</v>
+        <v>998.8</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.1149</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>1.98</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -1718,10 +1670,10 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>821.05</v>
+        <v>3770</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
@@ -1729,7 +1681,7 @@
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>844</v>
+        <v>4097.9</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -1740,19 +1692,19 @@
         <v>25</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>252.45</v>
+        <v>655.8</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>0.028</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>0.6</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -1761,10 +1713,10 @@
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>2426.1</v>
+        <v>821.05</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
@@ -1772,7 +1724,7 @@
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>2484.2</v>
+        <v>844</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -1783,39 +1735,39 @@
         <v>25</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>174.3</v>
+        <v>252.45</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.028</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>1410</v>
+        <v>2426.1</v>
       </c>
       <c r="D9" s="16" t="n">
         <v>3</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>1455.2</v>
+        <v>2484.2</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
@@ -1826,19 +1778,19 @@
         <v>25</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>135.6</v>
+        <v>174.3</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.0239</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>0.46</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -1847,10 +1799,10 @@
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>690</v>
+        <v>1410</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
@@ -1858,7 +1810,7 @@
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>660.45</v>
+        <v>1455.2</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
@@ -1869,19 +1821,19 @@
         <v>25</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>-206.85</v>
+        <v>135.6</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.0321</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -1890,10 +1842,10 @@
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>1839</v>
+        <v>690</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
@@ -1901,7 +1853,7 @@
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>1828.1</v>
+        <v>660.45</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
@@ -1912,19 +1864,19 @@
         <v>25</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>-21.8</v>
+        <v>-206.85</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>-0.0059</v>
+        <v>-0.0428</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>-0.1</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -1933,10 +1885,10 @@
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>1414</v>
+        <v>1839</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
@@ -1944,7 +1896,7 @@
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>1537.8</v>
+        <v>1828.1</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -1955,19 +1907,19 @@
         <v>25</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>371.4</v>
+        <v>-21.8</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>0.0876</v>
+        <v>-0.0059</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>1.38</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -1976,10 +1928,10 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>1300</v>
+        <v>1414</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
@@ -1987,7 +1939,7 @@
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>1389.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
@@ -1998,19 +1950,19 @@
         <v>25</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>356.4</v>
+        <v>371.4</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>0.0876</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>0.63</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -2019,10 +1971,10 @@
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>276.45</v>
+        <v>1300</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
@@ -2030,7 +1982,7 @@
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>330.1</v>
+        <v>1389.1</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
@@ -2041,19 +1993,19 @@
         <v>25</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>1019.35</v>
+        <v>356.4</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>3.1</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -2062,10 +2014,10 @@
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>1462.5</v>
+        <v>276.45</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
@@ -2073,7 +2025,7 @@
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>1564.7</v>
+        <v>330.1</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
@@ -2084,19 +2036,19 @@
         <v>25</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>306.6</v>
+        <v>1019.35</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.1941</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>1.78</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -2105,41 +2057,41 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>798</v>
+        <v>1462.5</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>750</v>
+        <v>1564.7</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H16" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>-288</v>
+        <v>306.6</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.0699</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>-0.92</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -2148,10 +2100,10 @@
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>260.45</v>
+        <v>798</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
@@ -2159,7 +2111,7 @@
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>257.85</v>
+        <v>750</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -2170,31 +2122,31 @@
         <v>23</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>-52.07</v>
+        <v>-288</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0602</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>-0.13</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>6500</v>
+        <v>260.45</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
@@ -2202,7 +2154,7 @@
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>6401.5</v>
+        <v>257.85</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -2210,65 +2162,65 @@
         </is>
       </c>
       <c r="H18" s="14" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>-98.5</v>
+        <v>-52.07</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.01</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>571.5</v>
+        <v>6500</v>
       </c>
       <c r="D19" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="n">
+        <v>6401.5</v>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="E19" s="14" t="inlineStr">
-        <is>
-          <t>2026-07-08</t>
-        </is>
-      </c>
-      <c r="F19" s="15" t="n">
-        <v>571.1</v>
-      </c>
-      <c r="G19" s="14" t="inlineStr">
-        <is>
-          <t>STOP_LOSS</t>
-        </is>
-      </c>
-      <c r="H19" s="14" t="n">
-        <v>2</v>
-      </c>
       <c r="I19" s="17" t="n">
-        <v>-6.4</v>
+        <v>-98.5</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.0152</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -2277,10 +2229,10 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>965</v>
+        <v>571.5</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
@@ -2288,7 +2240,7 @@
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>933</v>
+        <v>571.1</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -2299,19 +2251,19 @@
         <v>2</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>-288</v>
+        <v>-6.4</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0007</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -2320,18 +2272,18 @@
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>5479</v>
+        <v>965</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>5424</v>
+        <v>933</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -2339,42 +2291,42 @@
         </is>
       </c>
       <c r="H21" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>-55</v>
+        <v>-288</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0332</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>-0.18</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>960.1</v>
+        <v>5479</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>5424</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -2382,22 +2334,22 @@
         </is>
       </c>
       <c r="H22" s="14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>-516.79</v>
+        <v>-55</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.01</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
@@ -2406,18 +2358,18 @@
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>952.1</v>
+        <v>960.1</v>
       </c>
       <c r="D23" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>948.8</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -2425,42 +2377,42 @@
         </is>
       </c>
       <c r="H23" s="14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>-29.7</v>
+        <v>-516.79</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.0598</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>1475</v>
+        <v>952.1</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>1394.19</v>
+        <v>948.8</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -2468,42 +2420,42 @@
         </is>
       </c>
       <c r="H24" s="14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>-484.86</v>
+        <v>-29.7</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0035</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>-1</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>248.05</v>
+        <v>1475</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>242.8</v>
+        <v>1394.19</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -2511,22 +2463,22 @@
         </is>
       </c>
       <c r="H25" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>-110.25</v>
+        <v>-484.86</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0548</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>-0.3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
@@ -2535,10 +2487,10 @@
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>1039.2</v>
+        <v>248.05</v>
       </c>
       <c r="D26" s="16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
@@ -2546,7 +2498,7 @@
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>970</v>
+        <v>242.8</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
@@ -2557,19 +2509,19 @@
         <v>11</v>
       </c>
       <c r="I26" s="17" t="n">
-        <v>-346</v>
+        <v>-110.25</v>
       </c>
       <c r="J26" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
@@ -2578,10 +2530,10 @@
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>199.96</v>
+        <v>1039.2</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
@@ -2589,7 +2541,7 @@
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>193.31</v>
+        <v>970</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
@@ -2600,19 +2552,19 @@
         <v>11</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>-172.9</v>
+        <v>-346</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.06660000000000001</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
@@ -2621,10 +2573,10 @@
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>986.4</v>
+        <v>199.96</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
@@ -2632,7 +2584,7 @@
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>193.31</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
@@ -2643,17 +2595,60 @@
         <v>11</v>
       </c>
       <c r="I28" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J28" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K28" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D29" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F29" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H29" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I29" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J28" s="18" t="n">
+      <c r="J29" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K28" s="19" t="n">
+      <c r="K29" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I28">
+  <conditionalFormatting sqref="I2:I29">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2671,7 +2666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3343,6 +3338,31 @@
       </c>
       <c r="G26" s="14" t="n">
         <v>13</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="n">
+        <v>202796.29</v>
+      </c>
+      <c r="C27" s="20" t="n">
+        <v>100356.29</v>
+      </c>
+      <c r="D27" s="20" t="n">
+        <v>102440</v>
+      </c>
+      <c r="E27" s="20" t="n">
+        <v>99467.60000000001</v>
+      </c>
+      <c r="F27" s="20" t="n">
+        <v>-176.11</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -3425,18 +3445,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>9090.5</v>
+        <v>1954</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8589.5</v>
+        <v>1890.87</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -3445,10 +3465,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8206484570475396</v>
+        <v>0.8119140950792326</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -3463,18 +3483,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>7789</v>
+        <v>1778.5</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>7360.57</v>
+        <v>1705.94</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -3486,7 +3506,7 @@
         <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8339720600500417</v>
+        <v>0.804034612176814</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -3501,18 +3521,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1533.6</v>
+        <v>1378.2</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1450.07</v>
+        <v>1309.1</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -3521,10 +3541,10 @@
         <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8122685571309425</v>
+        <v>0.8243119266055046</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -3539,18 +3559,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>853.8</v>
+        <v>7673.5</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>797.86</v>
+        <v>7248.07</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -3562,7 +3582,7 @@
         <v>6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.818281901584654</v>
+        <v>0.818104670558799</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -3577,18 +3597,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>326.6</v>
+        <v>1393</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>310.44</v>
+        <v>1330.14</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -3597,10 +3617,10 @@
         <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8014512093411177</v>
+        <v>0.7574270225187657</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -3615,18 +3635,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1353.4</v>
+        <v>1564.2</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1288.41</v>
+        <v>1496.09</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -3635,10 +3655,10 @@
         <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.8078440366972477</v>
+        <v>0.7657756463719767</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3653,7 +3673,7 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
@@ -3661,10 +3681,10 @@
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1250.5</v>
+        <v>1240.3</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1175.64</v>
+        <v>1163.73</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -3673,10 +3693,10 @@
         <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.8031588824020016</v>
+        <v>0.7943160967472894</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3691,18 +3711,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1943</v>
+        <v>8935</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1876.67</v>
+        <v>8421.639999999999</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -3711,10 +3731,10 @@
         <v>5333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7778231859883237</v>
+        <v>0.7381463719766471</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3729,18 +3749,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1608.6</v>
+        <v>719.75</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1543.36</v>
+        <v>681.84</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -3749,10 +3769,10 @@
         <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7746497080900752</v>
+        <v>0.7422393661384488</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3767,18 +3787,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1819.4</v>
+        <v>586.05</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1751.19</v>
+        <v>549.63</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -3787,10 +3807,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.8</v>
+        <v>5.5</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7544787322768974</v>
+        <v>0.7647810675562969</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3805,18 +3825,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1489.9</v>
+        <v>853.2</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1414.13</v>
+        <v>822.04</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -3825,10 +3845,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7853336113427856</v>
+        <v>0.7169328607172645</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3843,18 +3863,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>CAPLIPOINT</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>2480.6</v>
+        <v>8862</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>2283.19</v>
+        <v>8593.639999999999</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -3863,10 +3883,10 @@
         <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7533236030025021</v>
+        <v>0.7132276897414511</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3881,18 +3901,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1577.8</v>
+        <v>2175.3</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1498.01</v>
+        <v>2070.47</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -3901,10 +3921,10 @@
         <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.736743119266055</v>
+        <v>0.7166722268557132</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3919,18 +3939,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1415.1</v>
+        <v>1466.1</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1358.21</v>
+        <v>1388.4</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -3939,10 +3959,10 @@
         <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7360425354462051</v>
+        <v>0.7555921601334445</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3957,18 +3977,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260722</v>
+        <v>20260723</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>2185.5</v>
+        <v>6130</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>2081.01</v>
+        <v>5799.29</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -3977,10 +3997,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.6</v>
+        <v>5.3</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7346267723102585</v>
+        <v>0.7091763969974979</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-24
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Thu 23 Jul 2026</t>
+          <t>As of Fri 24 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹202,796</t>
+          <t>₹202,256</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-1,369  (-0.67%)</t>
+          <t>₹-540  (-0.27%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.40%</t>
+          <t>+1.13%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.60%</t>
+          <t>-1.86%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹100,356</t>
+          <t>₹155,539</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹99,468</t>
+          <t>₹46,986</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹102,440</t>
+          <t>₹46,717</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹-176</t>
+          <t>₹+2,525</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -778,581 +778,293 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C2" s="7" t="n">
-        <v>420.3</v>
+        <v>7579.5</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E2" s="9" t="n">
-        <v>9246.6</v>
+        <v>7579.5</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>445.45</v>
+        <v>7520</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>9799.9</v>
+        <v>7520</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>553.2999999999995</v>
+        <v>-59.5</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.05983821080180818</v>
+        <v>-0.007850122039712382</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>386.74</v>
+        <v>7128.14</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>430.3857142857142</v>
+        <v>7289</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.03381812933951228</v>
+        <v>0.03071808510638298</v>
       </c>
       <c r="M2" s="13" t="n">
-        <v>16.71</v>
+        <v>209.96</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>1465</v>
+        <v>1798.5</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>8790</v>
+        <v>8992.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1612.8</v>
+        <v>1762.7</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9676.799999999999</v>
+        <v>8813.5</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>886.7999999999997</v>
+        <v>-178.9999999999998</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.1008873720136518</v>
+        <v>-0.01990547678621071</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>1365.41</v>
+        <v>1680.3</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>1506.7</v>
+        <v>1723.75</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.06578621031746026</v>
+        <v>0.0220967833437342</v>
       </c>
       <c r="M3" s="13" t="n">
-        <v>45.25</v>
+        <v>50.24</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>619.25</v>
+        <v>2415.2</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>9288.75</v>
+        <v>7245.6</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>719.75</v>
+        <v>2415.2</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>10796.25</v>
+        <v>7245.599999999999</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>1507.5</v>
+        <v>0</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.1622930964876867</v>
+        <v>0</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>591.46</v>
+        <v>2335.46</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>679.6178571428571</v>
+        <v>2349.7</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.05575844787376571</v>
+        <v>0.02711990725405764</v>
       </c>
       <c r="M4" s="13" t="n">
-        <v>14</v>
+        <v>49.27</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>8700</v>
+        <v>1269</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>8700</v>
+        <v>8883</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>8862</v>
+        <v>1232.9</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>8862</v>
+        <v>8630.300000000001</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>162</v>
+        <v>-252.6999999999994</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.01862068965517241</v>
+        <v>-0.02844759653270285</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>8339.209999999999</v>
+        <v>1182.49</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>8535.464285714286</v>
+        <v>1191.1</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.03684672921301216</v>
+        <v>0.03390380403925718</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>123.68</v>
+        <v>39.97</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>7579.5</v>
+        <v>8847</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>7579.5</v>
+        <v>8847</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>7673.5</v>
+        <v>8907.5</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>7673.5</v>
+        <v>8907.5</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>94</v>
+        <v>60.5</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.0124018734745036</v>
+        <v>0.006838476319656381</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>7128.14</v>
+        <v>8315.07</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>7289</v>
+        <v>8791</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.05010751286896462</v>
+        <v>0.01307886612405276</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>209.96</v>
+        <v>254.57</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>1798.5</v>
+        <v>5438</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>8992.5</v>
+        <v>5438</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1771.2</v>
+        <v>5600.5</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>8856</v>
+        <v>5600.5</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-136.4999999999998</v>
+        <v>162.5</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.01517931609674726</v>
+        <v>0.02988230967267378</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>1680.3</v>
+        <v>5157.93</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1722.657142857143</v>
+        <v>5381</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.02740676216285988</v>
+        <v>0.03919292920274976</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>50.24</v>
+        <v>143.39</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>JBCHEPHARM</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>2415.2</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E8" s="9" t="n">
-        <v>7245.6</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>2415.2</v>
-      </c>
-      <c r="G8" s="9" t="n">
-        <v>7245.599999999999</v>
-      </c>
-      <c r="H8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="7" t="n">
-        <v>2335.46</v>
-      </c>
-      <c r="K8" s="7" t="n">
-        <v>2349.7</v>
-      </c>
-      <c r="L8" s="12" t="n">
-        <v>0.02711990725405764</v>
-      </c>
-      <c r="M8" s="13" t="n">
-        <v>49.27</v>
-      </c>
-      <c r="N8" s="6" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>SAILIFE</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>1269</v>
-      </c>
-      <c r="D9" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="E9" s="9" t="n">
-        <v>8883</v>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>1240.3</v>
-      </c>
-      <c r="G9" s="9" t="n">
-        <v>8682.1</v>
-      </c>
-      <c r="H9" s="10" t="n">
-        <v>-200.9000000000003</v>
-      </c>
-      <c r="I9" s="11" t="n">
-        <v>-0.02261623325453116</v>
-      </c>
-      <c r="J9" s="7" t="n">
-        <v>1182.49</v>
-      </c>
-      <c r="K9" s="7" t="n">
-        <v>1187.221428571428</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>0.04279494592322152</v>
-      </c>
-      <c r="M9" s="13" t="n">
-        <v>39.97</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>FORTIS</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>961.85</v>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="E10" s="9" t="n">
-        <v>8656.65</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>943.65</v>
-      </c>
-      <c r="G10" s="9" t="n">
-        <v>8492.85</v>
-      </c>
-      <c r="H10" s="10" t="n">
-        <v>-163.8000000000004</v>
-      </c>
-      <c r="I10" s="11" t="n">
-        <v>-0.0189218693143422</v>
-      </c>
-      <c r="J10" s="7" t="n">
-        <v>920.8099999999999</v>
-      </c>
-      <c r="K10" s="7" t="n">
-        <v>935.6</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>0.008530705240290313</v>
-      </c>
-      <c r="M10" s="13" t="n">
-        <v>23.22</v>
-      </c>
-      <c r="N10" s="6" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>POLYCAB</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>8847</v>
-      </c>
-      <c r="D11" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="9" t="n">
-        <v>8847</v>
-      </c>
-      <c r="F11" s="7" t="n">
-        <v>8935</v>
-      </c>
-      <c r="G11" s="9" t="n">
-        <v>8935</v>
-      </c>
-      <c r="H11" s="10" t="n">
-        <v>88</v>
-      </c>
-      <c r="I11" s="11" t="n">
-        <v>0.009946874646772918</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>8315.07</v>
-      </c>
-      <c r="K11" s="7" t="n">
-        <v>8791</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>0.01611639619473979</v>
-      </c>
-      <c r="M11" s="13" t="n">
-        <v>254.57</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>PIDILITIND</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>1560</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>7800</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>1564.2</v>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>7821</v>
-      </c>
-      <c r="H12" s="10" t="n">
-        <v>21.00000000000023</v>
-      </c>
-      <c r="I12" s="11" t="n">
-        <v>0.002692307692307721</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>1504.37</v>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>1547.4</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>0.01074031453778286</v>
-      </c>
-      <c r="M12" s="13" t="n">
-        <v>30.61</v>
-      </c>
-      <c r="N12" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>CUMMINSIND</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>5438</v>
-      </c>
-      <c r="D13" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>5438</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>5599</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>5599</v>
-      </c>
-      <c r="H13" s="10" t="n">
-        <v>161</v>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>0.02960647296800294</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>5157.93</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>5381</v>
-      </c>
-      <c r="L13" s="12" t="n">
-        <v>0.03893552420075013</v>
-      </c>
-      <c r="M13" s="13" t="n">
-        <v>143.39</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H13">
+  <conditionalFormatting sqref="H2:H7">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1370,7 +1082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1446,457 +1158,457 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>900</v>
+        <v>420.3</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>887.1</v>
+        <v>448.6</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-129</v>
+        <v>622.6</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0143</v>
+        <v>0.0673</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-0.2</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>880.8</v>
+        <v>1465</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>832.9400000000001</v>
+        <v>1596.9</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-478.6</v>
+        <v>791.4</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0543</v>
+        <v>0.09</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-1</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>777</v>
+        <v>619.25</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>744.8</v>
+        <v>717.95</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-386.4</v>
+        <v>1480.5</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0414</v>
+        <v>0.1594</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-1</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>1114.9</v>
+        <v>8700</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>1050.57</v>
+        <v>8805.5</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-514.64</v>
+        <v>105.5</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.0577</v>
+        <v>0.0121</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-1</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>790</v>
+        <v>961.85</v>
       </c>
       <c r="D6" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>935.6</v>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="F6" s="15" t="n">
-        <v>880.8</v>
-      </c>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>TIME_STOP</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="n">
-        <v>25</v>
-      </c>
       <c r="I6" s="17" t="n">
-        <v>998.8</v>
+        <v>-236.25</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0273</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>1.79</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>3770</v>
+        <v>1560</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>4097.9</v>
+        <v>1547.4</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>655.8</v>
+        <v>-63</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>-0.0081</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>1.98</v>
+        <v>-0.23</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>821.05</v>
+        <v>900</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>844</v>
+        <v>887.1</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>252.45</v>
+        <v>-129</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>0.028</v>
+        <v>-0.0143</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>0.6</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>2426.1</v>
+        <v>880.8</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>2484.2</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>174.3</v>
+        <v>-478.6</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>0.0239</v>
+        <v>-0.0543</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>0.5</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1410</v>
+        <v>777</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>1455.2</v>
+        <v>744.8</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H10" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>135.6</v>
+        <v>-386.4</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>0.0321</v>
+        <v>-0.0414</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>0.46</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>690</v>
+        <v>1114.9</v>
       </c>
       <c r="D11" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="n">
+        <v>1050.57</v>
+      </c>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H11" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="E11" s="14" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="F11" s="15" t="n">
-        <v>660.45</v>
-      </c>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>TIME_STOP</t>
-        </is>
-      </c>
-      <c r="H11" s="14" t="n">
-        <v>25</v>
-      </c>
       <c r="I11" s="17" t="n">
-        <v>-206.85</v>
+        <v>-514.64</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>-0.0428</v>
+        <v>-0.0577</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>-0.38</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>1839</v>
+        <v>790</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>1828.1</v>
+        <v>880.8</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -1907,39 +1619,39 @@
         <v>25</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>-21.8</v>
+        <v>998.8</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>-0.0059</v>
+        <v>0.1149</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>-0.1</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>1414</v>
+        <v>3770</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>1537.8</v>
+        <v>4097.9</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
@@ -1950,39 +1662,39 @@
         <v>25</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>371.4</v>
+        <v>655.8</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>0.0876</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>1.38</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>1300</v>
+        <v>821.05</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>1389.1</v>
+        <v>844</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
@@ -1993,39 +1705,39 @@
         <v>25</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>356.4</v>
+        <v>252.45</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>0.028</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>0.63</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>276.45</v>
+        <v>2426.1</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>330.1</v>
+        <v>2484.2</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
@@ -2036,19 +1748,19 @@
         <v>25</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>1019.35</v>
+        <v>174.3</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.0239</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>3.1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -2057,7 +1769,7 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>1462.5</v>
+        <v>1410</v>
       </c>
       <c r="D16" s="16" t="n">
         <v>3</v>
@@ -2068,7 +1780,7 @@
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>1564.7</v>
+        <v>1455.2</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
@@ -2079,19 +1791,19 @@
         <v>25</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>306.6</v>
+        <v>135.6</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.0321</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>1.78</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -2100,41 +1812,41 @@
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>798</v>
+        <v>690</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>750</v>
+        <v>660.45</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H17" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>-288</v>
+        <v>-206.85</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>-0.0602</v>
+        <v>-0.0428</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>-0.92</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -2143,233 +1855,233 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>260.45</v>
+        <v>1839</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>257.85</v>
+        <v>1828.1</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H18" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>-52.07</v>
+        <v>-21.8</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0059</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>-0.13</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>6500</v>
+        <v>1414</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>6401.5</v>
+        <v>1537.8</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H19" s="14" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>-98.5</v>
+        <v>371.4</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>-0.0152</v>
+        <v>0.0876</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>-0.31</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>571.5</v>
+        <v>1300</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>571.1</v>
+        <v>1389.1</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H20" s="14" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>-6.4</v>
+        <v>356.4</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>-0.0007</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>-0.01</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>965</v>
+        <v>276.45</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>933</v>
+        <v>330.1</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H21" s="14" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>-288</v>
+        <v>1019.35</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>-0.0332</v>
+        <v>0.1941</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>-0.57</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>5479</v>
+        <v>1462.5</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>5424</v>
+        <v>1564.7</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H22" s="14" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>-55</v>
+        <v>306.6</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>-0.01</v>
+        <v>0.0699</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>-0.18</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>960.1</v>
+        <v>798</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>750</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -2377,42 +2089,42 @@
         </is>
       </c>
       <c r="H23" s="14" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>-516.79</v>
+        <v>-288</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.0602</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>952.1</v>
+        <v>260.45</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>948.8</v>
+        <v>257.85</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -2420,22 +2132,22 @@
         </is>
       </c>
       <c r="H24" s="14" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>-29.7</v>
+        <v>-52.07</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.01</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -2444,18 +2156,18 @@
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>1475</v>
+        <v>6500</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>1394.19</v>
+        <v>6401.5</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -2463,42 +2175,42 @@
         </is>
       </c>
       <c r="H25" s="14" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>-484.86</v>
+        <v>-98.5</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0152</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>-1</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>248.05</v>
+        <v>571.5</v>
       </c>
       <c r="D26" s="16" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>242.8</v>
+        <v>571.1</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
@@ -2506,42 +2218,42 @@
         </is>
       </c>
       <c r="H26" s="14" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="I26" s="17" t="n">
-        <v>-110.25</v>
+        <v>-6.4</v>
       </c>
       <c r="J26" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0007</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>-0.3</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>1039.2</v>
+        <v>965</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>970</v>
+        <v>933</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
@@ -2549,42 +2261,42 @@
         </is>
       </c>
       <c r="H27" s="14" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>-346</v>
+        <v>-288</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0332</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>199.96</v>
+        <v>5479</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>193.31</v>
+        <v>5424</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
@@ -2592,63 +2304,321 @@
         </is>
       </c>
       <c r="H28" s="14" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I28" s="17" t="n">
-        <v>-172.9</v>
+        <v>-55</v>
       </c>
       <c r="J28" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.01</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>960.1</v>
+      </c>
+      <c r="D29" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F29" s="15" t="n">
+        <v>902.6799999999999</v>
+      </c>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H29" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I29" s="17" t="n">
+        <v>-516.79</v>
+      </c>
+      <c r="J29" s="18" t="n">
+        <v>-0.0598</v>
+      </c>
+      <c r="K29" s="19" t="n">
+        <v>-0.87</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="n">
+        <v>952.1</v>
+      </c>
+      <c r="D30" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F30" s="15" t="n">
+        <v>948.8</v>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H30" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" s="17" t="n">
+        <v>-29.7</v>
+      </c>
+      <c r="J30" s="18" t="n">
+        <v>-0.0035</v>
+      </c>
+      <c r="K30" s="19" t="n">
+        <v>-0.06</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>RAINBOW</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="n">
+        <v>1475</v>
+      </c>
+      <c r="D31" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="F31" s="15" t="n">
+        <v>1394.19</v>
+      </c>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H31" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="I31" s="17" t="n">
+        <v>-484.86</v>
+      </c>
+      <c r="J31" s="18" t="n">
+        <v>-0.0548</v>
+      </c>
+      <c r="K31" s="19" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="n">
+        <v>248.05</v>
+      </c>
+      <c r="D32" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F32" s="15" t="n">
+        <v>242.8</v>
+      </c>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H32" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I32" s="17" t="n">
+        <v>-110.25</v>
+      </c>
+      <c r="J32" s="18" t="n">
+        <v>-0.0212</v>
+      </c>
+      <c r="K32" s="19" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="n">
+        <v>1039.2</v>
+      </c>
+      <c r="D33" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F33" s="15" t="n">
+        <v>970</v>
+      </c>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H33" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I33" s="17" t="n">
+        <v>-346</v>
+      </c>
+      <c r="J33" s="18" t="n">
+        <v>-0.06660000000000001</v>
+      </c>
+      <c r="K33" s="19" t="n">
+        <v>-0.82</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="n">
+        <v>199.96</v>
+      </c>
+      <c r="D34" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="E34" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F34" s="15" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="G34" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H34" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I34" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J34" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K34" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
           <t>SHYAMMETL</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="C29" s="15" t="n">
+      <c r="C35" s="15" t="n">
         <v>986.4</v>
       </c>
-      <c r="D29" s="16" t="n">
+      <c r="D35" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="E29" s="14" t="inlineStr">
+      <c r="E35" s="14" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="F29" s="15" t="n">
+      <c r="F35" s="15" t="n">
         <v>934.1900000000001</v>
       </c>
-      <c r="G29" s="14" t="inlineStr">
+      <c r="G35" s="14" t="inlineStr">
         <is>
           <t>STOP_LOSS</t>
         </is>
       </c>
-      <c r="H29" s="14" t="n">
+      <c r="H35" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="I29" s="17" t="n">
+      <c r="I35" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J29" s="18" t="n">
+      <c r="J35" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K29" s="19" t="n">
+      <c r="K35" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I29">
+  <conditionalFormatting sqref="I2:I35">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2666,7 +2636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3363,6 +3333,31 @@
       </c>
       <c r="G27" s="14" t="n">
         <v>12</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
+        <v>202256.44</v>
+      </c>
+      <c r="C28" s="20" t="n">
+        <v>155539.04</v>
+      </c>
+      <c r="D28" s="20" t="n">
+        <v>46717.4</v>
+      </c>
+      <c r="E28" s="20" t="n">
+        <v>46985.6</v>
+      </c>
+      <c r="F28" s="20" t="n">
+        <v>2524.64</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -3445,18 +3440,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1954</v>
+        <v>1601.2</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1890.87</v>
+        <v>1520.16</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -3465,10 +3460,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8119140950792326</v>
+        <v>0.8220482713633399</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -3483,18 +3478,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1778.5</v>
+        <v>1570.9</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1705.94</v>
+        <v>1499.44</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -3503,10 +3498,10 @@
         <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.804034612176814</v>
+        <v>0.7981082844096543</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -3521,18 +3516,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1378.2</v>
+        <v>867.7</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1309.1</v>
+        <v>814.9</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -3541,10 +3536,10 @@
         <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8243119266055046</v>
+        <v>0.7626696546935169</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -3559,18 +3554,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>7673.5</v>
+        <v>8805.5</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>7248.07</v>
+        <v>8540.639999999999</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -3579,10 +3574,10 @@
         <v>5333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.818104670558799</v>
+        <v>0.7742966563558699</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -3597,18 +3592,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1393</v>
+        <v>1768.3</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1330.14</v>
+        <v>1694.96</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -3617,10 +3612,10 @@
         <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7574270225187657</v>
+        <v>0.7615954379984429</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -3635,18 +3630,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1564.2</v>
+        <v>1410.6</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1496.09</v>
+        <v>1342.97</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -3655,10 +3650,10 @@
         <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7657756463719767</v>
+        <v>0.7423552806009722</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3673,18 +3668,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1240.3</v>
+        <v>1941.1</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1163.73</v>
+        <v>1876.83</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -3693,10 +3688,10 @@
         <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7943160967472894</v>
+        <v>0.7468857184942028</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3711,18 +3706,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>8935</v>
+        <v>717.95</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>8421.639999999999</v>
+        <v>676.71</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -3734,7 +3729,7 @@
         <v>5.7</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7381463719766471</v>
+        <v>0.7283883593207499</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3749,18 +3744,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>719.75</v>
+        <v>6407.5</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>681.84</v>
+        <v>6031.93</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -3772,7 +3767,7 @@
         <v>5.7</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7422393661384488</v>
+        <v>0.7375986364497191</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3787,18 +3782,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>APARINDS</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>586.05</v>
+        <v>13889</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>549.63</v>
+        <v>12710.43</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -3807,10 +3802,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7647810675562969</v>
+        <v>0.7303547755823496</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3825,18 +3820,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>853.2</v>
+        <v>1232.9</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>822.04</v>
+        <v>1157.97</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -3845,10 +3840,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7169328607172645</v>
+        <v>0.7616932853565641</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3863,18 +3858,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>8862</v>
+        <v>4091.3</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>8593.639999999999</v>
+        <v>3924.44</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -3883,10 +3878,10 @@
         <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7132276897414511</v>
+        <v>0.746445931443722</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3901,18 +3896,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>2175.3</v>
+        <v>855.6</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>2070.47</v>
+        <v>823.7</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -3924,7 +3919,7 @@
         <v>5.5</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7166722268557132</v>
+        <v>0.7241041180060181</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3939,7 +3934,7 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
@@ -3947,10 +3942,10 @@
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1466.1</v>
+        <v>1457.8</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1388.4</v>
+        <v>1376.6</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -3962,7 +3957,7 @@
         <v>5.4</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7555921601334445</v>
+        <v>0.7657229131157544</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3977,18 +3972,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260723</v>
+        <v>20260724</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>6130</v>
+        <v>1371</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>5799.29</v>
+        <v>1302.41</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -3997,10 +3992,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7091763969974979</v>
+        <v>0.7379111167224292</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-27
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Fri 24 Jul 2026</t>
+          <t>As of Mon 27 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹202,256</t>
+          <t>₹203,366</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-540  (-0.27%)</t>
+          <t>₹+1,109  (+0.55%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.13%</t>
+          <t>+1.68%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.86%</t>
+          <t>-1.33%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹155,539</t>
+          <t>₹114,571</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹46,986</t>
+          <t>₹87,954</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹46,717</t>
+          <t>₹88,795</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -796,16 +796,16 @@
         <v>7579.5</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>7520</v>
+        <v>7711</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>7520</v>
+        <v>7711</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>-59.5</v>
+        <v>131.5</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>-0.007850122039712382</v>
+        <v>0.01734942938188535</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>7128.14</v>
@@ -814,13 +814,13 @@
         <v>7289</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.03071808510638298</v>
+        <v>0.05472701335754118</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>209.96</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8992.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1762.7</v>
+        <v>1777.6</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8813.5</v>
+        <v>8888</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-178.9999999999998</v>
+        <v>-104.5000000000005</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.01990547678621071</v>
+        <v>-0.01162079510703369</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1680.3</v>
@@ -862,13 +862,13 @@
         <v>1723.75</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.0220967833437342</v>
+        <v>0.03029365436543662</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>50.24</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -916,7 +916,7 @@
         <v>49.27</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>8883</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1232.9</v>
+        <v>1287</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>8630.300000000001</v>
+        <v>9009</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>-252.6999999999994</v>
+        <v>126</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>-0.02844759653270285</v>
+        <v>0.01418439716312057</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1182.49</v>
@@ -958,13 +958,13 @@
         <v>1191.1</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.03390380403925718</v>
+        <v>0.07451437451437458</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>39.97</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>8847</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>8907.5</v>
+        <v>9010</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>8907.5</v>
+        <v>9010</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>60.5</v>
+        <v>163</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.006838476319656381</v>
+        <v>0.01842432462981802</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>8315.07</v>
@@ -1006,13 +1006,13 @@
         <v>8791</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.01307886612405276</v>
+        <v>0.02430632630410655</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>254.57</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>5438</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>5600.5</v>
+        <v>5629.5</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>5600.5</v>
+        <v>5629.5</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>162.5</v>
+        <v>191.5</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.02988230967267378</v>
+        <v>0.03521515262964325</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>5157.93</v>
@@ -1054,17 +1054,449 @@
         <v>5381</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.03919292920274976</v>
+        <v>0.04414246380673239</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>143.39</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>LAURUSLABS</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>1624.8</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>4874.4</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>1713.4</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>5140.200000000001</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>265.8000000000004</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>0.05452978828163475</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>1520.16</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>1520.16</v>
+      </c>
+      <c r="L8" s="12" t="n">
+        <v>0.1127816038286448</v>
+      </c>
+      <c r="M8" s="13" t="n">
+        <v>45.45</v>
+      </c>
+      <c r="N8" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>1588.9</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>4766.7</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>1611.3</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>4833.9</v>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>67.19999999999959</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>0.01409780351186347</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>1499.44</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>1499.44</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>0.06942220567243834</v>
+      </c>
+      <c r="M9" s="13" t="n">
+        <v>37.96</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>871.8</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>5230.8</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>877.3</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>5263.799999999999</v>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>0.006308786418903418</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>814.9</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>814.9</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>0.07112732246665905</v>
+      </c>
+      <c r="M10" s="13" t="n">
+        <v>25.57</v>
+      </c>
+      <c r="N10" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>1784</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>3568</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>1770.4</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>3540.8</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>-27.19999999999982</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>-0.007623318385650173</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>1694.96</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>1694.96</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>0.04261183913239949</v>
+      </c>
+      <c r="M11" s="13" t="n">
+        <v>35.32</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>1412.6</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>4237.8</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>1409.4</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>4228.200000000001</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>-9.599999999999454</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>-0.002265326348576963</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>1342.97</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>1342.97</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>0.04713353199943243</v>
+      </c>
+      <c r="M12" s="13" t="n">
+        <v>33.28</v>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>1948.5</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>3897</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>1973.7</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>3947.4</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>50.40000000000009</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0.01293302540415707</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>1876.83</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>1876.83</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>0.04908040735674121</v>
+      </c>
+      <c r="M13" s="13" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>SONACOMS</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>728.8</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>5101.6</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>720.9</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>5046.3</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>-55.29999999999984</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>-0.01083973655323817</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>676.71</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>676.71</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>0.06129837702871403</v>
+      </c>
+      <c r="M14" s="13" t="n">
+        <v>20.64</v>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>RADICO</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>4120</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>4120</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>4149.5</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>4149.5</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>0.007160194174757281</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>3924.44</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>3924.44</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>0.05423785998313049</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>85.14</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>MARICO</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>862</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>5172</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>858.65</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>5151.9</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>-20.10000000000014</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>-0.003886310904872416</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>823.7</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>823.7</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0.04070342980259702</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>15.94</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H7">
+  <conditionalFormatting sqref="H2:H16">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2636,7 +3068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3358,6 +3790,31 @@
       </c>
       <c r="G28" s="14" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>203365.84</v>
+      </c>
+      <c r="C29" s="20" t="n">
+        <v>114570.74</v>
+      </c>
+      <c r="D29" s="20" t="n">
+        <v>88795.10000000001</v>
+      </c>
+      <c r="E29" s="20" t="n">
+        <v>87953.89999999999</v>
+      </c>
+      <c r="F29" s="20" t="n">
+        <v>2524.64</v>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -3440,7 +3897,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -3448,10 +3905,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1601.2</v>
+        <v>1713.4</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1520.16</v>
+        <v>1622.5</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -3460,10 +3917,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8220482713633399</v>
+        <v>0.8545840961218778</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -3478,18 +3935,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1570.9</v>
+        <v>1973.7</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1499.44</v>
+        <v>1906.9</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -3498,10 +3955,10 @@
         <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.7981082844096543</v>
+        <v>0.795059234475938</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -3516,18 +3973,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>867.7</v>
+        <v>1287</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>814.9</v>
+        <v>1211.93</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -3536,10 +3993,10 @@
         <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7626696546935169</v>
+        <v>0.8276855417376849</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -3554,18 +4011,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>8805.5</v>
+        <v>1407.2</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>8540.639999999999</v>
+        <v>1339.17</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -3574,10 +4031,10 @@
         <v>5333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7742966563558699</v>
+        <v>0.8124139890158449</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -3592,7 +4049,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
@@ -3600,10 +4057,10 @@
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1768.3</v>
+        <v>1770.4</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1694.96</v>
+        <v>1699.76</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -3612,10 +4069,10 @@
         <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7615954379984429</v>
+        <v>0.7697830524167245</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -3630,18 +4087,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1410.6</v>
+        <v>1611.3</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1342.97</v>
+        <v>1535.39</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -3650,10 +4107,10 @@
         <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7423552806009722</v>
+        <v>0.7785156660985207</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -3668,18 +4125,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1941.1</v>
+        <v>7711</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1876.83</v>
+        <v>7290.14</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -3688,10 +4145,10 @@
         <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7468857184942028</v>
+        <v>0.7814374092544663</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -3706,18 +4163,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>717.95</v>
+        <v>1549.4</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>676.71</v>
+        <v>1473.29</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -3726,10 +4183,10 @@
         <v>5333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7283883593207499</v>
+        <v>0.7747459125055236</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -3744,18 +4201,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>6407.5</v>
+        <v>7414</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>6031.93</v>
+        <v>7092.29</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -3764,10 +4221,10 @@
         <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7375986364497191</v>
+        <v>0.7520106053910738</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -3782,18 +4239,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>APARINDS</t>
+          <t>CAPLIPOINT</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>13889</v>
+        <v>2621.4</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>12710.43</v>
+        <v>2419.96</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -3805,7 +4262,7 @@
         <v>5.7</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7303547755823496</v>
+        <v>0.7618584685310271</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -3820,18 +4277,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1232.9</v>
+        <v>4149.5</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1157.97</v>
+        <v>3979.23</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -3840,10 +4297,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7616932853565641</v>
+        <v>0.7499831660459146</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -3858,18 +4315,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>4091.3</v>
+        <v>2181.3</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>3924.44</v>
+        <v>2077.16</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -3878,10 +4335,10 @@
         <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.746445931443722</v>
+        <v>0.747351808597942</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -3896,18 +4353,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>855.6</v>
+        <v>452.75</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>823.7</v>
+        <v>422.64</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -3916,10 +4373,10 @@
         <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7241041180060181</v>
+        <v>0.7614860172968878</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -3934,18 +4391,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1457.8</v>
+        <v>1114.6</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1376.6</v>
+        <v>1061.64</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -3954,10 +4411,10 @@
         <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7657229131157544</v>
+        <v>0.7328430444205963</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -3972,18 +4429,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260724</v>
+        <v>20260727</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1371</v>
+        <v>1483.5</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1302.41</v>
+        <v>1403.6</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -3992,10 +4449,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7379111167224292</v>
+        <v>0.7271384382299098</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-28
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Mon 27 Jul 2026</t>
+          <t>As of Tue 28 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹203,366</t>
+          <t>₹203,488</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+1,109  (+0.55%)</t>
+          <t>₹+122  (+0.06%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.68%</t>
+          <t>+1.74%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.33%</t>
+          <t>-1.27%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹114,571</t>
+          <t>₹119,552</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹87,954</t>
+          <t>₹82,723</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹88,795</t>
+          <t>₹83,936</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+2,525</t>
+          <t>₹+2,275</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -796,16 +796,16 @@
         <v>7579.5</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>7711</v>
+        <v>7512.5</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>7711</v>
+        <v>7512.5</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>131.5</v>
+        <v>-67</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.01734942938188535</v>
+        <v>-0.008839633221188734</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>7128.14</v>
@@ -814,13 +814,13 @@
         <v>7289</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.05472701335754118</v>
+        <v>0.0297504159733777</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>209.96</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8992.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1777.6</v>
+        <v>1789</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8888</v>
+        <v>8945</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-104.5000000000005</v>
+        <v>-47.5</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.01162079510703369</v>
+        <v>-0.0052821795941062</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1680.3</v>
@@ -862,13 +862,13 @@
         <v>1723.75</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.03029365436543662</v>
+        <v>0.03647288988261611</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>50.24</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -916,7 +916,7 @@
         <v>49.27</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>8883</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1287</v>
+        <v>1300.5</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9009</v>
+        <v>9103.5</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>126</v>
+        <v>220.5</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.01418439716312057</v>
+        <v>0.02482269503546099</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1182.49</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1191.1</v>
+        <v>1191.342857142857</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.07451437451437458</v>
+        <v>0.08393475037073651</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>39.97</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>8847</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>9010</v>
+        <v>9121.5</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9010</v>
+        <v>9121.5</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>163</v>
+        <v>274.5</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.01842432462981802</v>
+        <v>0.03102746693794507</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>8315.07</v>
@@ -1006,13 +1006,13 @@
         <v>8791</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.02430632630410655</v>
+        <v>0.0362330757002686</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>254.57</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>5438</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>5629.5</v>
+        <v>5455.5</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>5629.5</v>
+        <v>5455.5</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>191.5</v>
+        <v>17.5</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.03521515262964325</v>
+        <v>0.003218094887826407</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>5157.93</v>
@@ -1054,13 +1054,13 @@
         <v>5381</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.04414246380673239</v>
+        <v>0.01365594354321327</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>143.39</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -1084,31 +1084,31 @@
         <v>4874.4</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1713.4</v>
+        <v>1758.9</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5140.200000000001</v>
+        <v>5276.700000000001</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>265.8000000000004</v>
+        <v>402.3000000000004</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.05452978828163475</v>
+        <v>0.08253323485967512</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1520.16</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>1520.16</v>
+        <v>1620.964285714286</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.1127816038286448</v>
+        <v>0.07842157842157843</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>45.45</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1132,37 +1132,37 @@
         <v>4766.7</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1611.3</v>
+        <v>1619.6</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4833.9</v>
+        <v>4858.799999999999</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>67.19999999999959</v>
+        <v>92.09999999999945</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.01409780351186347</v>
+        <v>0.01932154320599145</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1499.44</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>1499.44</v>
+        <v>1537.1</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.06942220567243834</v>
+        <v>0.05093850333415659</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>37.96</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1171,46 +1171,46 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>871.8</v>
+        <v>1784</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>5230.8</v>
+        <v>3568</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>877.3</v>
+        <v>1774.7</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>5263.799999999999</v>
+        <v>3549.4</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>33</v>
+        <v>-18.59999999999991</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.006308786418903418</v>
+        <v>-0.005213004484304907</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>814.9</v>
+        <v>1694.96</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>814.9</v>
+        <v>1752.1</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.07112732246665905</v>
+        <v>0.01273454668394666</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>25.57</v>
+        <v>35.32</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -1219,46 +1219,46 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>1784</v>
+        <v>1412.6</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>3568</v>
+        <v>4237.8</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>1770.4</v>
+        <v>1444.6</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>3540.8</v>
+        <v>4333.799999999999</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-27.19999999999982</v>
+        <v>96</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>-0.007623318385650173</v>
+        <v>0.02265326348577092</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>1694.96</v>
+        <v>1342.97</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>1694.96</v>
+        <v>1366.1</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.04261183913239949</v>
+        <v>0.05434030181365084</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>35.32</v>
+        <v>33.28</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1267,46 +1267,46 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>1412.6</v>
+        <v>1948.5</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>4237.8</v>
+        <v>3897</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>1409.4</v>
+        <v>1976.7</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4228.200000000001</v>
+        <v>3953.4</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-9.599999999999454</v>
+        <v>56.40000000000009</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.002265326348576963</v>
+        <v>0.01447267128560433</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>1342.97</v>
+        <v>1876.83</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>1342.97</v>
+        <v>1883.421428571429</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.04713353199943243</v>
+        <v>0.04718903800706796</v>
       </c>
       <c r="M12" s="13" t="n">
-        <v>33.28</v>
+        <v>33.4</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -1315,46 +1315,46 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>1948.5</v>
+        <v>728.8</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>3897</v>
+        <v>5101.6</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1973.7</v>
+        <v>713</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>3947.4</v>
+        <v>4991</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>50.40000000000009</v>
+        <v>-110.5999999999997</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.01293302540415707</v>
+        <v>-0.02167947310647634</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>1876.83</v>
+        <v>676.71</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>1876.83</v>
+        <v>676.71</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.04908040735674121</v>
+        <v>0.05089761570827484</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>33.4</v>
+        <v>20.64</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1363,46 +1363,46 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>728.8</v>
+        <v>4120</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>5101.6</v>
+        <v>4120</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>720.9</v>
+        <v>4289.7</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>5046.3</v>
+        <v>4289.7</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>-55.29999999999984</v>
+        <v>169.6999999999998</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>-0.01083973655323817</v>
+        <v>0.04118932038834947</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>676.71</v>
+        <v>3924.44</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>676.71</v>
+        <v>3994.028571428572</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.06129837702871403</v>
+        <v>0.06892589891400981</v>
       </c>
       <c r="M14" s="13" t="n">
-        <v>20.64</v>
+        <v>85.14</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
@@ -1411,92 +1411,44 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>4120</v>
+        <v>862</v>
       </c>
       <c r="D15" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>5172</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>883.25</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>5299.5</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>127.5</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>0.02465197215777262</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>823.7</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>832.5392857142857</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>0.05741377218875096</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>15.94</v>
+      </c>
+      <c r="N15" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="9" t="n">
-        <v>4120</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>4149.5</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>4149.5</v>
-      </c>
-      <c r="H15" s="10" t="n">
-        <v>29.5</v>
-      </c>
-      <c r="I15" s="11" t="n">
-        <v>0.007160194174757281</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>3924.44</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>3924.44</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>0.05423785998313049</v>
-      </c>
-      <c r="M15" s="13" t="n">
-        <v>85.14</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>MARICO</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>862</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <v>5172</v>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>858.65</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>5151.9</v>
-      </c>
-      <c r="H16" s="10" t="n">
-        <v>-20.10000000000014</v>
-      </c>
-      <c r="I16" s="11" t="n">
-        <v>-0.003886310904872416</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>823.7</v>
-      </c>
-      <c r="K16" s="7" t="n">
-        <v>823.7</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>0.04070342980259702</v>
-      </c>
-      <c r="M16" s="13" t="n">
-        <v>15.94</v>
-      </c>
-      <c r="N16" s="6" t="n">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H16">
+  <conditionalFormatting sqref="H2:H15">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1514,7 +1466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1590,50 +1542,50 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>420.3</v>
+        <v>871.8</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>448.6</v>
+        <v>830.15</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>622.6</v>
+        <v>-249.9</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>0.0673</v>
+        <v>-0.0478</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>0.84</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -1642,10 +1594,10 @@
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>1465</v>
+        <v>420.3</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
@@ -1653,7 +1605,7 @@
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>1596.9</v>
+        <v>448.6</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -1664,19 +1616,19 @@
         <v>25</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>791.4</v>
+        <v>622.6</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>0.09</v>
+        <v>0.0673</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>1.32</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -1685,10 +1637,10 @@
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>619.25</v>
+        <v>1465</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
@@ -1696,7 +1648,7 @@
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>717.95</v>
+        <v>1596.9</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1707,19 +1659,19 @@
         <v>25</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>1480.5</v>
+        <v>791.4</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>0.1594</v>
+        <v>0.09</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>3.55</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -1728,10 +1680,10 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>8700</v>
+        <v>619.25</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
@@ -1739,7 +1691,7 @@
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>8805.5</v>
+        <v>717.95</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1750,31 +1702,31 @@
         <v>25</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>105.5</v>
+        <v>1480.5</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>0.0121</v>
+        <v>0.1594</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>0.29</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>961.85</v>
+        <v>8700</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -1782,42 +1734,42 @@
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>935.6</v>
+        <v>8805.5</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>-236.25</v>
+        <v>105.5</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>-0.0273</v>
+        <v>0.0121</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>-0.64</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>1560</v>
+        <v>961.85</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
@@ -1825,7 +1777,7 @@
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>1547.4</v>
+        <v>935.6</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -1833,42 +1785,42 @@
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>-63</v>
+        <v>-236.25</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>-0.0081</v>
+        <v>-0.0273</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>-0.23</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>900</v>
+        <v>1560</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>887.1</v>
+        <v>1547.4</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -1876,42 +1828,42 @@
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>-129</v>
+        <v>-63</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>-0.0143</v>
+        <v>-0.0081</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.23</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>880.8</v>
+        <v>900</v>
       </c>
       <c r="D9" s="16" t="n">
         <v>10</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>832.9400000000001</v>
+        <v>887.1</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
@@ -1919,22 +1871,22 @@
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>-478.6</v>
+        <v>-129</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>-0.0543</v>
+        <v>-0.0143</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>-1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -1943,10 +1895,10 @@
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>777</v>
+        <v>880.8</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
@@ -1954,7 +1906,7 @@
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>744.8</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
@@ -1965,10 +1917,10 @@
         <v>2</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>-386.4</v>
+        <v>-478.6</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>-0.0414</v>
+        <v>-0.0543</v>
       </c>
       <c r="K10" s="19" t="n">
         <v>-1</v>
@@ -1977,27 +1929,27 @@
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>1114.9</v>
+        <v>777</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>1050.57</v>
+        <v>744.8</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
@@ -2005,13 +1957,13 @@
         </is>
       </c>
       <c r="H11" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>-514.64</v>
+        <v>-386.4</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>-0.0577</v>
+        <v>-0.0414</v>
       </c>
       <c r="K11" s="19" t="n">
         <v>-1</v>
@@ -2020,50 +1972,50 @@
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>790</v>
+        <v>1114.9</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>880.8</v>
+        <v>1050.57</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H12" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>998.8</v>
+        <v>-514.64</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0577</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -2072,10 +2024,10 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>3770</v>
+        <v>790</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
@@ -2083,7 +2035,7 @@
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>4097.9</v>
+        <v>880.8</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
@@ -2094,19 +2046,19 @@
         <v>25</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>655.8</v>
+        <v>998.8</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.1149</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>1.98</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -2115,10 +2067,10 @@
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>821.05</v>
+        <v>3770</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
@@ -2126,7 +2078,7 @@
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>844</v>
+        <v>4097.9</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
@@ -2137,19 +2089,19 @@
         <v>25</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>252.45</v>
+        <v>655.8</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>0.028</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>0.6</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -2158,10 +2110,10 @@
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>2426.1</v>
+        <v>821.05</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
@@ -2169,7 +2121,7 @@
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>2484.2</v>
+        <v>844</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
@@ -2180,39 +2132,39 @@
         <v>25</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>174.3</v>
+        <v>252.45</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.028</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>1410</v>
+        <v>2426.1</v>
       </c>
       <c r="D16" s="16" t="n">
         <v>3</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>1455.2</v>
+        <v>2484.2</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
@@ -2223,19 +2175,19 @@
         <v>25</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>135.6</v>
+        <v>174.3</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.0239</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>0.46</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -2244,10 +2196,10 @@
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>690</v>
+        <v>1410</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
@@ -2255,7 +2207,7 @@
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>660.45</v>
+        <v>1455.2</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -2266,19 +2218,19 @@
         <v>25</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>-206.85</v>
+        <v>135.6</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.0321</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -2287,10 +2239,10 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>1839</v>
+        <v>690</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
@@ -2298,7 +2250,7 @@
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>1828.1</v>
+        <v>660.45</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -2309,19 +2261,19 @@
         <v>25</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>-21.8</v>
+        <v>-206.85</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>-0.0059</v>
+        <v>-0.0428</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>-0.1</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -2330,10 +2282,10 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>1414</v>
+        <v>1839</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
@@ -2341,7 +2293,7 @@
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>1537.8</v>
+        <v>1828.1</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
@@ -2352,19 +2304,19 @@
         <v>25</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>371.4</v>
+        <v>-21.8</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>0.0876</v>
+        <v>-0.0059</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>1.38</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -2373,10 +2325,10 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>1300</v>
+        <v>1414</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
@@ -2384,7 +2336,7 @@
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>1389.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -2395,19 +2347,19 @@
         <v>25</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>356.4</v>
+        <v>371.4</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>0.0876</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>0.63</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -2416,10 +2368,10 @@
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>276.45</v>
+        <v>1300</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
@@ -2427,7 +2379,7 @@
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>330.1</v>
+        <v>1389.1</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -2438,19 +2390,19 @@
         <v>25</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>1019.35</v>
+        <v>356.4</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>3.1</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
@@ -2459,10 +2411,10 @@
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>1462.5</v>
+        <v>276.45</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
@@ -2470,7 +2422,7 @@
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>1564.7</v>
+        <v>330.1</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -2481,19 +2433,19 @@
         <v>25</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>306.6</v>
+        <v>1019.35</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.1941</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>1.78</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
@@ -2502,41 +2454,41 @@
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>798</v>
+        <v>1462.5</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>750</v>
+        <v>1564.7</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H23" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>-288</v>
+        <v>306.6</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.0699</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>-0.92</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -2545,10 +2497,10 @@
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>260.45</v>
+        <v>798</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
@@ -2556,7 +2508,7 @@
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>257.85</v>
+        <v>750</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -2567,31 +2519,31 @@
         <v>23</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>-52.07</v>
+        <v>-288</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0602</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>-0.13</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>6500</v>
+        <v>260.45</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
@@ -2599,7 +2551,7 @@
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>6401.5</v>
+        <v>257.85</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -2607,65 +2559,65 @@
         </is>
       </c>
       <c r="H25" s="14" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>-98.5</v>
+        <v>-52.07</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.01</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>571.5</v>
+        <v>6500</v>
       </c>
       <c r="D26" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>6401.5</v>
+      </c>
+      <c r="G26" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H26" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="E26" s="14" t="inlineStr">
-        <is>
-          <t>2026-07-08</t>
-        </is>
-      </c>
-      <c r="F26" s="15" t="n">
-        <v>571.1</v>
-      </c>
-      <c r="G26" s="14" t="inlineStr">
-        <is>
-          <t>STOP_LOSS</t>
-        </is>
-      </c>
-      <c r="H26" s="14" t="n">
-        <v>2</v>
-      </c>
       <c r="I26" s="17" t="n">
-        <v>-6.4</v>
+        <v>-98.5</v>
       </c>
       <c r="J26" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.0152</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
@@ -2674,10 +2626,10 @@
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>965</v>
+        <v>571.5</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
@@ -2685,7 +2637,7 @@
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>933</v>
+        <v>571.1</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
@@ -2696,19 +2648,19 @@
         <v>2</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>-288</v>
+        <v>-6.4</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0007</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
@@ -2717,18 +2669,18 @@
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>5479</v>
+        <v>965</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>5424</v>
+        <v>933</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
@@ -2736,42 +2688,42 @@
         </is>
       </c>
       <c r="H28" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I28" s="17" t="n">
-        <v>-55</v>
+        <v>-288</v>
       </c>
       <c r="J28" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0332</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>-0.18</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>960.1</v>
+        <v>5479</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F29" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>5424</v>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
@@ -2779,22 +2731,22 @@
         </is>
       </c>
       <c r="H29" s="14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I29" s="17" t="n">
-        <v>-516.79</v>
+        <v>-55</v>
       </c>
       <c r="J29" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.01</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
@@ -2803,18 +2755,18 @@
         </is>
       </c>
       <c r="C30" s="15" t="n">
-        <v>952.1</v>
+        <v>960.1</v>
       </c>
       <c r="D30" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F30" s="15" t="n">
-        <v>948.8</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
@@ -2822,42 +2774,42 @@
         </is>
       </c>
       <c r="H30" s="14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I30" s="17" t="n">
-        <v>-29.7</v>
+        <v>-516.79</v>
       </c>
       <c r="J30" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.0598</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>1475</v>
+        <v>952.1</v>
       </c>
       <c r="D31" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F31" s="15" t="n">
-        <v>1394.19</v>
+        <v>948.8</v>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
@@ -2865,42 +2817,42 @@
         </is>
       </c>
       <c r="H31" s="14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I31" s="17" t="n">
-        <v>-484.86</v>
+        <v>-29.7</v>
       </c>
       <c r="J31" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0035</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>-1</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C32" s="15" t="n">
-        <v>248.05</v>
+        <v>1475</v>
       </c>
       <c r="D32" s="16" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F32" s="15" t="n">
-        <v>242.8</v>
+        <v>1394.19</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
@@ -2908,22 +2860,22 @@
         </is>
       </c>
       <c r="H32" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I32" s="17" t="n">
-        <v>-110.25</v>
+        <v>-484.86</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0548</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>-0.3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
@@ -2932,10 +2884,10 @@
         </is>
       </c>
       <c r="C33" s="15" t="n">
-        <v>1039.2</v>
+        <v>248.05</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
@@ -2943,7 +2895,7 @@
         </is>
       </c>
       <c r="F33" s="15" t="n">
-        <v>970</v>
+        <v>242.8</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
@@ -2954,19 +2906,19 @@
         <v>11</v>
       </c>
       <c r="I33" s="17" t="n">
-        <v>-346</v>
+        <v>-110.25</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
@@ -2975,10 +2927,10 @@
         </is>
       </c>
       <c r="C34" s="15" t="n">
-        <v>199.96</v>
+        <v>1039.2</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
@@ -2986,7 +2938,7 @@
         </is>
       </c>
       <c r="F34" s="15" t="n">
-        <v>193.31</v>
+        <v>970</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
@@ -2997,19 +2949,19 @@
         <v>11</v>
       </c>
       <c r="I34" s="17" t="n">
-        <v>-172.9</v>
+        <v>-346</v>
       </c>
       <c r="J34" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.06660000000000001</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
@@ -3018,10 +2970,10 @@
         </is>
       </c>
       <c r="C35" s="15" t="n">
-        <v>986.4</v>
+        <v>199.96</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="E35" s="14" t="inlineStr">
         <is>
@@ -3029,7 +2981,7 @@
         </is>
       </c>
       <c r="F35" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>193.31</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
@@ -3040,17 +2992,60 @@
         <v>11</v>
       </c>
       <c r="I35" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J35" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K35" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D36" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E36" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F36" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G36" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H36" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I36" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J35" s="18" t="n">
+      <c r="J36" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K35" s="19" t="n">
+      <c r="K36" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I35">
+  <conditionalFormatting sqref="I2:I36">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3068,7 +3063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3815,6 +3810,31 @@
       </c>
       <c r="G29" s="14" t="n">
         <v>15</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>203487.54</v>
+      </c>
+      <c r="C30" s="20" t="n">
+        <v>119551.64</v>
+      </c>
+      <c r="D30" s="20" t="n">
+        <v>83935.89999999999</v>
+      </c>
+      <c r="E30" s="20" t="n">
+        <v>82723.10000000001</v>
+      </c>
+      <c r="F30" s="20" t="n">
+        <v>2274.74</v>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -3897,7 +3917,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -3905,10 +3925,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1713.4</v>
+        <v>1758.9</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1622.5</v>
+        <v>1666.94</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -3917,10 +3937,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8545840961218778</v>
+        <v>0.8320023988384573</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -3935,7 +3955,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
@@ -3943,10 +3963,10 @@
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1973.7</v>
+        <v>1976.7</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1906.9</v>
+        <v>1914.51</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -3958,7 +3978,7 @@
         <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.795059234475938</v>
+        <v>0.7870999305599393</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -3973,18 +3993,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1287</v>
+        <v>329.6</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1211.93</v>
+        <v>315.66</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -3993,10 +4013,10 @@
         <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8276855417376849</v>
+        <v>0.7909948866864465</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4011,18 +4031,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1407.2</v>
+        <v>9121.5</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1339.17</v>
+        <v>8633.07</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -4034,7 +4054,7 @@
         <v>5.9</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8124139890158449</v>
+        <v>0.7720903562485533</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -4049,18 +4069,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1770.4</v>
+        <v>883.25</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1699.76</v>
+        <v>849.4400000000001</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -4072,7 +4092,7 @@
         <v>5.9</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7697830524167245</v>
+        <v>0.7808829408917787</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -4087,18 +4107,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1611.3</v>
+        <v>4289.7</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1535.39</v>
+        <v>4092.59</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -4107,10 +4127,10 @@
         <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7785156660985207</v>
+        <v>0.7652273635923658</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -4125,18 +4145,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>7711</v>
+        <v>1300.5</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>7290.14</v>
+        <v>1227.73</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -4148,7 +4168,7 @@
         <v>5.8</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7814374092544663</v>
+        <v>0.7980051764408813</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -4163,18 +4183,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1549.4</v>
+        <v>2617.9</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1473.29</v>
+        <v>2487.06</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -4186,7 +4206,7 @@
         <v>5.8</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7747459125055236</v>
+        <v>0.7736716958104497</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -4201,18 +4221,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>7414</v>
+        <v>2162.7</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>7092.29</v>
+        <v>2061.74</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -4224,7 +4244,7 @@
         <v>5.8</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7520106053910738</v>
+        <v>0.7644645750478715</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -4239,18 +4259,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>CAPLIPOINT</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>2621.4</v>
+        <v>1619.6</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>2419.96</v>
+        <v>1549.03</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -4259,10 +4279,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7618584685310271</v>
+        <v>0.7634471729478358</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -4277,18 +4297,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>4149.5</v>
+        <v>8903</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>3979.23</v>
+        <v>8651.790000000001</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -4300,7 +4320,7 @@
         <v>5.7</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7499831660459146</v>
+        <v>0.7558561117774552</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -4315,18 +4335,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>2181.3</v>
+        <v>844.1</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>2077.16</v>
+        <v>790.04</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -4338,7 +4358,7 @@
         <v>5.7</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.747351808597942</v>
+        <v>0.7327820213370368</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -4353,18 +4373,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>452.75</v>
+        <v>1444.6</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>422.64</v>
+        <v>1378.7</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -4376,7 +4396,7 @@
         <v>5.6</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7614860172968878</v>
+        <v>0.7283157628937567</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -4391,18 +4411,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1114.6</v>
+        <v>1401.3</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1061.64</v>
+        <v>1334.74</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -4411,10 +4431,10 @@
         <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7328430444205963</v>
+        <v>0.7439208383309134</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -4429,18 +4449,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260727</v>
+        <v>20260728</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1483.5</v>
+        <v>452.1</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1403.6</v>
+        <v>421.68</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -4449,10 +4469,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.2</v>
+        <v>5.4</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7271384382299098</v>
+        <v>0.7245418008122383</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-29
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Tue 28 Jul 2026</t>
+          <t>As of Wed 29 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹203,488</t>
+          <t>₹203,734</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+122  (+0.06%)</t>
+          <t>₹+246  (+0.12%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.74%</t>
+          <t>+1.87%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.27%</t>
+          <t>-1.15%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹119,552</t>
+          <t>₹128,437</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹82,723</t>
+          <t>₹73,717</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹83,936</t>
+          <t>₹75,297</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+2,275</t>
+          <t>₹+2,154</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -796,31 +796,31 @@
         <v>7579.5</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>7512.5</v>
+        <v>7594.5</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>7512.5</v>
+        <v>7594.5</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>-67</v>
+        <v>15</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>-0.008839633221188734</v>
+        <v>0.001979022362952701</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>7128.14</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>7289</v>
+        <v>7332.464285714286</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.0297504159733777</v>
+        <v>0.03450335299041593</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>209.96</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8992.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1789</v>
+        <v>1774.5</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8945</v>
+        <v>8872.5</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-47.5</v>
+        <v>-120</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.0052821795941062</v>
+        <v>-0.01334445371142619</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1680.3</v>
@@ -862,13 +862,13 @@
         <v>1723.75</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.03647288988261611</v>
+        <v>0.02859960552268257</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>50.24</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -916,7 +916,7 @@
         <v>49.27</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>8883</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1300.5</v>
+        <v>1315.9</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9103.5</v>
+        <v>9211.300000000001</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>220.5</v>
+        <v>328.3000000000006</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.02482269503546099</v>
+        <v>0.03695823483057533</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1182.49</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1191.342857142857</v>
+        <v>1209.7</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.08393475037073651</v>
+        <v>0.08070522076145607</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>39.97</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>8847</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>9121.5</v>
+        <v>9047</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9121.5</v>
+        <v>9047</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>274.5</v>
+        <v>200</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.03102746693794507</v>
+        <v>0.02260653328812027</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>8315.07</v>
@@ -1006,67 +1006,67 @@
         <v>8791</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.0362330757002686</v>
+        <v>0.02829667293025312</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>254.57</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>5438</v>
+        <v>1624.8</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>5438</v>
+        <v>4874.4</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>5455.5</v>
+        <v>1781.3</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>5455.5</v>
+        <v>5343.9</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>17.5</v>
+        <v>469.5</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.003218094887826407</v>
+        <v>0.09631954702117183</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>5157.93</v>
+        <v>1520.16</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>5381</v>
+        <v>1647.864285714286</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.01365594354321327</v>
+        <v>0.074909175481791</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>143.39</v>
+        <v>45.45</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -1075,46 +1075,46 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>1624.8</v>
+        <v>1588.9</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>4874.4</v>
+        <v>4766.7</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1758.9</v>
+        <v>1629.9</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5276.700000000001</v>
+        <v>4889.700000000001</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>402.3000000000004</v>
+        <v>123</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.08253323485967512</v>
+        <v>0.02580401535653597</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>1520.16</v>
+        <v>1499.44</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>1620.964285714286</v>
+        <v>1537.1</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.07842157842157843</v>
+        <v>0.0569360083440703</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>45.45</v>
+        <v>37.96</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -1123,46 +1123,46 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>1588.9</v>
+        <v>1412.6</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>4766.7</v>
+        <v>4237.8</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1619.6</v>
+        <v>1474.3</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4858.799999999999</v>
+        <v>4422.9</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>92.09999999999945</v>
+        <v>185.1000000000001</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.01932154320599145</v>
+        <v>0.04367832365850209</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>1499.44</v>
+        <v>1342.97</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>1537.1</v>
+        <v>1370.992857142857</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.05093850333415659</v>
+        <v>0.07007199542640097</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>37.96</v>
+        <v>33.28</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1171,46 +1171,46 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1784</v>
+        <v>1948.5</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>3568</v>
+        <v>3897</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1774.7</v>
+        <v>1989.9</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>3549.4</v>
+        <v>3979.8</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>-18.59999999999991</v>
+        <v>82.80000000000018</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>-0.005213004484304907</v>
+        <v>0.02124711316397233</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>1694.96</v>
+        <v>1876.83</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1752.1</v>
+        <v>1903.371428571429</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.01273454668394666</v>
+        <v>0.04348387930477473</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>35.32</v>
+        <v>33.4</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -1219,46 +1219,46 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>1412.6</v>
+        <v>728.8</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>4237.8</v>
+        <v>5101.6</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>1444.6</v>
+        <v>720.5</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>4333.799999999999</v>
+        <v>5043.5</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>96</v>
+        <v>-58.09999999999968</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.02265326348577092</v>
+        <v>-0.01138858397365526</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>1342.97</v>
+        <v>676.71</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>1366.1</v>
+        <v>676.71</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.05434030181365084</v>
+        <v>0.06077723802914638</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>33.28</v>
+        <v>20.64</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1267,46 +1267,46 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>1948.5</v>
+        <v>4120</v>
       </c>
       <c r="D12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>4120</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>4373.8</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>4373.8</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>253.8000000000002</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>0.06160194174757286</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>3924.44</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>4053.142857142857</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>0.07331316997968432</v>
+      </c>
+      <c r="M12" s="13" t="n">
+        <v>85.14</v>
+      </c>
+      <c r="N12" s="6" t="n">
         <v>2</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>3897</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>1976.7</v>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>3953.4</v>
-      </c>
-      <c r="H12" s="10" t="n">
-        <v>56.40000000000009</v>
-      </c>
-      <c r="I12" s="11" t="n">
-        <v>0.01447267128560433</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>1876.83</v>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>1883.421428571429</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>0.04718903800706796</v>
-      </c>
-      <c r="M12" s="13" t="n">
-        <v>33.4</v>
-      </c>
-      <c r="N12" s="6" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -1315,140 +1315,44 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>728.8</v>
+        <v>862</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>5101.6</v>
+        <v>5172</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>713</v>
+        <v>878.7</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>4991</v>
+        <v>5272.200000000001</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-110.5999999999997</v>
+        <v>100.2000000000003</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.02167947310647634</v>
+        <v>0.01937354988399077</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>676.71</v>
+        <v>823.7</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>676.71</v>
+        <v>834.425</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.05089761570827484</v>
+        <v>0.05038693524524877</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>20.64</v>
+        <v>15.94</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>RADICO</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>4120</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="9" t="n">
-        <v>4120</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>4289.7</v>
-      </c>
-      <c r="G14" s="9" t="n">
-        <v>4289.7</v>
-      </c>
-      <c r="H14" s="10" t="n">
-        <v>169.6999999999998</v>
-      </c>
-      <c r="I14" s="11" t="n">
-        <v>0.04118932038834947</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>3924.44</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>3994.028571428572</v>
-      </c>
-      <c r="L14" s="12" t="n">
-        <v>0.06892589891400981</v>
-      </c>
-      <c r="M14" s="13" t="n">
-        <v>85.14</v>
-      </c>
-      <c r="N14" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>MARICO</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>862</v>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="E15" s="9" t="n">
-        <v>5172</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>883.25</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>5299.5</v>
-      </c>
-      <c r="H15" s="10" t="n">
-        <v>127.5</v>
-      </c>
-      <c r="I15" s="11" t="n">
-        <v>0.02465197215777262</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>823.7</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>832.5392857142857</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>0.05741377218875096</v>
-      </c>
-      <c r="M15" s="13" t="n">
-        <v>15.94</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H15">
+  <conditionalFormatting sqref="H2:H13">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1466,7 +1370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1542,27 +1446,27 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>871.8</v>
+        <v>5438</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>830.15</v>
+        <v>5381</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -1570,108 +1474,108 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-249.9</v>
+        <v>-57</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0478</v>
+        <v>-0.0105</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-0.73</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>420.3</v>
+        <v>1784</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>448.6</v>
+        <v>1752.1</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>622.6</v>
+        <v>-63.8</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>0.0673</v>
+        <v>-0.0179</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>0.84</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>1465</v>
+        <v>871.8</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>6</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>1596.9</v>
+        <v>830.15</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>791.4</v>
+        <v>-249.9</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>0.09</v>
+        <v>-0.0478</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>1.32</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -1680,10 +1584,10 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>619.25</v>
+        <v>420.3</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
@@ -1691,7 +1595,7 @@
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>717.95</v>
+        <v>448.6</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1702,19 +1606,19 @@
         <v>25</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>1480.5</v>
+        <v>622.6</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>0.1594</v>
+        <v>0.0673</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>3.55</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -1723,10 +1627,10 @@
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>8700</v>
+        <v>1465</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -1734,7 +1638,7 @@
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>8805.5</v>
+        <v>1596.9</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -1745,31 +1649,31 @@
         <v>25</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>105.5</v>
+        <v>791.4</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>0.0121</v>
+        <v>0.09</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>0.29</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>961.85</v>
+        <v>619.25</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
@@ -1777,42 +1681,42 @@
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>935.6</v>
+        <v>717.95</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>-236.25</v>
+        <v>1480.5</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>-0.0273</v>
+        <v>0.1594</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>-0.64</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>1560</v>
+        <v>8700</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
@@ -1820,50 +1724,50 @@
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>1547.4</v>
+        <v>8805.5</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>-63</v>
+        <v>105.5</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>-0.0081</v>
+        <v>0.0121</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>-0.23</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>900</v>
+        <v>961.85</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>887.1</v>
+        <v>935.6</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
@@ -1871,22 +1775,22 @@
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>-129</v>
+        <v>-236.25</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>-0.0143</v>
+        <v>-0.0273</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -1895,18 +1799,18 @@
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>880.8</v>
+        <v>1560</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>832.9400000000001</v>
+        <v>1547.4</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
@@ -1914,42 +1818,42 @@
         </is>
       </c>
       <c r="H10" s="14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>-478.6</v>
+        <v>-63</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>-0.0543</v>
+        <v>-0.0081</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>-1</v>
+        <v>-0.23</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>777</v>
+        <v>900</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>744.8</v>
+        <v>887.1</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
@@ -1957,42 +1861,42 @@
         </is>
       </c>
       <c r="H11" s="14" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>-386.4</v>
+        <v>-129</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>-0.0414</v>
+        <v>-0.0143</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>-1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>1114.9</v>
+        <v>880.8</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>1050.57</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -2000,13 +1904,13 @@
         </is>
       </c>
       <c r="H12" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>-514.64</v>
+        <v>-478.6</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>-0.0577</v>
+        <v>-0.0543</v>
       </c>
       <c r="K12" s="19" t="n">
         <v>-1</v>
@@ -2015,93 +1919,93 @@
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>790</v>
+        <v>777</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>880.8</v>
+        <v>744.8</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>998.8</v>
+        <v>-386.4</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0414</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>3770</v>
+        <v>1114.9</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>4097.9</v>
+        <v>1050.57</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H14" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>655.8</v>
+        <v>-514.64</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>-0.0577</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>1.98</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -2110,7 +2014,7 @@
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>821.05</v>
+        <v>790</v>
       </c>
       <c r="D15" s="16" t="n">
         <v>11</v>
@@ -2121,7 +2025,7 @@
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>844</v>
+        <v>880.8</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
@@ -2132,19 +2036,19 @@
         <v>25</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>252.45</v>
+        <v>998.8</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.028</v>
+        <v>0.1149</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>0.6</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -2153,10 +2057,10 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>2426.1</v>
+        <v>3770</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
@@ -2164,7 +2068,7 @@
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>2484.2</v>
+        <v>4097.9</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
@@ -2175,39 +2079,39 @@
         <v>25</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>174.3</v>
+        <v>655.8</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>0.5</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>1410</v>
+        <v>821.05</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>1455.2</v>
+        <v>844</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -2218,39 +2122,39 @@
         <v>25</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>135.6</v>
+        <v>252.45</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.028</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>0.46</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>690</v>
+        <v>2426.1</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>660.45</v>
+        <v>2484.2</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -2261,19 +2165,19 @@
         <v>25</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>-206.85</v>
+        <v>174.3</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.0239</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -2282,10 +2186,10 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>1839</v>
+        <v>1410</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
@@ -2293,7 +2197,7 @@
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>1828.1</v>
+        <v>1455.2</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
@@ -2304,19 +2208,19 @@
         <v>25</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>-21.8</v>
+        <v>135.6</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>-0.0059</v>
+        <v>0.0321</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>-0.1</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -2325,10 +2229,10 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>1414</v>
+        <v>690</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
@@ -2336,7 +2240,7 @@
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>1537.8</v>
+        <v>660.45</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -2347,19 +2251,19 @@
         <v>25</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>371.4</v>
+        <v>-206.85</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>0.0876</v>
+        <v>-0.0428</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>1.38</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -2368,10 +2272,10 @@
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>1300</v>
+        <v>1839</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
@@ -2379,7 +2283,7 @@
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>1389.1</v>
+        <v>1828.1</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -2390,19 +2294,19 @@
         <v>25</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>356.4</v>
+        <v>-21.8</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>-0.0059</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>0.63</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
@@ -2411,10 +2315,10 @@
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>276.45</v>
+        <v>1414</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
@@ -2422,7 +2326,7 @@
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>330.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -2433,19 +2337,19 @@
         <v>25</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>1019.35</v>
+        <v>371.4</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.0876</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>3.1</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
@@ -2454,10 +2358,10 @@
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>1462.5</v>
+        <v>1300</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
@@ -2465,7 +2369,7 @@
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>1564.7</v>
+        <v>1389.1</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -2476,19 +2380,19 @@
         <v>25</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>306.6</v>
+        <v>356.4</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>1.78</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -2497,41 +2401,41 @@
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>798</v>
+        <v>276.45</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>750</v>
+        <v>330.1</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H24" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>-288</v>
+        <v>1019.35</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.1941</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>-0.92</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -2540,53 +2444,53 @@
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>260.45</v>
+        <v>1462.5</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>257.85</v>
+        <v>1564.7</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H25" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>-52.07</v>
+        <v>306.6</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>-0.01</v>
+        <v>0.0699</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>-0.13</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>6500</v>
+        <v>798</v>
       </c>
       <c r="D26" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
@@ -2594,7 +2498,7 @@
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>6401.5</v>
+        <v>750</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
@@ -2602,34 +2506,34 @@
         </is>
       </c>
       <c r="H26" s="14" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I26" s="17" t="n">
-        <v>-98.5</v>
+        <v>-288</v>
       </c>
       <c r="J26" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.0602</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>571.5</v>
+        <v>260.45</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
@@ -2637,7 +2541,7 @@
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>571.1</v>
+        <v>257.85</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
@@ -2645,34 +2549,34 @@
         </is>
       </c>
       <c r="H27" s="14" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>-6.4</v>
+        <v>-52.07</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.01</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>965</v>
+        <v>6500</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
@@ -2680,7 +2584,7 @@
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>933</v>
+        <v>6401.5</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
@@ -2688,22 +2592,22 @@
         </is>
       </c>
       <c r="H28" s="14" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="I28" s="17" t="n">
-        <v>-288</v>
+        <v>-98.5</v>
       </c>
       <c r="J28" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0152</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -2712,18 +2616,18 @@
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>5479</v>
+        <v>571.5</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F29" s="15" t="n">
-        <v>5424</v>
+        <v>571.1</v>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
@@ -2731,42 +2635,42 @@
         </is>
       </c>
       <c r="H29" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I29" s="17" t="n">
-        <v>-55</v>
+        <v>-6.4</v>
       </c>
       <c r="J29" s="18" t="n">
+        <v>-0.0007</v>
+      </c>
+      <c r="K29" s="19" t="n">
         <v>-0.01</v>
-      </c>
-      <c r="K29" s="19" t="n">
-        <v>-0.18</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C30" s="15" t="n">
-        <v>960.1</v>
+        <v>965</v>
       </c>
       <c r="D30" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F30" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>933</v>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
@@ -2774,42 +2678,42 @@
         </is>
       </c>
       <c r="H30" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I30" s="17" t="n">
-        <v>-516.79</v>
+        <v>-288</v>
       </c>
       <c r="J30" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.0332</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>952.1</v>
+        <v>5479</v>
       </c>
       <c r="D31" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F31" s="15" t="n">
-        <v>948.8</v>
+        <v>5424</v>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
@@ -2820,39 +2724,39 @@
         <v>1</v>
       </c>
       <c r="I31" s="17" t="n">
-        <v>-29.7</v>
+        <v>-55</v>
       </c>
       <c r="J31" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.01</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C32" s="15" t="n">
-        <v>1475</v>
+        <v>960.1</v>
       </c>
       <c r="D32" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F32" s="15" t="n">
-        <v>1394.19</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
@@ -2860,42 +2764,42 @@
         </is>
       </c>
       <c r="H32" s="14" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I32" s="17" t="n">
-        <v>-484.86</v>
+        <v>-516.79</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0598</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>-1</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C33" s="15" t="n">
-        <v>248.05</v>
+        <v>952.1</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F33" s="15" t="n">
-        <v>242.8</v>
+        <v>948.8</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
@@ -2903,42 +2807,42 @@
         </is>
       </c>
       <c r="H33" s="14" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I33" s="17" t="n">
-        <v>-110.25</v>
+        <v>-29.7</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0035</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>-0.3</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C34" s="15" t="n">
-        <v>1039.2</v>
+        <v>1475</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F34" s="15" t="n">
-        <v>970</v>
+        <v>1394.19</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
@@ -2946,22 +2850,22 @@
         </is>
       </c>
       <c r="H34" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I34" s="17" t="n">
-        <v>-346</v>
+        <v>-484.86</v>
       </c>
       <c r="J34" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0548</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>-0.82</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
@@ -2970,10 +2874,10 @@
         </is>
       </c>
       <c r="C35" s="15" t="n">
-        <v>199.96</v>
+        <v>248.05</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E35" s="14" t="inlineStr">
         <is>
@@ -2981,7 +2885,7 @@
         </is>
       </c>
       <c r="F35" s="15" t="n">
-        <v>193.31</v>
+        <v>242.8</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
@@ -2992,19 +2896,19 @@
         <v>11</v>
       </c>
       <c r="I35" s="17" t="n">
-        <v>-172.9</v>
+        <v>-110.25</v>
       </c>
       <c r="J35" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.0212</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
@@ -3013,7 +2917,7 @@
         </is>
       </c>
       <c r="C36" s="15" t="n">
-        <v>986.4</v>
+        <v>1039.2</v>
       </c>
       <c r="D36" s="16" t="n">
         <v>5</v>
@@ -3024,7 +2928,7 @@
         </is>
       </c>
       <c r="F36" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>970</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
@@ -3035,17 +2939,103 @@
         <v>11</v>
       </c>
       <c r="I36" s="17" t="n">
+        <v>-346</v>
+      </c>
+      <c r="J36" s="18" t="n">
+        <v>-0.06660000000000001</v>
+      </c>
+      <c r="K36" s="19" t="n">
+        <v>-0.82</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C37" s="15" t="n">
+        <v>199.96</v>
+      </c>
+      <c r="D37" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F37" s="15" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="G37" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H37" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I37" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J37" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K37" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D38" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F38" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G38" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H38" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I38" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J36" s="18" t="n">
+      <c r="J38" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K36" s="19" t="n">
+      <c r="K38" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I36">
+  <conditionalFormatting sqref="I2:I38">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3063,7 +3053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3835,6 +3825,31 @@
       </c>
       <c r="G30" s="14" t="n">
         <v>14</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n">
+        <v>203733.54</v>
+      </c>
+      <c r="C31" s="20" t="n">
+        <v>128436.84</v>
+      </c>
+      <c r="D31" s="20" t="n">
+        <v>75296.7</v>
+      </c>
+      <c r="E31" s="20" t="n">
+        <v>73717.10000000001</v>
+      </c>
+      <c r="F31" s="20" t="n">
+        <v>2153.94</v>
+      </c>
+      <c r="G31" s="14" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -3917,7 +3932,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -3925,10 +3940,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1758.9</v>
+        <v>1781.3</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1666.94</v>
+        <v>1692.34</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -3937,10 +3952,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8320023988384573</v>
+        <v>0.8139448267154852</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -3955,18 +3970,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1976.7</v>
+        <v>1719.7</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1914.51</v>
+        <v>1646.99</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -3978,7 +3993,7 @@
         <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.7870999305599393</v>
+        <v>0.7954695621067693</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -3993,18 +4008,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>329.6</v>
+        <v>1590.7</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>315.66</v>
+        <v>1520.1</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -4013,10 +4028,10 @@
         <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7909948866864465</v>
+        <v>0.815125307745723</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4031,18 +4046,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>9121.5</v>
+        <v>878.7</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>8633.07</v>
+        <v>846.15</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -4054,7 +4069,7 @@
         <v>5.9</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7720903562485533</v>
+        <v>0.781255392125918</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -4069,18 +4084,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>883.25</v>
+        <v>4373.8</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>849.4400000000001</v>
+        <v>4160.03</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -4092,7 +4107,7 @@
         <v>5.9</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7808829408917787</v>
+        <v>0.7716095364349894</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -4107,18 +4122,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>4289.7</v>
+        <v>1474.3</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>4092.59</v>
+        <v>1405.43</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -4130,7 +4145,7 @@
         <v>5.9</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7652273635923658</v>
+        <v>0.7709393346379647</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -4145,18 +4160,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1300.5</v>
+        <v>449.35</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1227.73</v>
+        <v>419.51</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -4168,7 +4183,7 @@
         <v>5.8</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7980051764408813</v>
+        <v>0.7923500199903205</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -4183,18 +4198,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>2617.9</v>
+        <v>7784.5</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>2487.06</v>
+        <v>7441.93</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -4206,7 +4221,7 @@
         <v>5.8</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7736716958104497</v>
+        <v>0.7345432737832208</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -4221,18 +4236,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>2162.7</v>
+        <v>1315.9</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>2061.74</v>
+        <v>1245.1</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -4244,7 +4259,7 @@
         <v>5.8</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7644645750478715</v>
+        <v>0.7877522462807482</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -4259,18 +4274,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1619.6</v>
+        <v>1432.9</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1549.03</v>
+        <v>1367.39</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -4279,10 +4294,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7634471729478358</v>
+        <v>0.7847568545756791</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -4297,18 +4312,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>8903</v>
+        <v>2171.5</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>8651.790000000001</v>
+        <v>2073.54</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -4320,7 +4335,7 @@
         <v>5.7</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7558561117774552</v>
+        <v>0.7541695600025251</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -4335,18 +4350,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>844.1</v>
+        <v>1629.9</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>790.04</v>
+        <v>1560.16</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -4358,7 +4373,7 @@
         <v>5.7</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7327820213370368</v>
+        <v>0.7491761883719462</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -4373,18 +4388,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1444.6</v>
+        <v>2447</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1378.7</v>
+        <v>2338.04</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -4393,10 +4408,10 @@
         <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7283157628937567</v>
+        <v>0.7461271384382299</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -4411,18 +4426,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1401.3</v>
+        <v>841.85</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1334.74</v>
+        <v>787.36</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -4431,10 +4446,10 @@
         <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7439208383309134</v>
+        <v>0.7421395955642531</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -4449,18 +4464,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260728</v>
+        <v>20260729</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>452.1</v>
+        <v>8935</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>421.68</v>
+        <v>8698.07</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -4469,10 +4484,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7245418008122383</v>
+        <v>0.7407139700776466</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-30
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Wed 29 Jul 2026</t>
+          <t>As of Thu 30 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹203,734</t>
+          <t>₹203,625</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+246  (+0.12%)</t>
+          <t>₹-108  (-0.05%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.87%</t>
+          <t>+1.81%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.15%</t>
+          <t>-1.20%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹75,297</t>
+          <t>₹75,188</t>
         </is>
       </c>
     </row>
@@ -796,16 +796,16 @@
         <v>7579.5</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>7594.5</v>
+        <v>7386.5</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>7594.5</v>
+        <v>7386.5</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>15</v>
+        <v>-193</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.001979022362952701</v>
+        <v>-0.02546342106999143</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>7128.14</v>
@@ -814,13 +814,13 @@
         <v>7332.464285714286</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.03450335299041593</v>
+        <v>0.007315469340785726</v>
       </c>
       <c r="M2" s="13" t="n">
         <v>209.96</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8992.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1774.5</v>
+        <v>1758.8</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8872.5</v>
+        <v>8794</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-120</v>
+        <v>-198.5000000000002</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.01334445371142619</v>
+        <v>-0.02207395051431751</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1680.3</v>
@@ -862,13 +862,13 @@
         <v>1723.75</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.02859960552268257</v>
+        <v>0.01992836024562212</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>50.24</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -916,7 +916,7 @@
         <v>49.27</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>8883</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1315.9</v>
+        <v>1315.2</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9211.300000000001</v>
+        <v>9206.4</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>328.3000000000006</v>
+        <v>323.4000000000003</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.03695823483057533</v>
+        <v>0.03640661938534283</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1182.49</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1209.7</v>
+        <v>1218.4</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.08070522076145607</v>
+        <v>0.0736009732360097</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>39.97</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>8847</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>9047</v>
+        <v>8896</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9047</v>
+        <v>8896</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>200</v>
+        <v>49</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.02260653328812027</v>
+        <v>0.005538600655589465</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>8315.07</v>
@@ -1006,13 +1006,13 @@
         <v>8791</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.02829667293025312</v>
+        <v>0.01180305755395683</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>254.57</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -1051,16 +1051,16 @@
         <v>1520.16</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1647.864285714286</v>
+        <v>1651.785714285714</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.074909175481791</v>
+        <v>0.07270773351725467</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>45.45</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -1108,7 +1108,7 @@
         <v>37.96</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>4237.8</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1474.3</v>
+        <v>1466.4</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4422.9</v>
+        <v>4399.200000000001</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>185.1000000000001</v>
+        <v>161.4000000000005</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.04367832365850209</v>
+        <v>0.03808579923545249</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1342.97</v>
@@ -1150,13 +1150,13 @@
         <v>1370.992857142857</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.07007199542640097</v>
+        <v>0.06506215415789898</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>33.28</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>3897</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1989.9</v>
+        <v>2001.1</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>3979.8</v>
+        <v>4002.2</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>82.80000000000018</v>
+        <v>105.1999999999998</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.02124711316397233</v>
+        <v>0.0269951244547087</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1876.83</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1903.371428571429</v>
+        <v>1914.142857142857</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.04348387930477473</v>
+        <v>0.04345467135932377</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>33.4</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1228,31 +1228,31 @@
         <v>5101.6</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>720.5</v>
+        <v>763.75</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5043.5</v>
+        <v>5346.25</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-58.09999999999968</v>
+        <v>244.6500000000003</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>-0.01138858397365526</v>
+        <v>0.04795554335894628</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>676.71</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>676.71</v>
+        <v>696.6678571428571</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.06077723802914638</v>
+        <v>0.087832592938976</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>20.64</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4120</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>4373.8</v>
+        <v>4366.6</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4373.8</v>
+        <v>4366.6</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>253.8000000000002</v>
+        <v>246.6000000000004</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.06160194174757286</v>
+        <v>0.05985436893203892</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>3924.44</v>
@@ -1294,13 +1294,13 @@
         <v>4053.142857142857</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.07331316997968432</v>
+        <v>0.07178517447376527</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>85.14</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1324,31 +1324,31 @@
         <v>5172</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>878.7</v>
+        <v>885.35</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>5272.200000000001</v>
+        <v>5312.1</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>100.2000000000003</v>
+        <v>140.1000000000001</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.01937354988399077</v>
+        <v>0.0270881670533643</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>823.7</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>834.425</v>
+        <v>836.5035714285714</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.05038693524524877</v>
+        <v>0.05517188521085294</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>15.94</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -3053,7 +3053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3849,6 +3849,31 @@
         <v>2153.94</v>
       </c>
       <c r="G31" s="14" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="n">
+        <v>203625.29</v>
+      </c>
+      <c r="C32" s="20" t="n">
+        <v>128436.84</v>
+      </c>
+      <c r="D32" s="20" t="n">
+        <v>75188.45</v>
+      </c>
+      <c r="E32" s="20" t="n">
+        <v>73717.10000000001</v>
+      </c>
+      <c r="F32" s="20" t="n">
+        <v>2153.94</v>
+      </c>
+      <c r="G32" s="14" t="n">
         <v>12</v>
       </c>
     </row>
@@ -3932,18 +3957,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1781.3</v>
+        <v>333.75</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1692.34</v>
+        <v>319.94</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -3955,7 +3980,7 @@
         <v>6.2</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8139448267154852</v>
+        <v>0.8262442396313364</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -3970,18 +3995,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1719.7</v>
+        <v>1781.3</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1646.99</v>
+        <v>1694.96</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -3993,7 +4018,7 @@
         <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.7954695621067693</v>
+        <v>0.8038081273565145</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -4008,18 +4033,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1590.7</v>
+        <v>8988</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1520.1</v>
+        <v>8746.709999999999</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -4031,7 +4056,7 @@
         <v>6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.815125307745723</v>
+        <v>0.8015731043150398</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4046,18 +4071,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>878.7</v>
+        <v>1520.6</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>846.15</v>
+        <v>1446.5</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -4069,7 +4094,7 @@
         <v>5.9</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.781255392125918</v>
+        <v>0.8286730205278592</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -4084,7 +4109,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
@@ -4092,10 +4117,10 @@
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>4373.8</v>
+        <v>4366.6</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>4160.03</v>
+        <v>4142.76</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -4107,7 +4132,7 @@
         <v>5.9</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7716095364349894</v>
+        <v>0.7692930456640135</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -4122,18 +4147,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1474.3</v>
+        <v>2746.2</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1405.43</v>
+        <v>2630.03</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -4145,7 +4170,7 @@
         <v>5.9</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7709393346379647</v>
+        <v>0.7549172601591957</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -4160,18 +4185,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>449.35</v>
+        <v>1664.1</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>419.51</v>
+        <v>1589.03</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -4180,10 +4205,10 @@
         <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7923500199903205</v>
+        <v>0.762263301214914</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -4198,18 +4223,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>SYRMA</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>7784.5</v>
+        <v>1377.8</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>7441.93</v>
+        <v>1263.87</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -4218,10 +4243,10 @@
         <v>5333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7345432737832208</v>
+        <v>0.7438322161709259</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -4236,18 +4261,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1315.9</v>
+        <v>1576.3</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1245.1</v>
+        <v>1505.96</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -4259,7 +4284,7 @@
         <v>5.8</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7877522462807482</v>
+        <v>0.7729765395894428</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -4274,18 +4299,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1432.9</v>
+        <v>1629.9</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1367.39</v>
+        <v>1561.74</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -4294,10 +4319,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7847568545756791</v>
+        <v>0.7629587348135735</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -4312,18 +4337,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>2171.5</v>
+        <v>885.35</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>2073.54</v>
+        <v>852.79</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -4335,7 +4360,7 @@
         <v>5.7</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7541695600025251</v>
+        <v>0.7557415165479682</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -4350,18 +4375,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1629.9</v>
+        <v>1416.4</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1560.16</v>
+        <v>1349.1</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -4370,10 +4395,10 @@
         <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7491761883719462</v>
+        <v>0.7732268537913699</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -4388,18 +4413,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>2447</v>
+        <v>1315.2</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>2338.04</v>
+        <v>1250.2</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -4408,10 +4433,10 @@
         <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7461271384382299</v>
+        <v>0.7602031839128613</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -4426,18 +4451,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>841.85</v>
+        <v>7386.5</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>787.36</v>
+        <v>7003.5</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -4449,7 +4474,7 @@
         <v>5.6</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7421395955642531</v>
+        <v>0.7405310012568077</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -4464,18 +4489,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260729</v>
+        <v>20260730</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>8935</v>
+        <v>445.95</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>8698.07</v>
+        <v>416.01</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -4484,10 +4509,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7407139700776466</v>
+        <v>0.740736279849183</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-07-31
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Thu 30 Jul 2026</t>
+          <t>As of Fri 31 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹203,625</t>
+          <t>₹203,935</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-108  (-0.05%)</t>
+          <t>₹+310  (+0.15%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.81%</t>
+          <t>+1.97%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.20%</t>
+          <t>-1.05%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹128,437</t>
+          <t>₹144,743</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹73,717</t>
+          <t>₹57,145</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹75,188</t>
+          <t>₹59,192</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+2,154</t>
+          <t>₹+1,888</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -778,247 +778,247 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>JBCHEPHARM</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C2" s="7" t="n">
-        <v>7579.5</v>
+        <v>2415.2</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" s="9" t="n">
-        <v>7579.5</v>
+        <v>7245.6</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>7386.5</v>
+        <v>2415.2</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>7386.5</v>
+        <v>7245.599999999999</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>-193</v>
+        <v>0</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>-0.02546342106999143</v>
+        <v>0</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>7128.14</v>
+        <v>2335.46</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>7332.464285714286</v>
+        <v>2349.7</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>0.007315469340785726</v>
+        <v>0.02711990725405764</v>
       </c>
       <c r="M2" s="13" t="n">
-        <v>209.96</v>
+        <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>1798.5</v>
+        <v>1269</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>8992.5</v>
+        <v>8883</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1758.8</v>
+        <v>1315.1</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8794</v>
+        <v>9205.699999999999</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-198.5000000000002</v>
+        <v>322.6999999999994</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.02207395051431751</v>
+        <v>0.03632781717888094</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>1680.3</v>
+        <v>1182.49</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>1723.75</v>
+        <v>1218.4</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.01992836024562212</v>
+        <v>0.07353052999771867</v>
       </c>
       <c r="M3" s="13" t="n">
-        <v>50.24</v>
+        <v>39.97</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>JBCHEPHARM</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>2415.2</v>
+        <v>8847</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>7245.6</v>
+        <v>8847</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>2415.2</v>
+        <v>9106.5</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>7245.599999999999</v>
+        <v>9106.5</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>0</v>
+        <v>259.5</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0</v>
+        <v>0.02933197694133605</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>2335.46</v>
+        <v>8315.07</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>2349.7</v>
+        <v>8791</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.02711990725405764</v>
+        <v>0.03464558282545434</v>
       </c>
       <c r="M4" s="13" t="n">
-        <v>49.27</v>
+        <v>254.57</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>1269</v>
+        <v>1624.8</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>8883</v>
+        <v>4874.4</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1315.2</v>
+        <v>1816.2</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9206.4</v>
+        <v>5448.6</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>323.4000000000003</v>
+        <v>574.2000000000003</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.03640661938534283</v>
+        <v>0.1177991137370754</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>1182.49</v>
+        <v>1520.16</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1218.4</v>
+        <v>1685.614285714286</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.0736009732360097</v>
+        <v>0.07190051441785814</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>39.97</v>
+        <v>45.45</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>8847</v>
+        <v>1588.9</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>8847</v>
+        <v>4766.7</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>8896</v>
+        <v>1611.4</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>8896</v>
+        <v>4834.200000000001</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>49</v>
+        <v>67.5</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.005538600655589465</v>
+        <v>0.01416074013468437</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>8315.07</v>
+        <v>1499.44</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>8791</v>
+        <v>1537.1</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.01180305755395683</v>
+        <v>0.04610897356336116</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>254.57</v>
+        <v>37.96</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -1027,46 +1027,46 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>1624.8</v>
+        <v>1412.6</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>4874.4</v>
+        <v>4237.8</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1781.3</v>
+        <v>1473.2</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>5343.9</v>
+        <v>4419.6</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>469.5</v>
+        <v>181.8000000000004</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.09631954702117183</v>
+        <v>0.04289961772617878</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>1520.16</v>
+        <v>1342.97</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1651.785714285714</v>
+        <v>1372.342857142857</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.07270773351725467</v>
+        <v>0.06846126992746598</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>45.45</v>
+        <v>33.28</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -1075,46 +1075,46 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>1588.9</v>
+        <v>1948.5</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>4766.7</v>
+        <v>3897</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1629.9</v>
+        <v>1990.5</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>4889.700000000001</v>
+        <v>3981</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>123</v>
+        <v>84</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.02580401535653597</v>
+        <v>0.02155504234026174</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>1499.44</v>
+        <v>1876.83</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>1537.1</v>
+        <v>1914.142857142857</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.0569360083440703</v>
+        <v>0.03836078515807229</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>37.96</v>
+        <v>33.4</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -1123,46 +1123,46 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>1412.6</v>
+        <v>728.8</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>4237.8</v>
+        <v>5101.6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1466.4</v>
+        <v>769.4</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4399.200000000001</v>
+        <v>5385.8</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>161.4000000000005</v>
+        <v>284.2000000000002</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.03808579923545249</v>
+        <v>0.05570801317233812</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>1342.97</v>
+        <v>676.71</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>1370.992857142857</v>
+        <v>703.0999999999999</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.06506215415789898</v>
+        <v>0.08617104237067855</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>33.28</v>
+        <v>20.64</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1171,46 +1171,46 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1948.5</v>
+        <v>4120</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>3897</v>
+        <v>4120</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>2001.1</v>
+        <v>4340.8</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4002.2</v>
+        <v>4340.8</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>105.1999999999998</v>
+        <v>220.8000000000002</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.0269951244547087</v>
+        <v>0.05359223300970879</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>1876.83</v>
+        <v>3924.44</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1914.142857142857</v>
+        <v>4053.142857142857</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.04345467135932377</v>
+        <v>0.066268232320573</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>33.4</v>
+        <v>85.14</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -1219,140 +1219,44 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>728.8</v>
+        <v>862</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>5101.6</v>
+        <v>5172</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>763.75</v>
+        <v>870.65</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5346.25</v>
+        <v>5223.9</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>244.6500000000003</v>
+        <v>51.89999999999986</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.04795554335894628</v>
+        <v>0.01003480278422271</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>676.71</v>
+        <v>823.7</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>696.6678571428571</v>
+        <v>836.5035714285714</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.087832592938976</v>
+        <v>0.03921946657259358</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>20.64</v>
+        <v>15.94</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>RADICO</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>4120</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>4120</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>4366.6</v>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>4366.6</v>
-      </c>
-      <c r="H12" s="10" t="n">
-        <v>246.6000000000004</v>
-      </c>
-      <c r="I12" s="11" t="n">
-        <v>0.05985436893203892</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>3924.44</v>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>4053.142857142857</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>0.07178517447376527</v>
-      </c>
-      <c r="M12" s="13" t="n">
-        <v>85.14</v>
-      </c>
-      <c r="N12" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>MARICO</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>862</v>
-      </c>
-      <c r="D13" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>5172</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>885.35</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>5312.1</v>
-      </c>
-      <c r="H13" s="10" t="n">
-        <v>140.1000000000001</v>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>0.0270881670533643</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>823.7</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>836.5035714285714</v>
-      </c>
-      <c r="L13" s="12" t="n">
-        <v>0.05517188521085294</v>
-      </c>
-      <c r="M13" s="13" t="n">
-        <v>15.94</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H13">
+  <conditionalFormatting sqref="H2:H11">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1370,7 +1274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1446,113 +1350,113 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>5438</v>
+        <v>7579.5</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>5381</v>
+        <v>7567.5</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-57</v>
+        <v>-12</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0105</v>
+        <v>-0.0016</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>1784</v>
+        <v>1798.5</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>1752.1</v>
+        <v>1747.8</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-63.8</v>
+        <v>-253.5</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0179</v>
+        <v>-0.0282</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-0.36</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>871.8</v>
+        <v>5438</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>830.15</v>
+        <v>5381</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1560,108 +1464,108 @@
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-249.9</v>
+        <v>-57</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0478</v>
+        <v>-0.0105</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-0.73</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>420.3</v>
+        <v>1784</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>448.6</v>
+        <v>1752.1</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>622.6</v>
+        <v>-63.8</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>0.0673</v>
+        <v>-0.0179</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>0.84</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>1465</v>
+        <v>871.8</v>
       </c>
       <c r="D6" s="16" t="n">
         <v>6</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>1596.9</v>
+        <v>830.15</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>791.4</v>
+        <v>-249.9</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>0.09</v>
+        <v>-0.0478</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>1.32</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -1670,10 +1574,10 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>619.25</v>
+        <v>420.3</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
@@ -1681,7 +1585,7 @@
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>717.95</v>
+        <v>448.6</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -1692,19 +1596,19 @@
         <v>25</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>1480.5</v>
+        <v>622.6</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>0.1594</v>
+        <v>0.0673</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>3.55</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -1713,10 +1617,10 @@
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>8700</v>
+        <v>1465</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
@@ -1724,7 +1628,7 @@
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>8805.5</v>
+        <v>1596.9</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -1735,31 +1639,31 @@
         <v>25</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>105.5</v>
+        <v>791.4</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>0.0121</v>
+        <v>0.09</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>0.29</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>961.85</v>
+        <v>619.25</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
@@ -1767,42 +1671,42 @@
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>935.6</v>
+        <v>717.95</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>-236.25</v>
+        <v>1480.5</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>-0.0273</v>
+        <v>0.1594</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>-0.64</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1560</v>
+        <v>8700</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
@@ -1810,50 +1714,50 @@
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>1547.4</v>
+        <v>8805.5</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H10" s="14" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>-63</v>
+        <v>105.5</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>-0.0081</v>
+        <v>0.0121</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>-0.23</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>900</v>
+        <v>961.85</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>887.1</v>
+        <v>935.6</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
@@ -1861,22 +1765,22 @@
         </is>
       </c>
       <c r="H11" s="14" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>-129</v>
+        <v>-236.25</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>-0.0143</v>
+        <v>-0.0273</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -1885,18 +1789,18 @@
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>880.8</v>
+        <v>1560</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>832.9400000000001</v>
+        <v>1547.4</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -1904,42 +1808,42 @@
         </is>
       </c>
       <c r="H12" s="14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>-478.6</v>
+        <v>-63</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>-0.0543</v>
+        <v>-0.0081</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>-1</v>
+        <v>-0.23</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>777</v>
+        <v>900</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>744.8</v>
+        <v>887.1</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
@@ -1947,42 +1851,42 @@
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>-386.4</v>
+        <v>-129</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>-0.0414</v>
+        <v>-0.0143</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>-1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>1114.9</v>
+        <v>880.8</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>1050.57</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
@@ -1990,13 +1894,13 @@
         </is>
       </c>
       <c r="H14" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>-514.64</v>
+        <v>-478.6</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>-0.0577</v>
+        <v>-0.0543</v>
       </c>
       <c r="K14" s="19" t="n">
         <v>-1</v>
@@ -2005,93 +1909,93 @@
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>790</v>
+        <v>777</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>880.8</v>
+        <v>744.8</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H15" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>998.8</v>
+        <v>-386.4</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0414</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>3770</v>
+        <v>1114.9</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>4097.9</v>
+        <v>1050.57</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H16" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>655.8</v>
+        <v>-514.64</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>-0.0577</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>1.98</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -2100,7 +2004,7 @@
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>821.05</v>
+        <v>790</v>
       </c>
       <c r="D17" s="16" t="n">
         <v>11</v>
@@ -2111,7 +2015,7 @@
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>844</v>
+        <v>880.8</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -2122,19 +2026,19 @@
         <v>25</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>252.45</v>
+        <v>998.8</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>0.028</v>
+        <v>0.1149</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>0.6</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -2143,10 +2047,10 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>2426.1</v>
+        <v>3770</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
@@ -2154,7 +2058,7 @@
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>2484.2</v>
+        <v>4097.9</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -2165,39 +2069,39 @@
         <v>25</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>174.3</v>
+        <v>655.8</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>0.5</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>1410</v>
+        <v>821.05</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>1455.2</v>
+        <v>844</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
@@ -2208,39 +2112,39 @@
         <v>25</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>135.6</v>
+        <v>252.45</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.028</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>0.46</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>690</v>
+        <v>2426.1</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>660.45</v>
+        <v>2484.2</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -2251,19 +2155,19 @@
         <v>25</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>-206.85</v>
+        <v>174.3</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.0239</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -2272,10 +2176,10 @@
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>1839</v>
+        <v>1410</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
@@ -2283,7 +2187,7 @@
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>1828.1</v>
+        <v>1455.2</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -2294,19 +2198,19 @@
         <v>25</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>-21.8</v>
+        <v>135.6</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>-0.0059</v>
+        <v>0.0321</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>-0.1</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
@@ -2315,10 +2219,10 @@
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>1414</v>
+        <v>690</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
@@ -2326,7 +2230,7 @@
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>1537.8</v>
+        <v>660.45</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -2337,19 +2241,19 @@
         <v>25</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>371.4</v>
+        <v>-206.85</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>0.0876</v>
+        <v>-0.0428</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>1.38</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
@@ -2358,10 +2262,10 @@
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>1300</v>
+        <v>1839</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
@@ -2369,7 +2273,7 @@
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>1389.1</v>
+        <v>1828.1</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -2380,19 +2284,19 @@
         <v>25</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>356.4</v>
+        <v>-21.8</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>-0.0059</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>0.63</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -2401,10 +2305,10 @@
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>276.45</v>
+        <v>1414</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
@@ -2412,7 +2316,7 @@
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>330.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -2423,19 +2327,19 @@
         <v>25</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>1019.35</v>
+        <v>371.4</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.0876</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>3.1</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -2444,10 +2348,10 @@
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>1462.5</v>
+        <v>1300</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
@@ -2455,7 +2359,7 @@
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>1564.7</v>
+        <v>1389.1</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -2466,19 +2370,19 @@
         <v>25</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>306.6</v>
+        <v>356.4</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>1.78</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
@@ -2487,41 +2391,41 @@
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>798</v>
+        <v>276.45</v>
       </c>
       <c r="D26" s="16" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>750</v>
+        <v>330.1</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H26" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I26" s="17" t="n">
-        <v>-288</v>
+        <v>1019.35</v>
       </c>
       <c r="J26" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.1941</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>-0.92</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
@@ -2530,53 +2434,53 @@
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>260.45</v>
+        <v>1462.5</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>257.85</v>
+        <v>1564.7</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H27" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>-52.07</v>
+        <v>306.6</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>-0.01</v>
+        <v>0.0699</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>-0.13</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>6500</v>
+        <v>798</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
@@ -2584,7 +2488,7 @@
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>6401.5</v>
+        <v>750</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
@@ -2592,34 +2496,34 @@
         </is>
       </c>
       <c r="H28" s="14" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I28" s="17" t="n">
-        <v>-98.5</v>
+        <v>-288</v>
       </c>
       <c r="J28" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.0602</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>571.5</v>
+        <v>260.45</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
@@ -2627,7 +2531,7 @@
         </is>
       </c>
       <c r="F29" s="15" t="n">
-        <v>571.1</v>
+        <v>257.85</v>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
@@ -2635,34 +2539,34 @@
         </is>
       </c>
       <c r="H29" s="14" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="I29" s="17" t="n">
-        <v>-6.4</v>
+        <v>-52.07</v>
       </c>
       <c r="J29" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.01</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C30" s="15" t="n">
-        <v>965</v>
+        <v>6500</v>
       </c>
       <c r="D30" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
@@ -2670,7 +2574,7 @@
         </is>
       </c>
       <c r="F30" s="15" t="n">
-        <v>933</v>
+        <v>6401.5</v>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
@@ -2678,22 +2582,22 @@
         </is>
       </c>
       <c r="H30" s="14" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="I30" s="17" t="n">
-        <v>-288</v>
+        <v>-98.5</v>
       </c>
       <c r="J30" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0152</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
@@ -2702,18 +2606,18 @@
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>5479</v>
+        <v>571.5</v>
       </c>
       <c r="D31" s="16" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F31" s="15" t="n">
-        <v>5424</v>
+        <v>571.1</v>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
@@ -2721,42 +2625,42 @@
         </is>
       </c>
       <c r="H31" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I31" s="17" t="n">
-        <v>-55</v>
+        <v>-6.4</v>
       </c>
       <c r="J31" s="18" t="n">
+        <v>-0.0007</v>
+      </c>
+      <c r="K31" s="19" t="n">
         <v>-0.01</v>
-      </c>
-      <c r="K31" s="19" t="n">
-        <v>-0.18</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C32" s="15" t="n">
-        <v>960.1</v>
+        <v>965</v>
       </c>
       <c r="D32" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F32" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>933</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
@@ -2764,42 +2668,42 @@
         </is>
       </c>
       <c r="H32" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I32" s="17" t="n">
-        <v>-516.79</v>
+        <v>-288</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.0332</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C33" s="15" t="n">
-        <v>952.1</v>
+        <v>5479</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F33" s="15" t="n">
-        <v>948.8</v>
+        <v>5424</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
@@ -2810,39 +2714,39 @@
         <v>1</v>
       </c>
       <c r="I33" s="17" t="n">
-        <v>-29.7</v>
+        <v>-55</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.01</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C34" s="15" t="n">
-        <v>1475</v>
+        <v>960.1</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F34" s="15" t="n">
-        <v>1394.19</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
@@ -2850,42 +2754,42 @@
         </is>
       </c>
       <c r="H34" s="14" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I34" s="17" t="n">
-        <v>-484.86</v>
+        <v>-516.79</v>
       </c>
       <c r="J34" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0598</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>-1</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C35" s="15" t="n">
-        <v>248.05</v>
+        <v>952.1</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E35" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F35" s="15" t="n">
-        <v>242.8</v>
+        <v>948.8</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
@@ -2893,42 +2797,42 @@
         </is>
       </c>
       <c r="H35" s="14" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I35" s="17" t="n">
-        <v>-110.25</v>
+        <v>-29.7</v>
       </c>
       <c r="J35" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0035</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>-0.3</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C36" s="15" t="n">
-        <v>1039.2</v>
+        <v>1475</v>
       </c>
       <c r="D36" s="16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F36" s="15" t="n">
-        <v>970</v>
+        <v>1394.19</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
@@ -2936,22 +2840,22 @@
         </is>
       </c>
       <c r="H36" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I36" s="17" t="n">
-        <v>-346</v>
+        <v>-484.86</v>
       </c>
       <c r="J36" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0548</v>
       </c>
       <c r="K36" s="19" t="n">
-        <v>-0.82</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
@@ -2960,10 +2864,10 @@
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>199.96</v>
+        <v>248.05</v>
       </c>
       <c r="D37" s="16" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E37" s="14" t="inlineStr">
         <is>
@@ -2971,7 +2875,7 @@
         </is>
       </c>
       <c r="F37" s="15" t="n">
-        <v>193.31</v>
+        <v>242.8</v>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
@@ -2982,19 +2886,19 @@
         <v>11</v>
       </c>
       <c r="I37" s="17" t="n">
-        <v>-172.9</v>
+        <v>-110.25</v>
       </c>
       <c r="J37" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.0212</v>
       </c>
       <c r="K37" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
@@ -3003,7 +2907,7 @@
         </is>
       </c>
       <c r="C38" s="15" t="n">
-        <v>986.4</v>
+        <v>1039.2</v>
       </c>
       <c r="D38" s="16" t="n">
         <v>5</v>
@@ -3014,7 +2918,7 @@
         </is>
       </c>
       <c r="F38" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>970</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
@@ -3025,17 +2929,103 @@
         <v>11</v>
       </c>
       <c r="I38" s="17" t="n">
+        <v>-346</v>
+      </c>
+      <c r="J38" s="18" t="n">
+        <v>-0.06660000000000001</v>
+      </c>
+      <c r="K38" s="19" t="n">
+        <v>-0.82</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="n">
+        <v>199.96</v>
+      </c>
+      <c r="D39" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F39" s="15" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="G39" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H39" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I39" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J39" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K39" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C40" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D40" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F40" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G40" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H40" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I40" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J38" s="18" t="n">
+      <c r="J40" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K38" s="19" t="n">
+      <c r="K40" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I38">
+  <conditionalFormatting sqref="I2:I40">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3053,7 +3043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3875,6 +3865,31 @@
       </c>
       <c r="G32" s="14" t="n">
         <v>12</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B33" s="20" t="n">
+        <v>203935.04</v>
+      </c>
+      <c r="C33" s="20" t="n">
+        <v>144743.34</v>
+      </c>
+      <c r="D33" s="20" t="n">
+        <v>59191.7</v>
+      </c>
+      <c r="E33" s="20" t="n">
+        <v>57145.1</v>
+      </c>
+      <c r="F33" s="20" t="n">
+        <v>1888.44</v>
+      </c>
+      <c r="G33" s="14" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -3957,18 +3972,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>333.75</v>
+        <v>1816.2</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>319.94</v>
+        <v>1729.14</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -3977,10 +3992,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8262442396313364</v>
+        <v>0.8015982404692081</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -3995,18 +4010,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1781.3</v>
+        <v>2199.8</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1694.96</v>
+        <v>2105.19</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -4015,10 +4030,10 @@
         <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8038081273565145</v>
+        <v>0.8044742354419774</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -4033,18 +4048,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>8988</v>
+        <v>1696.5</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>8746.709999999999</v>
+        <v>1616.13</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -4056,7 +4071,7 @@
         <v>6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8015731043150398</v>
+        <v>0.7782509426057813</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4071,18 +4086,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1520.6</v>
+        <v>4591</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1446.5</v>
+        <v>4349.36</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -4094,7 +4109,7 @@
         <v>5.9</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8286730205278592</v>
+        <v>0.8061028487641391</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -4109,18 +4124,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>4366.6</v>
+        <v>1405.6</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>4142.76</v>
+        <v>1330.26</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -4132,7 +4147,7 @@
         <v>5.9</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7692930456640135</v>
+        <v>0.8100764558022622</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -4147,18 +4162,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>2746.2</v>
+        <v>1525.4</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>2630.03</v>
+        <v>1445.97</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -4170,7 +4185,7 @@
         <v>5.9</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7549172601591957</v>
+        <v>0.831400293255132</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -4185,18 +4200,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1664.1</v>
+        <v>8957</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1589.03</v>
+        <v>8724.57</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -4208,7 +4223,7 @@
         <v>5.9</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.762263301214914</v>
+        <v>0.7831954335986595</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -4223,18 +4238,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>SYRMA</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1377.8</v>
+        <v>333.4</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1263.87</v>
+        <v>319.33</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -4246,7 +4261,7 @@
         <v>5.9</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7438322161709259</v>
+        <v>0.777866568914956</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -4261,18 +4276,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1576.3</v>
+        <v>2469.6</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1505.96</v>
+        <v>2320.51</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -4281,10 +4296,10 @@
         <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7729765395894428</v>
+        <v>0.7708829074151655</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -4299,18 +4314,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1629.9</v>
+        <v>1990.5</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1561.74</v>
+        <v>1924.37</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -4319,10 +4334,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7629587348135735</v>
+        <v>0.7555927943024717</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -4337,7 +4352,7 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
@@ -4345,10 +4360,10 @@
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>885.35</v>
+        <v>870.65</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>852.79</v>
+        <v>836.71</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -4357,10 +4372,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7557415165479682</v>
+        <v>0.7653812316715543</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -4375,18 +4390,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1416.4</v>
+        <v>863.4</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1349.1</v>
+        <v>804.5700000000001</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -4395,10 +4410,10 @@
         <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7732268537913699</v>
+        <v>0.7366296606619187</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -4413,18 +4428,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1315.2</v>
+        <v>1098.5</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1250.2</v>
+        <v>1050.96</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -4433,10 +4448,10 @@
         <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7602031839128613</v>
+        <v>0.7388531629660662</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -4451,18 +4466,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>KAJARIACER</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>7386.5</v>
+        <v>1198.3</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>7003.5</v>
+        <v>1136.63</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -4474,7 +4489,7 @@
         <v>5.6</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7405310012568077</v>
+        <v>0.7502806870548806</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -4489,7 +4504,7 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260730</v>
+        <v>20260731</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
@@ -4497,10 +4512,10 @@
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>445.95</v>
+        <v>449.55</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>416.01</v>
+        <v>420.41</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -4509,10 +4524,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.740736279849183</v>
+        <v>0.7441767909509845</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-08-03
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Fri 31 Jul 2026</t>
+          <t>As of Mon 03 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹203,935</t>
+          <t>₹204,458</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+310  (+0.15%)</t>
+          <t>₹+522  (+0.26%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.97%</t>
+          <t>+2.23%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.05%</t>
+          <t>-0.80%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹144,743</t>
+          <t>₹121,711</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹57,145</t>
+          <t>₹80,177</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹59,192</t>
+          <t>₹82,746</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -844,31 +844,31 @@
         <v>8883</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1315.1</v>
+        <v>1333.4</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9205.699999999999</v>
+        <v>9333.800000000001</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>322.6999999999994</v>
+        <v>450.8000000000006</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.03632781717888094</v>
+        <v>0.05074862096138699</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1182.49</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>1218.4</v>
+        <v>1235.064285714286</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.07353052999771867</v>
+        <v>0.07374809830937033</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>39.97</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>8847</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>9106.5</v>
+        <v>9034</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9106.5</v>
+        <v>9034</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>259.5</v>
+        <v>187</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.02933197694133605</v>
+        <v>0.02113710862439245</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8315.07</v>
@@ -910,13 +910,13 @@
         <v>8791</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.03464558282545434</v>
+        <v>0.02689838388310826</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>254.57</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>4874.4</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1816.2</v>
+        <v>1811.4</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>5448.6</v>
+        <v>5434.200000000001</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>574.2000000000003</v>
+        <v>559.8000000000004</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.1177991137370754</v>
+        <v>0.1148449039881832</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1520.16</v>
@@ -958,13 +958,13 @@
         <v>1685.614285714286</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.07190051441785814</v>
+        <v>0.06944115837789223</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>45.45</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>4766.7</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1611.4</v>
+        <v>1642.5</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4834.200000000001</v>
+        <v>4927.5</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>67.5</v>
+        <v>160.7999999999997</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.01416074013468437</v>
+        <v>0.03373402983195916</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1499.44</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1537.1</v>
+        <v>1541.164285714286</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.04610897356336116</v>
+        <v>0.061696020874103</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>37.96</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -1036,31 +1036,31 @@
         <v>4237.8</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1473.2</v>
+        <v>1474.4</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>4419.6</v>
+        <v>4423.200000000001</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>181.8000000000004</v>
+        <v>185.4000000000005</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.04289961772617878</v>
+        <v>0.04374911510689522</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1342.97</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1372.342857142857</v>
+        <v>1373.064285714286</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.06846126992746598</v>
+        <v>0.06873013719866684</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>33.28</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>3897</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1990.5</v>
+        <v>1963.5</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>3981</v>
+        <v>3927</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>84</v>
+        <v>30</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.02155504234026174</v>
+        <v>0.007698229407236336</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1876.83</v>
@@ -1102,13 +1102,13 @@
         <v>1914.142857142857</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.03836078515807229</v>
+        <v>0.02513732765833608</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>33.4</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -1132,31 +1132,31 @@
         <v>5101.6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>769.4</v>
+        <v>785</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5385.8</v>
+        <v>5495</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>284.2000000000002</v>
+        <v>393.4000000000003</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.05570801317233812</v>
+        <v>0.07711306256860599</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>676.71</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>703.0999999999999</v>
+        <v>718.0464285714286</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.08617104237067855</v>
+        <v>0.08529117379435849</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>20.64</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>4120</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4340.8</v>
+        <v>4459.1</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4340.8</v>
+        <v>4459.1</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>220.8000000000002</v>
+        <v>339.1000000000004</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.05359223300970879</v>
+        <v>0.08230582524271854</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>3924.44</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>4053.142857142857</v>
+        <v>4121.021428571429</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.066268232320573</v>
+        <v>0.07581766980524572</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>85.14</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>5172</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>870.65</v>
+        <v>880.95</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5223.9</v>
+        <v>5285.700000000001</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>51.89999999999986</v>
+        <v>113.7000000000003</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.01003480278422271</v>
+        <v>0.02198375870069611</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>823.7</v>
@@ -1246,17 +1246,257 @@
         <v>836.5035714285714</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.03921946657259358</v>
+        <v>0.0504528390617273</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>15.94</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>BHARATFORG</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>2218</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>4436</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>2211</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>4422</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>-14</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>-0.003155996393146979</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>2105.19</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>2105.19</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>0.04785617367706917</v>
+      </c>
+      <c r="M12" s="13" t="n">
+        <v>46.56</v>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>1713.4</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>5140.2</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>1701</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>5103</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>-37.20000000000027</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>-0.007237072487451902</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>1616.13</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>1616.13</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>0.04989417989417983</v>
+      </c>
+      <c r="M13" s="13" t="n">
+        <v>39.53</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>AIAENG</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>4568</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>4568</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>4684.6</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>4684.6</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>116.6000000000004</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>0.02552539404553423</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>4349.36</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>4349.36</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>0.07156213977714226</v>
+      </c>
+      <c r="M14" s="13" t="n">
+        <v>130.39</v>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>MEDANTA</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>1412.6</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>4237.8</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>1444.9</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>4334.700000000001</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>96.90000000000055</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>0.02286563783095015</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>1330.26</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>1330.26</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>0.079341130874109</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>40.91</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>RAINBOW</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>1550</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>4650</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>1545.6</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>4636.799999999999</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>-13.20000000000027</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>-0.002838709677419414</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>1445.97</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>1445.97</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0.064460403726708</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>40.54</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H11">
+  <conditionalFormatting sqref="H2:H16">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3043,7 +3283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3890,6 +4130,31 @@
       </c>
       <c r="G33" s="14" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B34" s="20" t="n">
+        <v>204457.54</v>
+      </c>
+      <c r="C34" s="20" t="n">
+        <v>121711.34</v>
+      </c>
+      <c r="D34" s="20" t="n">
+        <v>82746.2</v>
+      </c>
+      <c r="E34" s="20" t="n">
+        <v>80177.10000000001</v>
+      </c>
+      <c r="F34" s="20" t="n">
+        <v>1888.44</v>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -3972,18 +4237,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1816.2</v>
+        <v>1554.7</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1729.14</v>
+        <v>1483.96</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -3992,10 +4257,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8015982404692081</v>
+        <v>0.8300146627565982</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -4010,18 +4275,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>2199.8</v>
+        <v>8820</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>2105.19</v>
+        <v>8576.209999999999</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -4030,10 +4295,10 @@
         <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8044742354419774</v>
+        <v>0.825852534562212</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -4048,18 +4313,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1696.5</v>
+        <v>1545.6</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1616.13</v>
+        <v>1464.53</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -4068,10 +4333,10 @@
         <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7782509426057813</v>
+        <v>0.8276152073732719</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4086,18 +4351,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>4591</v>
+        <v>1444.9</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>4349.36</v>
+        <v>1363.07</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -4109,7 +4374,7 @@
         <v>5.9</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8061028487641391</v>
+        <v>0.8028822790113113</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -4124,18 +4389,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1405.6</v>
+        <v>344.9</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1330.26</v>
+        <v>330.13</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -4147,7 +4412,7 @@
         <v>5.9</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8100764558022622</v>
+        <v>0.7910483870967742</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -4162,18 +4427,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1525.4</v>
+        <v>1811.4</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1445.97</v>
+        <v>1720.74</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -4185,7 +4450,7 @@
         <v>5.9</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.831400293255132</v>
+        <v>0.7816296606619187</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -4200,18 +4465,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>8957</v>
+        <v>1963.5</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>8724.57</v>
+        <v>1895.3</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -4223,7 +4488,7 @@
         <v>5.9</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7831954335986595</v>
+        <v>0.7540647255969837</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -4238,18 +4503,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>333.4</v>
+        <v>8585</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>319.33</v>
+        <v>8189.57</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -4261,7 +4526,7 @@
         <v>5.9</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.777866568914956</v>
+        <v>0.744024926686217</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -4276,18 +4541,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>2469.6</v>
+        <v>2393</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>2320.51</v>
+        <v>2276.17</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -4296,10 +4561,10 @@
         <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7708829074151655</v>
+        <v>0.7528341013824885</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -4314,18 +4579,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1990.5</v>
+        <v>880.95</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1924.37</v>
+        <v>846.0700000000001</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -4334,10 +4599,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7555927943024717</v>
+        <v>0.7402869710934228</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -4352,18 +4617,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>870.65</v>
+        <v>2211</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>836.71</v>
+        <v>2117.87</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -4372,10 +4637,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7653812316715543</v>
+        <v>0.7553990364474235</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -4390,18 +4655,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>863.4</v>
+        <v>940</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>804.5700000000001</v>
+        <v>902.99</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -4413,7 +4678,7 @@
         <v>5.7</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7366296606619187</v>
+        <v>0.7544093003770422</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -4428,18 +4693,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1098.5</v>
+        <v>458.2</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1050.96</v>
+        <v>428.51</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -4448,10 +4713,10 @@
         <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7388531629660662</v>
+        <v>0.7632677000418936</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -4466,18 +4731,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>KAJARIACER</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1198.3</v>
+        <v>1333.4</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1136.63</v>
+        <v>1267.84</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -4489,7 +4754,7 @@
         <v>5.6</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7502806870548806</v>
+        <v>0.7604461667364892</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -4504,18 +4769,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260731</v>
+        <v>20260803</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>449.55</v>
+        <v>727.6</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>420.41</v>
+        <v>688.25</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -4527,7 +4792,7 @@
         <v>5.5</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7441767909509845</v>
+        <v>0.7393475073313784</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-08-04
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Mon 03 Aug 2026</t>
+          <t>As of Tue 04 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹204,458</t>
+          <t>₹204,804</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+522  (+0.26%)</t>
+          <t>₹+347  (+0.17%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.23%</t>
+          <t>+2.40%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.80%</t>
+          <t>-0.63%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹82,746</t>
+          <t>₹83,093</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
@@ -844,31 +844,31 @@
         <v>8883</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1333.4</v>
+        <v>1366.4</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9333.800000000001</v>
+        <v>9564.800000000001</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>450.8000000000006</v>
+        <v>681.8000000000006</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.05074862096138699</v>
+        <v>0.07675334909377469</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1182.49</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>1235.064285714286</v>
+        <v>1262.214285714286</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.07374809830937033</v>
+        <v>0.07624832719973236</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>39.97</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>8847</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>9034</v>
+        <v>9176</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9034</v>
+        <v>9176</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>187</v>
+        <v>329</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.02113710862439245</v>
+        <v>0.03718774725895784</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8315.07</v>
@@ -910,13 +910,13 @@
         <v>8791</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.02689838388310826</v>
+        <v>0.04195727986050567</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>254.57</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>4874.4</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1811.4</v>
+        <v>1850</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>5434.200000000001</v>
+        <v>5550</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>559.8000000000004</v>
+        <v>675.6000000000001</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.1148449039881832</v>
+        <v>0.1386016740521911</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1520.16</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1685.614285714286</v>
+        <v>1710.95</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.06944115837789223</v>
+        <v>0.07516216216216214</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>45.45</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>4766.7</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1642.5</v>
+        <v>1620</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4927.5</v>
+        <v>4860</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>160.7999999999997</v>
+        <v>93.29999999999973</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.03373402983195916</v>
+        <v>0.01957328969727479</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1499.44</v>
@@ -1006,13 +1006,13 @@
         <v>1541.164285714286</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.061696020874103</v>
+        <v>0.0486640211640211</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>37.96</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>4237.8</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1474.4</v>
+        <v>1460</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>4423.200000000001</v>
+        <v>4380</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>185.4000000000005</v>
+        <v>142.2000000000003</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.04374911510689522</v>
+        <v>0.03355514653829824</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1342.97</v>
@@ -1054,13 +1054,13 @@
         <v>1373.064285714286</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.06873013719866684</v>
+        <v>0.05954500978473583</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>33.28</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>3897</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1963.5</v>
+        <v>1964</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>3927</v>
+        <v>3928</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.007698229407236336</v>
+        <v>0.007954837054144213</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1876.83</v>
@@ -1102,13 +1102,13 @@
         <v>1914.142857142857</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.02513732765833608</v>
+        <v>0.02538551061972652</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>33.4</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -1132,31 +1132,31 @@
         <v>5101.6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5495</v>
+        <v>5509</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>393.4000000000003</v>
+        <v>407.4000000000003</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.07711306256860599</v>
+        <v>0.07985729967069162</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>676.71</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>718.0464285714286</v>
+        <v>718.4928571428571</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.08529117379435849</v>
+        <v>0.08704846614630606</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>20.64</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>4120</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4459.1</v>
+        <v>4450</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4459.1</v>
+        <v>4450</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>339.1000000000004</v>
+        <v>330</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.08230582524271854</v>
+        <v>0.08009708737864078</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>3924.44</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>4121.021428571429</v>
+        <v>4121.085714285715</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.07581766980524572</v>
+        <v>0.07391332263242363</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>85.14</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>5172</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>880.95</v>
+        <v>875</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5285.700000000001</v>
+        <v>5250</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>113.7000000000003</v>
+        <v>78</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.02198375870069611</v>
+        <v>0.01508120649651972</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>823.7</v>
@@ -1246,13 +1246,13 @@
         <v>836.5035714285714</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.0504528390617273</v>
+        <v>0.043995918367347</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>15.94</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4436</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>2211</v>
+        <v>2195</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4422</v>
+        <v>4390</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-14</v>
+        <v>-46</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.003155996393146979</v>
+        <v>-0.01036970243462579</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>2105.19</v>
@@ -1294,13 +1294,13 @@
         <v>2105.19</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.04785617367706917</v>
+        <v>0.0409157175398633</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>46.56</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1324,31 +1324,31 @@
         <v>5140.2</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1701</v>
+        <v>1706.7</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>5103</v>
+        <v>5120.1</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-37.20000000000027</v>
+        <v>-20.10000000000014</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.007237072487451902</v>
+        <v>-0.003910353682736106</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1616.13</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>1616.13</v>
+        <v>1650</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.04989417989417983</v>
+        <v>0.03322200738266833</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>39.53</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1372,31 +1372,31 @@
         <v>4568</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>4684.6</v>
+        <v>4627</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4684.6</v>
+        <v>4627</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>116.6000000000004</v>
+        <v>59</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.02552539404553423</v>
+        <v>0.01291593695271454</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>4349.36</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>4349.36</v>
+        <v>4460</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.07156213977714226</v>
+        <v>0.0360925005403069</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>130.39</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>4237.8</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1444.9</v>
+        <v>1435.1</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>4334.700000000001</v>
+        <v>4305.299999999999</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>96.90000000000055</v>
+        <v>67.5</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.02286563783095015</v>
+        <v>0.01592807588843268</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>1330.26</v>
@@ -1438,13 +1438,13 @@
         <v>1330.26</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.079341130874109</v>
+        <v>0.07305414256846207</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>40.91</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1468,31 +1468,31 @@
         <v>4650</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>1545.6</v>
+        <v>1579</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>4636.799999999999</v>
+        <v>4737</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>-13.20000000000027</v>
+        <v>87</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>-0.002838709677419414</v>
+        <v>0.01870967741935484</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>1445.97</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>1445.97</v>
+        <v>1455.378571428571</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.064460403726708</v>
+        <v>0.07829096172984713</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>40.54</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3283,7 +3283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4154,6 +4154,31 @@
         <v>1888.44</v>
       </c>
       <c r="G34" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B35" s="20" t="n">
+        <v>204804.14</v>
+      </c>
+      <c r="C35" s="20" t="n">
+        <v>121711.34</v>
+      </c>
+      <c r="D35" s="20" t="n">
+        <v>83092.8</v>
+      </c>
+      <c r="E35" s="20" t="n">
+        <v>80177.10000000001</v>
+      </c>
+      <c r="F35" s="20" t="n">
+        <v>1888.44</v>
+      </c>
+      <c r="G35" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4237,7 +4262,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -4245,22 +4270,22 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1554.7</v>
+        <v>1585.9</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1483.96</v>
+        <v>1510.96</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.2</v>
+        <v>7.7</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8300146627565982</v>
+        <v>0.8316286133221618</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -4269,36 +4294,36 @@
       </c>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>8820</v>
+        <v>1620</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>8576.209999999999</v>
+        <v>1550.29</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.1</v>
+        <v>7.6</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.825852534562212</v>
+        <v>0.806587767071638</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -4307,36 +4332,36 @@
       </c>
       <c r="J3" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1545.6</v>
+        <v>9050</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1464.53</v>
+        <v>8780.290000000001</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>5.9</v>
+        <v>7.6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8276152073732719</v>
+        <v>0.8239243820695434</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4345,36 +4370,36 @@
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1444.9</v>
+        <v>459.4</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1363.07</v>
+        <v>429.08</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>5.9</v>
+        <v>7.5</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8028822790113113</v>
+        <v>0.824874319229158</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -4383,36 +4408,36 @@
       </c>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>344.9</v>
+        <v>1579</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>330.13</v>
+        <v>1496.59</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>5.9</v>
+        <v>7.5</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7910483870967742</v>
+        <v>0.8479681608713866</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -4421,36 +4446,36 @@
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1811.4</v>
+        <v>342.5</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1720.74</v>
+        <v>327.46</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.9</v>
+        <v>7.4</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7816296606619187</v>
+        <v>0.7843401759530793</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -4459,36 +4484,36 @@
       </c>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1963.5</v>
+        <v>8378</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1895.3</v>
+        <v>7953.93</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.9</v>
+        <v>7.3</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7540647255969837</v>
+        <v>0.7379671135316297</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -4497,36 +4522,36 @@
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>8585</v>
+        <v>591.2</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>8189.57</v>
+        <v>559.25</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.9</v>
+        <v>7.2</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.744024926686217</v>
+        <v>0.7876948051948053</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -4535,36 +4560,36 @@
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>2393</v>
+        <v>1366.4</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>2276.17</v>
+        <v>1296.94</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.8</v>
+        <v>7.2</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7528341013824885</v>
+        <v>0.7712767071638039</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -4573,36 +4598,36 @@
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>880.95</v>
+        <v>2195</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>846.0700000000001</v>
+        <v>2104.6</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.7</v>
+        <v>7.2</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7402869710934228</v>
+        <v>0.7528990364474236</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -4611,36 +4636,36 @@
       </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>2211</v>
+        <v>7629</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>2117.87</v>
+        <v>7207.79</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.7</v>
+        <v>7.2</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7553990364474235</v>
+        <v>0.7545747800586511</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -4649,36 +4674,36 @@
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>940</v>
+        <v>2410</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>902.99</v>
+        <v>2294.29</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.7</v>
+        <v>7.2</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7544093003770422</v>
+        <v>0.7369564306661082</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -4687,36 +4712,36 @@
       </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>458.2</v>
+        <v>1694.7</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>428.51</v>
+        <v>1577.39</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.6</v>
+        <v>7.1</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7632677000418936</v>
+        <v>0.76329702555509</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -4725,36 +4750,36 @@
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1333.4</v>
+        <v>825.7</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1267.84</v>
+        <v>768.47</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.6</v>
+        <v>7.1</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7604461667364892</v>
+        <v>0.7538395475492249</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -4763,36 +4788,36 @@
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260803</v>
+        <v>20260804</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>727.6</v>
+        <v>932.8</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>688.25</v>
+        <v>895.87</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0667</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>5333</v>
+        <v>13333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.5</v>
+        <v>7.1</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7393475073313784</v>
+        <v>0.744879555927943</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>
@@ -4801,7 +4826,7 @@
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>RISK_OFF</t>
+          <t>RISK_ON</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V5 daily refresh 2026-08-05
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Tue 04 Aug 2026</t>
+          <t>As of Wed 05 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹204,804</t>
+          <t>₹205,205</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+347  (+0.17%)</t>
+          <t>₹+401  (+0.20%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.40%</t>
+          <t>+2.60%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.63%</t>
+          <t>-0.43%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹83,093</t>
+          <t>₹83,494</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
@@ -844,31 +844,31 @@
         <v>8883</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1366.4</v>
+        <v>1394.3</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9564.800000000001</v>
+        <v>9760.1</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>681.8000000000006</v>
+        <v>877.0999999999997</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.07675334909377469</v>
+        <v>0.09873916469661147</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1182.49</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>1262.214285714286</v>
+        <v>1290.628571428571</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.07624832719973236</v>
+        <v>0.07435374637554944</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>39.97</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>8847</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>9176</v>
+        <v>9200</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9176</v>
+        <v>9200</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>329</v>
+        <v>353</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.03718774725895784</v>
+        <v>0.03990053125353227</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8315.07</v>
@@ -910,13 +910,13 @@
         <v>8791</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.04195727986050567</v>
+        <v>0.04445652173913044</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>254.57</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>4874.4</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1850</v>
+        <v>1835</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>5550</v>
+        <v>5505</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>675.6000000000001</v>
+        <v>630.6000000000001</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.1386016740521911</v>
+        <v>0.129369768586903</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1520.16</v>
@@ -958,13 +958,13 @@
         <v>1710.95</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.07516216216216214</v>
+        <v>0.06760217983651223</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>45.45</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>4766.7</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1620</v>
+        <v>1665</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4860</v>
+        <v>4995</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>93.29999999999973</v>
+        <v>228.2999999999997</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.01957328969727479</v>
+        <v>0.04789476996664353</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1499.44</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1541.164285714286</v>
+        <v>1555.2</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.0486640211640211</v>
+        <v>0.06594594594594592</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>37.96</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>4237.8</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1460</v>
+        <v>1458.8</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>4380</v>
+        <v>4376.4</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>142.2000000000003</v>
+        <v>138.6000000000001</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.03355514653829824</v>
+        <v>0.0327056491575818</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1342.97</v>
@@ -1054,13 +1054,13 @@
         <v>1373.064285714286</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.05954500978473583</v>
+        <v>0.0587713972345176</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>33.28</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>3897</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1964</v>
+        <v>1940</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>3928</v>
+        <v>3880</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>31</v>
+        <v>-17</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.007954837054144213</v>
+        <v>-0.004362329997433924</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1876.83</v>
@@ -1102,13 +1102,13 @@
         <v>1914.142857142857</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.02538551061972652</v>
+        <v>0.01332842415316644</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>33.4</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -1132,31 +1132,31 @@
         <v>5101.6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>787</v>
+        <v>814.6</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5509</v>
+        <v>5702.2</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>407.4000000000003</v>
+        <v>600.6000000000005</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.07985729967069162</v>
+        <v>0.1177277716794732</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>676.71</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>718.4928571428571</v>
+        <v>743.3392857142857</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.08704846614630606</v>
+        <v>0.08747939391813694</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>20.64</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>4120</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4450</v>
+        <v>4550</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4450</v>
+        <v>4550</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>330</v>
+        <v>430</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.08009708737864078</v>
+        <v>0.1043689320388349</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>3924.44</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>4121.085714285715</v>
+        <v>4194.607142857143</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.07391332263242363</v>
+        <v>0.07810832025117734</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>85.14</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>5172</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>875</v>
+        <v>852</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5250</v>
+        <v>5112</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>78</v>
+        <v>-60</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.01508120649651972</v>
+        <v>-0.01160092807424594</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>823.7</v>
@@ -1246,13 +1246,13 @@
         <v>836.5035714285714</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.043995918367347</v>
+        <v>0.01818829644533876</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>15.94</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4436</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>2195</v>
+        <v>2197.1</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4390</v>
+        <v>4394.2</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-46</v>
+        <v>-41.80000000000018</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.01036970243462579</v>
+        <v>-0.009422903516681735</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>2105.19</v>
@@ -1294,13 +1294,13 @@
         <v>2105.19</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.0409157175398633</v>
+        <v>0.04183241545673836</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>46.56</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>5140.2</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1706.7</v>
+        <v>1700</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>5120.1</v>
+        <v>5100</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-20.10000000000014</v>
+        <v>-40.20000000000027</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.003910353682736106</v>
+        <v>-0.007820707365472213</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1616.13</v>
@@ -1342,13 +1342,13 @@
         <v>1650</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.03322200738266833</v>
+        <v>0.02941176470588235</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>39.53</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>4568</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>4627</v>
+        <v>4646.6</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4627</v>
+        <v>4646.6</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>59</v>
+        <v>78.60000000000036</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.01291593695271454</v>
+        <v>0.01720665499124351</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>4349.36</v>
@@ -1390,13 +1390,13 @@
         <v>4460</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.0360925005403069</v>
+        <v>0.04015839538587362</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>130.39</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>4237.8</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1435.1</v>
+        <v>1410.3</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>4305.299999999999</v>
+        <v>4230.9</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>67.5</v>
+        <v>-6.899999999999864</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.01592807588843268</v>
+        <v>-0.001628203313039753</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>1330.26</v>
@@ -1438,13 +1438,13 @@
         <v>1330.26</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.07305414256846207</v>
+        <v>0.05675388215273344</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>40.91</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -1468,31 +1468,31 @@
         <v>4650</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>1579</v>
+        <v>1598.6</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>4737</v>
+        <v>4795.799999999999</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>87</v>
+        <v>145.7999999999997</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.01870967741935484</v>
+        <v>0.03135483870967736</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>1445.97</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>1455.378571428571</v>
+        <v>1470.071428571428</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.07829096172984713</v>
+        <v>0.08040070776214905</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>40.54</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -3283,7 +3283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4179,6 +4179,31 @@
         <v>1888.44</v>
       </c>
       <c r="G35" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B36" s="20" t="n">
+        <v>205205.14</v>
+      </c>
+      <c r="C36" s="20" t="n">
+        <v>121711.34</v>
+      </c>
+      <c r="D36" s="20" t="n">
+        <v>83493.8</v>
+      </c>
+      <c r="E36" s="20" t="n">
+        <v>80177.10000000001</v>
+      </c>
+      <c r="F36" s="20" t="n">
+        <v>1888.44</v>
+      </c>
+      <c r="G36" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4262,18 +4287,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1585.9</v>
+        <v>335.35</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1510.96</v>
+        <v>318.48</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0667</v>
@@ -4282,10 +4307,10 @@
         <v>13333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7.7</v>
+        <v>8</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8316286133221618</v>
+        <v>0.8663699204021785</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -4300,18 +4325,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1620</v>
+        <v>1598.6</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1550.29</v>
+        <v>1512.91</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0667</v>
@@ -4323,7 +4348,7 @@
         <v>7.6</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.806587767071638</v>
+        <v>0.8488144113950564</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -4338,7 +4363,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
@@ -4346,10 +4371,10 @@
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>9050</v>
+        <v>8910</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>8780.290000000001</v>
+        <v>8620.709999999999</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0667</v>
@@ -4361,7 +4386,7 @@
         <v>7.6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8239243820695434</v>
+        <v>0.818289694176791</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4376,18 +4401,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>459.4</v>
+        <v>1613.4</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>429.08</v>
+        <v>1533.37</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0667</v>
@@ -4396,10 +4421,10 @@
         <v>13333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.824874319229158</v>
+        <v>0.8121617092584835</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -4414,18 +4439,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1579</v>
+        <v>4550</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1496.59</v>
+        <v>4313.07</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0667</v>
@@ -4437,7 +4462,7 @@
         <v>7.5</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8479681608713866</v>
+        <v>0.8020213657310431</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -4452,18 +4477,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>342.5</v>
+        <v>1665</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>327.46</v>
+        <v>1591.8</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0667</v>
@@ -4472,10 +4497,10 @@
         <v>13333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>7.4</v>
+        <v>7.5</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7843401759530793</v>
+        <v>0.7939390448261416</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -4490,18 +4515,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>8378</v>
+        <v>1835</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>7953.93</v>
+        <v>1741.67</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0667</v>
@@ -4510,10 +4535,10 @@
         <v>13333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7379671135316297</v>
+        <v>0.7879775869291998</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -4528,18 +4553,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>591.2</v>
+        <v>852</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>559.25</v>
+        <v>811.64</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0667</v>
@@ -4548,10 +4573,10 @@
         <v>13333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7876948051948053</v>
+        <v>0.7874895266024299</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -4566,18 +4591,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1366.4</v>
+        <v>2388</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1296.94</v>
+        <v>2270</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0667</v>
@@ -4586,10 +4611,10 @@
         <v>13333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7712767071638039</v>
+        <v>0.7790647255969836</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -4604,18 +4629,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>2195</v>
+        <v>1765</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>2104.6</v>
+        <v>1640.06</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0667</v>
@@ -4624,10 +4649,10 @@
         <v>13333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7528990364474236</v>
+        <v>0.7892846669459572</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -4642,18 +4667,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>7629</v>
+        <v>925</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>7207.79</v>
+        <v>888.11</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0667</v>
@@ -4662,10 +4687,10 @@
         <v>13333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7545747800586511</v>
+        <v>0.7665018852115626</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -4680,18 +4705,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>2410</v>
+        <v>2197.1</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>2294.29</v>
+        <v>2106.54</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0667</v>
@@ -4703,7 +4728,7 @@
         <v>7.2</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7369564306661082</v>
+        <v>0.7599602010892332</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -4718,18 +4743,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1694.7</v>
+        <v>814.6</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1577.39</v>
+        <v>767.09</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0667</v>
@@ -4738,10 +4763,10 @@
         <v>13333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.76329702555509</v>
+        <v>0.7389327607875995</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -4756,18 +4781,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>825.7</v>
+        <v>584.1</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>768.47</v>
+        <v>551.5</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0667</v>
@@ -4776,10 +4801,10 @@
         <v>13333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7538395475492249</v>
+        <v>0.7574204021784667</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -4794,18 +4819,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260804</v>
+        <v>20260805</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>932.8</v>
+        <v>459.65</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>895.87</v>
+        <v>430.02</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0667</v>
@@ -4814,10 +4839,10 @@
         <v>13333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.744879555927943</v>
+        <v>0.7396470465018852</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-08-07
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Wed 05 Aug 2026</t>
+          <t>As of Fri 07 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹205,205</t>
+          <t>₹205,347</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+401  (+0.20%)</t>
+          <t>₹+142  (+0.07%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.60%</t>
+          <t>+2.67%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.43%</t>
+          <t>-0.36%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹121,711</t>
+          <t>₹131,268</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹80,177</t>
+          <t>₹71,294</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹83,494</t>
+          <t>₹74,079</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+1,888</t>
+          <t>₹+2,562</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,109 +820,109 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>1269</v>
+        <v>8847</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>8883</v>
+        <v>8847</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1394.3</v>
+        <v>9218</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9760.1</v>
+        <v>9218</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>877.0999999999997</v>
+        <v>371</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.09873916469661147</v>
+        <v>0.0419351192494631</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>1182.49</v>
+        <v>8315.07</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>1290.628571428571</v>
+        <v>8791</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.07435374637554944</v>
+        <v>0.04632241267086136</v>
       </c>
       <c r="M3" s="13" t="n">
-        <v>39.97</v>
+        <v>254.57</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>8847</v>
+        <v>1624.8</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>8847</v>
+        <v>4874.4</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>9200</v>
+        <v>1844.3</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9200</v>
+        <v>5532.9</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>353</v>
+        <v>658.5</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.03990053125353227</v>
+        <v>0.1350935499753816</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>8315.07</v>
+        <v>1520.16</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>8791</v>
+        <v>1717.442857142857</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.04445652173913044</v>
+        <v>0.06878335566726829</v>
       </c>
       <c r="M4" s="13" t="n">
-        <v>254.57</v>
+        <v>45.45</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -931,46 +931,46 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>1624.8</v>
+        <v>1588.9</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>4874.4</v>
+        <v>4766.7</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1835</v>
+        <v>1660</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>5505</v>
+        <v>4980</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>630.6000000000001</v>
+        <v>213.2999999999997</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.129369768586903</v>
+        <v>0.04474793882560256</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>1520.16</v>
+        <v>1499.44</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1710.95</v>
+        <v>1555.2</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.06760217983651223</v>
+        <v>0.06313253012048189</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>45.45</v>
+        <v>37.96</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -979,46 +979,46 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>1588.9</v>
+        <v>1412.6</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>4766.7</v>
+        <v>4237.8</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1665</v>
+        <v>1463.8</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4995</v>
+        <v>4391.4</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>228.2999999999997</v>
+        <v>153.6000000000001</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.04789476996664353</v>
+        <v>0.03624522157723351</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>1499.44</v>
+        <v>1342.97</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1555.2</v>
+        <v>1378.742857142857</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.06594594594594592</v>
+        <v>0.05810707942146653</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>37.96</v>
+        <v>33.28</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -1027,46 +1027,46 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>1412.6</v>
+        <v>1948.5</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>4237.8</v>
+        <v>3897</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1458.8</v>
+        <v>1945</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>4376.4</v>
+        <v>3890</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>138.6000000000001</v>
+        <v>-7</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.0327056491575818</v>
+        <v>-0.001796253528355145</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>1342.97</v>
+        <v>1876.83</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1373.064285714286</v>
+        <v>1914.142857142857</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.0587713972345176</v>
+        <v>0.01586485493940509</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>33.28</v>
+        <v>33.4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -1075,46 +1075,46 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>1948.5</v>
+        <v>728.8</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>3897</v>
+        <v>5101.6</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1940</v>
+        <v>818.05</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>3880</v>
+        <v>5726.349999999999</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>-17</v>
+        <v>624.75</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>-0.004362329997433924</v>
+        <v>0.1224615806805708</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>1876.83</v>
+        <v>676.71</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>1914.142857142857</v>
+        <v>743.3392857142857</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.01332842415316644</v>
+        <v>0.09132780916290482</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>33.4</v>
+        <v>20.64</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -1123,46 +1123,46 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>728.8</v>
+        <v>4120</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>5101.6</v>
+        <v>4120</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>814.6</v>
+        <v>4499</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5702.2</v>
+        <v>4499</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>600.6000000000005</v>
+        <v>379</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.1177277716794732</v>
+        <v>0.09199029126213593</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>676.71</v>
+        <v>3924.44</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>743.3392857142857</v>
+        <v>4194.607142857143</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.08747939391813694</v>
+        <v>0.06765789223001931</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>20.64</v>
+        <v>85.14</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1171,94 +1171,94 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>4120</v>
+        <v>862</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>4120</v>
+        <v>5172</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4550</v>
+        <v>862</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4550</v>
+        <v>5172</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>430</v>
+        <v>0</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.1043689320388349</v>
+        <v>0</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>3924.44</v>
+        <v>823.7</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>4194.607142857143</v>
+        <v>836.5035714285714</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.07810832025117734</v>
+        <v>0.02957822340072926</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>85.14</v>
+        <v>15.94</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>862</v>
+        <v>2218</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>5172</v>
+        <v>4436</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>852</v>
+        <v>2265.2</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5112</v>
+        <v>4530.4</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-60</v>
+        <v>94.39999999999964</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>-0.01160092807424594</v>
+        <v>0.02128043282236241</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>823.7</v>
+        <v>2105.19</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>836.5035714285714</v>
+        <v>2132.814285714285</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.01818829644533876</v>
+        <v>0.05844327842385443</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>15.94</v>
+        <v>46.56</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1267,46 +1267,46 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>2218</v>
+        <v>1713.4</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>4436</v>
+        <v>5140.2</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>2197.1</v>
+        <v>1693.5</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4394.2</v>
+        <v>5080.5</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-41.80000000000018</v>
+        <v>-59.70000000000027</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.009422903516681735</v>
+        <v>-0.01161433407260423</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>2105.19</v>
+        <v>1616.13</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>2105.19</v>
+        <v>1650</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.04183241545673836</v>
+        <v>0.02568644818423383</v>
       </c>
       <c r="M12" s="13" t="n">
-        <v>46.56</v>
+        <v>39.53</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -1315,46 +1315,46 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>1713.4</v>
+        <v>4568</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>5140.2</v>
+        <v>4568</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1700</v>
+        <v>4776</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>5100</v>
+        <v>4776</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-40.20000000000027</v>
+        <v>208</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.007820707365472213</v>
+        <v>0.04553415061295972</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>1616.13</v>
+        <v>4349.36</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>1650</v>
+        <v>4460</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.02941176470588235</v>
+        <v>0.0661641541038526</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>39.53</v>
+        <v>130.39</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1363,46 +1363,46 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>4568</v>
+        <v>1412.6</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>4568</v>
+        <v>4237.8</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>4646.6</v>
+        <v>1455.6</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4646.6</v>
+        <v>4366.799999999999</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>78.60000000000036</v>
+        <v>129</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.01720665499124351</v>
+        <v>0.03044032280900467</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>4349.36</v>
+        <v>1330.26</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>4460</v>
+        <v>1330.26</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.04015839538587362</v>
+        <v>0.08610882110469904</v>
       </c>
       <c r="M14" s="13" t="n">
-        <v>130.39</v>
+        <v>40.91</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
@@ -1411,92 +1411,44 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>1412.6</v>
+        <v>1550</v>
       </c>
       <c r="D15" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>4237.8</v>
+        <v>4650</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1410.3</v>
+        <v>1556.7</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>4230.9</v>
+        <v>4670.1</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>-6.899999999999864</v>
+        <v>20.10000000000014</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>-0.001628203313039753</v>
+        <v>0.00432258064516132</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>1330.26</v>
+        <v>1445.97</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>1330.26</v>
+        <v>1470.071428571428</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.05675388215273344</v>
+        <v>0.05564885426130378</v>
       </c>
       <c r="M15" s="13" t="n">
-        <v>40.91</v>
+        <v>40.54</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>RAINBOW</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>1550</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <v>4650</v>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>1598.6</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>4795.799999999999</v>
-      </c>
-      <c r="H16" s="10" t="n">
-        <v>145.7999999999997</v>
-      </c>
-      <c r="I16" s="11" t="n">
-        <v>0.03135483870967736</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>1445.97</v>
-      </c>
-      <c r="K16" s="7" t="n">
-        <v>1470.071428571428</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>0.08040070776214905</v>
-      </c>
-      <c r="M16" s="13" t="n">
-        <v>40.54</v>
-      </c>
-      <c r="N16" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H16">
+  <conditionalFormatting sqref="H2:H15">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1514,7 +1466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1590,27 +1542,27 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>7579.5</v>
+        <v>1269</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>7567.5</v>
+        <v>1365.2</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -1621,19 +1573,19 @@
         <v>25</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-12</v>
+        <v>673.4</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0016</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-0.03</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -1642,10 +1594,10 @@
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>1798.5</v>
+        <v>7579.5</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
@@ -1653,7 +1605,7 @@
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>1747.8</v>
+        <v>7567.5</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -1664,74 +1616,74 @@
         <v>25</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-253.5</v>
+        <v>-12</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0282</v>
+        <v>-0.0016</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-0.43</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>5438</v>
+        <v>1798.5</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>5381</v>
+        <v>1747.8</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-57</v>
+        <v>-253.5</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0105</v>
+        <v>-0.0282</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>1784</v>
+        <v>5438</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
@@ -1739,7 +1691,7 @@
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>1752.1</v>
+        <v>5381</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1747,22 +1699,22 @@
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-63.8</v>
+        <v>-57</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.0179</v>
+        <v>-0.0105</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-0.36</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -1771,18 +1723,18 @@
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>871.8</v>
+        <v>1784</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>830.15</v>
+        <v>1752.1</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -1790,65 +1742,65 @@
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>-249.9</v>
+        <v>-63.8</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>-0.0478</v>
+        <v>-0.0179</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>-0.73</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>420.3</v>
+        <v>871.8</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>448.6</v>
+        <v>830.15</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>622.6</v>
+        <v>-249.9</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>0.0673</v>
+        <v>-0.0478</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>0.84</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -1857,10 +1809,10 @@
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>1465</v>
+        <v>420.3</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
@@ -1868,7 +1820,7 @@
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>1596.9</v>
+        <v>448.6</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -1879,19 +1831,19 @@
         <v>25</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>791.4</v>
+        <v>622.6</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>0.09</v>
+        <v>0.0673</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>1.32</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -1900,10 +1852,10 @@
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>619.25</v>
+        <v>1465</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
@@ -1911,7 +1863,7 @@
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>717.95</v>
+        <v>1596.9</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
@@ -1922,19 +1874,19 @@
         <v>25</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>1480.5</v>
+        <v>791.4</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>0.1594</v>
+        <v>0.09</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>3.55</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -1943,10 +1895,10 @@
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>8700</v>
+        <v>619.25</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
@@ -1954,7 +1906,7 @@
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>8805.5</v>
+        <v>717.95</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
@@ -1965,31 +1917,31 @@
         <v>25</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>105.5</v>
+        <v>1480.5</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>0.0121</v>
+        <v>0.1594</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>0.29</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>961.85</v>
+        <v>8700</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
@@ -1997,42 +1949,42 @@
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>935.6</v>
+        <v>8805.5</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H11" s="14" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>-236.25</v>
+        <v>105.5</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>-0.0273</v>
+        <v>0.0121</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>-0.64</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>1560</v>
+        <v>961.85</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
@@ -2040,7 +1992,7 @@
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>1547.4</v>
+        <v>935.6</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -2048,42 +2000,42 @@
         </is>
       </c>
       <c r="H12" s="14" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>-63</v>
+        <v>-236.25</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>-0.0081</v>
+        <v>-0.0273</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>-0.23</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>900</v>
+        <v>1560</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>887.1</v>
+        <v>1547.4</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
@@ -2091,42 +2043,42 @@
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>-129</v>
+        <v>-63</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>-0.0143</v>
+        <v>-0.0081</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.23</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>880.8</v>
+        <v>900</v>
       </c>
       <c r="D14" s="16" t="n">
         <v>10</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>832.9400000000001</v>
+        <v>887.1</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
@@ -2134,22 +2086,22 @@
         </is>
       </c>
       <c r="H14" s="14" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>-478.6</v>
+        <v>-129</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>-0.0543</v>
+        <v>-0.0143</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>-1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -2158,10 +2110,10 @@
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>777</v>
+        <v>880.8</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
@@ -2169,7 +2121,7 @@
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>744.8</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
@@ -2180,10 +2132,10 @@
         <v>2</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>-386.4</v>
+        <v>-478.6</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>-0.0414</v>
+        <v>-0.0543</v>
       </c>
       <c r="K15" s="19" t="n">
         <v>-1</v>
@@ -2192,27 +2144,27 @@
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>1114.9</v>
+        <v>777</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>1050.57</v>
+        <v>744.8</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
@@ -2220,13 +2172,13 @@
         </is>
       </c>
       <c r="H16" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>-514.64</v>
+        <v>-386.4</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>-0.0577</v>
+        <v>-0.0414</v>
       </c>
       <c r="K16" s="19" t="n">
         <v>-1</v>
@@ -2235,50 +2187,50 @@
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>790</v>
+        <v>1114.9</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>880.8</v>
+        <v>1050.57</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H17" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>998.8</v>
+        <v>-514.64</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0577</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -2287,10 +2239,10 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>3770</v>
+        <v>790</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
@@ -2298,7 +2250,7 @@
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>4097.9</v>
+        <v>880.8</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -2309,19 +2261,19 @@
         <v>25</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>655.8</v>
+        <v>998.8</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.1149</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>1.98</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -2330,10 +2282,10 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>821.05</v>
+        <v>3770</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
@@ -2341,7 +2293,7 @@
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>844</v>
+        <v>4097.9</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
@@ -2352,19 +2304,19 @@
         <v>25</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>252.45</v>
+        <v>655.8</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>0.028</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>0.6</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -2373,10 +2325,10 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>2426.1</v>
+        <v>821.05</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
@@ -2384,7 +2336,7 @@
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>2484.2</v>
+        <v>844</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -2395,39 +2347,39 @@
         <v>25</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>174.3</v>
+        <v>252.45</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.028</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>1410</v>
+        <v>2426.1</v>
       </c>
       <c r="D21" s="16" t="n">
         <v>3</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>1455.2</v>
+        <v>2484.2</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -2438,19 +2390,19 @@
         <v>25</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>135.6</v>
+        <v>174.3</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.0239</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>0.46</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
@@ -2459,10 +2411,10 @@
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>690</v>
+        <v>1410</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
@@ -2470,7 +2422,7 @@
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>660.45</v>
+        <v>1455.2</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -2481,19 +2433,19 @@
         <v>25</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>-206.85</v>
+        <v>135.6</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.0321</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
@@ -2502,10 +2454,10 @@
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>1839</v>
+        <v>690</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
@@ -2513,7 +2465,7 @@
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>1828.1</v>
+        <v>660.45</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -2524,19 +2476,19 @@
         <v>25</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>-21.8</v>
+        <v>-206.85</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>-0.0059</v>
+        <v>-0.0428</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>-0.1</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -2545,10 +2497,10 @@
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>1414</v>
+        <v>1839</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
@@ -2556,7 +2508,7 @@
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>1537.8</v>
+        <v>1828.1</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -2567,19 +2519,19 @@
         <v>25</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>371.4</v>
+        <v>-21.8</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>0.0876</v>
+        <v>-0.0059</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>1.38</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -2588,10 +2540,10 @@
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>1300</v>
+        <v>1414</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
@@ -2599,7 +2551,7 @@
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>1389.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -2610,19 +2562,19 @@
         <v>25</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>356.4</v>
+        <v>371.4</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>0.0876</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>0.63</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
@@ -2631,10 +2583,10 @@
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>276.45</v>
+        <v>1300</v>
       </c>
       <c r="D26" s="16" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
@@ -2642,7 +2594,7 @@
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>330.1</v>
+        <v>1389.1</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
@@ -2653,19 +2605,19 @@
         <v>25</v>
       </c>
       <c r="I26" s="17" t="n">
-        <v>1019.35</v>
+        <v>356.4</v>
       </c>
       <c r="J26" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>3.1</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
@@ -2674,10 +2626,10 @@
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>1462.5</v>
+        <v>276.45</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
@@ -2685,7 +2637,7 @@
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>1564.7</v>
+        <v>330.1</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
@@ -2696,19 +2648,19 @@
         <v>25</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>306.6</v>
+        <v>1019.35</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.1941</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>1.78</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
@@ -2717,41 +2669,41 @@
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>798</v>
+        <v>1462.5</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>750</v>
+        <v>1564.7</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H28" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I28" s="17" t="n">
-        <v>-288</v>
+        <v>306.6</v>
       </c>
       <c r="J28" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.0699</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>-0.92</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -2760,10 +2712,10 @@
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>260.45</v>
+        <v>798</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
@@ -2771,7 +2723,7 @@
         </is>
       </c>
       <c r="F29" s="15" t="n">
-        <v>257.85</v>
+        <v>750</v>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
@@ -2782,31 +2734,31 @@
         <v>23</v>
       </c>
       <c r="I29" s="17" t="n">
-        <v>-52.07</v>
+        <v>-288</v>
       </c>
       <c r="J29" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0602</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>-0.13</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C30" s="15" t="n">
-        <v>6500</v>
+        <v>260.45</v>
       </c>
       <c r="D30" s="16" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
@@ -2814,7 +2766,7 @@
         </is>
       </c>
       <c r="F30" s="15" t="n">
-        <v>6401.5</v>
+        <v>257.85</v>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
@@ -2822,65 +2774,65 @@
         </is>
       </c>
       <c r="H30" s="14" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I30" s="17" t="n">
-        <v>-98.5</v>
+        <v>-52.07</v>
       </c>
       <c r="J30" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.01</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>571.5</v>
+        <v>6500</v>
       </c>
       <c r="D31" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="F31" s="15" t="n">
+        <v>6401.5</v>
+      </c>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H31" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="E31" s="14" t="inlineStr">
-        <is>
-          <t>2026-07-08</t>
-        </is>
-      </c>
-      <c r="F31" s="15" t="n">
-        <v>571.1</v>
-      </c>
-      <c r="G31" s="14" t="inlineStr">
-        <is>
-          <t>STOP_LOSS</t>
-        </is>
-      </c>
-      <c r="H31" s="14" t="n">
-        <v>2</v>
-      </c>
       <c r="I31" s="17" t="n">
-        <v>-6.4</v>
+        <v>-98.5</v>
       </c>
       <c r="J31" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.0152</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
@@ -2889,10 +2841,10 @@
         </is>
       </c>
       <c r="C32" s="15" t="n">
-        <v>965</v>
+        <v>571.5</v>
       </c>
       <c r="D32" s="16" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
@@ -2900,7 +2852,7 @@
         </is>
       </c>
       <c r="F32" s="15" t="n">
-        <v>933</v>
+        <v>571.1</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
@@ -2911,19 +2863,19 @@
         <v>2</v>
       </c>
       <c r="I32" s="17" t="n">
-        <v>-288</v>
+        <v>-6.4</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0007</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
@@ -2932,18 +2884,18 @@
         </is>
       </c>
       <c r="C33" s="15" t="n">
-        <v>5479</v>
+        <v>965</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F33" s="15" t="n">
-        <v>5424</v>
+        <v>933</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
@@ -2951,42 +2903,42 @@
         </is>
       </c>
       <c r="H33" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I33" s="17" t="n">
-        <v>-55</v>
+        <v>-288</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0332</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>-0.18</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C34" s="15" t="n">
-        <v>960.1</v>
+        <v>5479</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F34" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>5424</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
@@ -2994,22 +2946,22 @@
         </is>
       </c>
       <c r="H34" s="14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I34" s="17" t="n">
-        <v>-516.79</v>
+        <v>-55</v>
       </c>
       <c r="J34" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.01</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
@@ -3018,18 +2970,18 @@
         </is>
       </c>
       <c r="C35" s="15" t="n">
-        <v>952.1</v>
+        <v>960.1</v>
       </c>
       <c r="D35" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E35" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F35" s="15" t="n">
-        <v>948.8</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
@@ -3037,42 +2989,42 @@
         </is>
       </c>
       <c r="H35" s="14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I35" s="17" t="n">
-        <v>-29.7</v>
+        <v>-516.79</v>
       </c>
       <c r="J35" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.0598</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C36" s="15" t="n">
-        <v>1475</v>
+        <v>952.1</v>
       </c>
       <c r="D36" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F36" s="15" t="n">
-        <v>1394.19</v>
+        <v>948.8</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
@@ -3080,42 +3032,42 @@
         </is>
       </c>
       <c r="H36" s="14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I36" s="17" t="n">
-        <v>-484.86</v>
+        <v>-29.7</v>
       </c>
       <c r="J36" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0035</v>
       </c>
       <c r="K36" s="19" t="n">
-        <v>-1</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>248.05</v>
+        <v>1475</v>
       </c>
       <c r="D37" s="16" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E37" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F37" s="15" t="n">
-        <v>242.8</v>
+        <v>1394.19</v>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
@@ -3123,22 +3075,22 @@
         </is>
       </c>
       <c r="H37" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I37" s="17" t="n">
-        <v>-110.25</v>
+        <v>-484.86</v>
       </c>
       <c r="J37" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0548</v>
       </c>
       <c r="K37" s="19" t="n">
-        <v>-0.3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
@@ -3147,10 +3099,10 @@
         </is>
       </c>
       <c r="C38" s="15" t="n">
-        <v>1039.2</v>
+        <v>248.05</v>
       </c>
       <c r="D38" s="16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
@@ -3158,7 +3110,7 @@
         </is>
       </c>
       <c r="F38" s="15" t="n">
-        <v>970</v>
+        <v>242.8</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
@@ -3169,19 +3121,19 @@
         <v>11</v>
       </c>
       <c r="I38" s="17" t="n">
-        <v>-346</v>
+        <v>-110.25</v>
       </c>
       <c r="J38" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="K38" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
@@ -3190,10 +3142,10 @@
         </is>
       </c>
       <c r="C39" s="15" t="n">
-        <v>199.96</v>
+        <v>1039.2</v>
       </c>
       <c r="D39" s="16" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="E39" s="14" t="inlineStr">
         <is>
@@ -3201,7 +3153,7 @@
         </is>
       </c>
       <c r="F39" s="15" t="n">
-        <v>193.31</v>
+        <v>970</v>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
@@ -3212,19 +3164,19 @@
         <v>11</v>
       </c>
       <c r="I39" s="17" t="n">
-        <v>-172.9</v>
+        <v>-346</v>
       </c>
       <c r="J39" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.06660000000000001</v>
       </c>
       <c r="K39" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
@@ -3233,10 +3185,10 @@
         </is>
       </c>
       <c r="C40" s="15" t="n">
-        <v>986.4</v>
+        <v>199.96</v>
       </c>
       <c r="D40" s="16" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="E40" s="14" t="inlineStr">
         <is>
@@ -3244,7 +3196,7 @@
         </is>
       </c>
       <c r="F40" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>193.31</v>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
@@ -3255,17 +3207,60 @@
         <v>11</v>
       </c>
       <c r="I40" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J40" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K40" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D41" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F41" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G41" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H41" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I41" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J40" s="18" t="n">
+      <c r="J41" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K40" s="19" t="n">
+      <c r="K41" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I40">
+  <conditionalFormatting sqref="I2:I41">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3283,7 +3278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4205,6 +4200,31 @@
       </c>
       <c r="G36" s="14" t="n">
         <v>15</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B37" s="20" t="n">
+        <v>205346.79</v>
+      </c>
+      <c r="C37" s="20" t="n">
+        <v>131267.74</v>
+      </c>
+      <c r="D37" s="20" t="n">
+        <v>74079.05</v>
+      </c>
+      <c r="E37" s="20" t="n">
+        <v>71294.10000000001</v>
+      </c>
+      <c r="F37" s="20" t="n">
+        <v>2561.84</v>
+      </c>
+      <c r="G37" s="14" t="n">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -4287,18 +4307,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>335.35</v>
+        <v>2363.5</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>318.48</v>
+        <v>2250.39</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0667</v>
@@ -4307,10 +4327,10 @@
         <v>13333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>8</v>
+        <v>7.7</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8663699204021785</v>
+        <v>0.8238531629660661</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -4325,18 +4345,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1598.6</v>
+        <v>8945</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1512.91</v>
+        <v>8673.639999999999</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0667</v>
@@ -4348,7 +4368,7 @@
         <v>7.6</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8488144113950564</v>
+        <v>0.8277178466694597</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -4363,18 +4383,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>8910</v>
+        <v>873.85</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>8620.709999999999</v>
+        <v>814.59</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0667</v>
@@ -4386,7 +4406,7 @@
         <v>7.6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.818289694176791</v>
+        <v>0.8350387515710096</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4401,18 +4421,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1613.4</v>
+        <v>2265.2</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1533.37</v>
+        <v>2176.94</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0667</v>
@@ -4424,7 +4444,7 @@
         <v>7.6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8121617092584835</v>
+        <v>0.8088940092165898</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -4439,18 +4459,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>4550</v>
+        <v>1365.2</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>4313.07</v>
+        <v>1282.14</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0667</v>
@@ -4462,7 +4482,7 @@
         <v>7.5</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8020213657310431</v>
+        <v>0.8073428990364474</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -4477,18 +4497,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1665</v>
+        <v>1658</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1591.8</v>
+        <v>1569.16</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0667</v>
@@ -4500,7 +4520,7 @@
         <v>7.5</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7939390448261416</v>
+        <v>0.7919658567239213</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -4515,18 +4535,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1835</v>
+        <v>1556.7</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1741.67</v>
+        <v>1467.07</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0667</v>
@@ -4535,10 +4555,10 @@
         <v>13333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7879775869291998</v>
+        <v>0.8413625890238794</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -4553,18 +4573,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>852</v>
+        <v>1455.6</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>811.64</v>
+        <v>1363</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0667</v>
@@ -4573,10 +4593,10 @@
         <v>13333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7874895266024299</v>
+        <v>0.8128037285295349</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -4591,18 +4611,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>2388</v>
+        <v>477.6</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>2270</v>
+        <v>449.67</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0667</v>
@@ -4614,7 +4634,7 @@
         <v>7.4</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7790647255969836</v>
+        <v>0.8217396313364055</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -4629,18 +4649,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1765</v>
+        <v>1844.3</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1640.06</v>
+        <v>1755.93</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0667</v>
@@ -4649,10 +4669,10 @@
         <v>13333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7892846669459572</v>
+        <v>0.7719040636782573</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -4667,18 +4687,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>925</v>
+        <v>332</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>888.11</v>
+        <v>315.2</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0667</v>
@@ -4690,7 +4710,7 @@
         <v>7.3</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7665018852115626</v>
+        <v>0.782130289065773</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -4705,18 +4725,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>2197.1</v>
+        <v>1945</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>2106.54</v>
+        <v>1872.67</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0667</v>
@@ -4728,7 +4748,7 @@
         <v>7.2</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7599602010892332</v>
+        <v>0.7320192710515291</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -4743,18 +4763,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>814.6</v>
+        <v>4499</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>767.09</v>
+        <v>4253.81</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0667</v>
@@ -4763,10 +4783,10 @@
         <v>13333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7389327607875995</v>
+        <v>0.7397957687473816</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -4781,18 +4801,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>584.1</v>
+        <v>4776</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>551.5</v>
+        <v>4507.71</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0667</v>
@@ -4801,10 +4821,10 @@
         <v>13333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7574204021784667</v>
+        <v>0.7359614578969418</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -4819,18 +4839,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260805</v>
+        <v>20260807</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>459.65</v>
+        <v>721.65</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>430.02</v>
+        <v>678.91</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0667</v>
@@ -4839,10 +4859,10 @@
         <v>13333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7396470465018852</v>
+        <v>0.7292302052785924</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-08-10
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Fri 07 Aug 2026</t>
+          <t>As of Mon 10 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹205,347</t>
+          <t>₹204,926</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+142  (+0.07%)</t>
+          <t>₹-421  (-0.20%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.67%</t>
+          <t>+2.46%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.36%</t>
+          <t>-0.57%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹131,268</t>
+          <t>₹114,788</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹71,294</t>
+          <t>₹87,603</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹74,079</t>
+          <t>₹90,138</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+2,562</t>
+          <t>₹+2,391</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8847</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>9218</v>
+        <v>9275</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9218</v>
+        <v>9275</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>371</v>
+        <v>428</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.0419351192494631</v>
+        <v>0.04837798123657737</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8315.07</v>
@@ -862,13 +862,13 @@
         <v>8791</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.04632241267086136</v>
+        <v>0.0521832884097035</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>254.57</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -892,31 +892,31 @@
         <v>4874.4</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1844.3</v>
+        <v>1854</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>5532.9</v>
+        <v>5562</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>658.5</v>
+        <v>687.6000000000001</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.1350935499753816</v>
+        <v>0.1410635155096012</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1520.16</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1717.442857142857</v>
+        <v>1722.535714285714</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.06878335566726829</v>
+        <v>0.07090846047156731</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>45.45</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>4766.7</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1660</v>
+        <v>1685</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>4980</v>
+        <v>5055</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>213.2999999999997</v>
+        <v>288.2999999999997</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.04474793882560256</v>
+        <v>0.06048209453080742</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1499.44</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1555.2</v>
+        <v>1568.428571428571</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.06313253012048189</v>
+        <v>0.0691818567189489</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>37.96</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>4237.8</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1463.8</v>
+        <v>1467.7</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4391.4</v>
+        <v>4403.1</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>153.6000000000001</v>
+        <v>165.3000000000004</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.03624522157723351</v>
+        <v>0.0390060880645619</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1342.97</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1378.742857142857</v>
+        <v>1380.5</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.05810707942146653</v>
+        <v>0.05941268651631808</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>33.28</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>3897</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1945</v>
+        <v>1944.4</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>3890</v>
+        <v>3888.8</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-7</v>
+        <v>-8.199999999999818</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.001796253528355145</v>
+        <v>-0.002104182704644552</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1876.83</v>
@@ -1054,13 +1054,13 @@
         <v>1914.142857142857</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.01586485493940509</v>
+        <v>0.01556117201046234</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>33.4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>5101.6</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>818.05</v>
+        <v>812.5</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5726.349999999999</v>
+        <v>5687.5</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>624.75</v>
+        <v>585.9000000000003</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.1224615806805708</v>
+        <v>0.1148463227222833</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>676.71</v>
@@ -1102,13 +1102,13 @@
         <v>743.3392857142857</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.09132780916290482</v>
+        <v>0.08512087912087918</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>20.64</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>4120</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>4499</v>
+        <v>4550</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4499</v>
+        <v>4550</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>379</v>
+        <v>430</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.09199029126213593</v>
+        <v>0.1043689320388349</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>3924.44</v>
@@ -1150,13 +1150,13 @@
         <v>4194.607142857143</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.06765789223001931</v>
+        <v>0.07810832025117734</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>85.14</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>5172</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>862</v>
+        <v>863.5</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>5172</v>
+        <v>5181</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0</v>
+        <v>0.001740139211136891</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>823.7</v>
@@ -1198,19 +1198,19 @@
         <v>836.5035714285714</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.02957822340072926</v>
+        <v>0.0312639589709654</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>15.94</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -1219,46 +1219,46 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>2218</v>
+        <v>1713.4</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>4436</v>
+        <v>5140.2</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>2265.2</v>
+        <v>1681</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>4530.4</v>
+        <v>5043</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>94.39999999999964</v>
+        <v>-97.20000000000027</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.02128043282236241</v>
+        <v>-0.01890977004785811</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>2105.19</v>
+        <v>1616.13</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>2132.814285714285</v>
+        <v>1650</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.05844327842385443</v>
+        <v>0.01844140392623438</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>46.56</v>
+        <v>39.53</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1267,46 +1267,46 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>1713.4</v>
+        <v>4568</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>5140.2</v>
+        <v>4568</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>1693.5</v>
+        <v>4790.3</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>5080.5</v>
+        <v>4790.3</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-59.70000000000027</v>
+        <v>222.3000000000002</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.01161433407260423</v>
+        <v>0.04866462346760074</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>1616.13</v>
+        <v>4349.36</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>1650</v>
+        <v>4460</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.02568644818423383</v>
+        <v>0.06895184017702444</v>
       </c>
       <c r="M12" s="13" t="n">
-        <v>39.53</v>
+        <v>130.39</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -1315,46 +1315,46 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>4568</v>
+        <v>1412.6</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>4568</v>
+        <v>4237.8</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>4776</v>
+        <v>1476.2</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>4776</v>
+        <v>4428.6</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>208</v>
+        <v>190.8000000000004</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.04553415061295972</v>
+        <v>0.0450233611779698</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>4349.36</v>
+        <v>1330.26</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>4460</v>
+        <v>1335.778571428572</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.0661641541038526</v>
+        <v>0.0951235798478718</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>130.39</v>
+        <v>40.91</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1363,92 +1363,140 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>1412.6</v>
+        <v>1550</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>4237.8</v>
+        <v>4650</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1455.6</v>
+        <v>1538.6</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4366.799999999999</v>
+        <v>4615.799999999999</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>129</v>
+        <v>-34.20000000000027</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.03044032280900467</v>
+        <v>-0.007354838709677478</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>1330.26</v>
+        <v>1445.97</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>1330.26</v>
+        <v>1470.071428571428</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.08610882110469904</v>
+        <v>0.04453956286791334</v>
       </c>
       <c r="M14" s="13" t="n">
-        <v>40.91</v>
+        <v>40.54</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>1550</v>
+        <v>2360</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>4650</v>
+        <v>11800</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1556.7</v>
+        <v>2300</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>4670.1</v>
+        <v>11500</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>20.10000000000014</v>
+        <v>-300</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.00432258064516132</v>
+        <v>-0.02542372881355932</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>1445.97</v>
+        <v>2250.39</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>1470.071428571428</v>
+        <v>2250.39</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.05564885426130378</v>
+        <v>0.02156956521739136</v>
       </c>
       <c r="M15" s="13" t="n">
-        <v>40.54</v>
+        <v>62.34</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>4</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>8945</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>8945</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>8912</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>8912</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>-33</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>-0.00368921185019564</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>8673.639999999999</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>8673.639999999999</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0.02674596050269306</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>138.54</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H15">
+  <conditionalFormatting sqref="H2:H16">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1466,7 +1514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1542,70 +1590,70 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>1269</v>
+        <v>2218</v>
       </c>
       <c r="D2" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="n">
+        <v>2132.81</v>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="E2" s="14" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="F2" s="15" t="n">
-        <v>1365.2</v>
-      </c>
-      <c r="G2" s="14" t="inlineStr">
-        <is>
-          <t>TIME_STOP</t>
-        </is>
-      </c>
-      <c r="H2" s="14" t="n">
-        <v>25</v>
-      </c>
       <c r="I2" s="17" t="n">
-        <v>673.4</v>
+        <v>-170.37</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>0.07580000000000001</v>
+        <v>-0.0384</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>1.11</v>
+        <v>-0.76</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>7579.5</v>
+        <v>1269</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>7567.5</v>
+        <v>1365.2</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -1616,19 +1664,19 @@
         <v>25</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-12</v>
+        <v>673.4</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0016</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-0.03</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -1637,10 +1685,10 @@
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>1798.5</v>
+        <v>7579.5</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
@@ -1648,7 +1696,7 @@
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>1747.8</v>
+        <v>7567.5</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1659,74 +1707,74 @@
         <v>25</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-253.5</v>
+        <v>-12</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0282</v>
+        <v>-0.0016</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-0.43</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>5438</v>
+        <v>1798.5</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>5381</v>
+        <v>1747.8</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-57</v>
+        <v>-253.5</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.0105</v>
+        <v>-0.0282</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>1784</v>
+        <v>5438</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -1734,7 +1782,7 @@
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>1752.1</v>
+        <v>5381</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -1742,22 +1790,22 @@
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>-63.8</v>
+        <v>-57</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>-0.0179</v>
+        <v>-0.0105</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>-0.36</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -1766,18 +1814,18 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>871.8</v>
+        <v>1784</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>830.15</v>
+        <v>1752.1</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -1785,65 +1833,65 @@
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>-249.9</v>
+        <v>-63.8</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>-0.0478</v>
+        <v>-0.0179</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>-0.73</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>420.3</v>
+        <v>871.8</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>448.6</v>
+        <v>830.15</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>622.6</v>
+        <v>-249.9</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>0.0673</v>
+        <v>-0.0478</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>0.84</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -1852,10 +1900,10 @@
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>1465</v>
+        <v>420.3</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
@@ -1863,7 +1911,7 @@
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>1596.9</v>
+        <v>448.6</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
@@ -1874,19 +1922,19 @@
         <v>25</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>791.4</v>
+        <v>622.6</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>0.09</v>
+        <v>0.0673</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>1.32</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -1895,10 +1943,10 @@
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>619.25</v>
+        <v>1465</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
@@ -1906,7 +1954,7 @@
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>717.95</v>
+        <v>1596.9</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
@@ -1917,19 +1965,19 @@
         <v>25</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>1480.5</v>
+        <v>791.4</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>0.1594</v>
+        <v>0.09</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>3.55</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -1938,10 +1986,10 @@
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>8700</v>
+        <v>619.25</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
@@ -1949,7 +1997,7 @@
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>8805.5</v>
+        <v>717.95</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
@@ -1960,31 +2008,31 @@
         <v>25</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>105.5</v>
+        <v>1480.5</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>0.0121</v>
+        <v>0.1594</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>0.29</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>961.85</v>
+        <v>8700</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
@@ -1992,42 +2040,42 @@
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>935.6</v>
+        <v>8805.5</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H12" s="14" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>-236.25</v>
+        <v>105.5</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>-0.0273</v>
+        <v>0.0121</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>-0.64</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>1560</v>
+        <v>961.85</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
@@ -2035,7 +2083,7 @@
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>1547.4</v>
+        <v>935.6</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
@@ -2043,42 +2091,42 @@
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>-63</v>
+        <v>-236.25</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>-0.0081</v>
+        <v>-0.0273</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>-0.23</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>900</v>
+        <v>1560</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>887.1</v>
+        <v>1547.4</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
@@ -2086,42 +2134,42 @@
         </is>
       </c>
       <c r="H14" s="14" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>-129</v>
+        <v>-63</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>-0.0143</v>
+        <v>-0.0081</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.23</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>880.8</v>
+        <v>900</v>
       </c>
       <c r="D15" s="16" t="n">
         <v>10</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>832.9400000000001</v>
+        <v>887.1</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
@@ -2129,22 +2177,22 @@
         </is>
       </c>
       <c r="H15" s="14" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>-478.6</v>
+        <v>-129</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>-0.0543</v>
+        <v>-0.0143</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>-1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -2153,10 +2201,10 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>777</v>
+        <v>880.8</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
@@ -2164,7 +2212,7 @@
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>744.8</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
@@ -2175,10 +2223,10 @@
         <v>2</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>-386.4</v>
+        <v>-478.6</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>-0.0414</v>
+        <v>-0.0543</v>
       </c>
       <c r="K16" s="19" t="n">
         <v>-1</v>
@@ -2187,27 +2235,27 @@
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>1114.9</v>
+        <v>777</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>1050.57</v>
+        <v>744.8</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -2215,13 +2263,13 @@
         </is>
       </c>
       <c r="H17" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>-514.64</v>
+        <v>-386.4</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>-0.0577</v>
+        <v>-0.0414</v>
       </c>
       <c r="K17" s="19" t="n">
         <v>-1</v>
@@ -2230,50 +2278,50 @@
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>790</v>
+        <v>1114.9</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>880.8</v>
+        <v>1050.57</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H18" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>998.8</v>
+        <v>-514.64</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0577</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -2282,10 +2330,10 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>3770</v>
+        <v>790</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
@@ -2293,7 +2341,7 @@
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>4097.9</v>
+        <v>880.8</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
@@ -2304,19 +2352,19 @@
         <v>25</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>655.8</v>
+        <v>998.8</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.1149</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>1.98</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -2325,10 +2373,10 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>821.05</v>
+        <v>3770</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
@@ -2336,7 +2384,7 @@
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>844</v>
+        <v>4097.9</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -2347,19 +2395,19 @@
         <v>25</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>252.45</v>
+        <v>655.8</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>0.028</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>0.6</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -2368,10 +2416,10 @@
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>2426.1</v>
+        <v>821.05</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
@@ -2379,7 +2427,7 @@
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>2484.2</v>
+        <v>844</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -2390,39 +2438,39 @@
         <v>25</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>174.3</v>
+        <v>252.45</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.028</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>1410</v>
+        <v>2426.1</v>
       </c>
       <c r="D22" s="16" t="n">
         <v>3</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>1455.2</v>
+        <v>2484.2</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -2433,19 +2481,19 @@
         <v>25</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>135.6</v>
+        <v>174.3</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.0239</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>0.46</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
@@ -2454,10 +2502,10 @@
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>690</v>
+        <v>1410</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
@@ -2465,7 +2513,7 @@
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>660.45</v>
+        <v>1455.2</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -2476,19 +2524,19 @@
         <v>25</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>-206.85</v>
+        <v>135.6</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.0321</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -2497,10 +2545,10 @@
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>1839</v>
+        <v>690</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
@@ -2508,7 +2556,7 @@
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>1828.1</v>
+        <v>660.45</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -2519,19 +2567,19 @@
         <v>25</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>-21.8</v>
+        <v>-206.85</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>-0.0059</v>
+        <v>-0.0428</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>-0.1</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -2540,10 +2588,10 @@
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>1414</v>
+        <v>1839</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
@@ -2551,7 +2599,7 @@
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>1537.8</v>
+        <v>1828.1</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -2562,19 +2610,19 @@
         <v>25</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>371.4</v>
+        <v>-21.8</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>0.0876</v>
+        <v>-0.0059</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>1.38</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
@@ -2583,10 +2631,10 @@
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>1300</v>
+        <v>1414</v>
       </c>
       <c r="D26" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
@@ -2594,7 +2642,7 @@
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>1389.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
@@ -2605,19 +2653,19 @@
         <v>25</v>
       </c>
       <c r="I26" s="17" t="n">
-        <v>356.4</v>
+        <v>371.4</v>
       </c>
       <c r="J26" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>0.0876</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>0.63</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
@@ -2626,10 +2674,10 @@
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>276.45</v>
+        <v>1300</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
@@ -2637,7 +2685,7 @@
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>330.1</v>
+        <v>1389.1</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
@@ -2648,19 +2696,19 @@
         <v>25</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>1019.35</v>
+        <v>356.4</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>3.1</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
@@ -2669,10 +2717,10 @@
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>1462.5</v>
+        <v>276.45</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
@@ -2680,7 +2728,7 @@
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>1564.7</v>
+        <v>330.1</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
@@ -2691,19 +2739,19 @@
         <v>25</v>
       </c>
       <c r="I28" s="17" t="n">
-        <v>306.6</v>
+        <v>1019.35</v>
       </c>
       <c r="J28" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.1941</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>1.78</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -2712,41 +2760,41 @@
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>798</v>
+        <v>1462.5</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F29" s="15" t="n">
-        <v>750</v>
+        <v>1564.7</v>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H29" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I29" s="17" t="n">
-        <v>-288</v>
+        <v>306.6</v>
       </c>
       <c r="J29" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.0699</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>-0.92</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
@@ -2755,10 +2803,10 @@
         </is>
       </c>
       <c r="C30" s="15" t="n">
-        <v>260.45</v>
+        <v>798</v>
       </c>
       <c r="D30" s="16" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
@@ -2766,7 +2814,7 @@
         </is>
       </c>
       <c r="F30" s="15" t="n">
-        <v>257.85</v>
+        <v>750</v>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
@@ -2777,31 +2825,31 @@
         <v>23</v>
       </c>
       <c r="I30" s="17" t="n">
-        <v>-52.07</v>
+        <v>-288</v>
       </c>
       <c r="J30" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0602</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>-0.13</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>6500</v>
+        <v>260.45</v>
       </c>
       <c r="D31" s="16" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
@@ -2809,7 +2857,7 @@
         </is>
       </c>
       <c r="F31" s="15" t="n">
-        <v>6401.5</v>
+        <v>257.85</v>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
@@ -2817,65 +2865,65 @@
         </is>
       </c>
       <c r="H31" s="14" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I31" s="17" t="n">
-        <v>-98.5</v>
+        <v>-52.07</v>
       </c>
       <c r="J31" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.01</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C32" s="15" t="n">
-        <v>571.5</v>
+        <v>6500</v>
       </c>
       <c r="D32" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="F32" s="15" t="n">
+        <v>6401.5</v>
+      </c>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H32" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="E32" s="14" t="inlineStr">
-        <is>
-          <t>2026-07-08</t>
-        </is>
-      </c>
-      <c r="F32" s="15" t="n">
-        <v>571.1</v>
-      </c>
-      <c r="G32" s="14" t="inlineStr">
-        <is>
-          <t>STOP_LOSS</t>
-        </is>
-      </c>
-      <c r="H32" s="14" t="n">
-        <v>2</v>
-      </c>
       <c r="I32" s="17" t="n">
-        <v>-6.4</v>
+        <v>-98.5</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.0152</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
@@ -2884,10 +2932,10 @@
         </is>
       </c>
       <c r="C33" s="15" t="n">
-        <v>965</v>
+        <v>571.5</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
@@ -2895,7 +2943,7 @@
         </is>
       </c>
       <c r="F33" s="15" t="n">
-        <v>933</v>
+        <v>571.1</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
@@ -2906,19 +2954,19 @@
         <v>2</v>
       </c>
       <c r="I33" s="17" t="n">
-        <v>-288</v>
+        <v>-6.4</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0007</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
@@ -2927,18 +2975,18 @@
         </is>
       </c>
       <c r="C34" s="15" t="n">
-        <v>5479</v>
+        <v>965</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F34" s="15" t="n">
-        <v>5424</v>
+        <v>933</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
@@ -2946,42 +2994,42 @@
         </is>
       </c>
       <c r="H34" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I34" s="17" t="n">
-        <v>-55</v>
+        <v>-288</v>
       </c>
       <c r="J34" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0332</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>-0.18</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C35" s="15" t="n">
-        <v>960.1</v>
+        <v>5479</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E35" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F35" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>5424</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
@@ -2989,22 +3037,22 @@
         </is>
       </c>
       <c r="H35" s="14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I35" s="17" t="n">
-        <v>-516.79</v>
+        <v>-55</v>
       </c>
       <c r="J35" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.01</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
@@ -3013,18 +3061,18 @@
         </is>
       </c>
       <c r="C36" s="15" t="n">
-        <v>952.1</v>
+        <v>960.1</v>
       </c>
       <c r="D36" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F36" s="15" t="n">
-        <v>948.8</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
@@ -3032,42 +3080,42 @@
         </is>
       </c>
       <c r="H36" s="14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I36" s="17" t="n">
-        <v>-29.7</v>
+        <v>-516.79</v>
       </c>
       <c r="J36" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.0598</v>
       </c>
       <c r="K36" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>1475</v>
+        <v>952.1</v>
       </c>
       <c r="D37" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E37" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F37" s="15" t="n">
-        <v>1394.19</v>
+        <v>948.8</v>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
@@ -3075,42 +3123,42 @@
         </is>
       </c>
       <c r="H37" s="14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I37" s="17" t="n">
-        <v>-484.86</v>
+        <v>-29.7</v>
       </c>
       <c r="J37" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0035</v>
       </c>
       <c r="K37" s="19" t="n">
-        <v>-1</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C38" s="15" t="n">
-        <v>248.05</v>
+        <v>1475</v>
       </c>
       <c r="D38" s="16" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F38" s="15" t="n">
-        <v>242.8</v>
+        <v>1394.19</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
@@ -3118,22 +3166,22 @@
         </is>
       </c>
       <c r="H38" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I38" s="17" t="n">
-        <v>-110.25</v>
+        <v>-484.86</v>
       </c>
       <c r="J38" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0548</v>
       </c>
       <c r="K38" s="19" t="n">
-        <v>-0.3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
@@ -3142,10 +3190,10 @@
         </is>
       </c>
       <c r="C39" s="15" t="n">
-        <v>1039.2</v>
+        <v>248.05</v>
       </c>
       <c r="D39" s="16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E39" s="14" t="inlineStr">
         <is>
@@ -3153,7 +3201,7 @@
         </is>
       </c>
       <c r="F39" s="15" t="n">
-        <v>970</v>
+        <v>242.8</v>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
@@ -3164,19 +3212,19 @@
         <v>11</v>
       </c>
       <c r="I39" s="17" t="n">
-        <v>-346</v>
+        <v>-110.25</v>
       </c>
       <c r="J39" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="K39" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
@@ -3185,10 +3233,10 @@
         </is>
       </c>
       <c r="C40" s="15" t="n">
-        <v>199.96</v>
+        <v>1039.2</v>
       </c>
       <c r="D40" s="16" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="E40" s="14" t="inlineStr">
         <is>
@@ -3196,7 +3244,7 @@
         </is>
       </c>
       <c r="F40" s="15" t="n">
-        <v>193.31</v>
+        <v>970</v>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
@@ -3207,19 +3255,19 @@
         <v>11</v>
       </c>
       <c r="I40" s="17" t="n">
-        <v>-172.9</v>
+        <v>-346</v>
       </c>
       <c r="J40" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.06660000000000001</v>
       </c>
       <c r="K40" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
@@ -3228,10 +3276,10 @@
         </is>
       </c>
       <c r="C41" s="15" t="n">
-        <v>986.4</v>
+        <v>199.96</v>
       </c>
       <c r="D41" s="16" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="E41" s="14" t="inlineStr">
         <is>
@@ -3239,7 +3287,7 @@
         </is>
       </c>
       <c r="F41" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>193.31</v>
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
@@ -3250,17 +3298,60 @@
         <v>11</v>
       </c>
       <c r="I41" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J41" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K41" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D42" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F42" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G42" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H42" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I42" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J41" s="18" t="n">
+      <c r="J42" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K41" s="19" t="n">
+      <c r="K42" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I41">
+  <conditionalFormatting sqref="I2:I42">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3278,7 +3369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4225,6 +4316,31 @@
       </c>
       <c r="G37" s="14" t="n">
         <v>14</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B38" s="20" t="n">
+        <v>204926.07</v>
+      </c>
+      <c r="C38" s="20" t="n">
+        <v>114788.37</v>
+      </c>
+      <c r="D38" s="20" t="n">
+        <v>90137.7</v>
+      </c>
+      <c r="E38" s="20" t="n">
+        <v>87603.10000000001</v>
+      </c>
+      <c r="F38" s="20" t="n">
+        <v>2391.47</v>
+      </c>
+      <c r="G38" s="14" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -4307,18 +4423,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>2363.5</v>
+        <v>8912</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>2250.39</v>
+        <v>8634.93</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0667</v>
@@ -4327,10 +4443,10 @@
         <v>13333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7.7</v>
+        <v>7.8</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8238531629660661</v>
+        <v>0.839700460829493</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -4345,18 +4461,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>8945</v>
+        <v>2300</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>8673.639999999999</v>
+        <v>2175.33</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0667</v>
@@ -4365,10 +4481,10 @@
         <v>13333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>7.6</v>
+        <v>7.8</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8277178466694597</v>
+        <v>0.8246208630079598</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -4383,18 +4499,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>873.85</v>
+        <v>323.7</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>814.59</v>
+        <v>306.44</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0667</v>
@@ -4406,7 +4522,7 @@
         <v>7.6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8350387515710096</v>
+        <v>0.8182509426057814</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4421,18 +4537,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>2265.2</v>
+        <v>1426.2</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>2176.94</v>
+        <v>1331.1</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0667</v>
@@ -4444,7 +4560,7 @@
         <v>7.6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8088940092165898</v>
+        <v>0.8105090071219103</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -4459,18 +4575,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1365.2</v>
+        <v>2093.1</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1282.14</v>
+        <v>1975.91</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0667</v>
@@ -4482,7 +4598,7 @@
         <v>7.5</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8073428990364474</v>
+        <v>0.7640898617511521</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -4497,18 +4613,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1658</v>
+        <v>477.1</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1569.16</v>
+        <v>450.55</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0667</v>
@@ -4517,10 +4633,10 @@
         <v>13333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>7.5</v>
+        <v>7.3</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7919658567239213</v>
+        <v>0.7971784666945958</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -4535,18 +4651,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1556.7</v>
+        <v>1685.8</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1467.07</v>
+        <v>1575.7</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0667</v>
@@ -4555,10 +4671,10 @@
         <v>13333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.8413625890238794</v>
+        <v>0.8040029325513197</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -4573,18 +4689,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1455.6</v>
+        <v>1854</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1363</v>
+        <v>1766.36</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0667</v>
@@ -4593,10 +4709,10 @@
         <v>13333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.8128037285295349</v>
+        <v>0.7548586091328027</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -4611,18 +4727,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>477.6</v>
+        <v>582.55</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>449.67</v>
+        <v>552.0700000000001</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0667</v>
@@ -4631,10 +4747,10 @@
         <v>13333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.8217396313364055</v>
+        <v>0.7899193548387097</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -4649,18 +4765,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1844.3</v>
+        <v>4550</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1755.93</v>
+        <v>4300.4</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0667</v>
@@ -4669,10 +4785,10 @@
         <v>13333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7719040636782573</v>
+        <v>0.747930456640134</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -4687,18 +4803,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>332</v>
+        <v>855.15</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>315.2</v>
+        <v>797.7</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0667</v>
@@ -4707,10 +4823,10 @@
         <v>13333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.782130289065773</v>
+        <v>0.7782205697528278</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -4725,18 +4841,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1945</v>
+        <v>1538.6</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1872.67</v>
+        <v>1449.06</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0667</v>
@@ -4745,10 +4861,10 @@
         <v>13333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7320192710515291</v>
+        <v>0.7910096355257646</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -4763,18 +4879,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>4499</v>
+        <v>1476.2</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>4253.81</v>
+        <v>1382.59</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0667</v>
@@ -4786,7 +4902,7 @@
         <v>7.1</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7397957687473816</v>
+        <v>0.7604367406786762</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -4801,18 +4917,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>4776</v>
+        <v>736.1</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>4507.71</v>
+        <v>690.74</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0667</v>
@@ -4821,10 +4937,10 @@
         <v>13333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.9</v>
+        <v>7.1</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7359614578969418</v>
+        <v>0.7523408043569334</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -4839,18 +4955,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260807</v>
+        <v>20260810</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>INDHOTEL</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>721.65</v>
+        <v>728.7</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>678.91</v>
+        <v>701.6900000000001</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0667</v>
@@ -4859,10 +4975,10 @@
         <v>13333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.8</v>
+        <v>7.1</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7292302052785924</v>
+        <v>0.7375984499371596</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-08-11
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Mon 10 Aug 2026</t>
+          <t>As of Tue 11 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹204,926</t>
+          <t>₹204,026</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-421  (-0.20%)</t>
+          <t>₹-900  (-0.44%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.46%</t>
+          <t>+2.01%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-0.57%</t>
+          <t>-1.01%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹114,788</t>
+          <t>₹123,462</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹87,603</t>
+          <t>₹78,658</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹90,138</t>
+          <t>₹80,564</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+2,391</t>
+          <t>₹+2,120</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8847</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>9275</v>
+        <v>9125</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9275</v>
+        <v>9125</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>428</v>
+        <v>278</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.04837798123657737</v>
+        <v>0.03142308127048717</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8315.07</v>
@@ -862,13 +862,13 @@
         <v>8791</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.0521832884097035</v>
+        <v>0.0366027397260274</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>254.57</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -892,31 +892,31 @@
         <v>4874.4</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1854</v>
+        <v>1858</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>5562</v>
+        <v>5574</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>687.6000000000001</v>
+        <v>699.6000000000001</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.1410635155096012</v>
+        <v>0.1435253569670114</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1520.16</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1722.535714285714</v>
+        <v>1726.814285714286</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.07090846047156731</v>
+        <v>0.07060587421190222</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>45.45</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>4766.7</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1685</v>
+        <v>1685.8</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>5055</v>
+        <v>5057.4</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>288.2999999999997</v>
+        <v>290.6999999999996</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.06048209453080742</v>
+        <v>0.06098558751337394</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1499.44</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1568.428571428571</v>
+        <v>1574.2</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.0691818567189489</v>
+        <v>0.06620002372760715</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>37.96</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>4237.8</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1467.7</v>
+        <v>1463</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4403.1</v>
+        <v>4389</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>165.3000000000004</v>
+        <v>151.2000000000003</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.0390060880645619</v>
+        <v>0.03567888999008927</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1342.97</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1380.5</v>
+        <v>1385.685714285714</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.05941268651631808</v>
+        <v>0.05284640171858215</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>33.28</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>3897</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1944.4</v>
+        <v>1942</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>3888.8</v>
+        <v>3884</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-8.199999999999818</v>
+        <v>-13</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.002104182704644552</v>
+        <v>-0.003335899409802412</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1876.83</v>
@@ -1054,13 +1054,13 @@
         <v>1914.142857142857</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.01556117201046234</v>
+        <v>0.01434456377813743</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>33.4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>5101.6</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>812.5</v>
+        <v>800</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5687.5</v>
+        <v>5600</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>585.9000000000003</v>
+        <v>498.4000000000003</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.1148463227222833</v>
+        <v>0.09769484083424815</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>676.71</v>
@@ -1102,13 +1102,13 @@
         <v>743.3392857142857</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.08512087912087918</v>
+        <v>0.07082589285714291</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>20.64</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>4120</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>4550</v>
+        <v>4545</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4550</v>
+        <v>4545</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.1043689320388349</v>
+        <v>0.1031553398058252</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>3924.44</v>
@@ -1150,13 +1150,13 @@
         <v>4194.607142857143</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.07810832025117734</v>
+        <v>0.07709413798522703</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>85.14</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>5172</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>863.5</v>
+        <v>855</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>5181</v>
+        <v>5130</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>9</v>
+        <v>-42</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.001740139211136891</v>
+        <v>-0.008120649651972157</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>823.7</v>
@@ -1198,13 +1198,13 @@
         <v>836.5035714285714</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.0312639589709654</v>
+        <v>0.02163324979114459</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>15.94</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>5140.2</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>1681</v>
+        <v>1668.2</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5043</v>
+        <v>5004.6</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-97.20000000000027</v>
+        <v>-135.6000000000001</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>-0.01890977004785811</v>
+        <v>-0.02638029648651806</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>1616.13</v>
@@ -1246,13 +1246,13 @@
         <v>1650</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.01844140392623438</v>
+        <v>0.01090996283419257</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>39.53</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4568</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>4790.3</v>
+        <v>4781.6</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4790.3</v>
+        <v>4781.6</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>222.3000000000002</v>
+        <v>213.6000000000004</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.04866462346760074</v>
+        <v>0.04676007005253949</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>4349.36</v>
@@ -1294,13 +1294,13 @@
         <v>4460</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.06895184017702444</v>
+        <v>0.06725782164965709</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>130.39</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>4237.8</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1476.2</v>
+        <v>1440.4</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>4428.6</v>
+        <v>4321.200000000001</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>190.8000000000004</v>
+        <v>83.40000000000055</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.0450233611779698</v>
+        <v>0.01968002265326362</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1330.26</v>
@@ -1342,13 +1342,13 @@
         <v>1335.778571428572</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.0951235798478718</v>
+        <v>0.07263359384298</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>40.91</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>4650</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1538.6</v>
+        <v>1504.1</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4615.799999999999</v>
+        <v>4512.299999999999</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>-34.20000000000027</v>
+        <v>-137.7000000000003</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>-0.007354838709677478</v>
+        <v>-0.02961290322580651</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1445.97</v>
@@ -1390,13 +1390,13 @@
         <v>1470.071428571428</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.04453956286791334</v>
+        <v>0.02262387569215575</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>40.54</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>11800</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>2300</v>
+        <v>2278.9</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>11500</v>
+        <v>11394.5</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>-300</v>
+        <v>-405.4999999999995</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>-0.02542372881355932</v>
+        <v>-0.03436440677966098</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>2250.39</v>
@@ -1438,65 +1438,17 @@
         <v>2250.39</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.02156956521739136</v>
+        <v>0.01251042169467735</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>62.34</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>APOLLOHOSP</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>8945</v>
-      </c>
-      <c r="D16" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="9" t="n">
-        <v>8945</v>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>8912</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>8912</v>
-      </c>
-      <c r="H16" s="10" t="n">
-        <v>-33</v>
-      </c>
-      <c r="I16" s="11" t="n">
-        <v>-0.00368921185019564</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>8673.639999999999</v>
-      </c>
-      <c r="K16" s="7" t="n">
-        <v>8673.639999999999</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>0.02674596050269306</v>
-      </c>
-      <c r="M16" s="13" t="n">
-        <v>138.54</v>
-      </c>
-      <c r="N16" s="6" t="n">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H16">
+  <conditionalFormatting sqref="H2:H15">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1514,7 +1466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1590,27 +1542,27 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>2218</v>
+        <v>8945</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>2132.81</v>
+        <v>8673.639999999999</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -1618,85 +1570,85 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-170.37</v>
+        <v>-271.36</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0384</v>
+        <v>-0.0303</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-0.76</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>1269</v>
+        <v>2218</v>
       </c>
       <c r="D3" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="F3" s="15" t="n">
+        <v>2132.81</v>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="E3" s="14" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="F3" s="15" t="n">
-        <v>1365.2</v>
-      </c>
-      <c r="G3" s="14" t="inlineStr">
-        <is>
-          <t>TIME_STOP</t>
-        </is>
-      </c>
-      <c r="H3" s="14" t="n">
-        <v>25</v>
-      </c>
       <c r="I3" s="17" t="n">
-        <v>673.4</v>
+        <v>-170.37</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>0.07580000000000001</v>
+        <v>-0.0384</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>1.11</v>
+        <v>-0.76</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>7579.5</v>
+        <v>1269</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>7567.5</v>
+        <v>1365.2</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1707,19 +1659,19 @@
         <v>25</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-12</v>
+        <v>673.4</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0016</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-0.03</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -1728,10 +1680,10 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>1798.5</v>
+        <v>7579.5</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
@@ -1739,7 +1691,7 @@
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>1747.8</v>
+        <v>7567.5</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1750,74 +1702,74 @@
         <v>25</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-253.5</v>
+        <v>-12</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.0282</v>
+        <v>-0.0016</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-0.43</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>5438</v>
+        <v>1798.5</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>5381</v>
+        <v>1747.8</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>-57</v>
+        <v>-253.5</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>-0.0105</v>
+        <v>-0.0282</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>1784</v>
+        <v>5438</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
@@ -1825,7 +1777,7 @@
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>1752.1</v>
+        <v>5381</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -1833,22 +1785,22 @@
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>-63.8</v>
+        <v>-57</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>-0.0179</v>
+        <v>-0.0105</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>-0.36</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -1857,18 +1809,18 @@
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>871.8</v>
+        <v>1784</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>830.15</v>
+        <v>1752.1</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -1876,65 +1828,65 @@
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>-249.9</v>
+        <v>-63.8</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>-0.0478</v>
+        <v>-0.0179</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>-0.73</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>420.3</v>
+        <v>871.8</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>448.6</v>
+        <v>830.15</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>622.6</v>
+        <v>-249.9</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>0.0673</v>
+        <v>-0.0478</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>0.84</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -1943,10 +1895,10 @@
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1465</v>
+        <v>420.3</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
@@ -1954,7 +1906,7 @@
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>1596.9</v>
+        <v>448.6</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
@@ -1965,19 +1917,19 @@
         <v>25</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>791.4</v>
+        <v>622.6</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>0.09</v>
+        <v>0.0673</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>1.32</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -1986,10 +1938,10 @@
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>619.25</v>
+        <v>1465</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
@@ -1997,7 +1949,7 @@
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>717.95</v>
+        <v>1596.9</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
@@ -2008,19 +1960,19 @@
         <v>25</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>1480.5</v>
+        <v>791.4</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>0.1594</v>
+        <v>0.09</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>3.55</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -2029,10 +1981,10 @@
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>8700</v>
+        <v>619.25</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
@@ -2040,7 +1992,7 @@
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>8805.5</v>
+        <v>717.95</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -2051,31 +2003,31 @@
         <v>25</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>105.5</v>
+        <v>1480.5</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>0.0121</v>
+        <v>0.1594</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>0.29</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>961.85</v>
+        <v>8700</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
@@ -2083,42 +2035,42 @@
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>935.6</v>
+        <v>8805.5</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>-236.25</v>
+        <v>105.5</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>-0.0273</v>
+        <v>0.0121</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>-0.64</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>1560</v>
+        <v>961.85</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
@@ -2126,7 +2078,7 @@
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>1547.4</v>
+        <v>935.6</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
@@ -2134,42 +2086,42 @@
         </is>
       </c>
       <c r="H14" s="14" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>-63</v>
+        <v>-236.25</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>-0.0081</v>
+        <v>-0.0273</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>-0.23</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>900</v>
+        <v>1560</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>887.1</v>
+        <v>1547.4</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
@@ -2177,42 +2129,42 @@
         </is>
       </c>
       <c r="H15" s="14" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>-129</v>
+        <v>-63</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>-0.0143</v>
+        <v>-0.0081</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.23</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>880.8</v>
+        <v>900</v>
       </c>
       <c r="D16" s="16" t="n">
         <v>10</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>832.9400000000001</v>
+        <v>887.1</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
@@ -2220,22 +2172,22 @@
         </is>
       </c>
       <c r="H16" s="14" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>-478.6</v>
+        <v>-129</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>-0.0543</v>
+        <v>-0.0143</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>-1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -2244,10 +2196,10 @@
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>777</v>
+        <v>880.8</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
@@ -2255,7 +2207,7 @@
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>744.8</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -2266,10 +2218,10 @@
         <v>2</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>-386.4</v>
+        <v>-478.6</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>-0.0414</v>
+        <v>-0.0543</v>
       </c>
       <c r="K17" s="19" t="n">
         <v>-1</v>
@@ -2278,27 +2230,27 @@
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>1114.9</v>
+        <v>777</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>1050.57</v>
+        <v>744.8</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -2306,13 +2258,13 @@
         </is>
       </c>
       <c r="H18" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>-514.64</v>
+        <v>-386.4</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>-0.0577</v>
+        <v>-0.0414</v>
       </c>
       <c r="K18" s="19" t="n">
         <v>-1</v>
@@ -2321,50 +2273,50 @@
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>790</v>
+        <v>1114.9</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>880.8</v>
+        <v>1050.57</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H19" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>998.8</v>
+        <v>-514.64</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0577</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -2373,10 +2325,10 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>3770</v>
+        <v>790</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
@@ -2384,7 +2336,7 @@
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>4097.9</v>
+        <v>880.8</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -2395,19 +2347,19 @@
         <v>25</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>655.8</v>
+        <v>998.8</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.1149</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>1.98</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -2416,10 +2368,10 @@
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>821.05</v>
+        <v>3770</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
@@ -2427,7 +2379,7 @@
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>844</v>
+        <v>4097.9</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -2438,19 +2390,19 @@
         <v>25</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>252.45</v>
+        <v>655.8</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>0.028</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>0.6</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
@@ -2459,10 +2411,10 @@
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>2426.1</v>
+        <v>821.05</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
@@ -2470,7 +2422,7 @@
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>2484.2</v>
+        <v>844</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -2481,39 +2433,39 @@
         <v>25</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>174.3</v>
+        <v>252.45</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.028</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>1410</v>
+        <v>2426.1</v>
       </c>
       <c r="D23" s="16" t="n">
         <v>3</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>1455.2</v>
+        <v>2484.2</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -2524,19 +2476,19 @@
         <v>25</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>135.6</v>
+        <v>174.3</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.0239</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>0.46</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -2545,10 +2497,10 @@
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>690</v>
+        <v>1410</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
@@ -2556,7 +2508,7 @@
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>660.45</v>
+        <v>1455.2</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -2567,19 +2519,19 @@
         <v>25</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>-206.85</v>
+        <v>135.6</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.0321</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -2588,10 +2540,10 @@
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>1839</v>
+        <v>690</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
@@ -2599,7 +2551,7 @@
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>1828.1</v>
+        <v>660.45</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -2610,19 +2562,19 @@
         <v>25</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>-21.8</v>
+        <v>-206.85</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>-0.0059</v>
+        <v>-0.0428</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>-0.1</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
@@ -2631,10 +2583,10 @@
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>1414</v>
+        <v>1839</v>
       </c>
       <c r="D26" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
@@ -2642,7 +2594,7 @@
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>1537.8</v>
+        <v>1828.1</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
@@ -2653,19 +2605,19 @@
         <v>25</v>
       </c>
       <c r="I26" s="17" t="n">
-        <v>371.4</v>
+        <v>-21.8</v>
       </c>
       <c r="J26" s="18" t="n">
-        <v>0.0876</v>
+        <v>-0.0059</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>1.38</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
@@ -2674,10 +2626,10 @@
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>1300</v>
+        <v>1414</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
@@ -2685,7 +2637,7 @@
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>1389.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
@@ -2696,19 +2648,19 @@
         <v>25</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>356.4</v>
+        <v>371.4</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>0.0876</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>0.63</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
@@ -2717,10 +2669,10 @@
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>276.45</v>
+        <v>1300</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
@@ -2728,7 +2680,7 @@
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>330.1</v>
+        <v>1389.1</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
@@ -2739,19 +2691,19 @@
         <v>25</v>
       </c>
       <c r="I28" s="17" t="n">
-        <v>1019.35</v>
+        <v>356.4</v>
       </c>
       <c r="J28" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>3.1</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -2760,10 +2712,10 @@
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>1462.5</v>
+        <v>276.45</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
@@ -2771,7 +2723,7 @@
         </is>
       </c>
       <c r="F29" s="15" t="n">
-        <v>1564.7</v>
+        <v>330.1</v>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
@@ -2782,19 +2734,19 @@
         <v>25</v>
       </c>
       <c r="I29" s="17" t="n">
-        <v>306.6</v>
+        <v>1019.35</v>
       </c>
       <c r="J29" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.1941</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>1.78</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
@@ -2803,41 +2755,41 @@
         </is>
       </c>
       <c r="C30" s="15" t="n">
-        <v>798</v>
+        <v>1462.5</v>
       </c>
       <c r="D30" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F30" s="15" t="n">
-        <v>750</v>
+        <v>1564.7</v>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H30" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I30" s="17" t="n">
-        <v>-288</v>
+        <v>306.6</v>
       </c>
       <c r="J30" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.0699</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>-0.92</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
@@ -2846,10 +2798,10 @@
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>260.45</v>
+        <v>798</v>
       </c>
       <c r="D31" s="16" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
@@ -2857,7 +2809,7 @@
         </is>
       </c>
       <c r="F31" s="15" t="n">
-        <v>257.85</v>
+        <v>750</v>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
@@ -2868,31 +2820,31 @@
         <v>23</v>
       </c>
       <c r="I31" s="17" t="n">
-        <v>-52.07</v>
+        <v>-288</v>
       </c>
       <c r="J31" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0602</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>-0.13</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C32" s="15" t="n">
-        <v>6500</v>
+        <v>260.45</v>
       </c>
       <c r="D32" s="16" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
@@ -2900,7 +2852,7 @@
         </is>
       </c>
       <c r="F32" s="15" t="n">
-        <v>6401.5</v>
+        <v>257.85</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
@@ -2908,65 +2860,65 @@
         </is>
       </c>
       <c r="H32" s="14" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I32" s="17" t="n">
-        <v>-98.5</v>
+        <v>-52.07</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.01</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C33" s="15" t="n">
-        <v>571.5</v>
+        <v>6500</v>
       </c>
       <c r="D33" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="F33" s="15" t="n">
+        <v>6401.5</v>
+      </c>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H33" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="E33" s="14" t="inlineStr">
-        <is>
-          <t>2026-07-08</t>
-        </is>
-      </c>
-      <c r="F33" s="15" t="n">
-        <v>571.1</v>
-      </c>
-      <c r="G33" s="14" t="inlineStr">
-        <is>
-          <t>STOP_LOSS</t>
-        </is>
-      </c>
-      <c r="H33" s="14" t="n">
-        <v>2</v>
-      </c>
       <c r="I33" s="17" t="n">
-        <v>-6.4</v>
+        <v>-98.5</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.0152</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
@@ -2975,10 +2927,10 @@
         </is>
       </c>
       <c r="C34" s="15" t="n">
-        <v>965</v>
+        <v>571.5</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
@@ -2986,7 +2938,7 @@
         </is>
       </c>
       <c r="F34" s="15" t="n">
-        <v>933</v>
+        <v>571.1</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
@@ -2997,19 +2949,19 @@
         <v>2</v>
       </c>
       <c r="I34" s="17" t="n">
-        <v>-288</v>
+        <v>-6.4</v>
       </c>
       <c r="J34" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0007</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
@@ -3018,18 +2970,18 @@
         </is>
       </c>
       <c r="C35" s="15" t="n">
-        <v>5479</v>
+        <v>965</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E35" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F35" s="15" t="n">
-        <v>5424</v>
+        <v>933</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
@@ -3037,42 +2989,42 @@
         </is>
       </c>
       <c r="H35" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I35" s="17" t="n">
-        <v>-55</v>
+        <v>-288</v>
       </c>
       <c r="J35" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0332</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>-0.18</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C36" s="15" t="n">
-        <v>960.1</v>
+        <v>5479</v>
       </c>
       <c r="D36" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F36" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>5424</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
@@ -3080,22 +3032,22 @@
         </is>
       </c>
       <c r="H36" s="14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I36" s="17" t="n">
-        <v>-516.79</v>
+        <v>-55</v>
       </c>
       <c r="J36" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.01</v>
       </c>
       <c r="K36" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
@@ -3104,18 +3056,18 @@
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>952.1</v>
+        <v>960.1</v>
       </c>
       <c r="D37" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E37" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F37" s="15" t="n">
-        <v>948.8</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
@@ -3123,42 +3075,42 @@
         </is>
       </c>
       <c r="H37" s="14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I37" s="17" t="n">
-        <v>-29.7</v>
+        <v>-516.79</v>
       </c>
       <c r="J37" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.0598</v>
       </c>
       <c r="K37" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C38" s="15" t="n">
-        <v>1475</v>
+        <v>952.1</v>
       </c>
       <c r="D38" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F38" s="15" t="n">
-        <v>1394.19</v>
+        <v>948.8</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
@@ -3166,42 +3118,42 @@
         </is>
       </c>
       <c r="H38" s="14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I38" s="17" t="n">
-        <v>-484.86</v>
+        <v>-29.7</v>
       </c>
       <c r="J38" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0035</v>
       </c>
       <c r="K38" s="19" t="n">
-        <v>-1</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C39" s="15" t="n">
-        <v>248.05</v>
+        <v>1475</v>
       </c>
       <c r="D39" s="16" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E39" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F39" s="15" t="n">
-        <v>242.8</v>
+        <v>1394.19</v>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
@@ -3209,22 +3161,22 @@
         </is>
       </c>
       <c r="H39" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I39" s="17" t="n">
-        <v>-110.25</v>
+        <v>-484.86</v>
       </c>
       <c r="J39" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0548</v>
       </c>
       <c r="K39" s="19" t="n">
-        <v>-0.3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
@@ -3233,10 +3185,10 @@
         </is>
       </c>
       <c r="C40" s="15" t="n">
-        <v>1039.2</v>
+        <v>248.05</v>
       </c>
       <c r="D40" s="16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E40" s="14" t="inlineStr">
         <is>
@@ -3244,7 +3196,7 @@
         </is>
       </c>
       <c r="F40" s="15" t="n">
-        <v>970</v>
+        <v>242.8</v>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
@@ -3255,19 +3207,19 @@
         <v>11</v>
       </c>
       <c r="I40" s="17" t="n">
-        <v>-346</v>
+        <v>-110.25</v>
       </c>
       <c r="J40" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="K40" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
@@ -3276,10 +3228,10 @@
         </is>
       </c>
       <c r="C41" s="15" t="n">
-        <v>199.96</v>
+        <v>1039.2</v>
       </c>
       <c r="D41" s="16" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="E41" s="14" t="inlineStr">
         <is>
@@ -3287,7 +3239,7 @@
         </is>
       </c>
       <c r="F41" s="15" t="n">
-        <v>193.31</v>
+        <v>970</v>
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
@@ -3298,19 +3250,19 @@
         <v>11</v>
       </c>
       <c r="I41" s="17" t="n">
-        <v>-172.9</v>
+        <v>-346</v>
       </c>
       <c r="J41" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.06660000000000001</v>
       </c>
       <c r="K41" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
@@ -3319,10 +3271,10 @@
         </is>
       </c>
       <c r="C42" s="15" t="n">
-        <v>986.4</v>
+        <v>199.96</v>
       </c>
       <c r="D42" s="16" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="E42" s="14" t="inlineStr">
         <is>
@@ -3330,7 +3282,7 @@
         </is>
       </c>
       <c r="F42" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>193.31</v>
       </c>
       <c r="G42" s="14" t="inlineStr">
         <is>
@@ -3341,17 +3293,60 @@
         <v>11</v>
       </c>
       <c r="I42" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J42" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K42" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D43" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E43" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F43" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G43" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H43" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I43" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J42" s="18" t="n">
+      <c r="J43" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K42" s="19" t="n">
+      <c r="K43" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I42">
+  <conditionalFormatting sqref="I2:I43">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3369,7 +3364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4341,6 +4336,31 @@
       </c>
       <c r="G38" s="14" t="n">
         <v>15</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B39" s="20" t="n">
+        <v>204026.21</v>
+      </c>
+      <c r="C39" s="20" t="n">
+        <v>123462.01</v>
+      </c>
+      <c r="D39" s="20" t="n">
+        <v>80564.2</v>
+      </c>
+      <c r="E39" s="20" t="n">
+        <v>78658.10000000001</v>
+      </c>
+      <c r="F39" s="20" t="n">
+        <v>2120.11</v>
+      </c>
+      <c r="G39" s="14" t="n">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -4423,7 +4443,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -4431,10 +4451,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>8912</v>
+        <v>8750.5</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8634.93</v>
+        <v>8439.290000000001</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0667</v>
@@ -4443,10 +4463,10 @@
         <v>13333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7.8</v>
+        <v>7.7</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.839700460829493</v>
+        <v>0.8291987850858817</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -4461,18 +4481,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>2300</v>
+        <v>467.3</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>2175.33</v>
+        <v>439.77</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0667</v>
@@ -4481,10 +4501,10 @@
         <v>13333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>7.8</v>
+        <v>7.4</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8246208630079598</v>
+        <v>0.8096784666945958</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -4499,7 +4519,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
@@ -4507,10 +4527,10 @@
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>323.7</v>
+        <v>325</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>306.44</v>
+        <v>308.38</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0667</v>
@@ -4519,10 +4539,10 @@
         <v>13333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8182509426057814</v>
+        <v>0.7859928780896523</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4537,18 +4557,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1426.2</v>
+        <v>45185</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1331.1</v>
+        <v>42830.71</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0667</v>
@@ -4557,10 +4577,10 @@
         <v>13333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8105090071219103</v>
+        <v>0.7531242144951822</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -4575,7 +4595,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
@@ -4583,10 +4603,10 @@
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>2093.1</v>
+        <v>2051</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1975.91</v>
+        <v>1922.26</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0667</v>
@@ -4595,10 +4615,10 @@
         <v>13333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7640898617511521</v>
+        <v>0.761409719312945</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -4613,18 +4633,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>KAJARIACER</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>477.1</v>
+        <v>1225.6</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>450.55</v>
+        <v>1154.4</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0667</v>
@@ -4636,7 +4656,7 @@
         <v>7.3</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7971784666945958</v>
+        <v>0.801707163803938</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -4651,18 +4671,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1685.8</v>
+        <v>2278.9</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1575.7</v>
+        <v>2164.1</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0667</v>
@@ -4674,7 +4694,7 @@
         <v>7.3</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.8040029325513197</v>
+        <v>0.760608504398827</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -4689,7 +4709,7 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
@@ -4697,10 +4717,10 @@
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1854</v>
+        <v>1858</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1766.36</v>
+        <v>1770.54</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0667</v>
@@ -4712,7 +4732,7 @@
         <v>7.3</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7548586091328027</v>
+        <v>0.7601015919564307</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -4727,18 +4747,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>582.55</v>
+        <v>1748.4</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>552.0700000000001</v>
+        <v>1638.59</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0667</v>
@@ -4747,10 +4767,10 @@
         <v>13333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7899193548387097</v>
+        <v>0.7802492668621701</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -4765,18 +4785,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>4550</v>
+        <v>1444.4</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>4300.4</v>
+        <v>1347.24</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0667</v>
@@ -4788,7 +4808,7 @@
         <v>7.2</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.747930456640134</v>
+        <v>0.7663709677419355</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -4803,18 +4823,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>855.15</v>
+        <v>1504.1</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>797.7</v>
+        <v>1413.66</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0667</v>
@@ -4823,10 +4843,10 @@
         <v>13333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>7.2</v>
+        <v>7</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7782205697528278</v>
+        <v>0.7739956011730205</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -4841,18 +4861,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>KPIL</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1538.6</v>
+        <v>1347.7</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1449.06</v>
+        <v>1277.33</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0667</v>
@@ -4861,10 +4881,10 @@
         <v>13333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7910096355257646</v>
+        <v>0.7478508588186008</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -4879,18 +4899,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1476.2</v>
+        <v>984.8</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1382.59</v>
+        <v>934.86</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0667</v>
@@ -4899,10 +4919,10 @@
         <v>13333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7604367406786762</v>
+        <v>0.7290416841223293</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -4917,18 +4937,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>CPPLUS</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>736.1</v>
+        <v>3805.5</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>690.74</v>
+        <v>3506.37</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0667</v>
@@ -4937,10 +4957,10 @@
         <v>13333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7523408043569334</v>
+        <v>0.7229388353581903</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -4955,18 +4975,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260810</v>
+        <v>20260811</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>INDHOTEL</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>728.7</v>
+        <v>721.45</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>701.6900000000001</v>
+        <v>674.51</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0667</v>
@@ -4975,10 +4995,10 @@
         <v>13333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7375984499371596</v>
+        <v>0.7208912861332216</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-08-12
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Tue 11 Aug 2026</t>
+          <t>As of Wed 12 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹204,026</t>
+          <t>₹203,574</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-900  (-0.44%)</t>
+          <t>₹-452  (-0.22%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+2.01%</t>
+          <t>+1.79%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.01%</t>
+          <t>-1.22%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹123,462</t>
+          <t>₹139,664</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹78,658</t>
+          <t>₹61,718</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹80,564</t>
+          <t>₹63,910</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+2,120</t>
+          <t>₹+1,382</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8847</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>9125</v>
+        <v>9289</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9125</v>
+        <v>9289</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>278</v>
+        <v>442</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.03142308127048717</v>
+        <v>0.04996043856674579</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8315.07</v>
@@ -862,13 +862,13 @@
         <v>8791</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.0366027397260274</v>
+        <v>0.05361179890192701</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>254.57</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>4874.4</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1858</v>
+        <v>1850</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>5574</v>
+        <v>5550</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>699.6000000000001</v>
+        <v>675.6000000000001</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.1435253569670114</v>
+        <v>0.1386016740521911</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1520.16</v>
@@ -910,13 +910,13 @@
         <v>1726.814285714286</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.07060587421190222</v>
+        <v>0.0665868725868726</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>45.45</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>4766.7</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1685.8</v>
+        <v>1701.5</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>5057.4</v>
+        <v>5104.5</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>290.6999999999996</v>
+        <v>337.7999999999997</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.06098558751337394</v>
+        <v>0.07086663729624262</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1499.44</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1574.2</v>
+        <v>1595.9</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.06620002372760715</v>
+        <v>0.0620628856890978</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>37.96</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -1003,16 +1003,16 @@
         <v>1342.97</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1385.685714285714</v>
+        <v>1395.992857142857</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.05284640171858215</v>
+        <v>0.04580119128991302</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>33.28</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>3897</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1942</v>
+        <v>1944</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>3884</v>
+        <v>3888</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-13</v>
+        <v>-9</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.003335899409802412</v>
+        <v>-0.002309468822170901</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1876.83</v>
@@ -1054,13 +1054,13 @@
         <v>1914.142857142857</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.01434456377813743</v>
+        <v>0.01535861258083482</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>33.4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>5101.6</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>800</v>
+        <v>804.5</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5600</v>
+        <v>5631.5</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>498.4000000000003</v>
+        <v>529.9000000000003</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.09769484083424815</v>
+        <v>0.1038693743139408</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>676.71</v>
@@ -1102,13 +1102,13 @@
         <v>743.3392857142857</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.07082589285714291</v>
+        <v>0.07602326200834597</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>20.64</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>4120</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>4545</v>
+        <v>4533</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4545</v>
+        <v>4533</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>425</v>
+        <v>413</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.1031553398058252</v>
+        <v>0.1002427184466019</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>3924.44</v>
@@ -1150,13 +1150,13 @@
         <v>4194.607142857143</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.07709413798522703</v>
+        <v>0.07465097223535339</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>85.14</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -1204,13 +1204,13 @@
         <v>15.94</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -1219,46 +1219,46 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>1713.4</v>
+        <v>4568</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>5140.2</v>
+        <v>4568</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>1668.2</v>
+        <v>4523</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5004.6</v>
+        <v>4523</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-135.6000000000001</v>
+        <v>-45</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>-0.02638029648651806</v>
+        <v>-0.009851138353765323</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>1616.13</v>
+        <v>4349.36</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>1650</v>
+        <v>4460</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.01090996283419257</v>
+        <v>0.01392880831306655</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>39.53</v>
+        <v>130.39</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1267,46 +1267,46 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>4568</v>
+        <v>1412.6</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>4568</v>
+        <v>4237.8</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>4781.6</v>
+        <v>1393.5</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4781.6</v>
+        <v>4180.5</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>213.6000000000004</v>
+        <v>-57.29999999999973</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.04676007005253949</v>
+        <v>-0.01352116664306945</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>4349.36</v>
+        <v>1330.26</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>4460</v>
+        <v>1335.778571428572</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.06725782164965709</v>
+        <v>0.04142190783740819</v>
       </c>
       <c r="M12" s="13" t="n">
-        <v>130.39</v>
+        <v>40.91</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -1315,140 +1315,44 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>1412.6</v>
+        <v>1550</v>
       </c>
       <c r="D13" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>4237.8</v>
+        <v>4650</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1440.4</v>
+        <v>1482</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>4321.200000000001</v>
+        <v>4446</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>83.40000000000055</v>
+        <v>-204</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.01968002265326362</v>
+        <v>-0.04387096774193548</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>1330.26</v>
+        <v>1445.97</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>1335.778571428572</v>
+        <v>1470.071428571428</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.07263359384298</v>
+        <v>0.008048968575284452</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>40.91</v>
+        <v>40.54</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>RAINBOW</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>1550</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E14" s="9" t="n">
-        <v>4650</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>1504.1</v>
-      </c>
-      <c r="G14" s="9" t="n">
-        <v>4512.299999999999</v>
-      </c>
-      <c r="H14" s="10" t="n">
-        <v>-137.7000000000003</v>
-      </c>
-      <c r="I14" s="11" t="n">
-        <v>-0.02961290322580651</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>1445.97</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>1470.071428571428</v>
-      </c>
-      <c r="L14" s="12" t="n">
-        <v>0.02262387569215575</v>
-      </c>
-      <c r="M14" s="13" t="n">
-        <v>40.54</v>
-      </c>
-      <c r="N14" s="6" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>LUPIN</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>2360</v>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="E15" s="9" t="n">
-        <v>11800</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>2278.9</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>11394.5</v>
-      </c>
-      <c r="H15" s="10" t="n">
-        <v>-405.4999999999995</v>
-      </c>
-      <c r="I15" s="11" t="n">
-        <v>-0.03436440677966098</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>2250.39</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>2250.39</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>0.01251042169467735</v>
-      </c>
-      <c r="M15" s="13" t="n">
-        <v>62.34</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H15">
+  <conditionalFormatting sqref="H2:H13">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1466,7 +1370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1542,27 +1446,27 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>8945</v>
+        <v>1713.4</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>8673.639999999999</v>
+        <v>1650</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -1570,171 +1474,171 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-271.36</v>
+        <v>-190.2</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0303</v>
+        <v>-0.037</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-1</v>
+        <v>-0.65</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>2218</v>
+        <v>2360</v>
       </c>
       <c r="D3" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F3" s="15" t="n">
+        <v>2250.39</v>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="14" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="F3" s="15" t="n">
-        <v>2132.81</v>
-      </c>
-      <c r="G3" s="14" t="inlineStr">
-        <is>
-          <t>STOP_LOSS</t>
-        </is>
-      </c>
-      <c r="H3" s="14" t="n">
-        <v>7</v>
-      </c>
       <c r="I3" s="17" t="n">
-        <v>-170.37</v>
+        <v>-548.05</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0384</v>
+        <v>-0.0464</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-0.76</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>1269</v>
+        <v>8945</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>1365.2</v>
+        <v>8673.639999999999</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>673.4</v>
+        <v>-271.36</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>0.07580000000000001</v>
+        <v>-0.0303</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>1.11</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>7579.5</v>
+        <v>2218</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>7567.5</v>
+        <v>2132.81</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-12</v>
+        <v>-170.37</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.0016</v>
+        <v>-0.0384</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-0.03</v>
+        <v>-0.76</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>1798.5</v>
+        <v>1269</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>1747.8</v>
+        <v>1365.2</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -1745,125 +1649,125 @@
         <v>25</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>-253.5</v>
+        <v>673.4</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>-0.0282</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>-0.43</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>5438</v>
+        <v>7579.5</v>
       </c>
       <c r="D7" s="16" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>5381</v>
+        <v>7567.5</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>-57</v>
+        <v>-12</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>-0.0105</v>
+        <v>-0.0016</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>1784</v>
+        <v>1798.5</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>1752.1</v>
+        <v>1747.8</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>-63.8</v>
+        <v>-253.5</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>-0.0179</v>
+        <v>-0.0282</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>-0.36</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>871.8</v>
+        <v>5438</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>830.15</v>
+        <v>5381</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
@@ -1871,108 +1775,108 @@
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>-249.9</v>
+        <v>-57</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>-0.0478</v>
+        <v>-0.0105</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>-0.73</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>420.3</v>
+        <v>1784</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>448.6</v>
+        <v>1752.1</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H10" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>622.6</v>
+        <v>-63.8</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>0.0673</v>
+        <v>-0.0179</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>0.84</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>1465</v>
+        <v>871.8</v>
       </c>
       <c r="D11" s="16" t="n">
         <v>6</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>1596.9</v>
+        <v>830.15</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H11" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>791.4</v>
+        <v>-249.9</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>0.09</v>
+        <v>-0.0478</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>1.32</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -1981,10 +1885,10 @@
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>619.25</v>
+        <v>420.3</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
@@ -1992,7 +1896,7 @@
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>717.95</v>
+        <v>448.6</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -2003,19 +1907,19 @@
         <v>25</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>1480.5</v>
+        <v>622.6</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>0.1594</v>
+        <v>0.0673</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>3.55</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -2024,10 +1928,10 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>8700</v>
+        <v>1465</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
@@ -2035,7 +1939,7 @@
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>8805.5</v>
+        <v>1596.9</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
@@ -2046,31 +1950,31 @@
         <v>25</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>105.5</v>
+        <v>791.4</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>0.0121</v>
+        <v>0.09</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>0.29</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>961.85</v>
+        <v>619.25</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
@@ -2078,42 +1982,42 @@
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>935.6</v>
+        <v>717.95</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H14" s="14" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>-236.25</v>
+        <v>1480.5</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>-0.0273</v>
+        <v>0.1594</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>-0.64</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>1560</v>
+        <v>8700</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
@@ -2121,50 +2025,50 @@
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>1547.4</v>
+        <v>8805.5</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H15" s="14" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>-63</v>
+        <v>105.5</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>-0.0081</v>
+        <v>0.0121</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>-0.23</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>900</v>
+        <v>961.85</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>887.1</v>
+        <v>935.6</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
@@ -2172,22 +2076,22 @@
         </is>
       </c>
       <c r="H16" s="14" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>-129</v>
+        <v>-236.25</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>-0.0143</v>
+        <v>-0.0273</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -2196,18 +2100,18 @@
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>880.8</v>
+        <v>1560</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>832.9400000000001</v>
+        <v>1547.4</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -2215,42 +2119,42 @@
         </is>
       </c>
       <c r="H17" s="14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>-478.6</v>
+        <v>-63</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>-0.0543</v>
+        <v>-0.0081</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>-1</v>
+        <v>-0.23</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>777</v>
+        <v>900</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>744.8</v>
+        <v>887.1</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -2258,42 +2162,42 @@
         </is>
       </c>
       <c r="H18" s="14" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>-386.4</v>
+        <v>-129</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>-0.0414</v>
+        <v>-0.0143</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>-1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>1114.9</v>
+        <v>880.8</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>1050.57</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
@@ -2301,13 +2205,13 @@
         </is>
       </c>
       <c r="H19" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>-514.64</v>
+        <v>-478.6</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>-0.0577</v>
+        <v>-0.0543</v>
       </c>
       <c r="K19" s="19" t="n">
         <v>-1</v>
@@ -2316,93 +2220,93 @@
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>790</v>
+        <v>777</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>880.8</v>
+        <v>744.8</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H20" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>998.8</v>
+        <v>-386.4</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0414</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>3770</v>
+        <v>1114.9</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>4097.9</v>
+        <v>1050.57</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H21" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>655.8</v>
+        <v>-514.64</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>-0.0577</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>1.98</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
@@ -2411,7 +2315,7 @@
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>821.05</v>
+        <v>790</v>
       </c>
       <c r="D22" s="16" t="n">
         <v>11</v>
@@ -2422,7 +2326,7 @@
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>844</v>
+        <v>880.8</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -2433,19 +2337,19 @@
         <v>25</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>252.45</v>
+        <v>998.8</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>0.028</v>
+        <v>0.1149</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>0.6</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
@@ -2454,10 +2358,10 @@
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>2426.1</v>
+        <v>3770</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
@@ -2465,7 +2369,7 @@
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>2484.2</v>
+        <v>4097.9</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -2476,39 +2380,39 @@
         <v>25</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>174.3</v>
+        <v>655.8</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>0.5</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>1410</v>
+        <v>821.05</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>1455.2</v>
+        <v>844</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -2519,39 +2423,39 @@
         <v>25</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>135.6</v>
+        <v>252.45</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.028</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>0.46</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>690</v>
+        <v>2426.1</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>660.45</v>
+        <v>2484.2</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -2562,19 +2466,19 @@
         <v>25</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>-206.85</v>
+        <v>174.3</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.0239</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
@@ -2583,10 +2487,10 @@
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>1839</v>
+        <v>1410</v>
       </c>
       <c r="D26" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
@@ -2594,7 +2498,7 @@
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>1828.1</v>
+        <v>1455.2</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
@@ -2605,19 +2509,19 @@
         <v>25</v>
       </c>
       <c r="I26" s="17" t="n">
-        <v>-21.8</v>
+        <v>135.6</v>
       </c>
       <c r="J26" s="18" t="n">
-        <v>-0.0059</v>
+        <v>0.0321</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>-0.1</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
@@ -2626,10 +2530,10 @@
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>1414</v>
+        <v>690</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
@@ -2637,7 +2541,7 @@
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>1537.8</v>
+        <v>660.45</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
@@ -2648,19 +2552,19 @@
         <v>25</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>371.4</v>
+        <v>-206.85</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>0.0876</v>
+        <v>-0.0428</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>1.38</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
@@ -2669,10 +2573,10 @@
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>1300</v>
+        <v>1839</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
@@ -2680,7 +2584,7 @@
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>1389.1</v>
+        <v>1828.1</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
@@ -2691,19 +2595,19 @@
         <v>25</v>
       </c>
       <c r="I28" s="17" t="n">
-        <v>356.4</v>
+        <v>-21.8</v>
       </c>
       <c r="J28" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>-0.0059</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>0.63</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -2712,10 +2616,10 @@
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>276.45</v>
+        <v>1414</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
@@ -2723,7 +2627,7 @@
         </is>
       </c>
       <c r="F29" s="15" t="n">
-        <v>330.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
@@ -2734,19 +2638,19 @@
         <v>25</v>
       </c>
       <c r="I29" s="17" t="n">
-        <v>1019.35</v>
+        <v>371.4</v>
       </c>
       <c r="J29" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.0876</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>3.1</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
@@ -2755,10 +2659,10 @@
         </is>
       </c>
       <c r="C30" s="15" t="n">
-        <v>1462.5</v>
+        <v>1300</v>
       </c>
       <c r="D30" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
@@ -2766,7 +2670,7 @@
         </is>
       </c>
       <c r="F30" s="15" t="n">
-        <v>1564.7</v>
+        <v>1389.1</v>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
@@ -2777,19 +2681,19 @@
         <v>25</v>
       </c>
       <c r="I30" s="17" t="n">
-        <v>306.6</v>
+        <v>356.4</v>
       </c>
       <c r="J30" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>1.78</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
@@ -2798,41 +2702,41 @@
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>798</v>
+        <v>276.45</v>
       </c>
       <c r="D31" s="16" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F31" s="15" t="n">
-        <v>750</v>
+        <v>330.1</v>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H31" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I31" s="17" t="n">
-        <v>-288</v>
+        <v>1019.35</v>
       </c>
       <c r="J31" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.1941</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>-0.92</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
@@ -2841,53 +2745,53 @@
         </is>
       </c>
       <c r="C32" s="15" t="n">
-        <v>260.45</v>
+        <v>1462.5</v>
       </c>
       <c r="D32" s="16" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F32" s="15" t="n">
-        <v>257.85</v>
+        <v>1564.7</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H32" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I32" s="17" t="n">
-        <v>-52.07</v>
+        <v>306.6</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>-0.01</v>
+        <v>0.0699</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>-0.13</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C33" s="15" t="n">
-        <v>6500</v>
+        <v>798</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
@@ -2895,7 +2799,7 @@
         </is>
       </c>
       <c r="F33" s="15" t="n">
-        <v>6401.5</v>
+        <v>750</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
@@ -2903,34 +2807,34 @@
         </is>
       </c>
       <c r="H33" s="14" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I33" s="17" t="n">
-        <v>-98.5</v>
+        <v>-288</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.0602</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C34" s="15" t="n">
-        <v>571.5</v>
+        <v>260.45</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
@@ -2938,7 +2842,7 @@
         </is>
       </c>
       <c r="F34" s="15" t="n">
-        <v>571.1</v>
+        <v>257.85</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
@@ -2946,34 +2850,34 @@
         </is>
       </c>
       <c r="H34" s="14" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="I34" s="17" t="n">
-        <v>-6.4</v>
+        <v>-52.07</v>
       </c>
       <c r="J34" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.01</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C35" s="15" t="n">
-        <v>965</v>
+        <v>6500</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E35" s="14" t="inlineStr">
         <is>
@@ -2981,7 +2885,7 @@
         </is>
       </c>
       <c r="F35" s="15" t="n">
-        <v>933</v>
+        <v>6401.5</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
@@ -2989,22 +2893,22 @@
         </is>
       </c>
       <c r="H35" s="14" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="I35" s="17" t="n">
-        <v>-288</v>
+        <v>-98.5</v>
       </c>
       <c r="J35" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0152</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
@@ -3013,18 +2917,18 @@
         </is>
       </c>
       <c r="C36" s="15" t="n">
-        <v>5479</v>
+        <v>571.5</v>
       </c>
       <c r="D36" s="16" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F36" s="15" t="n">
-        <v>5424</v>
+        <v>571.1</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
@@ -3032,42 +2936,42 @@
         </is>
       </c>
       <c r="H36" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I36" s="17" t="n">
-        <v>-55</v>
+        <v>-6.4</v>
       </c>
       <c r="J36" s="18" t="n">
+        <v>-0.0007</v>
+      </c>
+      <c r="K36" s="19" t="n">
         <v>-0.01</v>
-      </c>
-      <c r="K36" s="19" t="n">
-        <v>-0.18</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>960.1</v>
+        <v>965</v>
       </c>
       <c r="D37" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E37" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F37" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>933</v>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
@@ -3075,42 +2979,42 @@
         </is>
       </c>
       <c r="H37" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I37" s="17" t="n">
-        <v>-516.79</v>
+        <v>-288</v>
       </c>
       <c r="J37" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.0332</v>
       </c>
       <c r="K37" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C38" s="15" t="n">
-        <v>952.1</v>
+        <v>5479</v>
       </c>
       <c r="D38" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F38" s="15" t="n">
-        <v>948.8</v>
+        <v>5424</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
@@ -3121,39 +3025,39 @@
         <v>1</v>
       </c>
       <c r="I38" s="17" t="n">
-        <v>-29.7</v>
+        <v>-55</v>
       </c>
       <c r="J38" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.01</v>
       </c>
       <c r="K38" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C39" s="15" t="n">
-        <v>1475</v>
+        <v>960.1</v>
       </c>
       <c r="D39" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E39" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F39" s="15" t="n">
-        <v>1394.19</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
@@ -3161,42 +3065,42 @@
         </is>
       </c>
       <c r="H39" s="14" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I39" s="17" t="n">
-        <v>-484.86</v>
+        <v>-516.79</v>
       </c>
       <c r="J39" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0598</v>
       </c>
       <c r="K39" s="19" t="n">
-        <v>-1</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C40" s="15" t="n">
-        <v>248.05</v>
+        <v>952.1</v>
       </c>
       <c r="D40" s="16" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E40" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F40" s="15" t="n">
-        <v>242.8</v>
+        <v>948.8</v>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
@@ -3204,42 +3108,42 @@
         </is>
       </c>
       <c r="H40" s="14" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I40" s="17" t="n">
-        <v>-110.25</v>
+        <v>-29.7</v>
       </c>
       <c r="J40" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0035</v>
       </c>
       <c r="K40" s="19" t="n">
-        <v>-0.3</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C41" s="15" t="n">
-        <v>1039.2</v>
+        <v>1475</v>
       </c>
       <c r="D41" s="16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E41" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F41" s="15" t="n">
-        <v>970</v>
+        <v>1394.19</v>
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
@@ -3247,22 +3151,22 @@
         </is>
       </c>
       <c r="H41" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I41" s="17" t="n">
-        <v>-346</v>
+        <v>-484.86</v>
       </c>
       <c r="J41" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0548</v>
       </c>
       <c r="K41" s="19" t="n">
-        <v>-0.82</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
@@ -3271,10 +3175,10 @@
         </is>
       </c>
       <c r="C42" s="15" t="n">
-        <v>199.96</v>
+        <v>248.05</v>
       </c>
       <c r="D42" s="16" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E42" s="14" t="inlineStr">
         <is>
@@ -3282,7 +3186,7 @@
         </is>
       </c>
       <c r="F42" s="15" t="n">
-        <v>193.31</v>
+        <v>242.8</v>
       </c>
       <c r="G42" s="14" t="inlineStr">
         <is>
@@ -3293,19 +3197,19 @@
         <v>11</v>
       </c>
       <c r="I42" s="17" t="n">
-        <v>-172.9</v>
+        <v>-110.25</v>
       </c>
       <c r="J42" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.0212</v>
       </c>
       <c r="K42" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
@@ -3314,7 +3218,7 @@
         </is>
       </c>
       <c r="C43" s="15" t="n">
-        <v>986.4</v>
+        <v>1039.2</v>
       </c>
       <c r="D43" s="16" t="n">
         <v>5</v>
@@ -3325,7 +3229,7 @@
         </is>
       </c>
       <c r="F43" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>970</v>
       </c>
       <c r="G43" s="14" t="inlineStr">
         <is>
@@ -3336,17 +3240,103 @@
         <v>11</v>
       </c>
       <c r="I43" s="17" t="n">
+        <v>-346</v>
+      </c>
+      <c r="J43" s="18" t="n">
+        <v>-0.06660000000000001</v>
+      </c>
+      <c r="K43" s="19" t="n">
+        <v>-0.82</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="n">
+        <v>199.96</v>
+      </c>
+      <c r="D44" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F44" s="15" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="G44" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H44" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I44" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J44" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K44" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C45" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D45" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F45" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G45" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H45" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I45" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J43" s="18" t="n">
+      <c r="J45" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K43" s="19" t="n">
+      <c r="K45" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I43">
+  <conditionalFormatting sqref="I2:I45">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3364,7 +3354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4361,6 +4351,31 @@
       </c>
       <c r="G39" s="14" t="n">
         <v>14</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B40" s="20" t="n">
+        <v>203574.06</v>
+      </c>
+      <c r="C40" s="20" t="n">
+        <v>139663.96</v>
+      </c>
+      <c r="D40" s="20" t="n">
+        <v>63910.1</v>
+      </c>
+      <c r="E40" s="20" t="n">
+        <v>61717.9</v>
+      </c>
+      <c r="F40" s="20" t="n">
+        <v>1381.86</v>
+      </c>
+      <c r="G40" s="14" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -4443,7 +4458,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -4451,10 +4466,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>8750.5</v>
+        <v>8597</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8439.290000000001</v>
+        <v>8267.209999999999</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0667</v>
@@ -4463,10 +4478,10 @@
         <v>13333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7.7</v>
+        <v>8</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8291987850858817</v>
+        <v>0.8647947214076246</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -4481,7 +4496,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
@@ -4489,10 +4504,10 @@
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>467.3</v>
+        <v>467.4</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>439.77</v>
+        <v>439.69</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0667</v>
@@ -4504,7 +4519,7 @@
         <v>7.4</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8096784666945958</v>
+        <v>0.8205718475073314</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -4519,18 +4534,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>KAJARIACER</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>325</v>
+        <v>1252.2</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>308.38</v>
+        <v>1179.06</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0667</v>
@@ -4542,7 +4557,7 @@
         <v>7.4</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7859928780896523</v>
+        <v>0.8024518223711772</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4557,18 +4572,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>45185</v>
+        <v>4523</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>42830.71</v>
+        <v>4223.53</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0667</v>
@@ -4577,10 +4592,10 @@
         <v>13333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7531242144951822</v>
+        <v>0.7852251780477586</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -4595,18 +4610,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>2051</v>
+        <v>46480</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1922.26</v>
+        <v>44149.29</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0667</v>
@@ -4615,10 +4630,10 @@
         <v>13333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.761409719312945</v>
+        <v>0.7531168831168831</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -4633,18 +4648,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>KAJARIACER</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1225.6</v>
+        <v>2081.5</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1154.4</v>
+        <v>1954.07</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0667</v>
@@ -4656,7 +4671,7 @@
         <v>7.3</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.801707163803938</v>
+        <v>0.7475617930456641</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -4671,18 +4686,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>2278.9</v>
+        <v>8600</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>2164.1</v>
+        <v>8148.86</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0667</v>
@@ -4694,7 +4709,7 @@
         <v>7.3</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.760608504398827</v>
+        <v>0.7450293255131966</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -4709,18 +4724,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1858</v>
+        <v>1701.5</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1770.54</v>
+        <v>1631.1</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0667</v>
@@ -4729,10 +4744,10 @@
         <v>13333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>7.3</v>
+        <v>7.1</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7601015919564307</v>
+        <v>0.7316579388353582</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -4747,18 +4762,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>CAPLIPOINT</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1748.4</v>
+        <v>2472.4</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1638.59</v>
+        <v>2293.7</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0667</v>
@@ -4767,10 +4782,10 @@
         <v>13333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7802492668621701</v>
+        <v>0.7432048596564726</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -4785,18 +4800,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1444.4</v>
+        <v>1482</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1347.24</v>
+        <v>1391.81</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0667</v>
@@ -4805,10 +4820,10 @@
         <v>13333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>7.2</v>
+        <v>7</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7663709677419355</v>
+        <v>0.7678906577293674</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -4823,18 +4838,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>PHOENIXLTD</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1504.1</v>
+        <v>1905</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1413.66</v>
+        <v>1808.04</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0667</v>
@@ -4846,7 +4861,7 @@
         <v>7</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7739956011730205</v>
+        <v>0.7301550062840385</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -4861,18 +4876,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>KPIL</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1347.7</v>
+        <v>2433.1</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1277.33</v>
+        <v>2311.96</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0667</v>
@@ -4884,7 +4899,7 @@
         <v>7</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7478508588186008</v>
+        <v>0.7194574780058651</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -4899,18 +4914,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>984.8</v>
+        <v>575.55</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>934.86</v>
+        <v>547.47</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0667</v>
@@ -4919,10 +4934,10 @@
         <v>13333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7290416841223293</v>
+        <v>0.739206116464181</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -4937,18 +4952,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>CPPLUS</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>3805.5</v>
+        <v>736.3</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>3506.37</v>
+        <v>688.59</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0667</v>
@@ -4957,10 +4972,10 @@
         <v>13333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7229388353581903</v>
+        <v>0.7339317134478425</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -4975,18 +4990,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260811</v>
+        <v>20260812</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>721.45</v>
+        <v>1766.6</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>674.51</v>
+        <v>1656.27</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0667</v>
@@ -4995,10 +5010,10 @@
         <v>13333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7208912861332216</v>
+        <v>0.7334939254294093</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-08-13
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Wed 12 Aug 2026</t>
+          <t>As of Thu 13 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹203,574</t>
+          <t>₹203,653</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-452  (-0.22%)</t>
+          <t>₹+79  (+0.04%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.79%</t>
+          <t>+1.83%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.22%</t>
+          <t>-1.19%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹139,664</t>
+          <t>₹148,534</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹61,718</t>
+          <t>₹52,500</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹63,910</t>
+          <t>₹55,119</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+1,382</t>
+          <t>₹+1,034</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8847</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>9289</v>
+        <v>9297</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9289</v>
+        <v>9297</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>442</v>
+        <v>450</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.04996043856674579</v>
+        <v>0.0508646998982706</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8315.07</v>
@@ -862,13 +862,13 @@
         <v>8791</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.05361179890192701</v>
+        <v>0.05442615897601377</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>254.57</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -892,31 +892,31 @@
         <v>4874.4</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1850</v>
+        <v>1851.7</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>5550</v>
+        <v>5555.1</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>675.6000000000001</v>
+        <v>680.7000000000003</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.1386016740521911</v>
+        <v>0.1396479566715904</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1520.16</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1726.814285714286</v>
+        <v>1731.464285714286</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.0665868725868726</v>
+        <v>0.06493261018832126</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>45.45</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>4766.7</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1701.5</v>
+        <v>1696.1</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>5104.5</v>
+        <v>5088.299999999999</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>337.7999999999997</v>
+        <v>321.5999999999995</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.07086663729624262</v>
+        <v>0.06746805966391832</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1499.44</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1595.9</v>
+        <v>1601.707142857143</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.0620628856890978</v>
+        <v>0.05565288434812636</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>37.96</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>4237.8</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1463</v>
+        <v>1458.8</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4389</v>
+        <v>4376.4</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>151.2000000000003</v>
+        <v>138.6000000000001</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.03567888999008927</v>
+        <v>0.0327056491575818</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1342.97</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1395.992857142857</v>
+        <v>1405.957142857143</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.04580119128991302</v>
+        <v>0.0362235105174506</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>33.28</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -1036,31 +1036,31 @@
         <v>3897</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1944</v>
+        <v>1932</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>3888</v>
+        <v>3864</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-9</v>
+        <v>-33</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.002309468822170901</v>
+        <v>-0.008468052347959968</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1876.83</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1914.142857142857</v>
+        <v>1922.5</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.01535861258083482</v>
+        <v>0.004917184265010352</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>33.4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -1084,31 +1084,31 @@
         <v>5101.6</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>804.5</v>
+        <v>799.9</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5631.5</v>
+        <v>5599.3</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>529.9000000000003</v>
+        <v>497.7000000000002</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.1038693743139408</v>
+        <v>0.09755762897914383</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>676.71</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>743.3392857142857</v>
+        <v>745.6214285714285</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.07602326200834597</v>
+        <v>0.06785669637276093</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>20.64</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -1132,31 +1132,31 @@
         <v>4120</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>4533</v>
+        <v>4675.2</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4533</v>
+        <v>4675.2</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>413</v>
+        <v>555.1999999999998</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.1002427184466019</v>
+        <v>0.134757281553398</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>3924.44</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>4194.607142857143</v>
+        <v>4303.007142857143</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.07465097223535339</v>
+        <v>0.07961003960105602</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>85.14</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>5172</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>855</v>
+        <v>864.45</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>5130</v>
+        <v>5186.700000000001</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>-42</v>
+        <v>14.70000000000027</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>-0.008120649651972157</v>
+        <v>0.002842227378190308</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>823.7</v>
@@ -1198,19 +1198,19 @@
         <v>836.5035714285714</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.02163324979114459</v>
+        <v>0.03232856564454702</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>15.94</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -1219,140 +1219,44 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>4568</v>
+        <v>1412.6</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>4568</v>
+        <v>4237.8</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>4523</v>
+        <v>1410.4</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>4523</v>
+        <v>4231.200000000001</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-45</v>
+        <v>-6.599999999999454</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>-0.009851138353765323</v>
+        <v>-0.001557411864646622</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>4349.36</v>
+        <v>1330.26</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>4460</v>
+        <v>1335.778571428572</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.01392880831306655</v>
+        <v>0.05290798962806891</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>130.39</v>
+        <v>40.91</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>MEDANTA</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>1412.6</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>4237.8</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>1393.5</v>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>4180.5</v>
-      </c>
-      <c r="H12" s="10" t="n">
-        <v>-57.29999999999973</v>
-      </c>
-      <c r="I12" s="11" t="n">
-        <v>-0.01352116664306945</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>1330.26</v>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>1335.778571428572</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>0.04142190783740819</v>
-      </c>
-      <c r="M12" s="13" t="n">
-        <v>40.91</v>
-      </c>
-      <c r="N12" s="6" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>RAINBOW</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>1550</v>
-      </c>
-      <c r="D13" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>4650</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>1482</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>4446</v>
-      </c>
-      <c r="H13" s="10" t="n">
-        <v>-204</v>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>-0.04387096774193548</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>1445.97</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>1470.071428571428</v>
-      </c>
-      <c r="L13" s="12" t="n">
-        <v>0.008048968575284452</v>
-      </c>
-      <c r="M13" s="13" t="n">
-        <v>40.54</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H13">
+  <conditionalFormatting sqref="H2:H11">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1370,7 +1274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1446,7 +1350,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -1455,18 +1359,18 @@
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>1713.4</v>
+        <v>4568</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>1650</v>
+        <v>4460</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -1474,42 +1378,42 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-190.2</v>
+        <v>-108</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.037</v>
+        <v>-0.0236</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-0.65</v>
+        <v>-0.49</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>2360</v>
+        <v>1550</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>2250.39</v>
+        <v>1470.07</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -1517,42 +1421,42 @@
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-548.05</v>
+        <v>-239.79</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0464</v>
+        <v>-0.0516</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-1</v>
+        <v>-0.77</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>8945</v>
+        <v>1713.4</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>8673.639999999999</v>
+        <v>1650</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1560,171 +1464,171 @@
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-271.36</v>
+        <v>-190.2</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0303</v>
+        <v>-0.037</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-1</v>
+        <v>-0.65</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>2218</v>
+        <v>2360</v>
       </c>
       <c r="D5" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="n">
+        <v>2250.39</v>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="F5" s="15" t="n">
-        <v>2132.81</v>
-      </c>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>STOP_LOSS</t>
-        </is>
-      </c>
-      <c r="H5" s="14" t="n">
-        <v>7</v>
-      </c>
       <c r="I5" s="17" t="n">
-        <v>-170.37</v>
+        <v>-548.05</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.0384</v>
+        <v>-0.0464</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-0.76</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>1269</v>
+        <v>8945</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>1365.2</v>
+        <v>8673.639999999999</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>673.4</v>
+        <v>-271.36</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>0.07580000000000001</v>
+        <v>-0.0303</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>1.11</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>7579.5</v>
+        <v>2218</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>7567.5</v>
+        <v>2132.81</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>-12</v>
+        <v>-170.37</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>-0.0016</v>
+        <v>-0.0384</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>-0.03</v>
+        <v>-0.76</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>1798.5</v>
+        <v>1269</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>1747.8</v>
+        <v>1365.2</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -1735,125 +1639,125 @@
         <v>25</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>-253.5</v>
+        <v>673.4</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>-0.0282</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>-0.43</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>5438</v>
+        <v>7579.5</v>
       </c>
       <c r="D9" s="16" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>5381</v>
+        <v>7567.5</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>-57</v>
+        <v>-12</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>-0.0105</v>
+        <v>-0.0016</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1784</v>
+        <v>1798.5</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>1752.1</v>
+        <v>1747.8</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H10" s="14" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>-63.8</v>
+        <v>-253.5</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>-0.0179</v>
+        <v>-0.0282</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>-0.36</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>871.8</v>
+        <v>5438</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>830.15</v>
+        <v>5381</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
@@ -1861,108 +1765,108 @@
         </is>
       </c>
       <c r="H11" s="14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>-249.9</v>
+        <v>-57</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>-0.0478</v>
+        <v>-0.0105</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>-0.73</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>420.3</v>
+        <v>1784</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>448.6</v>
+        <v>1752.1</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H12" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>622.6</v>
+        <v>-63.8</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>0.0673</v>
+        <v>-0.0179</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>0.84</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>1465</v>
+        <v>871.8</v>
       </c>
       <c r="D13" s="16" t="n">
         <v>6</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>1596.9</v>
+        <v>830.15</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>791.4</v>
+        <v>-249.9</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>0.09</v>
+        <v>-0.0478</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>1.32</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -1971,10 +1875,10 @@
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>619.25</v>
+        <v>420.3</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
@@ -1982,7 +1886,7 @@
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>717.95</v>
+        <v>448.6</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
@@ -1993,19 +1897,19 @@
         <v>25</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>1480.5</v>
+        <v>622.6</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>0.1594</v>
+        <v>0.0673</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>3.55</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -2014,10 +1918,10 @@
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>8700</v>
+        <v>1465</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
@@ -2025,7 +1929,7 @@
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>8805.5</v>
+        <v>1596.9</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
@@ -2036,31 +1940,31 @@
         <v>25</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>105.5</v>
+        <v>791.4</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.0121</v>
+        <v>0.09</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>0.29</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>961.85</v>
+        <v>619.25</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
@@ -2068,42 +1972,42 @@
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>935.6</v>
+        <v>717.95</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H16" s="14" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>-236.25</v>
+        <v>1480.5</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>-0.0273</v>
+        <v>0.1594</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>-0.64</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>1560</v>
+        <v>8700</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
@@ -2111,50 +2015,50 @@
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>1547.4</v>
+        <v>8805.5</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H17" s="14" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>-63</v>
+        <v>105.5</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>-0.0081</v>
+        <v>0.0121</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>-0.23</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>900</v>
+        <v>961.85</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>887.1</v>
+        <v>935.6</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -2162,22 +2066,22 @@
         </is>
       </c>
       <c r="H18" s="14" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>-129</v>
+        <v>-236.25</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>-0.0143</v>
+        <v>-0.0273</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -2186,18 +2090,18 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>880.8</v>
+        <v>1560</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>832.9400000000001</v>
+        <v>1547.4</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
@@ -2205,42 +2109,42 @@
         </is>
       </c>
       <c r="H19" s="14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>-478.6</v>
+        <v>-63</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>-0.0543</v>
+        <v>-0.0081</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>-1</v>
+        <v>-0.23</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>777</v>
+        <v>900</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>744.8</v>
+        <v>887.1</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -2248,42 +2152,42 @@
         </is>
       </c>
       <c r="H20" s="14" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>-386.4</v>
+        <v>-129</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>-0.0414</v>
+        <v>-0.0143</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>-1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>1114.9</v>
+        <v>880.8</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>1050.57</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -2291,13 +2195,13 @@
         </is>
       </c>
       <c r="H21" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>-514.64</v>
+        <v>-478.6</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>-0.0577</v>
+        <v>-0.0543</v>
       </c>
       <c r="K21" s="19" t="n">
         <v>-1</v>
@@ -2306,93 +2210,93 @@
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>790</v>
+        <v>777</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>880.8</v>
+        <v>744.8</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H22" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>998.8</v>
+        <v>-386.4</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0414</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>3770</v>
+        <v>1114.9</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>4097.9</v>
+        <v>1050.57</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H23" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>655.8</v>
+        <v>-514.64</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>-0.0577</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>1.98</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -2401,7 +2305,7 @@
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>821.05</v>
+        <v>790</v>
       </c>
       <c r="D24" s="16" t="n">
         <v>11</v>
@@ -2412,7 +2316,7 @@
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>844</v>
+        <v>880.8</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -2423,19 +2327,19 @@
         <v>25</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>252.45</v>
+        <v>998.8</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>0.028</v>
+        <v>0.1149</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>0.6</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -2444,10 +2348,10 @@
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>2426.1</v>
+        <v>3770</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
@@ -2455,7 +2359,7 @@
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>2484.2</v>
+        <v>4097.9</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -2466,39 +2370,39 @@
         <v>25</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>174.3</v>
+        <v>655.8</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>0.5</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>1410</v>
+        <v>821.05</v>
       </c>
       <c r="D26" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>1455.2</v>
+        <v>844</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
@@ -2509,39 +2413,39 @@
         <v>25</v>
       </c>
       <c r="I26" s="17" t="n">
-        <v>135.6</v>
+        <v>252.45</v>
       </c>
       <c r="J26" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.028</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>0.46</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>690</v>
+        <v>2426.1</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>660.45</v>
+        <v>2484.2</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
@@ -2552,19 +2456,19 @@
         <v>25</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>-206.85</v>
+        <v>174.3</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.0239</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
@@ -2573,10 +2477,10 @@
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>1839</v>
+        <v>1410</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
@@ -2584,7 +2488,7 @@
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>1828.1</v>
+        <v>1455.2</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
@@ -2595,19 +2499,19 @@
         <v>25</v>
       </c>
       <c r="I28" s="17" t="n">
-        <v>-21.8</v>
+        <v>135.6</v>
       </c>
       <c r="J28" s="18" t="n">
-        <v>-0.0059</v>
+        <v>0.0321</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>-0.1</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -2616,10 +2520,10 @@
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>1414</v>
+        <v>690</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
@@ -2627,7 +2531,7 @@
         </is>
       </c>
       <c r="F29" s="15" t="n">
-        <v>1537.8</v>
+        <v>660.45</v>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
@@ -2638,19 +2542,19 @@
         <v>25</v>
       </c>
       <c r="I29" s="17" t="n">
-        <v>371.4</v>
+        <v>-206.85</v>
       </c>
       <c r="J29" s="18" t="n">
-        <v>0.0876</v>
+        <v>-0.0428</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>1.38</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
@@ -2659,10 +2563,10 @@
         </is>
       </c>
       <c r="C30" s="15" t="n">
-        <v>1300</v>
+        <v>1839</v>
       </c>
       <c r="D30" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
@@ -2670,7 +2574,7 @@
         </is>
       </c>
       <c r="F30" s="15" t="n">
-        <v>1389.1</v>
+        <v>1828.1</v>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
@@ -2681,19 +2585,19 @@
         <v>25</v>
       </c>
       <c r="I30" s="17" t="n">
-        <v>356.4</v>
+        <v>-21.8</v>
       </c>
       <c r="J30" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>-0.0059</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>0.63</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
@@ -2702,10 +2606,10 @@
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>276.45</v>
+        <v>1414</v>
       </c>
       <c r="D31" s="16" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
@@ -2713,7 +2617,7 @@
         </is>
       </c>
       <c r="F31" s="15" t="n">
-        <v>330.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
@@ -2724,19 +2628,19 @@
         <v>25</v>
       </c>
       <c r="I31" s="17" t="n">
-        <v>1019.35</v>
+        <v>371.4</v>
       </c>
       <c r="J31" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.0876</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>3.1</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
@@ -2745,10 +2649,10 @@
         </is>
       </c>
       <c r="C32" s="15" t="n">
-        <v>1462.5</v>
+        <v>1300</v>
       </c>
       <c r="D32" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
@@ -2756,7 +2660,7 @@
         </is>
       </c>
       <c r="F32" s="15" t="n">
-        <v>1564.7</v>
+        <v>1389.1</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
@@ -2767,19 +2671,19 @@
         <v>25</v>
       </c>
       <c r="I32" s="17" t="n">
-        <v>306.6</v>
+        <v>356.4</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>1.78</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
@@ -2788,41 +2692,41 @@
         </is>
       </c>
       <c r="C33" s="15" t="n">
-        <v>798</v>
+        <v>276.45</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F33" s="15" t="n">
-        <v>750</v>
+        <v>330.1</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H33" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I33" s="17" t="n">
-        <v>-288</v>
+        <v>1019.35</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.1941</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>-0.92</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
@@ -2831,53 +2735,53 @@
         </is>
       </c>
       <c r="C34" s="15" t="n">
-        <v>260.45</v>
+        <v>1462.5</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F34" s="15" t="n">
-        <v>257.85</v>
+        <v>1564.7</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H34" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I34" s="17" t="n">
-        <v>-52.07</v>
+        <v>306.6</v>
       </c>
       <c r="J34" s="18" t="n">
-        <v>-0.01</v>
+        <v>0.0699</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>-0.13</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C35" s="15" t="n">
-        <v>6500</v>
+        <v>798</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E35" s="14" t="inlineStr">
         <is>
@@ -2885,7 +2789,7 @@
         </is>
       </c>
       <c r="F35" s="15" t="n">
-        <v>6401.5</v>
+        <v>750</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
@@ -2893,34 +2797,34 @@
         </is>
       </c>
       <c r="H35" s="14" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I35" s="17" t="n">
-        <v>-98.5</v>
+        <v>-288</v>
       </c>
       <c r="J35" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.0602</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C36" s="15" t="n">
-        <v>571.5</v>
+        <v>260.45</v>
       </c>
       <c r="D36" s="16" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
@@ -2928,7 +2832,7 @@
         </is>
       </c>
       <c r="F36" s="15" t="n">
-        <v>571.1</v>
+        <v>257.85</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
@@ -2936,34 +2840,34 @@
         </is>
       </c>
       <c r="H36" s="14" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="I36" s="17" t="n">
-        <v>-6.4</v>
+        <v>-52.07</v>
       </c>
       <c r="J36" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.01</v>
       </c>
       <c r="K36" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>965</v>
+        <v>6500</v>
       </c>
       <c r="D37" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E37" s="14" t="inlineStr">
         <is>
@@ -2971,7 +2875,7 @@
         </is>
       </c>
       <c r="F37" s="15" t="n">
-        <v>933</v>
+        <v>6401.5</v>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
@@ -2979,22 +2883,22 @@
         </is>
       </c>
       <c r="H37" s="14" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="I37" s="17" t="n">
-        <v>-288</v>
+        <v>-98.5</v>
       </c>
       <c r="J37" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0152</v>
       </c>
       <c r="K37" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
@@ -3003,18 +2907,18 @@
         </is>
       </c>
       <c r="C38" s="15" t="n">
-        <v>5479</v>
+        <v>571.5</v>
       </c>
       <c r="D38" s="16" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F38" s="15" t="n">
-        <v>5424</v>
+        <v>571.1</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
@@ -3022,42 +2926,42 @@
         </is>
       </c>
       <c r="H38" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I38" s="17" t="n">
-        <v>-55</v>
+        <v>-6.4</v>
       </c>
       <c r="J38" s="18" t="n">
+        <v>-0.0007</v>
+      </c>
+      <c r="K38" s="19" t="n">
         <v>-0.01</v>
-      </c>
-      <c r="K38" s="19" t="n">
-        <v>-0.18</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C39" s="15" t="n">
-        <v>960.1</v>
+        <v>965</v>
       </c>
       <c r="D39" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E39" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F39" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>933</v>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
@@ -3065,42 +2969,42 @@
         </is>
       </c>
       <c r="H39" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I39" s="17" t="n">
-        <v>-516.79</v>
+        <v>-288</v>
       </c>
       <c r="J39" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.0332</v>
       </c>
       <c r="K39" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C40" s="15" t="n">
-        <v>952.1</v>
+        <v>5479</v>
       </c>
       <c r="D40" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E40" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F40" s="15" t="n">
-        <v>948.8</v>
+        <v>5424</v>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
@@ -3111,39 +3015,39 @@
         <v>1</v>
       </c>
       <c r="I40" s="17" t="n">
-        <v>-29.7</v>
+        <v>-55</v>
       </c>
       <c r="J40" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.01</v>
       </c>
       <c r="K40" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C41" s="15" t="n">
-        <v>1475</v>
+        <v>960.1</v>
       </c>
       <c r="D41" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E41" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F41" s="15" t="n">
-        <v>1394.19</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
@@ -3151,42 +3055,42 @@
         </is>
       </c>
       <c r="H41" s="14" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I41" s="17" t="n">
-        <v>-484.86</v>
+        <v>-516.79</v>
       </c>
       <c r="J41" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0598</v>
       </c>
       <c r="K41" s="19" t="n">
-        <v>-1</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C42" s="15" t="n">
-        <v>248.05</v>
+        <v>952.1</v>
       </c>
       <c r="D42" s="16" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E42" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F42" s="15" t="n">
-        <v>242.8</v>
+        <v>948.8</v>
       </c>
       <c r="G42" s="14" t="inlineStr">
         <is>
@@ -3194,42 +3098,42 @@
         </is>
       </c>
       <c r="H42" s="14" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I42" s="17" t="n">
-        <v>-110.25</v>
+        <v>-29.7</v>
       </c>
       <c r="J42" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0035</v>
       </c>
       <c r="K42" s="19" t="n">
-        <v>-0.3</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C43" s="15" t="n">
-        <v>1039.2</v>
+        <v>1475</v>
       </c>
       <c r="D43" s="16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E43" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F43" s="15" t="n">
-        <v>970</v>
+        <v>1394.19</v>
       </c>
       <c r="G43" s="14" t="inlineStr">
         <is>
@@ -3237,22 +3141,22 @@
         </is>
       </c>
       <c r="H43" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I43" s="17" t="n">
-        <v>-346</v>
+        <v>-484.86</v>
       </c>
       <c r="J43" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0548</v>
       </c>
       <c r="K43" s="19" t="n">
-        <v>-0.82</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
@@ -3261,10 +3165,10 @@
         </is>
       </c>
       <c r="C44" s="15" t="n">
-        <v>199.96</v>
+        <v>248.05</v>
       </c>
       <c r="D44" s="16" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E44" s="14" t="inlineStr">
         <is>
@@ -3272,7 +3176,7 @@
         </is>
       </c>
       <c r="F44" s="15" t="n">
-        <v>193.31</v>
+        <v>242.8</v>
       </c>
       <c r="G44" s="14" t="inlineStr">
         <is>
@@ -3283,19 +3187,19 @@
         <v>11</v>
       </c>
       <c r="I44" s="17" t="n">
-        <v>-172.9</v>
+        <v>-110.25</v>
       </c>
       <c r="J44" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.0212</v>
       </c>
       <c r="K44" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
@@ -3304,7 +3208,7 @@
         </is>
       </c>
       <c r="C45" s="15" t="n">
-        <v>986.4</v>
+        <v>1039.2</v>
       </c>
       <c r="D45" s="16" t="n">
         <v>5</v>
@@ -3315,7 +3219,7 @@
         </is>
       </c>
       <c r="F45" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>970</v>
       </c>
       <c r="G45" s="14" t="inlineStr">
         <is>
@@ -3326,17 +3230,103 @@
         <v>11</v>
       </c>
       <c r="I45" s="17" t="n">
+        <v>-346</v>
+      </c>
+      <c r="J45" s="18" t="n">
+        <v>-0.06660000000000001</v>
+      </c>
+      <c r="K45" s="19" t="n">
+        <v>-0.82</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="n">
+        <v>199.96</v>
+      </c>
+      <c r="D46" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="E46" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F46" s="15" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="G46" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H46" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I46" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J46" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K46" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C47" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D47" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F47" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G47" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H47" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I47" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J45" s="18" t="n">
+      <c r="J47" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K45" s="19" t="n">
+      <c r="K47" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I45">
+  <conditionalFormatting sqref="I2:I47">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3354,7 +3344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4376,6 +4366,31 @@
       </c>
       <c r="G40" s="14" t="n">
         <v>12</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B41" s="20" t="n">
+        <v>203652.97</v>
+      </c>
+      <c r="C41" s="20" t="n">
+        <v>148534.17</v>
+      </c>
+      <c r="D41" s="20" t="n">
+        <v>55118.8</v>
+      </c>
+      <c r="E41" s="20" t="n">
+        <v>52499.9</v>
+      </c>
+      <c r="F41" s="20" t="n">
+        <v>1034.07</v>
+      </c>
+      <c r="G41" s="14" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -4458,7 +4473,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -4466,22 +4481,22 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>8597</v>
+        <v>8600</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8267.209999999999</v>
+        <v>8248.07</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>8</v>
+        <v>7.2</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8647947214076246</v>
+        <v>0.8581723921240051</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -4490,36 +4505,36 @@
       </c>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>467.4</v>
+        <v>1796.3</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>439.69</v>
+        <v>1672.19</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>7.4</v>
+        <v>7</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8205718475073314</v>
+        <v>0.8402262253875158</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -4528,36 +4543,36 @@
       </c>
       <c r="J3" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>KAJARIACER</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1252.2</v>
+        <v>479.45</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1179.06</v>
+        <v>450.59</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>7.4</v>
+        <v>6.9</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8024518223711772</v>
+        <v>0.8459949727691662</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4566,36 +4581,36 @@
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>OBEROIRLTY</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>4523</v>
+        <v>1846</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>4223.53</v>
+        <v>1764.51</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>7.3</v>
+        <v>6.8</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7852251780477586</v>
+        <v>0.8189715123586091</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -4604,36 +4619,36 @@
       </c>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>46480</v>
+        <v>857.55</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>44149.29</v>
+        <v>806.47</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>7.3</v>
+        <v>6.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7531168831168831</v>
+        <v>0.8223271889400922</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -4642,36 +4657,36 @@
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>2081.5</v>
+        <v>331.15</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1954.07</v>
+        <v>314.13</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>7.3</v>
+        <v>6.7</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7475617930456641</v>
+        <v>0.7946763720150817</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -4680,36 +4695,36 @@
       </c>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>8600</v>
+        <v>712.05</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>8148.86</v>
+        <v>661.02</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>7.3</v>
+        <v>6.5</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7450293255131966</v>
+        <v>0.7495821114369501</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -4718,36 +4733,36 @@
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1701.5</v>
+        <v>4675.2</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1631.1</v>
+        <v>4427.07</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>7.1</v>
+        <v>6.5</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7316579388353582</v>
+        <v>0.7663552576455802</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -4756,36 +4771,36 @@
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>CAPLIPOINT</t>
+          <t>KAJARIACER</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>2472.4</v>
+        <v>1260.9</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>2293.7</v>
+        <v>1189.9</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>7.1</v>
+        <v>6.4</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7432048596564726</v>
+        <v>0.7776633850020946</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -4794,36 +4809,36 @@
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1482</v>
+        <v>4435.1</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1391.81</v>
+        <v>4125.37</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>7</v>
+        <v>6.4</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7678906577293674</v>
+        <v>0.7747235023041475</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -4832,36 +4847,36 @@
       </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>PHOENIXLTD</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1905</v>
+        <v>1851.7</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1808.04</v>
+        <v>1767.34</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>7</v>
+        <v>6.4</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7301550062840385</v>
+        <v>0.7423900293255132</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -4870,36 +4885,36 @@
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>2433.1</v>
+        <v>46750</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>2311.96</v>
+        <v>44410</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>7</v>
+        <v>6.4</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7194574780058651</v>
+        <v>0.7369176790950985</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -4908,36 +4923,36 @@
       </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>575.55</v>
+        <v>1663.4</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>547.47</v>
+        <v>1583.19</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.739206116464181</v>
+        <v>0.7315039798910766</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -4946,36 +4961,36 @@
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>INDHOTEL</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>736.3</v>
+        <v>721.75</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>688.59</v>
+        <v>696.5700000000001</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7339317134478425</v>
+        <v>0.7264463762044407</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -4984,36 +4999,36 @@
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260812</v>
+        <v>20260813</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1766.6</v>
+        <v>1453</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1656.27</v>
+        <v>1364.64</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.0667</v>
+        <v>0.0467</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>13333</v>
+        <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.9</v>
+        <v>6.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7334939254294093</v>
+        <v>0.7711426476749057</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>
@@ -5022,7 +5037,7 @@
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>RISK_ON</t>
+          <t>RISK_NEU</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V5 daily refresh 2026-08-14
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Thu 13 Aug 2026</t>
+          <t>As of Fri 14 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹203,653</t>
+          <t>₹203,309</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+79  (+0.04%)</t>
+          <t>₹-344  (-0.17%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.83%</t>
+          <t>+1.65%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.19%</t>
+          <t>-1.35%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹148,534</t>
+          <t>₹161,619</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹52,500</t>
+          <t>₹39,756</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹55,119</t>
+          <t>₹41,690</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+1,034</t>
+          <t>₹+1,375</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,61 +820,61 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>8847</v>
+        <v>1624.8</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>8847</v>
+        <v>4874.4</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>9297</v>
+        <v>1787.3</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9297</v>
+        <v>5361.9</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>450</v>
+        <v>487.5</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.0508646998982706</v>
+        <v>0.1000123092072871</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>8315.07</v>
+        <v>1520.16</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>8791</v>
+        <v>1743.85</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.05442615897601377</v>
+        <v>0.02431041235382983</v>
       </c>
       <c r="M3" s="13" t="n">
-        <v>254.57</v>
+        <v>45.45</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -883,46 +883,46 @@
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>1624.8</v>
+        <v>1588.9</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>4874.4</v>
+        <v>4766.7</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1851.7</v>
+        <v>1693</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>5555.1</v>
+        <v>5079</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>680.7000000000003</v>
+        <v>312.2999999999997</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.1396479566715904</v>
+        <v>0.06551702435647297</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>1520.16</v>
+        <v>1499.44</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1731.464285714286</v>
+        <v>1607.792857142857</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.06493261018832126</v>
+        <v>0.05032908615306735</v>
       </c>
       <c r="M4" s="13" t="n">
-        <v>45.45</v>
+        <v>37.96</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -931,46 +931,46 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>1588.9</v>
+        <v>1412.6</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>4766.7</v>
+        <v>4237.8</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1696.1</v>
+        <v>1450</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>5088.299999999999</v>
+        <v>4350</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>321.5999999999995</v>
+        <v>112.2000000000003</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.06746805966391832</v>
+        <v>0.02647600169899483</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>1499.44</v>
+        <v>1342.97</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1601.707142857143</v>
+        <v>1406</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.05565288434812636</v>
+        <v>0.0303448275862069</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>37.96</v>
+        <v>33.28</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -979,46 +979,46 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>1412.6</v>
+        <v>728.8</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>4237.8</v>
+        <v>5101.6</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1458.8</v>
+        <v>792</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4376.4</v>
+        <v>5544</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>138.6000000000001</v>
+        <v>442.4000000000003</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.0327056491575818</v>
+        <v>0.08671789242590566</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>1342.97</v>
+        <v>676.71</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1405.957142857143</v>
+        <v>746.5642857142857</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.0362235105174506</v>
+        <v>0.05736832611832615</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>33.28</v>
+        <v>20.64</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -1027,46 +1027,46 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>1948.5</v>
+        <v>4120</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>3897</v>
+        <v>4120</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1932</v>
+        <v>4650</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>3864</v>
+        <v>4650</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-33</v>
+        <v>530</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.008468052347959968</v>
+        <v>0.1286407766990291</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>1876.83</v>
+        <v>3924.44</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1922.5</v>
+        <v>4305.171428571429</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.004917184265010352</v>
+        <v>0.07415668202764972</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>33.4</v>
+        <v>85.14</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -1075,188 +1075,92 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>728.8</v>
+        <v>862</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>5101.6</v>
+        <v>5172</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>799.9</v>
+        <v>865.2</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5599.3</v>
+        <v>5191.200000000001</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>497.7000000000002</v>
+        <v>19.20000000000027</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.09755762897914383</v>
+        <v>0.003712296983758754</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>676.71</v>
+        <v>823.7</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>745.6214285714285</v>
+        <v>836.5035714285714</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.06785669637276093</v>
+        <v>0.03316739317086069</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>20.64</v>
+        <v>15.94</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>4120</v>
+        <v>1412.6</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>4120</v>
+        <v>4237.8</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>4675.2</v>
+        <v>1422.6</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4675.2</v>
+        <v>4267.799999999999</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>555.1999999999998</v>
+        <v>30</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.134757281553398</v>
+        <v>0.007079144839303412</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>3924.44</v>
+        <v>1330.26</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>4303.007142857143</v>
+        <v>1335.778571428572</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.07961003960105602</v>
+        <v>0.06103010584242107</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>85.14</v>
+        <v>40.91</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>MARICO</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>862</v>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="E10" s="9" t="n">
-        <v>5172</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>864.45</v>
-      </c>
-      <c r="G10" s="9" t="n">
-        <v>5186.700000000001</v>
-      </c>
-      <c r="H10" s="10" t="n">
-        <v>14.70000000000027</v>
-      </c>
-      <c r="I10" s="11" t="n">
-        <v>0.002842227378190308</v>
-      </c>
-      <c r="J10" s="7" t="n">
-        <v>823.7</v>
-      </c>
-      <c r="K10" s="7" t="n">
-        <v>836.5035714285714</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>0.03232856564454702</v>
-      </c>
-      <c r="M10" s="13" t="n">
-        <v>15.94</v>
-      </c>
-      <c r="N10" s="6" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>MEDANTA</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>1412.6</v>
-      </c>
-      <c r="D11" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E11" s="9" t="n">
-        <v>4237.8</v>
-      </c>
-      <c r="F11" s="7" t="n">
-        <v>1410.4</v>
-      </c>
-      <c r="G11" s="9" t="n">
-        <v>4231.200000000001</v>
-      </c>
-      <c r="H11" s="10" t="n">
-        <v>-6.599999999999454</v>
-      </c>
-      <c r="I11" s="11" t="n">
-        <v>-0.001557411864646622</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>1330.26</v>
-      </c>
-      <c r="K11" s="7" t="n">
-        <v>1335.778571428572</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>0.05290798962806891</v>
-      </c>
-      <c r="M11" s="13" t="n">
-        <v>40.91</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H11">
+  <conditionalFormatting sqref="H2:H9">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1274,7 +1178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1350,70 +1254,70 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>4568</v>
+        <v>8847</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>4460</v>
+        <v>9240</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-108</v>
+        <v>393</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0236</v>
+        <v>0.0444</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-0.49</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>1550</v>
+        <v>1948.5</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>1470.07</v>
+        <v>1922.5</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -1421,22 +1325,22 @@
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-239.79</v>
+        <v>-52</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0516</v>
+        <v>-0.0133</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-0.77</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -1445,18 +1349,18 @@
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>1713.4</v>
+        <v>4568</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>1650</v>
+        <v>4460</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1464,42 +1368,42 @@
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-190.2</v>
+        <v>-108</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.037</v>
+        <v>-0.0236</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-0.65</v>
+        <v>-0.49</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>2360</v>
+        <v>1550</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>2250.39</v>
+        <v>1470.07</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1507,42 +1411,42 @@
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-548.05</v>
+        <v>-239.79</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.0464</v>
+        <v>-0.0516</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-1</v>
+        <v>-0.77</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>8945</v>
+        <v>1713.4</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>8673.639999999999</v>
+        <v>1650</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -1550,171 +1454,171 @@
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>-271.36</v>
+        <v>-190.2</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>-0.0303</v>
+        <v>-0.037</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>-1</v>
+        <v>-0.65</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>2218</v>
+        <v>2360</v>
       </c>
       <c r="D7" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>2250.39</v>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="F7" s="15" t="n">
-        <v>2132.81</v>
-      </c>
-      <c r="G7" s="14" t="inlineStr">
-        <is>
-          <t>STOP_LOSS</t>
-        </is>
-      </c>
-      <c r="H7" s="14" t="n">
-        <v>7</v>
-      </c>
       <c r="I7" s="17" t="n">
-        <v>-170.37</v>
+        <v>-548.05</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>-0.0384</v>
+        <v>-0.0464</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>-0.76</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>1269</v>
+        <v>8945</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>1365.2</v>
+        <v>8673.639999999999</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>673.4</v>
+        <v>-271.36</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>0.07580000000000001</v>
+        <v>-0.0303</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>1.11</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>7579.5</v>
+        <v>2218</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>7567.5</v>
+        <v>2132.81</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>-12</v>
+        <v>-170.37</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>-0.0016</v>
+        <v>-0.0384</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>-0.03</v>
+        <v>-0.76</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1798.5</v>
+        <v>1269</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>1747.8</v>
+        <v>1365.2</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
@@ -1725,125 +1629,125 @@
         <v>25</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>-253.5</v>
+        <v>673.4</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>-0.0282</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>-0.43</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>5438</v>
+        <v>7579.5</v>
       </c>
       <c r="D11" s="16" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>5381</v>
+        <v>7567.5</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H11" s="14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>-57</v>
+        <v>-12</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>-0.0105</v>
+        <v>-0.0016</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>1784</v>
+        <v>1798.5</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>1752.1</v>
+        <v>1747.8</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H12" s="14" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>-63.8</v>
+        <v>-253.5</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>-0.0179</v>
+        <v>-0.0282</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>-0.36</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>871.8</v>
+        <v>5438</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>830.15</v>
+        <v>5381</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
@@ -1851,108 +1755,108 @@
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>-249.9</v>
+        <v>-57</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>-0.0478</v>
+        <v>-0.0105</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>-0.73</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>420.3</v>
+        <v>1784</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>448.6</v>
+        <v>1752.1</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H14" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>622.6</v>
+        <v>-63.8</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>0.0673</v>
+        <v>-0.0179</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>0.84</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>1465</v>
+        <v>871.8</v>
       </c>
       <c r="D15" s="16" t="n">
         <v>6</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>1596.9</v>
+        <v>830.15</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H15" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>791.4</v>
+        <v>-249.9</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.09</v>
+        <v>-0.0478</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>1.32</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -1961,10 +1865,10 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>619.25</v>
+        <v>420.3</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
@@ -1972,7 +1876,7 @@
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>717.95</v>
+        <v>448.6</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
@@ -1983,19 +1887,19 @@
         <v>25</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>1480.5</v>
+        <v>622.6</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>0.1594</v>
+        <v>0.0673</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>3.55</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -2004,10 +1908,10 @@
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>8700</v>
+        <v>1465</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
@@ -2015,7 +1919,7 @@
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>8805.5</v>
+        <v>1596.9</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -2026,31 +1930,31 @@
         <v>25</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>105.5</v>
+        <v>791.4</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>0.0121</v>
+        <v>0.09</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>0.29</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>961.85</v>
+        <v>619.25</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
@@ -2058,42 +1962,42 @@
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>935.6</v>
+        <v>717.95</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H18" s="14" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>-236.25</v>
+        <v>1480.5</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>-0.0273</v>
+        <v>0.1594</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>-0.64</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>1560</v>
+        <v>8700</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
@@ -2101,50 +2005,50 @@
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>1547.4</v>
+        <v>8805.5</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H19" s="14" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>-63</v>
+        <v>105.5</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>-0.0081</v>
+        <v>0.0121</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>-0.23</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>900</v>
+        <v>961.85</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>887.1</v>
+        <v>935.6</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -2152,22 +2056,22 @@
         </is>
       </c>
       <c r="H20" s="14" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>-129</v>
+        <v>-236.25</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>-0.0143</v>
+        <v>-0.0273</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -2176,18 +2080,18 @@
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>880.8</v>
+        <v>1560</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>832.9400000000001</v>
+        <v>1547.4</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -2195,42 +2099,42 @@
         </is>
       </c>
       <c r="H21" s="14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>-478.6</v>
+        <v>-63</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>-0.0543</v>
+        <v>-0.0081</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>-1</v>
+        <v>-0.23</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>777</v>
+        <v>900</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>744.8</v>
+        <v>887.1</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -2238,42 +2142,42 @@
         </is>
       </c>
       <c r="H22" s="14" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>-386.4</v>
+        <v>-129</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>-0.0414</v>
+        <v>-0.0143</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>-1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>1114.9</v>
+        <v>880.8</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>1050.57</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -2281,13 +2185,13 @@
         </is>
       </c>
       <c r="H23" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>-514.64</v>
+        <v>-478.6</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>-0.0577</v>
+        <v>-0.0543</v>
       </c>
       <c r="K23" s="19" t="n">
         <v>-1</v>
@@ -2296,93 +2200,93 @@
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>790</v>
+        <v>777</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>880.8</v>
+        <v>744.8</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H24" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>998.8</v>
+        <v>-386.4</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0414</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>3770</v>
+        <v>1114.9</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>4097.9</v>
+        <v>1050.57</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H25" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>655.8</v>
+        <v>-514.64</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>-0.0577</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>1.98</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
@@ -2391,7 +2295,7 @@
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>821.05</v>
+        <v>790</v>
       </c>
       <c r="D26" s="16" t="n">
         <v>11</v>
@@ -2402,7 +2306,7 @@
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>844</v>
+        <v>880.8</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
@@ -2413,19 +2317,19 @@
         <v>25</v>
       </c>
       <c r="I26" s="17" t="n">
-        <v>252.45</v>
+        <v>998.8</v>
       </c>
       <c r="J26" s="18" t="n">
-        <v>0.028</v>
+        <v>0.1149</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>0.6</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
@@ -2434,10 +2338,10 @@
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>2426.1</v>
+        <v>3770</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
@@ -2445,7 +2349,7 @@
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>2484.2</v>
+        <v>4097.9</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
@@ -2456,39 +2360,39 @@
         <v>25</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>174.3</v>
+        <v>655.8</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>0.5</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>1410</v>
+        <v>821.05</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>1455.2</v>
+        <v>844</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
@@ -2499,39 +2403,39 @@
         <v>25</v>
       </c>
       <c r="I28" s="17" t="n">
-        <v>135.6</v>
+        <v>252.45</v>
       </c>
       <c r="J28" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.028</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>0.46</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>690</v>
+        <v>2426.1</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F29" s="15" t="n">
-        <v>660.45</v>
+        <v>2484.2</v>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
@@ -2542,19 +2446,19 @@
         <v>25</v>
       </c>
       <c r="I29" s="17" t="n">
-        <v>-206.85</v>
+        <v>174.3</v>
       </c>
       <c r="J29" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.0239</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
@@ -2563,10 +2467,10 @@
         </is>
       </c>
       <c r="C30" s="15" t="n">
-        <v>1839</v>
+        <v>1410</v>
       </c>
       <c r="D30" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
@@ -2574,7 +2478,7 @@
         </is>
       </c>
       <c r="F30" s="15" t="n">
-        <v>1828.1</v>
+        <v>1455.2</v>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
@@ -2585,19 +2489,19 @@
         <v>25</v>
       </c>
       <c r="I30" s="17" t="n">
-        <v>-21.8</v>
+        <v>135.6</v>
       </c>
       <c r="J30" s="18" t="n">
-        <v>-0.0059</v>
+        <v>0.0321</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>-0.1</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
@@ -2606,10 +2510,10 @@
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>1414</v>
+        <v>690</v>
       </c>
       <c r="D31" s="16" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
@@ -2617,7 +2521,7 @@
         </is>
       </c>
       <c r="F31" s="15" t="n">
-        <v>1537.8</v>
+        <v>660.45</v>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
@@ -2628,19 +2532,19 @@
         <v>25</v>
       </c>
       <c r="I31" s="17" t="n">
-        <v>371.4</v>
+        <v>-206.85</v>
       </c>
       <c r="J31" s="18" t="n">
-        <v>0.0876</v>
+        <v>-0.0428</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>1.38</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
@@ -2649,10 +2553,10 @@
         </is>
       </c>
       <c r="C32" s="15" t="n">
-        <v>1300</v>
+        <v>1839</v>
       </c>
       <c r="D32" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
@@ -2660,7 +2564,7 @@
         </is>
       </c>
       <c r="F32" s="15" t="n">
-        <v>1389.1</v>
+        <v>1828.1</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
@@ -2671,19 +2575,19 @@
         <v>25</v>
       </c>
       <c r="I32" s="17" t="n">
-        <v>356.4</v>
+        <v>-21.8</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>-0.0059</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>0.63</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
@@ -2692,10 +2596,10 @@
         </is>
       </c>
       <c r="C33" s="15" t="n">
-        <v>276.45</v>
+        <v>1414</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
@@ -2703,7 +2607,7 @@
         </is>
       </c>
       <c r="F33" s="15" t="n">
-        <v>330.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
@@ -2714,19 +2618,19 @@
         <v>25</v>
       </c>
       <c r="I33" s="17" t="n">
-        <v>1019.35</v>
+        <v>371.4</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.0876</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>3.1</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
@@ -2735,10 +2639,10 @@
         </is>
       </c>
       <c r="C34" s="15" t="n">
-        <v>1462.5</v>
+        <v>1300</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
@@ -2746,7 +2650,7 @@
         </is>
       </c>
       <c r="F34" s="15" t="n">
-        <v>1564.7</v>
+        <v>1389.1</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
@@ -2757,19 +2661,19 @@
         <v>25</v>
       </c>
       <c r="I34" s="17" t="n">
-        <v>306.6</v>
+        <v>356.4</v>
       </c>
       <c r="J34" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>1.78</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
@@ -2778,41 +2682,41 @@
         </is>
       </c>
       <c r="C35" s="15" t="n">
-        <v>798</v>
+        <v>276.45</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="E35" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F35" s="15" t="n">
-        <v>750</v>
+        <v>330.1</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H35" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I35" s="17" t="n">
-        <v>-288</v>
+        <v>1019.35</v>
       </c>
       <c r="J35" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.1941</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>-0.92</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
@@ -2821,53 +2725,53 @@
         </is>
       </c>
       <c r="C36" s="15" t="n">
-        <v>260.45</v>
+        <v>1462.5</v>
       </c>
       <c r="D36" s="16" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F36" s="15" t="n">
-        <v>257.85</v>
+        <v>1564.7</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H36" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I36" s="17" t="n">
-        <v>-52.07</v>
+        <v>306.6</v>
       </c>
       <c r="J36" s="18" t="n">
-        <v>-0.01</v>
+        <v>0.0699</v>
       </c>
       <c r="K36" s="19" t="n">
-        <v>-0.13</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>6500</v>
+        <v>798</v>
       </c>
       <c r="D37" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E37" s="14" t="inlineStr">
         <is>
@@ -2875,7 +2779,7 @@
         </is>
       </c>
       <c r="F37" s="15" t="n">
-        <v>6401.5</v>
+        <v>750</v>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
@@ -2883,34 +2787,34 @@
         </is>
       </c>
       <c r="H37" s="14" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I37" s="17" t="n">
-        <v>-98.5</v>
+        <v>-288</v>
       </c>
       <c r="J37" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.0602</v>
       </c>
       <c r="K37" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C38" s="15" t="n">
-        <v>571.5</v>
+        <v>260.45</v>
       </c>
       <c r="D38" s="16" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
@@ -2918,7 +2822,7 @@
         </is>
       </c>
       <c r="F38" s="15" t="n">
-        <v>571.1</v>
+        <v>257.85</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
@@ -2926,34 +2830,34 @@
         </is>
       </c>
       <c r="H38" s="14" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="I38" s="17" t="n">
-        <v>-6.4</v>
+        <v>-52.07</v>
       </c>
       <c r="J38" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.01</v>
       </c>
       <c r="K38" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C39" s="15" t="n">
-        <v>965</v>
+        <v>6500</v>
       </c>
       <c r="D39" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E39" s="14" t="inlineStr">
         <is>
@@ -2961,7 +2865,7 @@
         </is>
       </c>
       <c r="F39" s="15" t="n">
-        <v>933</v>
+        <v>6401.5</v>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
@@ -2969,22 +2873,22 @@
         </is>
       </c>
       <c r="H39" s="14" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="I39" s="17" t="n">
-        <v>-288</v>
+        <v>-98.5</v>
       </c>
       <c r="J39" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0152</v>
       </c>
       <c r="K39" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
@@ -2993,18 +2897,18 @@
         </is>
       </c>
       <c r="C40" s="15" t="n">
-        <v>5479</v>
+        <v>571.5</v>
       </c>
       <c r="D40" s="16" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E40" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F40" s="15" t="n">
-        <v>5424</v>
+        <v>571.1</v>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
@@ -3012,42 +2916,42 @@
         </is>
       </c>
       <c r="H40" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I40" s="17" t="n">
-        <v>-55</v>
+        <v>-6.4</v>
       </c>
       <c r="J40" s="18" t="n">
+        <v>-0.0007</v>
+      </c>
+      <c r="K40" s="19" t="n">
         <v>-0.01</v>
-      </c>
-      <c r="K40" s="19" t="n">
-        <v>-0.18</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C41" s="15" t="n">
-        <v>960.1</v>
+        <v>965</v>
       </c>
       <c r="D41" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E41" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F41" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>933</v>
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
@@ -3055,42 +2959,42 @@
         </is>
       </c>
       <c r="H41" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I41" s="17" t="n">
-        <v>-516.79</v>
+        <v>-288</v>
       </c>
       <c r="J41" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.0332</v>
       </c>
       <c r="K41" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C42" s="15" t="n">
-        <v>952.1</v>
+        <v>5479</v>
       </c>
       <c r="D42" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E42" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F42" s="15" t="n">
-        <v>948.8</v>
+        <v>5424</v>
       </c>
       <c r="G42" s="14" t="inlineStr">
         <is>
@@ -3101,39 +3005,39 @@
         <v>1</v>
       </c>
       <c r="I42" s="17" t="n">
-        <v>-29.7</v>
+        <v>-55</v>
       </c>
       <c r="J42" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.01</v>
       </c>
       <c r="K42" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C43" s="15" t="n">
-        <v>1475</v>
+        <v>960.1</v>
       </c>
       <c r="D43" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E43" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F43" s="15" t="n">
-        <v>1394.19</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G43" s="14" t="inlineStr">
         <is>
@@ -3141,42 +3045,42 @@
         </is>
       </c>
       <c r="H43" s="14" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I43" s="17" t="n">
-        <v>-484.86</v>
+        <v>-516.79</v>
       </c>
       <c r="J43" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0598</v>
       </c>
       <c r="K43" s="19" t="n">
-        <v>-1</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C44" s="15" t="n">
-        <v>248.05</v>
+        <v>952.1</v>
       </c>
       <c r="D44" s="16" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E44" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F44" s="15" t="n">
-        <v>242.8</v>
+        <v>948.8</v>
       </c>
       <c r="G44" s="14" t="inlineStr">
         <is>
@@ -3184,42 +3088,42 @@
         </is>
       </c>
       <c r="H44" s="14" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I44" s="17" t="n">
-        <v>-110.25</v>
+        <v>-29.7</v>
       </c>
       <c r="J44" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0035</v>
       </c>
       <c r="K44" s="19" t="n">
-        <v>-0.3</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C45" s="15" t="n">
-        <v>1039.2</v>
+        <v>1475</v>
       </c>
       <c r="D45" s="16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E45" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F45" s="15" t="n">
-        <v>970</v>
+        <v>1394.19</v>
       </c>
       <c r="G45" s="14" t="inlineStr">
         <is>
@@ -3227,22 +3131,22 @@
         </is>
       </c>
       <c r="H45" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I45" s="17" t="n">
-        <v>-346</v>
+        <v>-484.86</v>
       </c>
       <c r="J45" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0548</v>
       </c>
       <c r="K45" s="19" t="n">
-        <v>-0.82</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B46" s="14" t="inlineStr">
@@ -3251,10 +3155,10 @@
         </is>
       </c>
       <c r="C46" s="15" t="n">
-        <v>199.96</v>
+        <v>248.05</v>
       </c>
       <c r="D46" s="16" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E46" s="14" t="inlineStr">
         <is>
@@ -3262,7 +3166,7 @@
         </is>
       </c>
       <c r="F46" s="15" t="n">
-        <v>193.31</v>
+        <v>242.8</v>
       </c>
       <c r="G46" s="14" t="inlineStr">
         <is>
@@ -3273,19 +3177,19 @@
         <v>11</v>
       </c>
       <c r="I46" s="17" t="n">
-        <v>-172.9</v>
+        <v>-110.25</v>
       </c>
       <c r="J46" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.0212</v>
       </c>
       <c r="K46" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B47" s="14" t="inlineStr">
@@ -3294,7 +3198,7 @@
         </is>
       </c>
       <c r="C47" s="15" t="n">
-        <v>986.4</v>
+        <v>1039.2</v>
       </c>
       <c r="D47" s="16" t="n">
         <v>5</v>
@@ -3305,7 +3209,7 @@
         </is>
       </c>
       <c r="F47" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>970</v>
       </c>
       <c r="G47" s="14" t="inlineStr">
         <is>
@@ -3316,17 +3220,103 @@
         <v>11</v>
       </c>
       <c r="I47" s="17" t="n">
+        <v>-346</v>
+      </c>
+      <c r="J47" s="18" t="n">
+        <v>-0.06660000000000001</v>
+      </c>
+      <c r="K47" s="19" t="n">
+        <v>-0.82</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="14" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C48" s="15" t="n">
+        <v>199.96</v>
+      </c>
+      <c r="D48" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="E48" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F48" s="15" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="G48" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H48" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I48" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J48" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K48" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C49" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D49" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E49" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F49" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G49" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H49" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I49" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J47" s="18" t="n">
+      <c r="J49" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K47" s="19" t="n">
+      <c r="K49" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I47">
+  <conditionalFormatting sqref="I2:I49">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3344,7 +3334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4391,6 +4381,31 @@
       </c>
       <c r="G41" s="14" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B42" s="20" t="n">
+        <v>203308.67</v>
+      </c>
+      <c r="C42" s="20" t="n">
+        <v>161619.17</v>
+      </c>
+      <c r="D42" s="20" t="n">
+        <v>41689.5</v>
+      </c>
+      <c r="E42" s="20" t="n">
+        <v>39755.9</v>
+      </c>
+      <c r="F42" s="20" t="n">
+        <v>1375.07</v>
+      </c>
+      <c r="G42" s="14" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -4473,7 +4488,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -4481,10 +4496,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>8600</v>
+        <v>8920.5</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8248.07</v>
+        <v>8537.139999999999</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -4496,7 +4511,7 @@
         <v>7.2</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8581723921240051</v>
+        <v>0.8516045245077504</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -4511,18 +4526,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1796.3</v>
+        <v>502.8</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1672.19</v>
+        <v>471.54</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -4531,10 +4546,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8402262253875158</v>
+        <v>0.8435106828655217</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -4549,18 +4564,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>479.45</v>
+        <v>1461.8</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>450.59</v>
+        <v>1369.97</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -4569,10 +4584,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8459949727691662</v>
+        <v>0.8479136992040218</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4587,18 +4602,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>OBEROIRLTY</t>
+          <t>KAJARIACER</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1846</v>
+        <v>1253.4</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1764.51</v>
+        <v>1182.47</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -4607,10 +4622,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.8</v>
+        <v>6.6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8189715123586091</v>
+        <v>0.8112997486384583</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -4625,18 +4640,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>857.55</v>
+        <v>1734.2</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>806.47</v>
+        <v>1605.14</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -4645,10 +4660,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8223271889400922</v>
+        <v>0.8059237536656891</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -4663,18 +4678,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>331.15</v>
+        <v>1787.3</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>314.13</v>
+        <v>1711.2</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -4683,10 +4698,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7946763720150817</v>
+        <v>0.7472957687473817</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -4701,7 +4716,7 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
@@ -4709,10 +4724,10 @@
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>712.05</v>
+        <v>720.05</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>661.02</v>
+        <v>664.91</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -4724,7 +4739,7 @@
         <v>6.5</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7495821114369501</v>
+        <v>0.7559614578969419</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -4739,18 +4754,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>OBEROIRLTY</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>4675.2</v>
+        <v>1846</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>4427.07</v>
+        <v>1765.23</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -4759,10 +4774,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7663552576455802</v>
+        <v>0.7618160871386678</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -4777,18 +4792,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>KAJARIACER</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1260.9</v>
+        <v>4482.8</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1189.9</v>
+        <v>4159.54</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -4800,7 +4815,7 @@
         <v>6.4</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7776633850020946</v>
+        <v>0.7641359447004609</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -4815,18 +4830,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>4435.1</v>
+        <v>609.5</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>4125.37</v>
+        <v>577.99</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -4838,7 +4853,7 @@
         <v>6.4</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7747235023041475</v>
+        <v>0.7303581901968998</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -4853,18 +4868,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>3MINDIA</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1851.7</v>
+        <v>35340</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1767.34</v>
+        <v>33437.86</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -4873,10 +4888,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7423900293255132</v>
+        <v>0.7398617511520736</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -4891,7 +4906,7 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
@@ -4899,10 +4914,10 @@
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>46750</v>
+        <v>47100</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>44410</v>
+        <v>44788.57</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -4911,10 +4926,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7369176790950985</v>
+        <v>0.7247308336824465</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -4929,18 +4944,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1663.4</v>
+        <v>999.6</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1583.19</v>
+        <v>953.89</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -4949,10 +4964,10 @@
         <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7315039798910766</v>
+        <v>0.7173408043569334</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -4967,18 +4982,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>INDHOTEL</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>721.75</v>
+        <v>4650</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>696.5700000000001</v>
+        <v>4403.31</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -4987,10 +5002,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7264463762044407</v>
+        <v>0.7158850020946795</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -5005,18 +5020,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260813</v>
+        <v>20260814</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1453</v>
+        <v>858.4</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1364.64</v>
+        <v>809.79</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -5025,10 +5040,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.2</v>
+        <v>6</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7711426476749057</v>
+        <v>0.7125387515710097</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-08-17
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Fri 14 Aug 2026</t>
+          <t>As of Mon 17 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹203,309</t>
+          <t>₹203,857</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-344  (-0.17%)</t>
+          <t>₹+548  (+0.27%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.65%</t>
+          <t>+1.93%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.35%</t>
+          <t>-1.09%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹161,619</t>
+          <t>₹99,287</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹39,756</t>
+          <t>₹102,088</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹41,690</t>
+          <t>₹104,570</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>4874.4</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1787.3</v>
+        <v>1809.7</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>5361.9</v>
+        <v>5429.1</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>487.5</v>
+        <v>554.7000000000003</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.1000123092072871</v>
+        <v>0.1137986213687839</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1520.16</v>
@@ -862,13 +862,13 @@
         <v>1743.85</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.02431041235382983</v>
+        <v>0.03638724650494565</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>45.45</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>4766.7</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1693</v>
+        <v>1669</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>5079</v>
+        <v>5007</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>312.2999999999997</v>
+        <v>240.2999999999997</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.06551702435647297</v>
+        <v>0.0504122348794763</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1499.44</v>
@@ -910,13 +910,13 @@
         <v>1607.792857142857</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.05032908615306735</v>
+        <v>0.03667294359325526</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>37.96</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>4237.8</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1450</v>
+        <v>1431.5</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>4350</v>
+        <v>4294.5</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>112.2000000000003</v>
+        <v>56.70000000000027</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.02647600169899483</v>
+        <v>0.01337958374628351</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1342.97</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1406</v>
+        <v>1408.592857142857</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.0303448275862069</v>
+        <v>0.01600219549922658</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>33.28</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>5101.6</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>792</v>
+        <v>805.1</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>5544</v>
+        <v>5635.7</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>442.4000000000003</v>
+        <v>534.1000000000005</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.08671789242590566</v>
+        <v>0.1046926454445665</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>676.71</v>
@@ -1006,13 +1006,13 @@
         <v>746.5642857142857</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.05736832611832615</v>
+        <v>0.07270614120694861</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>20.64</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
@@ -1036,31 +1036,31 @@
         <v>4120</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>4650</v>
+        <v>4693.4</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>4650</v>
+        <v>4693.4</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>530</v>
+        <v>573.3999999999996</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.1286407766990291</v>
+        <v>0.1391747572815533</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>3924.44</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>4305.171428571429</v>
+        <v>4363.871428571429</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.07415668202764972</v>
+        <v>0.07021105625528849</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>85.14</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>5172</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>865.2</v>
+        <v>852.05</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5191.200000000001</v>
+        <v>5112.299999999999</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>19.20000000000027</v>
+        <v>-59.70000000000027</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.003712296983758754</v>
+        <v>-0.01154292343387476</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>823.7</v>
@@ -1102,13 +1102,13 @@
         <v>836.5035714285714</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.03316739317086069</v>
+        <v>0.01824591112191606</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>15.94</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>4237.8</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1422.6</v>
+        <v>1415.1</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4267.799999999999</v>
+        <v>4245.299999999999</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>30</v>
+        <v>7.5</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.007079144839303412</v>
+        <v>0.001769786209825853</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1330.26</v>
@@ -1150,17 +1150,353 @@
         <v>1335.778571428572</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.06103010584242107</v>
+        <v>0.05605358530946804</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>40.91</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>8917.5</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>8917.5</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>8825.5</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>8825.5</v>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>-92</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>-0.01031679282310064</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>8537.139999999999</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>8537.139999999999</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>0.03267350291768178</v>
+      </c>
+      <c r="M10" s="13" t="n">
+        <v>194.79</v>
+      </c>
+      <c r="N10" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>HONASA</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>507</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>9126</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>481.65</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>8669.699999999999</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>-456.3000000000004</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>-0.05000000000000004</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>471.54</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>471.54</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>0.02099034568670187</v>
+      </c>
+      <c r="M11" s="13" t="n">
+        <v>16.89</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>RAINBOW</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>1423.8</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>8542.799999999999</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>1478.5</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>8871</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>328.2000000000003</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>0.03841831717937916</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>1369.97</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>1369.97</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>0.07340547852553261</v>
+      </c>
+      <c r="M12" s="13" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>KAJARIACER</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>1259</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>8813</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>1251.6</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>8761.199999999999</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>-51.80000000000064</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>-0.005877680698967507</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>1182.47</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>1182.47</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>0.05523330137424088</v>
+      </c>
+      <c r="M13" s="13" t="n">
+        <v>35.73</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>IPCALAB</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>1805.9</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>9029.5</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>1884.6</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>9423</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>393.4999999999991</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>0.0435793787031396</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>1605.14</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>1605.14</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>0.1482861084580281</v>
+      </c>
+      <c r="M14" s="13" t="n">
+        <v>73.94</v>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>MINDACORP</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>721.55</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>8658.6</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>725.15</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>8701.799999999999</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>43.20000000000027</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>0.004989259233594378</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>664.91</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>664.91</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>0.08307246776528995</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>27.21</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>OBEROIRLTY</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>1849</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>9245</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>1931</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>9655</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>410</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>0.04434829637641969</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>1765.23</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>1765.23</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0.0858467115484205</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>45.92</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H9">
+  <conditionalFormatting sqref="H2:H16">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3334,7 +3670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4406,6 +4742,31 @@
       </c>
       <c r="G42" s="14" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="n">
+        <v>203856.87</v>
+      </c>
+      <c r="C43" s="20" t="n">
+        <v>99286.77</v>
+      </c>
+      <c r="D43" s="20" t="n">
+        <v>104570.1</v>
+      </c>
+      <c r="E43" s="20" t="n">
+        <v>102088.3</v>
+      </c>
+      <c r="F43" s="20" t="n">
+        <v>1375.07</v>
+      </c>
+      <c r="G43" s="14" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -4488,30 +4849,30 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>OBEROIRLTY</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>8920.5</v>
+        <v>1931</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8537.139999999999</v>
+        <v>1839.16</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>9333</v>
+        <v>9343</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7.2</v>
+        <v>6.9</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8516045245077504</v>
+        <v>0.8246847507331377</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -4526,30 +4887,30 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>KAJARIACER</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>502.8</v>
+        <v>1251.6</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>471.54</v>
+        <v>1180.14</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>9333</v>
+        <v>9343</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8435106828655217</v>
+        <v>0.840359237536657</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -4564,30 +4925,30 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1461.8</v>
+        <v>481.65</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1369.97</v>
+        <v>447.86</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>9333</v>
+        <v>9343</v>
       </c>
       <c r="G4" s="14" t="n">
         <v>6.8</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8479136992040218</v>
+        <v>0.8216610808546293</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4602,30 +4963,30 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>KAJARIACER</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1253.4</v>
+        <v>1884.6</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1182.47</v>
+        <v>1736.73</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>9333</v>
+        <v>9343</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.6</v>
+        <v>6.8</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8112997486384583</v>
+        <v>0.7737526183493926</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -4640,30 +5001,30 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1734.2</v>
+        <v>8825.5</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1605.14</v>
+        <v>8435.93</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>9333</v>
+        <v>9343</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.6</v>
+        <v>6.8</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8059237536656891</v>
+        <v>0.8088772517804776</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -4678,30 +5039,30 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1787.3</v>
+        <v>1478.5</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1711.2</v>
+        <v>1381.5</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>9333</v>
+        <v>9343</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7472957687473817</v>
+        <v>0.835852534562212</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -4716,30 +5077,30 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>PHOENIXLTD</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>720.05</v>
+        <v>1929.8</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>664.91</v>
+        <v>1834.26</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>9333</v>
+        <v>9343</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7559614578969419</v>
+        <v>0.7843003770423125</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -4754,30 +5115,30 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>OBEROIRLTY</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1846</v>
+        <v>2093</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1765.23</v>
+        <v>1968.3</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>9333</v>
+        <v>9343</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7618160871386678</v>
+        <v>0.7639327607875995</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -4792,30 +5153,30 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>4482.8</v>
+        <v>1809.7</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>4159.54</v>
+        <v>1733.56</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>9333</v>
+        <v>9343</v>
       </c>
       <c r="G10" s="14" t="n">
         <v>6.4</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7641359447004609</v>
+        <v>0.7277346041055718</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -4830,30 +5191,30 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>CPPLUS</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>609.5</v>
+        <v>3343.1</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>577.99</v>
+        <v>3003.61</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.046</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>9333</v>
+        <v>9200</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7303581901968998</v>
+        <v>0.719075198994554</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -4868,30 +5229,30 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>3MINDIA</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>35340</v>
+        <v>861.55</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>33437.86</v>
+        <v>810.76</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>9333</v>
+        <v>9343</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7398617511520736</v>
+        <v>0.7320842061164642</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -4906,30 +5267,30 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>47100</v>
+        <v>805.1</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>44788.57</v>
+        <v>756.65</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>9333</v>
+        <v>9343</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7247308336824465</v>
+        <v>0.7143485546711353</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -4944,30 +5305,30 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>999.6</v>
+        <v>46970</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>953.89</v>
+        <v>44647.14</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>9333</v>
+        <v>9343</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>6.2</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7173408043569334</v>
+        <v>0.7127010892333473</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -4982,30 +5343,30 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>4650</v>
+        <v>1627.2</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>4403.31</v>
+        <v>1543.94</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>9333</v>
+        <v>9343</v>
       </c>
       <c r="G15" s="14" t="n">
         <v>6.2</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7158850020946795</v>
+        <v>0.7095915374947632</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -5020,30 +5381,30 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260814</v>
+        <v>20260817</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>858.4</v>
+        <v>725.15</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>809.79</v>
+        <v>670.72</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>9333</v>
+        <v>9343</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7125387515710097</v>
+        <v>0.7078581901968999</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-08-18
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Mon 17 Aug 2026</t>
+          <t>As of Tue 18 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹203,857</t>
+          <t>₹203,449</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+548  (+0.27%)</t>
+          <t>₹-408  (-0.20%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.93%</t>
+          <t>+1.72%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.09%</t>
+          <t>-1.29%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹99,287</t>
+          <t>₹107,774</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹102,088</t>
+          <t>₹92,962</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹104,570</t>
+          <t>₹95,674</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+1,375</t>
+          <t>₹+737</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3">
@@ -844,31 +844,31 @@
         <v>4874.4</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1809.7</v>
+        <v>1814</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>5429.1</v>
+        <v>5442</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>554.7000000000003</v>
+        <v>567.6000000000001</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.1137986213687839</v>
+        <v>0.1164451009354998</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1520.16</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>1743.85</v>
+        <v>1748.307142857143</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.03638724650494565</v>
+        <v>0.03621436446684526</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>45.45</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -892,31 +892,31 @@
         <v>4766.7</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1669</v>
+        <v>1674</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>5007</v>
+        <v>5022</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>240.2999999999997</v>
+        <v>255.2999999999997</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.0504122348794763</v>
+        <v>0.05355906602051728</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1499.44</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1607.792857142857</v>
+        <v>1607.985714285714</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.03667294359325526</v>
+        <v>0.03943505717699253</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>37.96</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>4237.8</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1431.5</v>
+        <v>1431.1</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>4294.5</v>
+        <v>4293.299999999999</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>56.70000000000027</v>
+        <v>55.5</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.01337958374628351</v>
+        <v>0.01309641795271131</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1342.97</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1408.592857142857</v>
+        <v>1417.164285714286</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.01600219549922658</v>
+        <v>0.009737764157441188</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>33.28</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>5101.6</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>805.1</v>
+        <v>824</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>5635.7</v>
+        <v>5768</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>534.1000000000005</v>
+        <v>666.4000000000003</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.1046926454445665</v>
+        <v>0.1306256860592756</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>676.71</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>746.5642857142857</v>
+        <v>749.4821428571429</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.07270614120694861</v>
+        <v>0.09043429264909844</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>20.64</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -1036,31 +1036,31 @@
         <v>4120</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>4693.4</v>
+        <v>4732.9</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>4693.4</v>
+        <v>4732.9</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>573.3999999999996</v>
+        <v>612.8999999999996</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.1391747572815533</v>
+        <v>0.14876213592233</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>3924.44</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>4363.871428571429</v>
+        <v>4419.785714285714</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.07021105625528849</v>
+        <v>0.06615696205588242</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>85.14</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
@@ -1084,31 +1084,31 @@
         <v>5172</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>852.05</v>
+        <v>841.55</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5112.299999999999</v>
+        <v>5049.299999999999</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>-59.70000000000027</v>
+        <v>-122.7000000000003</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>-0.01154292343387476</v>
+        <v>-0.023723897911833</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>823.7</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>836.5035714285714</v>
+        <v>837.2</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.01824591112191606</v>
+        <v>0.005169033331352753</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>15.94</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>4237.8</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1415.1</v>
+        <v>1442.7</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4245.299999999999</v>
+        <v>4328.1</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>7.5</v>
+        <v>90.30000000000041</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.001769786209825853</v>
+        <v>0.02130822596630337</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1330.26</v>
@@ -1150,13 +1150,13 @@
         <v>1335.778571428572</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.05605358530946804</v>
+        <v>0.07411203200348537</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>40.91</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>8917.5</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>8825.5</v>
+        <v>8817</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>8825.5</v>
+        <v>8817</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>-92</v>
+        <v>-100.5</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>-0.01031679282310064</v>
+        <v>-0.0112699747687132</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>8537.139999999999</v>
@@ -1198,19 +1198,19 @@
         <v>8537.139999999999</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.03267350291768178</v>
+        <v>0.03174095497334701</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>194.79</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -1219,46 +1219,46 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>507</v>
+        <v>1423.8</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>9126</v>
+        <v>8542.799999999999</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>481.65</v>
+        <v>1458.7</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8669.699999999999</v>
+        <v>8752.200000000001</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-456.3000000000004</v>
+        <v>209.4000000000005</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>-0.05000000000000004</v>
+        <v>0.02451186964461307</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>471.54</v>
+        <v>1369.97</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>471.54</v>
+        <v>1414.5</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.02099034568670187</v>
+        <v>0.03030095290327007</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>16.89</v>
+        <v>48.5</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>KAJARIACER</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1267,46 +1267,46 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>1423.8</v>
+        <v>1259</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>8542.799999999999</v>
+        <v>8813</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>1478.5</v>
+        <v>1225.8</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>8871</v>
+        <v>8580.6</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>328.2000000000003</v>
+        <v>-232.4000000000003</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.03841831717937916</v>
+        <v>-0.02637013502779988</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>1369.97</v>
+        <v>1182.47</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>1369.97</v>
+        <v>1182.47</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.07340547852553261</v>
+        <v>0.03534834393865225</v>
       </c>
       <c r="M12" s="13" t="n">
-        <v>48.5</v>
+        <v>35.73</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>KAJARIACER</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -1315,46 +1315,46 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>1259</v>
+        <v>1805.9</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>8813</v>
+        <v>9029.5</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1251.6</v>
+        <v>1882.1</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>8761.199999999999</v>
+        <v>9410.5</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-51.80000000000064</v>
+        <v>380.9999999999991</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.005877680698967507</v>
+        <v>0.0421950274101555</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>1182.47</v>
+        <v>1605.14</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>1182.47</v>
+        <v>1674.4</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.05523330137424088</v>
+        <v>0.1103554540141331</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>35.73</v>
+        <v>73.94</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1363,46 +1363,46 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>1805.9</v>
+        <v>721.55</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>9029.5</v>
+        <v>8658.6</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1884.6</v>
+        <v>745.25</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>9423</v>
+        <v>8943</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>393.4999999999991</v>
+        <v>284.4000000000005</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.0435793787031396</v>
+        <v>0.03284595662116284</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>1605.14</v>
+        <v>664.91</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>1605.14</v>
+        <v>664.91</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.1482861084580281</v>
+        <v>0.1078027507547803</v>
       </c>
       <c r="M14" s="13" t="n">
-        <v>73.94</v>
+        <v>27.21</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>OBEROIRLTY</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
@@ -1411,92 +1411,44 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>721.55</v>
+        <v>1849</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>8658.6</v>
+        <v>9245</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>725.15</v>
+        <v>1858</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>8701.799999999999</v>
+        <v>9290</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>43.20000000000027</v>
+        <v>45</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.004989259233594378</v>
+        <v>0.00486749594375338</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>664.91</v>
+        <v>1765.23</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>664.91</v>
+        <v>1765.23</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.08307246776528995</v>
+        <v>0.04993003229278793</v>
       </c>
       <c r="M15" s="13" t="n">
-        <v>27.21</v>
+        <v>45.92</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>OBEROIRLTY</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>1849</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <v>9245</v>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>1931</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>9655</v>
-      </c>
-      <c r="H16" s="10" t="n">
-        <v>410</v>
-      </c>
-      <c r="I16" s="11" t="n">
-        <v>0.04434829637641969</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>1765.23</v>
-      </c>
-      <c r="K16" s="7" t="n">
-        <v>1765.23</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>0.0858467115484205</v>
-      </c>
-      <c r="M16" s="13" t="n">
-        <v>45.92</v>
-      </c>
-      <c r="N16" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H16">
+  <conditionalFormatting sqref="H2:H15">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1514,7 +1466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1590,62 +1542,62 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>8847</v>
+        <v>507</v>
       </c>
       <c r="D2" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="n">
+        <v>471.54</v>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="14" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="F2" s="15" t="n">
-        <v>9240</v>
-      </c>
-      <c r="G2" s="14" t="inlineStr">
-        <is>
-          <t>TIME_STOP</t>
-        </is>
-      </c>
-      <c r="H2" s="14" t="n">
-        <v>25</v>
-      </c>
       <c r="I2" s="17" t="n">
-        <v>393</v>
+        <v>-638.28</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>0.0444</v>
+        <v>-0.0699</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>0.74</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>1948.5</v>
+        <v>8847</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
@@ -1653,50 +1605,50 @@
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>1922.5</v>
+        <v>9240</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-52</v>
+        <v>393</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0133</v>
+        <v>0.0444</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-0.36</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>4568</v>
+        <v>1948.5</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>4460</v>
+        <v>1922.5</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1704,22 +1656,22 @@
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-108</v>
+        <v>-52</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0236</v>
+        <v>-0.0133</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-0.49</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -1728,10 +1680,10 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>1550</v>
+        <v>4568</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
@@ -1739,7 +1691,7 @@
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>1470.07</v>
+        <v>4460</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1750,19 +1702,19 @@
         <v>10</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-239.79</v>
+        <v>-108</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.0516</v>
+        <v>-0.0236</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-0.77</v>
+        <v>-0.49</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -1771,18 +1723,18 @@
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>1713.4</v>
+        <v>1550</v>
       </c>
       <c r="D6" s="16" t="n">
         <v>3</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>1650</v>
+        <v>1470.07</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -1790,34 +1742,34 @@
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>-190.2</v>
+        <v>-239.79</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>-0.037</v>
+        <v>-0.0516</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>-0.65</v>
+        <v>-0.77</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>2360</v>
+        <v>1713.4</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
@@ -1825,7 +1777,7 @@
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>2250.39</v>
+        <v>1650</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -1833,22 +1785,22 @@
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>-548.05</v>
+        <v>-190.2</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>-0.0464</v>
+        <v>-0.037</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>-1</v>
+        <v>-0.65</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -1857,18 +1809,18 @@
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>8945</v>
+        <v>2360</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>8673.639999999999</v>
+        <v>2250.39</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -1876,13 +1828,13 @@
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>-271.36</v>
+        <v>-548.05</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>-0.0303</v>
+        <v>-0.0464</v>
       </c>
       <c r="K8" s="19" t="n">
         <v>-1</v>
@@ -1891,27 +1843,27 @@
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>2218</v>
+        <v>8945</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>2132.81</v>
+        <v>8673.639999999999</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
@@ -1919,85 +1871,85 @@
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>-170.37</v>
+        <v>-271.36</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>-0.0384</v>
+        <v>-0.0303</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>-0.76</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1269</v>
+        <v>2218</v>
       </c>
       <c r="D10" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>2132.81</v>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="F10" s="15" t="n">
-        <v>1365.2</v>
-      </c>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>TIME_STOP</t>
-        </is>
-      </c>
-      <c r="H10" s="14" t="n">
-        <v>25</v>
-      </c>
       <c r="I10" s="17" t="n">
-        <v>673.4</v>
+        <v>-170.37</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>0.07580000000000001</v>
+        <v>-0.0384</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>1.11</v>
+        <v>-0.76</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>7579.5</v>
+        <v>1269</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>7567.5</v>
+        <v>1365.2</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
@@ -2008,19 +1960,19 @@
         <v>25</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>-12</v>
+        <v>673.4</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>-0.0016</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>-0.03</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -2029,10 +1981,10 @@
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>1798.5</v>
+        <v>7579.5</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
@@ -2040,7 +1992,7 @@
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>1747.8</v>
+        <v>7567.5</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -2051,74 +2003,74 @@
         <v>25</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>-253.5</v>
+        <v>-12</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>-0.0282</v>
+        <v>-0.0016</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>-0.43</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>5438</v>
+        <v>1798.5</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>5381</v>
+        <v>1747.8</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>-57</v>
+        <v>-253.5</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>-0.0105</v>
+        <v>-0.0282</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>1784</v>
+        <v>5438</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
@@ -2126,7 +2078,7 @@
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>1752.1</v>
+        <v>5381</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
@@ -2134,22 +2086,22 @@
         </is>
       </c>
       <c r="H14" s="14" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>-63.8</v>
+        <v>-57</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>-0.0179</v>
+        <v>-0.0105</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>-0.36</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -2158,18 +2110,18 @@
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>871.8</v>
+        <v>1784</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>830.15</v>
+        <v>1752.1</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
@@ -2177,65 +2129,65 @@
         </is>
       </c>
       <c r="H15" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>-249.9</v>
+        <v>-63.8</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>-0.0478</v>
+        <v>-0.0179</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>-0.73</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>420.3</v>
+        <v>871.8</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>448.6</v>
+        <v>830.15</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H16" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>622.6</v>
+        <v>-249.9</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>0.0673</v>
+        <v>-0.0478</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>0.84</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -2244,10 +2196,10 @@
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>1465</v>
+        <v>420.3</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
@@ -2255,7 +2207,7 @@
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>1596.9</v>
+        <v>448.6</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -2266,19 +2218,19 @@
         <v>25</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>791.4</v>
+        <v>622.6</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>0.09</v>
+        <v>0.0673</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>1.32</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -2287,10 +2239,10 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>619.25</v>
+        <v>1465</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
@@ -2298,7 +2250,7 @@
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>717.95</v>
+        <v>1596.9</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -2309,19 +2261,19 @@
         <v>25</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>1480.5</v>
+        <v>791.4</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>0.1594</v>
+        <v>0.09</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>3.55</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -2330,10 +2282,10 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>8700</v>
+        <v>619.25</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
@@ -2341,7 +2293,7 @@
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>8805.5</v>
+        <v>717.95</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
@@ -2352,31 +2304,31 @@
         <v>25</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>105.5</v>
+        <v>1480.5</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>0.0121</v>
+        <v>0.1594</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>0.29</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>961.85</v>
+        <v>8700</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
@@ -2384,42 +2336,42 @@
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>935.6</v>
+        <v>8805.5</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H20" s="14" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>-236.25</v>
+        <v>105.5</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>-0.0273</v>
+        <v>0.0121</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>-0.64</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>1560</v>
+        <v>961.85</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
@@ -2427,7 +2379,7 @@
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>1547.4</v>
+        <v>935.6</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -2435,42 +2387,42 @@
         </is>
       </c>
       <c r="H21" s="14" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>-63</v>
+        <v>-236.25</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>-0.0081</v>
+        <v>-0.0273</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>-0.23</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>900</v>
+        <v>1560</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>887.1</v>
+        <v>1547.4</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -2478,42 +2430,42 @@
         </is>
       </c>
       <c r="H22" s="14" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>-129</v>
+        <v>-63</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>-0.0143</v>
+        <v>-0.0081</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.23</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>880.8</v>
+        <v>900</v>
       </c>
       <c r="D23" s="16" t="n">
         <v>10</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>832.9400000000001</v>
+        <v>887.1</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -2521,22 +2473,22 @@
         </is>
       </c>
       <c r="H23" s="14" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>-478.6</v>
+        <v>-129</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>-0.0543</v>
+        <v>-0.0143</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>-1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -2545,10 +2497,10 @@
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>777</v>
+        <v>880.8</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
@@ -2556,7 +2508,7 @@
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>744.8</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -2567,10 +2519,10 @@
         <v>2</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>-386.4</v>
+        <v>-478.6</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>-0.0414</v>
+        <v>-0.0543</v>
       </c>
       <c r="K24" s="19" t="n">
         <v>-1</v>
@@ -2579,27 +2531,27 @@
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>1114.9</v>
+        <v>777</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>1050.57</v>
+        <v>744.8</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -2607,13 +2559,13 @@
         </is>
       </c>
       <c r="H25" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>-514.64</v>
+        <v>-386.4</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>-0.0577</v>
+        <v>-0.0414</v>
       </c>
       <c r="K25" s="19" t="n">
         <v>-1</v>
@@ -2622,50 +2574,50 @@
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>790</v>
+        <v>1114.9</v>
       </c>
       <c r="D26" s="16" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>880.8</v>
+        <v>1050.57</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H26" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I26" s="17" t="n">
-        <v>998.8</v>
+        <v>-514.64</v>
       </c>
       <c r="J26" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0577</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
@@ -2674,10 +2626,10 @@
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>3770</v>
+        <v>790</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
@@ -2685,7 +2637,7 @@
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>4097.9</v>
+        <v>880.8</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
@@ -2696,19 +2648,19 @@
         <v>25</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>655.8</v>
+        <v>998.8</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.1149</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>1.98</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
@@ -2717,10 +2669,10 @@
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>821.05</v>
+        <v>3770</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
@@ -2728,7 +2680,7 @@
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>844</v>
+        <v>4097.9</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
@@ -2739,19 +2691,19 @@
         <v>25</v>
       </c>
       <c r="I28" s="17" t="n">
-        <v>252.45</v>
+        <v>655.8</v>
       </c>
       <c r="J28" s="18" t="n">
-        <v>0.028</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>0.6</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -2760,10 +2712,10 @@
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>2426.1</v>
+        <v>821.05</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
@@ -2771,7 +2723,7 @@
         </is>
       </c>
       <c r="F29" s="15" t="n">
-        <v>2484.2</v>
+        <v>844</v>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
@@ -2782,39 +2734,39 @@
         <v>25</v>
       </c>
       <c r="I29" s="17" t="n">
-        <v>174.3</v>
+        <v>252.45</v>
       </c>
       <c r="J29" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.028</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C30" s="15" t="n">
-        <v>1410</v>
+        <v>2426.1</v>
       </c>
       <c r="D30" s="16" t="n">
         <v>3</v>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F30" s="15" t="n">
-        <v>1455.2</v>
+        <v>2484.2</v>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
@@ -2825,19 +2777,19 @@
         <v>25</v>
       </c>
       <c r="I30" s="17" t="n">
-        <v>135.6</v>
+        <v>174.3</v>
       </c>
       <c r="J30" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.0239</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>0.46</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
@@ -2846,10 +2798,10 @@
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>690</v>
+        <v>1410</v>
       </c>
       <c r="D31" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
@@ -2857,7 +2809,7 @@
         </is>
       </c>
       <c r="F31" s="15" t="n">
-        <v>660.45</v>
+        <v>1455.2</v>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
@@ -2868,19 +2820,19 @@
         <v>25</v>
       </c>
       <c r="I31" s="17" t="n">
-        <v>-206.85</v>
+        <v>135.6</v>
       </c>
       <c r="J31" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.0321</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
@@ -2889,10 +2841,10 @@
         </is>
       </c>
       <c r="C32" s="15" t="n">
-        <v>1839</v>
+        <v>690</v>
       </c>
       <c r="D32" s="16" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
@@ -2900,7 +2852,7 @@
         </is>
       </c>
       <c r="F32" s="15" t="n">
-        <v>1828.1</v>
+        <v>660.45</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
@@ -2911,19 +2863,19 @@
         <v>25</v>
       </c>
       <c r="I32" s="17" t="n">
-        <v>-21.8</v>
+        <v>-206.85</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>-0.0059</v>
+        <v>-0.0428</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>-0.1</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
@@ -2932,10 +2884,10 @@
         </is>
       </c>
       <c r="C33" s="15" t="n">
-        <v>1414</v>
+        <v>1839</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
@@ -2943,7 +2895,7 @@
         </is>
       </c>
       <c r="F33" s="15" t="n">
-        <v>1537.8</v>
+        <v>1828.1</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
@@ -2954,19 +2906,19 @@
         <v>25</v>
       </c>
       <c r="I33" s="17" t="n">
-        <v>371.4</v>
+        <v>-21.8</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>0.0876</v>
+        <v>-0.0059</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>1.38</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
@@ -2975,10 +2927,10 @@
         </is>
       </c>
       <c r="C34" s="15" t="n">
-        <v>1300</v>
+        <v>1414</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
@@ -2986,7 +2938,7 @@
         </is>
       </c>
       <c r="F34" s="15" t="n">
-        <v>1389.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
@@ -2997,19 +2949,19 @@
         <v>25</v>
       </c>
       <c r="I34" s="17" t="n">
-        <v>356.4</v>
+        <v>371.4</v>
       </c>
       <c r="J34" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>0.0876</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>0.63</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
@@ -3018,10 +2970,10 @@
         </is>
       </c>
       <c r="C35" s="15" t="n">
-        <v>276.45</v>
+        <v>1300</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E35" s="14" t="inlineStr">
         <is>
@@ -3029,7 +2981,7 @@
         </is>
       </c>
       <c r="F35" s="15" t="n">
-        <v>330.1</v>
+        <v>1389.1</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
@@ -3040,19 +2992,19 @@
         <v>25</v>
       </c>
       <c r="I35" s="17" t="n">
-        <v>1019.35</v>
+        <v>356.4</v>
       </c>
       <c r="J35" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>3.1</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
@@ -3061,10 +3013,10 @@
         </is>
       </c>
       <c r="C36" s="15" t="n">
-        <v>1462.5</v>
+        <v>276.45</v>
       </c>
       <c r="D36" s="16" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
@@ -3072,7 +3024,7 @@
         </is>
       </c>
       <c r="F36" s="15" t="n">
-        <v>1564.7</v>
+        <v>330.1</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
@@ -3083,19 +3035,19 @@
         <v>25</v>
       </c>
       <c r="I36" s="17" t="n">
-        <v>306.6</v>
+        <v>1019.35</v>
       </c>
       <c r="J36" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.1941</v>
       </c>
       <c r="K36" s="19" t="n">
-        <v>1.78</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
@@ -3104,41 +3056,41 @@
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>798</v>
+        <v>1462.5</v>
       </c>
       <c r="D37" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E37" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F37" s="15" t="n">
-        <v>750</v>
+        <v>1564.7</v>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H37" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I37" s="17" t="n">
-        <v>-288</v>
+        <v>306.6</v>
       </c>
       <c r="J37" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.0699</v>
       </c>
       <c r="K37" s="19" t="n">
-        <v>-0.92</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
@@ -3147,10 +3099,10 @@
         </is>
       </c>
       <c r="C38" s="15" t="n">
-        <v>260.45</v>
+        <v>798</v>
       </c>
       <c r="D38" s="16" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
@@ -3158,7 +3110,7 @@
         </is>
       </c>
       <c r="F38" s="15" t="n">
-        <v>257.85</v>
+        <v>750</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
@@ -3169,31 +3121,31 @@
         <v>23</v>
       </c>
       <c r="I38" s="17" t="n">
-        <v>-52.07</v>
+        <v>-288</v>
       </c>
       <c r="J38" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0602</v>
       </c>
       <c r="K38" s="19" t="n">
-        <v>-0.13</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C39" s="15" t="n">
-        <v>6500</v>
+        <v>260.45</v>
       </c>
       <c r="D39" s="16" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E39" s="14" t="inlineStr">
         <is>
@@ -3201,7 +3153,7 @@
         </is>
       </c>
       <c r="F39" s="15" t="n">
-        <v>6401.5</v>
+        <v>257.85</v>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
@@ -3209,65 +3161,65 @@
         </is>
       </c>
       <c r="H39" s="14" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I39" s="17" t="n">
-        <v>-98.5</v>
+        <v>-52.07</v>
       </c>
       <c r="J39" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.01</v>
       </c>
       <c r="K39" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C40" s="15" t="n">
-        <v>571.5</v>
+        <v>6500</v>
       </c>
       <c r="D40" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="F40" s="15" t="n">
+        <v>6401.5</v>
+      </c>
+      <c r="G40" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H40" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="E40" s="14" t="inlineStr">
-        <is>
-          <t>2026-07-08</t>
-        </is>
-      </c>
-      <c r="F40" s="15" t="n">
-        <v>571.1</v>
-      </c>
-      <c r="G40" s="14" t="inlineStr">
-        <is>
-          <t>STOP_LOSS</t>
-        </is>
-      </c>
-      <c r="H40" s="14" t="n">
-        <v>2</v>
-      </c>
       <c r="I40" s="17" t="n">
-        <v>-6.4</v>
+        <v>-98.5</v>
       </c>
       <c r="J40" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.0152</v>
       </c>
       <c r="K40" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
@@ -3276,10 +3228,10 @@
         </is>
       </c>
       <c r="C41" s="15" t="n">
-        <v>965</v>
+        <v>571.5</v>
       </c>
       <c r="D41" s="16" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E41" s="14" t="inlineStr">
         <is>
@@ -3287,7 +3239,7 @@
         </is>
       </c>
       <c r="F41" s="15" t="n">
-        <v>933</v>
+        <v>571.1</v>
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
@@ -3298,19 +3250,19 @@
         <v>2</v>
       </c>
       <c r="I41" s="17" t="n">
-        <v>-288</v>
+        <v>-6.4</v>
       </c>
       <c r="J41" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0007</v>
       </c>
       <c r="K41" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
@@ -3319,18 +3271,18 @@
         </is>
       </c>
       <c r="C42" s="15" t="n">
-        <v>5479</v>
+        <v>965</v>
       </c>
       <c r="D42" s="16" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E42" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F42" s="15" t="n">
-        <v>5424</v>
+        <v>933</v>
       </c>
       <c r="G42" s="14" t="inlineStr">
         <is>
@@ -3338,42 +3290,42 @@
         </is>
       </c>
       <c r="H42" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I42" s="17" t="n">
-        <v>-55</v>
+        <v>-288</v>
       </c>
       <c r="J42" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0332</v>
       </c>
       <c r="K42" s="19" t="n">
-        <v>-0.18</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C43" s="15" t="n">
-        <v>960.1</v>
+        <v>5479</v>
       </c>
       <c r="D43" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E43" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F43" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>5424</v>
       </c>
       <c r="G43" s="14" t="inlineStr">
         <is>
@@ -3381,22 +3333,22 @@
         </is>
       </c>
       <c r="H43" s="14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I43" s="17" t="n">
-        <v>-516.79</v>
+        <v>-55</v>
       </c>
       <c r="J43" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.01</v>
       </c>
       <c r="K43" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
@@ -3405,18 +3357,18 @@
         </is>
       </c>
       <c r="C44" s="15" t="n">
-        <v>952.1</v>
+        <v>960.1</v>
       </c>
       <c r="D44" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E44" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F44" s="15" t="n">
-        <v>948.8</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G44" s="14" t="inlineStr">
         <is>
@@ -3424,42 +3376,42 @@
         </is>
       </c>
       <c r="H44" s="14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I44" s="17" t="n">
-        <v>-29.7</v>
+        <v>-516.79</v>
       </c>
       <c r="J44" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.0598</v>
       </c>
       <c r="K44" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C45" s="15" t="n">
-        <v>1475</v>
+        <v>952.1</v>
       </c>
       <c r="D45" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E45" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F45" s="15" t="n">
-        <v>1394.19</v>
+        <v>948.8</v>
       </c>
       <c r="G45" s="14" t="inlineStr">
         <is>
@@ -3467,42 +3419,42 @@
         </is>
       </c>
       <c r="H45" s="14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I45" s="17" t="n">
-        <v>-484.86</v>
+        <v>-29.7</v>
       </c>
       <c r="J45" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0035</v>
       </c>
       <c r="K45" s="19" t="n">
-        <v>-1</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C46" s="15" t="n">
-        <v>248.05</v>
+        <v>1475</v>
       </c>
       <c r="D46" s="16" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E46" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F46" s="15" t="n">
-        <v>242.8</v>
+        <v>1394.19</v>
       </c>
       <c r="G46" s="14" t="inlineStr">
         <is>
@@ -3510,22 +3462,22 @@
         </is>
       </c>
       <c r="H46" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I46" s="17" t="n">
-        <v>-110.25</v>
+        <v>-484.86</v>
       </c>
       <c r="J46" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0548</v>
       </c>
       <c r="K46" s="19" t="n">
-        <v>-0.3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B47" s="14" t="inlineStr">
@@ -3534,10 +3486,10 @@
         </is>
       </c>
       <c r="C47" s="15" t="n">
-        <v>1039.2</v>
+        <v>248.05</v>
       </c>
       <c r="D47" s="16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E47" s="14" t="inlineStr">
         <is>
@@ -3545,7 +3497,7 @@
         </is>
       </c>
       <c r="F47" s="15" t="n">
-        <v>970</v>
+        <v>242.8</v>
       </c>
       <c r="G47" s="14" t="inlineStr">
         <is>
@@ -3556,19 +3508,19 @@
         <v>11</v>
       </c>
       <c r="I47" s="17" t="n">
-        <v>-346</v>
+        <v>-110.25</v>
       </c>
       <c r="J47" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="K47" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B48" s="14" t="inlineStr">
@@ -3577,10 +3529,10 @@
         </is>
       </c>
       <c r="C48" s="15" t="n">
-        <v>199.96</v>
+        <v>1039.2</v>
       </c>
       <c r="D48" s="16" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="E48" s="14" t="inlineStr">
         <is>
@@ -3588,7 +3540,7 @@
         </is>
       </c>
       <c r="F48" s="15" t="n">
-        <v>193.31</v>
+        <v>970</v>
       </c>
       <c r="G48" s="14" t="inlineStr">
         <is>
@@ -3599,19 +3551,19 @@
         <v>11</v>
       </c>
       <c r="I48" s="17" t="n">
-        <v>-172.9</v>
+        <v>-346</v>
       </c>
       <c r="J48" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.06660000000000001</v>
       </c>
       <c r="K48" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B49" s="14" t="inlineStr">
@@ -3620,10 +3572,10 @@
         </is>
       </c>
       <c r="C49" s="15" t="n">
-        <v>986.4</v>
+        <v>199.96</v>
       </c>
       <c r="D49" s="16" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="E49" s="14" t="inlineStr">
         <is>
@@ -3631,7 +3583,7 @@
         </is>
       </c>
       <c r="F49" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>193.31</v>
       </c>
       <c r="G49" s="14" t="inlineStr">
         <is>
@@ -3642,17 +3594,60 @@
         <v>11</v>
       </c>
       <c r="I49" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J49" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K49" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D50" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E50" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F50" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G50" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H50" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I50" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J49" s="18" t="n">
+      <c r="J50" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K49" s="19" t="n">
+      <c r="K50" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I49">
+  <conditionalFormatting sqref="I2:I50">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3670,7 +3665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4767,6 +4762,31 @@
       </c>
       <c r="G43" s="14" t="n">
         <v>15</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B44" s="20" t="n">
+        <v>203448.99</v>
+      </c>
+      <c r="C44" s="20" t="n">
+        <v>107774.49</v>
+      </c>
+      <c r="D44" s="20" t="n">
+        <v>95674.5</v>
+      </c>
+      <c r="E44" s="20" t="n">
+        <v>92962.3</v>
+      </c>
+      <c r="F44" s="20" t="n">
+        <v>736.79</v>
+      </c>
+      <c r="G44" s="14" t="n">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -4849,30 +4869,30 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>OBEROIRLTY</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1931</v>
+        <v>8817</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1839.16</v>
+        <v>8419.790000000001</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>9343</v>
+        <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
         <v>6.9</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8246847507331377</v>
+        <v>0.8124036447423545</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -4887,30 +4907,30 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>KAJARIACER</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1251.6</v>
+        <v>48730</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1180.14</v>
+        <v>46372.86</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>9343</v>
+        <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.840359237536657</v>
+        <v>0.8117919983242563</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -4925,30 +4945,30 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>OBEROIRLTY</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>481.65</v>
+        <v>1858</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>447.86</v>
+        <v>1755.91</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>9343</v>
+        <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
         <v>6.8</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8216610808546293</v>
+        <v>0.7973963133640554</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -4963,30 +4983,30 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1884.6</v>
+        <v>474.6</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1736.73</v>
+        <v>440.61</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>9343</v>
+        <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.8</v>
+        <v>6.6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7737526183493926</v>
+        <v>0.784082530372853</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -5001,30 +5021,30 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>8825.5</v>
+        <v>4732.9</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>8435.93</v>
+        <v>4524.16</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>9343</v>
+        <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.8</v>
+        <v>6.6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8088772517804776</v>
+        <v>0.783596564725597</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -5039,30 +5059,30 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1478.5</v>
+        <v>824</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1381.5</v>
+        <v>774.3200000000001</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>9343</v>
+        <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.835852534562212</v>
+        <v>0.7695601173020528</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -5077,30 +5097,30 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>PHOENIXLTD</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1929.8</v>
+        <v>2628.4</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1834.26</v>
+        <v>2519.46</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>9343</v>
+        <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7843003770423125</v>
+        <v>0.7324423963133641</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -5115,30 +5135,30 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>2093</v>
+        <v>745.25</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1968.3</v>
+        <v>688.01</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>9343</v>
+        <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7639327607875995</v>
+        <v>0.740608504398827</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -5153,30 +5173,30 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1809.7</v>
+        <v>1917.1</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1733.56</v>
+        <v>1823.1</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>9343</v>
+        <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7277346041055718</v>
+        <v>0.7286049434436531</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -5191,30 +5211,30 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>CPPLUS</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>3343.1</v>
+        <v>2098.9</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>3003.61</v>
+        <v>1974.04</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.046</v>
+        <v>0.0467</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>9200</v>
+        <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
         <v>6.3</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.719075198994554</v>
+        <v>0.7214327607875995</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -5229,30 +5249,30 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>861.55</v>
+        <v>1882.1</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>810.76</v>
+        <v>1732.99</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>9343</v>
+        <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7320842061164642</v>
+        <v>0.7240029325513198</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -5267,30 +5287,30 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>SYRMA</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>805.1</v>
+        <v>1500.1</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>756.65</v>
+        <v>1385.17</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>9343</v>
+        <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7143485546711353</v>
+        <v>0.7166139505655635</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -5305,30 +5325,30 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>46970</v>
+        <v>851.2</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>44647.14</v>
+        <v>801.99</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>9343</v>
+        <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>6.2</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7127010892333473</v>
+        <v>0.7368726434855467</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -5343,30 +5363,30 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>PHOENIXLTD</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1627.2</v>
+        <v>1940</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1543.94</v>
+        <v>1857.64</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>9343</v>
+        <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
         <v>6.2</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7095915374947632</v>
+        <v>0.7265573942186846</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -5381,30 +5401,30 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260817</v>
+        <v>20260818</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>725.15</v>
+        <v>1458.7</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>670.72</v>
+        <v>1362.41</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>9343</v>
+        <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7078581901968999</v>
+        <v>0.735053414327608</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-08-19
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Tue 18 Aug 2026</t>
+          <t>As of Wed 19 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹203,449</t>
+          <t>₹203,156</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-408  (-0.20%)</t>
+          <t>₹-293  (-0.14%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.72%</t>
+          <t>+1.58%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.29%</t>
+          <t>-1.43%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹107,774</t>
+          <t>₹112,026</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹92,962</t>
+          <t>₹88,724</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹95,674</t>
+          <t>₹91,130</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+737</t>
+          <t>₹+750</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>4874.4</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1814</v>
+        <v>1801.8</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>5442</v>
+        <v>5405.4</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>567.6000000000001</v>
+        <v>531</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.1164451009354998</v>
+        <v>0.1089364844903988</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1520.16</v>
@@ -862,13 +862,13 @@
         <v>1748.307142857143</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.03621436446684526</v>
+        <v>0.02968856540285118</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>45.45</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>4766.7</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1674</v>
+        <v>1650</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>5022</v>
+        <v>4950</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>255.2999999999997</v>
+        <v>183.2999999999997</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.05355906602051728</v>
+        <v>0.03845427654352061</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1499.44</v>
@@ -910,19 +910,19 @@
         <v>1607.985714285714</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.03943505717699253</v>
+        <v>0.02546320346320334</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>37.96</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -931,46 +931,46 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>1412.6</v>
+        <v>728.8</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>4237.8</v>
+        <v>5101.6</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1431.1</v>
+        <v>823.5</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>4293.299999999999</v>
+        <v>5764.5</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>55.5</v>
+        <v>662.9000000000003</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.01309641795271131</v>
+        <v>0.1299396267837542</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>1342.97</v>
+        <v>676.71</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1417.164285714286</v>
+        <v>757.9892857142856</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.009737764157441188</v>
+        <v>0.07955156561713947</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>33.28</v>
+        <v>20.64</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -979,46 +979,46 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>728.8</v>
+        <v>4120</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>5101.6</v>
+        <v>4120</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>824</v>
+        <v>4696</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>5768</v>
+        <v>4696</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>666.4000000000003</v>
+        <v>576</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.1306256860592756</v>
+        <v>0.1398058252427185</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>676.71</v>
+        <v>3924.44</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>749.4821428571429</v>
+        <v>4428.228571428571</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.09043429264909844</v>
+        <v>0.05702117303480178</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>20.64</v>
+        <v>85.14</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -1027,142 +1027,142 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>4120</v>
+        <v>862</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>4120</v>
+        <v>5172</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>4732.9</v>
+        <v>850</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>4732.9</v>
+        <v>5100</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>612.8999999999996</v>
+        <v>-72</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.14876213592233</v>
+        <v>-0.01392111368909513</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>3924.44</v>
+        <v>823.7</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>4419.785714285714</v>
+        <v>839.05</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.06615696205588242</v>
+        <v>0.01288235294117652</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>85.14</v>
+        <v>15.94</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>862</v>
+        <v>1412.6</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>5172</v>
+        <v>4237.8</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>841.55</v>
+        <v>1417.2</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5049.299999999999</v>
+        <v>4251.6</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>-122.7000000000003</v>
+        <v>13.80000000000041</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>-0.023723897911833</v>
+        <v>0.003256406626079666</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>823.7</v>
+        <v>1330.26</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>837.2</v>
+        <v>1335.778571428572</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.005169033331352753</v>
+        <v>0.05745232047094859</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>15.94</v>
+        <v>40.91</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>1412.6</v>
+        <v>8917.5</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>4237.8</v>
+        <v>8917.5</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1442.7</v>
+        <v>8750</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4328.1</v>
+        <v>8750</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>90.30000000000041</v>
+        <v>-167.5</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.02130822596630337</v>
+        <v>-0.01878329128118867</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>1330.26</v>
+        <v>8537.139999999999</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>1335.778571428572</v>
+        <v>8537.139999999999</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.07411203200348537</v>
+        <v>0.02432685714285721</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>40.91</v>
+        <v>194.79</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1171,46 +1171,46 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>8917.5</v>
+        <v>1423.8</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>8917.5</v>
+        <v>8542.799999999999</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>8817</v>
+        <v>1461.8</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>8817</v>
+        <v>8770.799999999999</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>-100.5</v>
+        <v>228</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>-0.0112699747687132</v>
+        <v>0.02668914173338952</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>8537.139999999999</v>
+        <v>1369.97</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>8537.139999999999</v>
+        <v>1414.5</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.03174095497334701</v>
+        <v>0.03235736762895058</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>194.79</v>
+        <v>48.5</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>KAJARIACER</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -1219,46 +1219,46 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>1423.8</v>
+        <v>1259</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>8542.799999999999</v>
+        <v>8813</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>1458.7</v>
+        <v>1208.9</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8752.200000000001</v>
+        <v>8462.300000000001</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>209.4000000000005</v>
+        <v>-350.6999999999994</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.02451186964461307</v>
+        <v>-0.03979348689436053</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>1369.97</v>
+        <v>1182.47</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>1414.5</v>
+        <v>1182.47</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.03030095290327007</v>
+        <v>0.02186285052527096</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>48.5</v>
+        <v>35.73</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>KAJARIACER</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1267,46 +1267,46 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>1259</v>
+        <v>1805.9</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>8813</v>
+        <v>9029.5</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>1225.8</v>
+        <v>1903.7</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>8580.6</v>
+        <v>9518.5</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-232.4000000000003</v>
+        <v>488.9999999999998</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.02637013502779988</v>
+        <v>0.05415582258153826</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>1182.47</v>
+        <v>1605.14</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>1182.47</v>
+        <v>1674.4</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.03534834393865225</v>
+        <v>0.1204496506802542</v>
       </c>
       <c r="M12" s="13" t="n">
-        <v>35.73</v>
+        <v>73.94</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -1315,46 +1315,46 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>1805.9</v>
+        <v>721.55</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>9029.5</v>
+        <v>8658.6</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1882.1</v>
+        <v>738.9</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>9410.5</v>
+        <v>8866.799999999999</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>380.9999999999991</v>
+        <v>208.2000000000003</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.0421950274101555</v>
+        <v>0.02404545769523945</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>1605.14</v>
+        <v>664.91</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>1674.4</v>
+        <v>664.91</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.1103554540141331</v>
+        <v>0.1001353363107322</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>73.94</v>
+        <v>27.21</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>OBEROIRLTY</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1363,92 +1363,44 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>721.55</v>
+        <v>1849</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>8658.6</v>
+        <v>9245</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>745.25</v>
+        <v>1869.7</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>8943</v>
+        <v>9348.5</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>284.4000000000005</v>
+        <v>103.5000000000002</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.03284595662116284</v>
+        <v>0.0111952406706328</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>664.91</v>
+        <v>1765.23</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>664.91</v>
+        <v>1765.23</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.1078027507547803</v>
+        <v>0.0558752741081457</v>
       </c>
       <c r="M14" s="13" t="n">
-        <v>27.21</v>
+        <v>45.92</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>OBEROIRLTY</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>1849</v>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="E15" s="9" t="n">
-        <v>9245</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>1858</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>9290</v>
-      </c>
-      <c r="H15" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="I15" s="11" t="n">
-        <v>0.00486749594375338</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>1765.23</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>1765.23</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>0.04993003229278793</v>
-      </c>
-      <c r="M15" s="13" t="n">
-        <v>45.92</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H15">
+  <conditionalFormatting sqref="H2:H14">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1466,7 +1418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1542,27 +1494,27 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>507</v>
+        <v>1412.6</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>471.54</v>
+        <v>1417.16</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -1570,77 +1522,77 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-638.28</v>
+        <v>13.69</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0699</v>
+        <v>0.0032</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-1</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>8847</v>
+        <v>507</v>
       </c>
       <c r="D3" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="F3" s="15" t="n">
+        <v>471.54</v>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="14" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="F3" s="15" t="n">
-        <v>9240</v>
-      </c>
-      <c r="G3" s="14" t="inlineStr">
-        <is>
-          <t>TIME_STOP</t>
-        </is>
-      </c>
-      <c r="H3" s="14" t="n">
-        <v>25</v>
-      </c>
       <c r="I3" s="17" t="n">
-        <v>393</v>
+        <v>-638.28</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>0.0444</v>
+        <v>-0.0699</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>0.74</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>1948.5</v>
+        <v>8847</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
@@ -1648,50 +1600,50 @@
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>1922.5</v>
+        <v>9240</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-52</v>
+        <v>393</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0133</v>
+        <v>0.0444</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-0.36</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>4568</v>
+        <v>1948.5</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>4460</v>
+        <v>1922.5</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1699,22 +1651,22 @@
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-108</v>
+        <v>-52</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.0236</v>
+        <v>-0.0133</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-0.49</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -1723,10 +1675,10 @@
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>1550</v>
+        <v>4568</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -1734,7 +1686,7 @@
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>1470.07</v>
+        <v>4460</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -1745,19 +1697,19 @@
         <v>10</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>-239.79</v>
+        <v>-108</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>-0.0516</v>
+        <v>-0.0236</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>-0.77</v>
+        <v>-0.49</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -1766,18 +1718,18 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>1713.4</v>
+        <v>1550</v>
       </c>
       <c r="D7" s="16" t="n">
         <v>3</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>1650</v>
+        <v>1470.07</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -1785,34 +1737,34 @@
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>-190.2</v>
+        <v>-239.79</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>-0.037</v>
+        <v>-0.0516</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>-0.65</v>
+        <v>-0.77</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>2360</v>
+        <v>1713.4</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
@@ -1820,7 +1772,7 @@
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>2250.39</v>
+        <v>1650</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -1828,22 +1780,22 @@
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>-548.05</v>
+        <v>-190.2</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>-0.0464</v>
+        <v>-0.037</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>-1</v>
+        <v>-0.65</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -1852,18 +1804,18 @@
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>8945</v>
+        <v>2360</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>8673.639999999999</v>
+        <v>2250.39</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
@@ -1871,13 +1823,13 @@
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>-271.36</v>
+        <v>-548.05</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>-0.0303</v>
+        <v>-0.0464</v>
       </c>
       <c r="K9" s="19" t="n">
         <v>-1</v>
@@ -1886,27 +1838,27 @@
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>2218</v>
+        <v>8945</v>
   